<commit_message>
chore: update snapshots 2026-04-07
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -434,16 +434,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -808,6 +809,386 @@
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="15" customHeight="1">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:39 UTC</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:39 UTC</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:39 UTC</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="15" customHeight="1">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:39 UTC</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:39 UTC</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:39 UTC</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:39 UTC</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:39 UTC</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:39 UTC</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:39 UTC</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -824,32 +1205,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>File</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Last Updated</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Line Count</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -858,18 +1245,23 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>amc.com/ads.txt</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-04-07 18:24 UTC</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:39 UTC</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
         <v>1111</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -878,18 +1270,23 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>amc.com/app-ads.txt</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-04-07 18:24 UTC</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:39 UTC</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
         <v>1022</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -898,18 +1295,23 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>bbca.com/ads.txt</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-04-07 18:24 UTC</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:39 UTC</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
         <v>1111</v>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -918,18 +1320,23 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>bbca.com/app-ads.txt</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-04-07 18:24 UTC</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:39 UTC</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
         <v>1022</v>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -938,18 +1345,23 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>ifc.com/ads.txt</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-04-07 18:24 UTC</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:39 UTC</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
         <v>1111</v>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -958,18 +1370,23 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>ifc.com/app-ads.txt</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-04-07 18:24 UTC</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:39 UTC</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
         <v>1022</v>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -978,18 +1395,23 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>sundancetv.com/ads.txt</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-04-07 18:24 UTC</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:39 UTC</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
         <v>1111</v>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -998,18 +1420,23 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>sundancetv.com/app-ads.txt</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-04-07 18:24 UTC</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:39 UTC</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
         <v>19</v>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -1018,18 +1445,23 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>wetv.com/ads.txt</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2026-04-07 18:24 UTC</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:39 UTC</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
         <v>1111</v>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -1038,18 +1470,23 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>wetv.com/app-ads.txt</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2026-04-07 18:24 UTC</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-04-07 18:39 UTC</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
         <v>1022</v>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
         </is>

</xml_diff>

<commit_message>
chore: update snapshots 2026-04-08
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -8,16 +8,17 @@
   </bookViews>
   <sheets>
     <sheet name="Change Log" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Current Snapshot" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="amc_com_ads_txt" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="amc_com_app-ads_txt" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="bbca_com_ads_txt" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="bbca_com_app-ads_txt" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ifc_com_ads_txt" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="ifc_com_app-ads_txt" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="sundancetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="wetv_com_ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="wetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="amc_com_ads_txt" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="amc_com_app-ads_txt" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="bbca_com_ads_txt" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="bbca_com_app-ads_txt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ifc_com_ads_txt" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ifc_com_app-ads_txt" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -52,7 +53,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -74,6 +75,11 @@
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -87,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -96,6 +102,7 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -461,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H61"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2866,6 +2873,374 @@
 #Xapads: media.net, 8CU406385, RESELLER</t>
         </is>
       </c>
+    </row>
+    <row r="62" ht="15" customHeight="1">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-04-08 10:09 UTC</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>0</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="15" customHeight="1">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-04-08 10:09 UTC</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="15" customHeight="1">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-04-08 10:09 UTC</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="15" customHeight="1">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-04-08 10:09 UTC</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="15" customHeight="1">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-04-08 10:09 UTC</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="15" customHeight="1">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-04-08 10:09 UTC</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="15" customHeight="1">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-04-08 10:09 UTC</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="15" customHeight="1">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-08 10:09 UTC</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F69" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.e41d8e80af8e1fe013af.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.1e4883d8d49bff6089da.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.74920a00d5b66942eb04.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3c96d4aa1f359505e0ae.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.e41d8e80af8e1fe013af.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.1e4883d8d49bff6089da.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.871b8323c49607557945.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3c96d4aa1f359505e0ae.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="15" customHeight="1">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-04-08 10:09 UTC</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="15" customHeight="1">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-08 10:09 UTC</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="inlineStr">
+        <is>
+          <t>Error: HTTPSConnectionPool(host='www.wetv.com', port=443): Read timed out. (read timeout=15)</t>
+        </is>
+      </c>
+      <c r="E71" s="6" t="inlineStr"/>
+      <c r="F71" s="6" t="inlineStr"/>
+      <c r="G71" s="6" t="inlineStr"/>
+      <c r="H71" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3186,7 +3561,307 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Line Count</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-04-08 10:09 UTC</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1127</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-04-08 10:09 UTC</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1040</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-04-08 10:09 UTC</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1127</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-04-08 10:09 UTC</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1040</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-04-08 10:09 UTC</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1127</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-04-08 10:09 UTC</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1040</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-04-08 10:09 UTC</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1127</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-04-08 10:09 UTC</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>19</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-04-08 10:09 UTC</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1127</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-04-08 10:09 UTC</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Error: HTTPSConnectionPool(host='www.wetv.com', port=443): Read timed out. (read timeout=15)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3219,267 +3894,29 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Sonobi</t>
+          <t>(no section)</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>oxiem.com, 7d3ac7564a, DIRECT, d1a215d9eb5aee9e</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.e41d8e80af8e1fe013af.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.1e4883d8d49bff6089da.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.74920a00d5b66942eb04.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3c96d4aa1f359505e0ae.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>#Sonobi</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>oxiem.com, 7d3ac7564a, DIRECT, b7aba0bfd04aa6b6</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>#MyCode</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>connatix.com, 101557, DIRECT, 2af98acdee0e81ed</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>#MyCode</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 166226, RESELLER, 5d62403b186f2ace</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>#MyCode</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 535072-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>#MyCode</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>appnexus.com, 17444, RESELLER, f5ab79cb980f11d1</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>#MyCode</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>themediagrid.com, PCE1BO, RESELLER, 35d5010d7789b49d</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>#MyCode</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>loopme.com, 11186, RESELLER, 6c8d5f95897a5a3b</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>videoheroes.tv, 212796, DIRECT, 064bc410192443d8</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>video.unrulymedia.com, 170071695, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 534963-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>lkqd.net, 1100060074, RESELLER, 59c49fa9598a0117</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>- Removed</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>conversantmedia.com, 100718, RESELLER, 03113cd04947736d</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>safex.tv, 5078, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>media.net, 8CU406385, RESELLER</t>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.e41d8e80af8e1fe013af.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.1e4883d8d49bff6089da.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.871b8323c49607557945.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3c96d4aa1f359505e0ae.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -3494,290 +3931,300 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Partner</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>File</t>
+          <t>Section</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Last Updated</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Line Count</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
+          <t>Line Content</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>AMC Networks</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>amc.com/ads.txt</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2026-04-07 21:33 UTC</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>1127</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>#Sonobi</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>oxiem.com, 7d3ac7564a, DIRECT, d1a215d9eb5aee9e</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>AMC Networks</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>amc.com/app-ads.txt</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2026-04-07 21:33 UTC</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>1040</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>#Sonobi</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>oxiem.com, 7d3ac7564a, DIRECT, b7aba0bfd04aa6b6</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>BBC America</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>bbca.com/ads.txt</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2026-04-07 21:33 UTC</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>1127</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>#MyCode</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>connatix.com, 101557, DIRECT, 2af98acdee0e81ed</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>BBC America</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>bbca.com/app-ads.txt</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2026-04-07 21:33 UTC</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>1040</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>#MyCode</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>pubmatic.com, 166226, RESELLER, 5d62403b186f2ace</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>IFC</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>ifc.com/ads.txt</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>2026-04-07 21:33 UTC</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>1127</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>#MyCode</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 535072-r-524565, RESELLER</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>IFC</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>ifc.com/app-ads.txt</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>2026-04-07 21:33 UTC</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>1040</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>#MyCode</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>appnexus.com, 17444, RESELLER, f5ab79cb980f11d1</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Sundance TV</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>sundancetv.com/ads.txt</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2026-04-07 21:33 UTC</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>1127</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>#MyCode</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>themediagrid.com, PCE1BO, RESELLER, 35d5010d7789b49d</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Sundance TV</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>sundancetv.com/app-ads.txt</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>2026-04-07 21:33 UTC</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>19</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>#MyCode</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>loopme.com, 11186, RESELLER, 6c8d5f95897a5a3b</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>WE tv</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>wetv.com/ads.txt</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>2026-04-07 21:33 UTC</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>1127</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>videoheroes.tv, 212796, DIRECT, 064bc410192443d8</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>WE tv</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>wetv.com/app-ads.txt</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>2026-04-07 21:33 UTC</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>1040</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>video.unrulymedia.com, 170071695, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 534963-r-524565, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>lkqd.net, 1100060074, RESELLER, 59c49fa9598a0117</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>conversantmedia.com, 100718, RESELLER, 03113cd04947736d</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>safex.tv, 5078, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>media.net, 8CU406385, RESELLER</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-04-09
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3617,6 +3617,386 @@
         </is>
       </c>
       <c r="H81" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="15" customHeight="1">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-04-09 10:14 UTC</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>0</v>
+      </c>
+      <c r="F82" t="n">
+        <v>0</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="15" customHeight="1">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-04-09 10:14 UTC</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>0</v>
+      </c>
+      <c r="F83" t="n">
+        <v>0</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="15" customHeight="1">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-04-09 10:14 UTC</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>0</v>
+      </c>
+      <c r="F84" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="15" customHeight="1">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-04-09 10:14 UTC</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>0</v>
+      </c>
+      <c r="F85" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="15" customHeight="1">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-04-09 10:14 UTC</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="15" customHeight="1">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-04-09 10:14 UTC</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>0</v>
+      </c>
+      <c r="F87" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="15" customHeight="1">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-04-09 10:14 UTC</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>0</v>
+      </c>
+      <c r="F88" t="n">
+        <v>0</v>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="15" customHeight="1">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-09 10:14 UTC</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F89" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G89" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.1ee2046668ca9007aca9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.ade6382deac3f393ccbf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.64bc1e17cca094288e2f.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H89" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.e41d8e80af8e1fe013af.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.1e4883d8d49bff6089da.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.95e2e36a83a7a8a8d971.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="15" customHeight="1">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-04-09 10:14 UTC</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>0</v>
+      </c>
+      <c r="F90" t="n">
+        <v>0</v>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="15" customHeight="1">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-04-09 10:14 UTC</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>0</v>
+      </c>
+      <c r="F91" t="n">
+        <v>0</v>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3991,7 +4371,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-08 14:45 UTC</t>
+          <t>2026-04-09 10:14 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -4016,7 +4396,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-04-08 14:45 UTC</t>
+          <t>2026-04-09 10:14 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -4041,7 +4421,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-04-08 14:45 UTC</t>
+          <t>2026-04-09 10:14 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -4066,7 +4446,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-08 14:45 UTC</t>
+          <t>2026-04-09 10:14 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -4091,7 +4471,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-04-08 14:45 UTC</t>
+          <t>2026-04-09 10:14 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -4116,7 +4496,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-04-08 14:45 UTC</t>
+          <t>2026-04-09 10:14 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -4141,7 +4521,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-04-08 14:45 UTC</t>
+          <t>2026-04-09 10:14 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -4166,7 +4546,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-04-08 14:45 UTC</t>
+          <t>2026-04-09 10:14 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -4191,7 +4571,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-08 14:45 UTC</t>
+          <t>2026-04-09 10:14 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -4216,7 +4596,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-08 14:45 UTC</t>
+          <t>2026-04-09 10:14 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -4277,7 +4657,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.e41d8e80af8e1fe013af.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.1e4883d8d49bff6089da.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.95e2e36a83a7a8a8d971.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.1ee2046668ca9007aca9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.ade6382deac3f393ccbf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.64bc1e17cca094288e2f.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -4294,7 +4674,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.e41d8e80af8e1fe013af.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.1e4883d8d49bff6089da.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.74920a00d5b66942eb04.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3c96d4aa1f359505e0ae.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.e41d8e80af8e1fe013af.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.1e4883d8d49bff6089da.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.95e2e36a83a7a8a8d971.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-04-10
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H101"/>
+  <dimension ref="A1:H111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4377,6 +4377,386 @@
         </is>
       </c>
       <c r="H101" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="15" customHeight="1">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-04-10 10:08 UTC</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>0</v>
+      </c>
+      <c r="F102" t="n">
+        <v>0</v>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="15" customHeight="1">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-04-10 10:08 UTC</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>0</v>
+      </c>
+      <c r="F103" t="n">
+        <v>0</v>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="15" customHeight="1">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-04-10 10:08 UTC</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>0</v>
+      </c>
+      <c r="F104" t="n">
+        <v>0</v>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="15" customHeight="1">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-04-10 10:08 UTC</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>0</v>
+      </c>
+      <c r="F105" t="n">
+        <v>0</v>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="15" customHeight="1">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-04-10 10:08 UTC</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F106" t="n">
+        <v>0</v>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="15" customHeight="1">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-04-10 10:08 UTC</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>0</v>
+      </c>
+      <c r="F107" t="n">
+        <v>0</v>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="15" customHeight="1">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-04-10 10:08 UTC</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>0</v>
+      </c>
+      <c r="F108" t="n">
+        <v>0</v>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="15" customHeight="1">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-10 10:08 UTC</t>
+        </is>
+      </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E109" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F109" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G109" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.1ee2046668ca9007aca9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.ade6382deac3f393ccbf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.c8a0bdaecce7501db5c5.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H109" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.1ee2046668ca9007aca9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.ade6382deac3f393ccbf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.61ff6ab92cfea372a5a8.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="15" customHeight="1">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-04-10 10:08 UTC</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E110" t="n">
+        <v>0</v>
+      </c>
+      <c r="F110" t="n">
+        <v>0</v>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="15" customHeight="1">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-04-10 10:08 UTC</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>0</v>
+      </c>
+      <c r="F111" t="n">
+        <v>0</v>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4751,7 +5131,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-09 12:20 UTC</t>
+          <t>2026-04-10 10:08 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -4776,7 +5156,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-04-09 12:20 UTC</t>
+          <t>2026-04-10 10:08 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -4801,7 +5181,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-04-09 12:20 UTC</t>
+          <t>2026-04-10 10:08 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -4826,7 +5206,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-09 12:20 UTC</t>
+          <t>2026-04-10 10:08 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -4851,7 +5231,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-04-09 12:20 UTC</t>
+          <t>2026-04-10 10:08 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -4876,7 +5256,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-04-09 12:20 UTC</t>
+          <t>2026-04-10 10:08 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -4901,7 +5281,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-04-09 12:20 UTC</t>
+          <t>2026-04-10 10:08 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -4926,7 +5306,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-04-09 12:20 UTC</t>
+          <t>2026-04-10 10:08 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -4951,7 +5331,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-09 12:20 UTC</t>
+          <t>2026-04-10 10:08 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -4976,7 +5356,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-09 12:20 UTC</t>
+          <t>2026-04-10 10:08 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -5037,7 +5417,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.1ee2046668ca9007aca9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.ade6382deac3f393ccbf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.61ff6ab92cfea372a5a8.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.1ee2046668ca9007aca9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.ade6382deac3f393ccbf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.c8a0bdaecce7501db5c5.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -5054,7 +5434,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.1ee2046668ca9007aca9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.ade6382deac3f393ccbf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.64bc1e17cca094288e2f.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.1ee2046668ca9007aca9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.ade6382deac3f393ccbf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.61ff6ab92cfea372a5a8.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-04-11
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H111"/>
+  <dimension ref="A1:H121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4757,6 +4757,386 @@
         </is>
       </c>
       <c r="H111" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="15" customHeight="1">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-04-11 09:42 UTC</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>0</v>
+      </c>
+      <c r="F112" t="n">
+        <v>0</v>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="15" customHeight="1">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-04-11 09:42 UTC</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>0</v>
+      </c>
+      <c r="F113" t="n">
+        <v>0</v>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="15" customHeight="1">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-04-11 09:42 UTC</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>0</v>
+      </c>
+      <c r="F114" t="n">
+        <v>0</v>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="15" customHeight="1">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-04-11 09:42 UTC</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E115" t="n">
+        <v>0</v>
+      </c>
+      <c r="F115" t="n">
+        <v>0</v>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="15" customHeight="1">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-04-11 09:42 UTC</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>0</v>
+      </c>
+      <c r="F116" t="n">
+        <v>0</v>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="15" customHeight="1">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-04-11 09:42 UTC</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E117" t="n">
+        <v>0</v>
+      </c>
+      <c r="F117" t="n">
+        <v>0</v>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="15" customHeight="1">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-04-11 09:42 UTC</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>0</v>
+      </c>
+      <c r="F118" t="n">
+        <v>0</v>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="15" customHeight="1">
+      <c r="A119" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-11 09:42 UTC</t>
+        </is>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D119" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E119" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F119" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G119" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.1ee2046668ca9007aca9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.fa2cb02e63563e8675d3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.784bd1e03285776dc597.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H119" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.1ee2046668ca9007aca9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.ade6382deac3f393ccbf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.c8a0bdaecce7501db5c5.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="15" customHeight="1">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-04-11 09:42 UTC</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E120" t="n">
+        <v>0</v>
+      </c>
+      <c r="F120" t="n">
+        <v>0</v>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="15" customHeight="1">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-04-11 09:42 UTC</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E121" t="n">
+        <v>0</v>
+      </c>
+      <c r="F121" t="n">
+        <v>0</v>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5131,7 +5511,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-10 10:08 UTC</t>
+          <t>2026-04-11 09:42 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -5156,7 +5536,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-04-10 10:08 UTC</t>
+          <t>2026-04-11 09:42 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -5181,7 +5561,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-04-10 10:08 UTC</t>
+          <t>2026-04-11 09:42 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -5206,7 +5586,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-10 10:08 UTC</t>
+          <t>2026-04-11 09:42 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -5231,7 +5611,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-04-10 10:08 UTC</t>
+          <t>2026-04-11 09:42 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -5256,7 +5636,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-04-10 10:08 UTC</t>
+          <t>2026-04-11 09:42 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -5281,7 +5661,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-04-10 10:08 UTC</t>
+          <t>2026-04-11 09:42 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -5306,7 +5686,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-04-10 10:08 UTC</t>
+          <t>2026-04-11 09:42 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -5331,7 +5711,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-10 10:08 UTC</t>
+          <t>2026-04-11 09:42 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -5356,7 +5736,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-10 10:08 UTC</t>
+          <t>2026-04-11 09:42 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -5417,7 +5797,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.1ee2046668ca9007aca9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.ade6382deac3f393ccbf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.c8a0bdaecce7501db5c5.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.1ee2046668ca9007aca9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.fa2cb02e63563e8675d3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.784bd1e03285776dc597.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -5434,7 +5814,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.1ee2046668ca9007aca9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.ade6382deac3f393ccbf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.61ff6ab92cfea372a5a8.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.1ee2046668ca9007aca9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.ade6382deac3f393ccbf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.c8a0bdaecce7501db5c5.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-04-12
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H121"/>
+  <dimension ref="A1:H131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5137,6 +5137,386 @@
         </is>
       </c>
       <c r="H121" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="15" customHeight="1">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-04-12 09:48 UTC</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E122" t="n">
+        <v>0</v>
+      </c>
+      <c r="F122" t="n">
+        <v>0</v>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="15" customHeight="1">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-04-12 09:48 UTC</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E123" t="n">
+        <v>0</v>
+      </c>
+      <c r="F123" t="n">
+        <v>0</v>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="15" customHeight="1">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-04-12 09:48 UTC</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E124" t="n">
+        <v>0</v>
+      </c>
+      <c r="F124" t="n">
+        <v>0</v>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="15" customHeight="1">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-04-12 09:48 UTC</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E125" t="n">
+        <v>0</v>
+      </c>
+      <c r="F125" t="n">
+        <v>0</v>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="15" customHeight="1">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-04-12 09:48 UTC</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>0</v>
+      </c>
+      <c r="F126" t="n">
+        <v>0</v>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="15" customHeight="1">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-04-12 09:48 UTC</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>0</v>
+      </c>
+      <c r="F127" t="n">
+        <v>0</v>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="15" customHeight="1">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-04-12 09:48 UTC</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>0</v>
+      </c>
+      <c r="F128" t="n">
+        <v>0</v>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="15" customHeight="1">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-04-12 09:48 UTC</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>0</v>
+      </c>
+      <c r="F129" t="n">
+        <v>0</v>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="15" customHeight="1">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-04-12 09:48 UTC</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>0</v>
+      </c>
+      <c r="F130" t="n">
+        <v>0</v>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="15" customHeight="1">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-04-12 09:48 UTC</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>0</v>
+      </c>
+      <c r="F131" t="n">
+        <v>0</v>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5461,6 +5841,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.1ee2046668ca9007aca9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.fa2cb02e63563e8675d3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.784bd1e03285776dc597.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.1ee2046668ca9007aca9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.ade6382deac3f393ccbf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.c8a0bdaecce7501db5c5.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5511,7 +5961,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-11 09:42 UTC</t>
+          <t>2026-04-12 09:48 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -5536,7 +5986,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-04-11 09:42 UTC</t>
+          <t>2026-04-12 09:48 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -5561,7 +6011,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-04-11 09:42 UTC</t>
+          <t>2026-04-12 09:48 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -5586,7 +6036,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-11 09:42 UTC</t>
+          <t>2026-04-12 09:48 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -5611,7 +6061,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-04-11 09:42 UTC</t>
+          <t>2026-04-12 09:48 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -5636,7 +6086,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-04-11 09:42 UTC</t>
+          <t>2026-04-12 09:48 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -5661,7 +6111,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-04-11 09:42 UTC</t>
+          <t>2026-04-12 09:48 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -5686,7 +6136,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-04-11 09:42 UTC</t>
+          <t>2026-04-12 09:48 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -5711,7 +6161,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-11 09:42 UTC</t>
+          <t>2026-04-12 09:48 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -5736,7 +6186,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-11 09:42 UTC</t>
+          <t>2026-04-12 09:48 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -5745,76 +6195,6 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.1ee2046668ca9007aca9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.fa2cb02e63563e8675d3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.784bd1e03285776dc597.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.1ee2046668ca9007aca9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.ade6382deac3f393ccbf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.c8a0bdaecce7501db5c5.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-04-13
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H131"/>
+  <dimension ref="A1:H141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5517,6 +5517,386 @@
         </is>
       </c>
       <c r="H131" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="15" customHeight="1">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-04-13 10:48 UTC</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>0</v>
+      </c>
+      <c r="F132" t="n">
+        <v>0</v>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="15" customHeight="1">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-04-13 10:48 UTC</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>0</v>
+      </c>
+      <c r="F133" t="n">
+        <v>0</v>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="15" customHeight="1">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-04-13 10:48 UTC</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>0</v>
+      </c>
+      <c r="F134" t="n">
+        <v>0</v>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="15" customHeight="1">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-04-13 10:48 UTC</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>0</v>
+      </c>
+      <c r="F135" t="n">
+        <v>0</v>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="15" customHeight="1">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-04-13 10:48 UTC</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E136" t="n">
+        <v>0</v>
+      </c>
+      <c r="F136" t="n">
+        <v>0</v>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="15" customHeight="1">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-04-13 10:48 UTC</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E137" t="n">
+        <v>0</v>
+      </c>
+      <c r="F137" t="n">
+        <v>0</v>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="15" customHeight="1">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-04-13 10:48 UTC</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E138" t="n">
+        <v>0</v>
+      </c>
+      <c r="F138" t="n">
+        <v>0</v>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="15" customHeight="1">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-04-13 10:48 UTC</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E139" t="n">
+        <v>0</v>
+      </c>
+      <c r="F139" t="n">
+        <v>0</v>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="15" customHeight="1">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-04-13 10:48 UTC</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E140" t="n">
+        <v>0</v>
+      </c>
+      <c r="F140" t="n">
+        <v>0</v>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="15" customHeight="1">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-04-13 10:48 UTC</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E141" t="n">
+        <v>0</v>
+      </c>
+      <c r="F141" t="n">
+        <v>0</v>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5961,7 +6341,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-12 09:48 UTC</t>
+          <t>2026-04-13 10:48 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -5986,7 +6366,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-04-12 09:48 UTC</t>
+          <t>2026-04-13 10:48 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -6011,7 +6391,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-04-12 09:48 UTC</t>
+          <t>2026-04-13 10:48 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -6036,7 +6416,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-12 09:48 UTC</t>
+          <t>2026-04-13 10:48 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -6061,7 +6441,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-04-12 09:48 UTC</t>
+          <t>2026-04-13 10:48 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -6086,7 +6466,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-04-12 09:48 UTC</t>
+          <t>2026-04-13 10:48 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -6111,7 +6491,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-04-12 09:48 UTC</t>
+          <t>2026-04-13 10:48 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -6136,7 +6516,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-04-12 09:48 UTC</t>
+          <t>2026-04-13 10:48 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -6161,7 +6541,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-12 09:48 UTC</t>
+          <t>2026-04-13 10:48 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -6186,7 +6566,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-12 09:48 UTC</t>
+          <t>2026-04-13 10:48 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">

</xml_diff>

<commit_message>
chore: update snapshots 2026-04-14
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H141"/>
+  <dimension ref="A1:H151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -5897,6 +5897,386 @@
         </is>
       </c>
       <c r="H141" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="15" customHeight="1">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-04-14 10:16 UTC</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E142" t="n">
+        <v>0</v>
+      </c>
+      <c r="F142" t="n">
+        <v>0</v>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="15" customHeight="1">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-04-14 10:16 UTC</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>0</v>
+      </c>
+      <c r="F143" t="n">
+        <v>0</v>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="15" customHeight="1">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-04-14 10:16 UTC</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E144" t="n">
+        <v>0</v>
+      </c>
+      <c r="F144" t="n">
+        <v>0</v>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="15" customHeight="1">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-04-14 10:16 UTC</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E145" t="n">
+        <v>0</v>
+      </c>
+      <c r="F145" t="n">
+        <v>0</v>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="15" customHeight="1">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-04-14 10:16 UTC</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>0</v>
+      </c>
+      <c r="F146" t="n">
+        <v>0</v>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="15" customHeight="1">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-04-14 10:16 UTC</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>0</v>
+      </c>
+      <c r="F147" t="n">
+        <v>0</v>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="15" customHeight="1">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-04-14 10:16 UTC</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>0</v>
+      </c>
+      <c r="F148" t="n">
+        <v>0</v>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="15" customHeight="1">
+      <c r="A149" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-14 10:16 UTC</t>
+        </is>
+      </c>
+      <c r="B149" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C149" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D149" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E149" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F149" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G149" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.c421acb53eb153fcd99b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.eac6f59c7f9ed48b5640.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.36503702c27564dd1876.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.8865d79e3145093956d2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.b7333e46c13cdfe0d523.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H149" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.1ee2046668ca9007aca9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.fa2cb02e63563e8675d3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.784bd1e03285776dc597.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="15" customHeight="1">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-04-14 10:16 UTC</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E150" t="n">
+        <v>0</v>
+      </c>
+      <c r="F150" t="n">
+        <v>0</v>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="15" customHeight="1">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-04-14 10:16 UTC</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E151" t="n">
+        <v>0</v>
+      </c>
+      <c r="F151" t="n">
+        <v>0</v>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -6221,76 +6601,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.1ee2046668ca9007aca9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.fa2cb02e63563e8675d3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.784bd1e03285776dc597.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.1ee2046668ca9007aca9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.ade6382deac3f393ccbf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.c8a0bdaecce7501db5c5.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6341,7 +6651,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-13 10:48 UTC</t>
+          <t>2026-04-14 10:16 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -6366,7 +6676,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-04-13 10:48 UTC</t>
+          <t>2026-04-14 10:16 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -6391,7 +6701,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-04-13 10:48 UTC</t>
+          <t>2026-04-14 10:16 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -6416,7 +6726,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-13 10:48 UTC</t>
+          <t>2026-04-14 10:16 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -6441,7 +6751,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-04-13 10:48 UTC</t>
+          <t>2026-04-14 10:16 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -6466,7 +6776,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-04-13 10:48 UTC</t>
+          <t>2026-04-14 10:16 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -6491,7 +6801,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-04-13 10:48 UTC</t>
+          <t>2026-04-14 10:16 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -6516,7 +6826,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-04-13 10:48 UTC</t>
+          <t>2026-04-14 10:16 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -6541,7 +6851,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-13 10:48 UTC</t>
+          <t>2026-04-14 10:16 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -6566,7 +6876,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-13 10:48 UTC</t>
+          <t>2026-04-14 10:16 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -6575,6 +6885,76 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.c421acb53eb153fcd99b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.eac6f59c7f9ed48b5640.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.36503702c27564dd1876.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.8865d79e3145093956d2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.b7333e46c13cdfe0d523.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.1ee2046668ca9007aca9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.fa2cb02e63563e8675d3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.784bd1e03285776dc597.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-04-15
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H151"/>
+  <dimension ref="A1:H161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -6277,6 +6277,386 @@
         </is>
       </c>
       <c r="H151" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="15" customHeight="1">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-04-15 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E152" t="n">
+        <v>0</v>
+      </c>
+      <c r="F152" t="n">
+        <v>0</v>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="15" customHeight="1">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>2026-04-15 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E153" t="n">
+        <v>0</v>
+      </c>
+      <c r="F153" t="n">
+        <v>0</v>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="15" customHeight="1">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>2026-04-15 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E154" t="n">
+        <v>0</v>
+      </c>
+      <c r="F154" t="n">
+        <v>0</v>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="15" customHeight="1">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>2026-04-15 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E155" t="n">
+        <v>0</v>
+      </c>
+      <c r="F155" t="n">
+        <v>0</v>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="15" customHeight="1">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2026-04-15 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E156" t="n">
+        <v>0</v>
+      </c>
+      <c r="F156" t="n">
+        <v>0</v>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="15" customHeight="1">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>2026-04-15 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E157" t="n">
+        <v>0</v>
+      </c>
+      <c r="F157" t="n">
+        <v>0</v>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" ht="15" customHeight="1">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>2026-04-15 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E158" t="n">
+        <v>0</v>
+      </c>
+      <c r="F158" t="n">
+        <v>0</v>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" ht="15" customHeight="1">
+      <c r="A159" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-15 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B159" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C159" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D159" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E159" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F159" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G159" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.07ce253117f319a04257.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.5181f866c94bfef28c47.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.b8cbd5b0e9bffb44dbb6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7c91461537dc955217af.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.0a957cbed93cf36c985d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H159" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.c421acb53eb153fcd99b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.eac6f59c7f9ed48b5640.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.36503702c27564dd1876.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.8865d79e3145093956d2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.b7333e46c13cdfe0d523.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="15" customHeight="1">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>2026-04-15 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E160" t="n">
+        <v>0</v>
+      </c>
+      <c r="F160" t="n">
+        <v>0</v>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" ht="15" customHeight="1">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>2026-04-15 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E161" t="n">
+        <v>0</v>
+      </c>
+      <c r="F161" t="n">
+        <v>0</v>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -6651,7 +7031,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-14 10:16 UTC</t>
+          <t>2026-04-15 10:17 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -6676,7 +7056,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-04-14 10:16 UTC</t>
+          <t>2026-04-15 10:17 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -6701,7 +7081,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-04-14 10:16 UTC</t>
+          <t>2026-04-15 10:17 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -6726,7 +7106,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-14 10:16 UTC</t>
+          <t>2026-04-15 10:17 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -6751,7 +7131,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-04-14 10:16 UTC</t>
+          <t>2026-04-15 10:17 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -6776,7 +7156,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-04-14 10:16 UTC</t>
+          <t>2026-04-15 10:17 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -6801,7 +7181,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-04-14 10:16 UTC</t>
+          <t>2026-04-15 10:17 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -6826,7 +7206,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-04-14 10:16 UTC</t>
+          <t>2026-04-15 10:17 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -6851,7 +7231,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-14 10:16 UTC</t>
+          <t>2026-04-15 10:17 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -6876,7 +7256,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-14 10:16 UTC</t>
+          <t>2026-04-15 10:17 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -6937,7 +7317,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.c421acb53eb153fcd99b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.eac6f59c7f9ed48b5640.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.36503702c27564dd1876.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.8865d79e3145093956d2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.b7333e46c13cdfe0d523.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.07ce253117f319a04257.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.5181f866c94bfef28c47.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.b8cbd5b0e9bffb44dbb6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7c91461537dc955217af.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.0a957cbed93cf36c985d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -6954,7 +7334,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.1ee2046668ca9007aca9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.d276055840356a4c6779.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c72dfebc62e768e3c2ba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.fa2cb02e63563e8675d3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.784bd1e03285776dc597.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4766.50337c2ffca49f286ae2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9851.c421acb53eb153fcd99b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8502.eac6f59c7f9ed48b5640.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.36503702c27564dd1876.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/3319.8865d79e3145093956d2.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.b7333e46c13cdfe0d523.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9851.374c2a76e4002104c6b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/3319.622d7009bd006d474e0e.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-04-16
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H171"/>
+  <dimension ref="A1:H181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -7037,6 +7037,386 @@
         </is>
       </c>
       <c r="H171" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" ht="15" customHeight="1">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>2026-04-16 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E172" t="n">
+        <v>0</v>
+      </c>
+      <c r="F172" t="n">
+        <v>0</v>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="173" ht="15" customHeight="1">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>2026-04-16 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E173" t="n">
+        <v>0</v>
+      </c>
+      <c r="F173" t="n">
+        <v>0</v>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="174" ht="15" customHeight="1">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>2026-04-16 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E174" t="n">
+        <v>0</v>
+      </c>
+      <c r="F174" t="n">
+        <v>0</v>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="175" ht="15" customHeight="1">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>2026-04-16 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E175" t="n">
+        <v>0</v>
+      </c>
+      <c r="F175" t="n">
+        <v>0</v>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="176" ht="15" customHeight="1">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>2026-04-16 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E176" t="n">
+        <v>0</v>
+      </c>
+      <c r="F176" t="n">
+        <v>0</v>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="177" ht="15" customHeight="1">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>2026-04-16 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E177" t="n">
+        <v>0</v>
+      </c>
+      <c r="F177" t="n">
+        <v>0</v>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="178" ht="15" customHeight="1">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>2026-04-16 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E178" t="n">
+        <v>0</v>
+      </c>
+      <c r="F178" t="n">
+        <v>0</v>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="179" ht="15" customHeight="1">
+      <c r="A179" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-16 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B179" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C179" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D179" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E179" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F179" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G179" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.f3bd1b5b095bb64711ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.5f8f57924d402881318d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3978fb6ce2deb4c39aa0.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H179" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.f3bd1b5b095bb64711ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f436ea78c738b6e75306.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3978fb6ce2deb4c39aa0.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" ht="15" customHeight="1">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>2026-04-16 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E180" t="n">
+        <v>0</v>
+      </c>
+      <c r="F180" t="n">
+        <v>0</v>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="181" ht="15" customHeight="1">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>2026-04-16 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E181" t="n">
+        <v>0</v>
+      </c>
+      <c r="F181" t="n">
+        <v>0</v>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -7411,7 +7791,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-15 18:51 UTC</t>
+          <t>2026-04-16 10:17 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -7436,7 +7816,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-04-15 18:51 UTC</t>
+          <t>2026-04-16 10:17 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -7461,7 +7841,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-04-15 18:51 UTC</t>
+          <t>2026-04-16 10:17 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -7486,7 +7866,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-15 18:51 UTC</t>
+          <t>2026-04-16 10:17 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -7511,7 +7891,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-04-15 18:51 UTC</t>
+          <t>2026-04-16 10:17 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -7536,7 +7916,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-04-15 18:51 UTC</t>
+          <t>2026-04-16 10:17 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -7561,7 +7941,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-04-15 18:51 UTC</t>
+          <t>2026-04-16 10:17 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -7586,7 +7966,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-04-15 18:51 UTC</t>
+          <t>2026-04-16 10:17 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -7611,7 +7991,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-15 18:51 UTC</t>
+          <t>2026-04-16 10:17 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -7636,7 +8016,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-15 18:51 UTC</t>
+          <t>2026-04-16 10:17 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -7697,7 +8077,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.f3bd1b5b095bb64711ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f436ea78c738b6e75306.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3978fb6ce2deb4c39aa0.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.f3bd1b5b095bb64711ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.5f8f57924d402881318d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3978fb6ce2deb4c39aa0.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -7714,7 +8094,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.07ce253117f319a04257.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.5181f866c94bfef28c47.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.b8cbd5b0e9bffb44dbb6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7c91461537dc955217af.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.0a957cbed93cf36c985d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.13b7645709c4445d6063.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.f3bd1b5b095bb64711ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f436ea78c738b6e75306.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3978fb6ce2deb4c39aa0.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-04-17
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H181"/>
+  <dimension ref="A1:H191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -7417,6 +7417,386 @@
         </is>
       </c>
       <c r="H181" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="182" ht="15" customHeight="1">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>2026-04-17 10:15 UTC</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E182" t="n">
+        <v>0</v>
+      </c>
+      <c r="F182" t="n">
+        <v>0</v>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="183" ht="15" customHeight="1">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>2026-04-17 10:15 UTC</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E183" t="n">
+        <v>0</v>
+      </c>
+      <c r="F183" t="n">
+        <v>0</v>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="184" ht="15" customHeight="1">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>2026-04-17 10:15 UTC</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E184" t="n">
+        <v>0</v>
+      </c>
+      <c r="F184" t="n">
+        <v>0</v>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="185" ht="15" customHeight="1">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>2026-04-17 10:15 UTC</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E185" t="n">
+        <v>0</v>
+      </c>
+      <c r="F185" t="n">
+        <v>0</v>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="186" ht="15" customHeight="1">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>2026-04-17 10:15 UTC</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E186" t="n">
+        <v>0</v>
+      </c>
+      <c r="F186" t="n">
+        <v>0</v>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="187" ht="15" customHeight="1">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>2026-04-17 10:15 UTC</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E187" t="n">
+        <v>0</v>
+      </c>
+      <c r="F187" t="n">
+        <v>0</v>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="188" ht="15" customHeight="1">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>2026-04-17 10:15 UTC</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E188" t="n">
+        <v>0</v>
+      </c>
+      <c r="F188" t="n">
+        <v>0</v>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="189" ht="15" customHeight="1">
+      <c r="A189" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-17 10:15 UTC</t>
+        </is>
+      </c>
+      <c r="B189" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C189" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D189" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E189" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F189" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G189" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.f3bd1b5b095bb64711ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.a198328c15c6d468eaf3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3978fb6ce2deb4c39aa0.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H189" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.f3bd1b5b095bb64711ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.5f8f57924d402881318d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3978fb6ce2deb4c39aa0.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="190" ht="15" customHeight="1">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>2026-04-17 10:15 UTC</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E190" t="n">
+        <v>0</v>
+      </c>
+      <c r="F190" t="n">
+        <v>0</v>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" ht="15" customHeight="1">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>2026-04-17 10:15 UTC</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E191" t="n">
+        <v>0</v>
+      </c>
+      <c r="F191" t="n">
+        <v>0</v>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -7791,7 +8171,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-16 10:17 UTC</t>
+          <t>2026-04-17 10:15 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -7816,7 +8196,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-04-16 10:17 UTC</t>
+          <t>2026-04-17 10:15 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -7841,7 +8221,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-04-16 10:17 UTC</t>
+          <t>2026-04-17 10:15 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -7866,7 +8246,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-16 10:17 UTC</t>
+          <t>2026-04-17 10:15 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -7891,7 +8271,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-04-16 10:17 UTC</t>
+          <t>2026-04-17 10:15 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -7916,7 +8296,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-04-16 10:17 UTC</t>
+          <t>2026-04-17 10:15 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -7941,7 +8321,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-04-16 10:17 UTC</t>
+          <t>2026-04-17 10:15 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -7966,7 +8346,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-04-16 10:17 UTC</t>
+          <t>2026-04-17 10:15 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -7991,7 +8371,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-16 10:17 UTC</t>
+          <t>2026-04-17 10:15 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -8016,7 +8396,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-16 10:17 UTC</t>
+          <t>2026-04-17 10:15 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -8077,7 +8457,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.f3bd1b5b095bb64711ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.5f8f57924d402881318d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3978fb6ce2deb4c39aa0.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.f3bd1b5b095bb64711ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.a198328c15c6d468eaf3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3978fb6ce2deb4c39aa0.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -8094,7 +8474,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.f3bd1b5b095bb64711ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f436ea78c738b6e75306.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3978fb6ce2deb4c39aa0.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.f3bd1b5b095bb64711ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.5f8f57924d402881318d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3978fb6ce2deb4c39aa0.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-04-18
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H191"/>
+  <dimension ref="A1:H201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -7797,6 +7797,386 @@
         </is>
       </c>
       <c r="H191" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="192" ht="15" customHeight="1">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>2026-04-18 09:50 UTC</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E192" t="n">
+        <v>0</v>
+      </c>
+      <c r="F192" t="n">
+        <v>0</v>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="193" ht="15" customHeight="1">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>2026-04-18 09:50 UTC</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E193" t="n">
+        <v>0</v>
+      </c>
+      <c r="F193" t="n">
+        <v>0</v>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" ht="15" customHeight="1">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>2026-04-18 09:50 UTC</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E194" t="n">
+        <v>0</v>
+      </c>
+      <c r="F194" t="n">
+        <v>0</v>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="195" ht="15" customHeight="1">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>2026-04-18 09:50 UTC</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E195" t="n">
+        <v>0</v>
+      </c>
+      <c r="F195" t="n">
+        <v>0</v>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="196" ht="15" customHeight="1">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>2026-04-18 09:50 UTC</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E196" t="n">
+        <v>0</v>
+      </c>
+      <c r="F196" t="n">
+        <v>0</v>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="197" ht="15" customHeight="1">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>2026-04-18 09:50 UTC</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E197" t="n">
+        <v>0</v>
+      </c>
+      <c r="F197" t="n">
+        <v>0</v>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="198" ht="15" customHeight="1">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>2026-04-18 09:50 UTC</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E198" t="n">
+        <v>0</v>
+      </c>
+      <c r="F198" t="n">
+        <v>0</v>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="199" ht="15" customHeight="1">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2026-04-18 09:50 UTC</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E199" t="n">
+        <v>0</v>
+      </c>
+      <c r="F199" t="n">
+        <v>0</v>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="200" ht="15" customHeight="1">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2026-04-18 09:50 UTC</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E200" t="n">
+        <v>0</v>
+      </c>
+      <c r="F200" t="n">
+        <v>0</v>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="201" ht="15" customHeight="1">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2026-04-18 09:50 UTC</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E201" t="n">
+        <v>0</v>
+      </c>
+      <c r="F201" t="n">
+        <v>0</v>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -8121,6 +8501,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.f3bd1b5b095bb64711ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.a198328c15c6d468eaf3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3978fb6ce2deb4c39aa0.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.f3bd1b5b095bb64711ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.5f8f57924d402881318d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3978fb6ce2deb4c39aa0.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -8171,7 +8621,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-17 10:15 UTC</t>
+          <t>2026-04-18 09:50 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -8196,7 +8646,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-04-17 10:15 UTC</t>
+          <t>2026-04-18 09:50 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -8221,7 +8671,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-04-17 10:15 UTC</t>
+          <t>2026-04-18 09:50 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -8246,7 +8696,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-17 10:15 UTC</t>
+          <t>2026-04-18 09:50 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -8271,7 +8721,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-04-17 10:15 UTC</t>
+          <t>2026-04-18 09:50 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -8296,7 +8746,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-04-17 10:15 UTC</t>
+          <t>2026-04-18 09:50 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -8321,7 +8771,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-04-17 10:15 UTC</t>
+          <t>2026-04-18 09:50 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -8346,7 +8796,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-04-17 10:15 UTC</t>
+          <t>2026-04-18 09:50 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -8371,7 +8821,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-17 10:15 UTC</t>
+          <t>2026-04-18 09:50 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -8396,7 +8846,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-17 10:15 UTC</t>
+          <t>2026-04-18 09:50 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -8405,76 +8855,6 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.f3bd1b5b095bb64711ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.a198328c15c6d468eaf3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3978fb6ce2deb4c39aa0.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.f3bd1b5b095bb64711ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.5f8f57924d402881318d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3978fb6ce2deb4c39aa0.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-04-19
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H201"/>
+  <dimension ref="A1:H211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -8177,6 +8177,386 @@
         </is>
       </c>
       <c r="H201" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="202" ht="15" customHeight="1">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>2026-04-19 09:49 UTC</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E202" t="n">
+        <v>0</v>
+      </c>
+      <c r="F202" t="n">
+        <v>0</v>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="203" ht="15" customHeight="1">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2026-04-19 09:49 UTC</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E203" t="n">
+        <v>0</v>
+      </c>
+      <c r="F203" t="n">
+        <v>0</v>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="204" ht="15" customHeight="1">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>2026-04-19 09:49 UTC</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E204" t="n">
+        <v>0</v>
+      </c>
+      <c r="F204" t="n">
+        <v>0</v>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="205" ht="15" customHeight="1">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2026-04-19 09:49 UTC</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E205" t="n">
+        <v>0</v>
+      </c>
+      <c r="F205" t="n">
+        <v>0</v>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="206" ht="15" customHeight="1">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2026-04-19 09:49 UTC</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E206" t="n">
+        <v>0</v>
+      </c>
+      <c r="F206" t="n">
+        <v>0</v>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="207" ht="15" customHeight="1">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2026-04-19 09:49 UTC</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E207" t="n">
+        <v>0</v>
+      </c>
+      <c r="F207" t="n">
+        <v>0</v>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="208" ht="15" customHeight="1">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2026-04-19 09:49 UTC</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E208" t="n">
+        <v>0</v>
+      </c>
+      <c r="F208" t="n">
+        <v>0</v>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="209" ht="15" customHeight="1">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2026-04-19 09:49 UTC</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E209" t="n">
+        <v>0</v>
+      </c>
+      <c r="F209" t="n">
+        <v>0</v>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="210" ht="15" customHeight="1">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2026-04-19 09:49 UTC</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E210" t="n">
+        <v>0</v>
+      </c>
+      <c r="F210" t="n">
+        <v>0</v>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="211" ht="15" customHeight="1">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>2026-04-19 09:49 UTC</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E211" t="n">
+        <v>0</v>
+      </c>
+      <c r="F211" t="n">
+        <v>0</v>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -8621,7 +9001,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-18 09:50 UTC</t>
+          <t>2026-04-19 09:49 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -8646,7 +9026,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-04-18 09:50 UTC</t>
+          <t>2026-04-19 09:49 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -8671,7 +9051,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-04-18 09:50 UTC</t>
+          <t>2026-04-19 09:49 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -8696,7 +9076,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-18 09:50 UTC</t>
+          <t>2026-04-19 09:49 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -8721,7 +9101,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-04-18 09:50 UTC</t>
+          <t>2026-04-19 09:49 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -8746,7 +9126,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-04-18 09:50 UTC</t>
+          <t>2026-04-19 09:49 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -8771,7 +9151,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-04-18 09:50 UTC</t>
+          <t>2026-04-19 09:49 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -8796,7 +9176,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-04-18 09:50 UTC</t>
+          <t>2026-04-19 09:49 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -8821,7 +9201,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-18 09:50 UTC</t>
+          <t>2026-04-19 09:49 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -8846,7 +9226,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-18 09:50 UTC</t>
+          <t>2026-04-19 09:49 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">

</xml_diff>

<commit_message>
chore: update snapshots 2026-04-20
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H211"/>
+  <dimension ref="A1:H221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -8557,6 +8557,386 @@
         </is>
       </c>
       <c r="H211" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="212" ht="15" customHeight="1">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>2026-04-20 10:50 UTC</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E212" t="n">
+        <v>0</v>
+      </c>
+      <c r="F212" t="n">
+        <v>0</v>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="213" ht="15" customHeight="1">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>2026-04-20 10:50 UTC</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E213" t="n">
+        <v>0</v>
+      </c>
+      <c r="F213" t="n">
+        <v>0</v>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="214" ht="15" customHeight="1">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>2026-04-20 10:50 UTC</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E214" t="n">
+        <v>0</v>
+      </c>
+      <c r="F214" t="n">
+        <v>0</v>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="215" ht="15" customHeight="1">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>2026-04-20 10:50 UTC</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E215" t="n">
+        <v>0</v>
+      </c>
+      <c r="F215" t="n">
+        <v>0</v>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="216" ht="15" customHeight="1">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>2026-04-20 10:50 UTC</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E216" t="n">
+        <v>0</v>
+      </c>
+      <c r="F216" t="n">
+        <v>0</v>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="217" ht="15" customHeight="1">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>2026-04-20 10:50 UTC</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E217" t="n">
+        <v>0</v>
+      </c>
+      <c r="F217" t="n">
+        <v>0</v>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="218" ht="15" customHeight="1">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>2026-04-20 10:50 UTC</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E218" t="n">
+        <v>0</v>
+      </c>
+      <c r="F218" t="n">
+        <v>0</v>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="219" ht="15" customHeight="1">
+      <c r="A219" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-20 10:50 UTC</t>
+        </is>
+      </c>
+      <c r="B219" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C219" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D219" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E219" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F219" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G219" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.276ff2ba54c8e48abf3a.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.eeea495b597ca09b845b.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H219" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.f3bd1b5b095bb64711ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.a198328c15c6d468eaf3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3978fb6ce2deb4c39aa0.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="220" ht="15" customHeight="1">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>2026-04-20 10:50 UTC</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E220" t="n">
+        <v>0</v>
+      </c>
+      <c r="F220" t="n">
+        <v>0</v>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="221" ht="15" customHeight="1">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>2026-04-20 10:50 UTC</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E221" t="n">
+        <v>0</v>
+      </c>
+      <c r="F221" t="n">
+        <v>0</v>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -8881,76 +9261,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.f3bd1b5b095bb64711ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.a198328c15c6d468eaf3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3978fb6ce2deb4c39aa0.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.f3bd1b5b095bb64711ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.5f8f57924d402881318d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3978fb6ce2deb4c39aa0.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -9001,7 +9311,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-19 09:49 UTC</t>
+          <t>2026-04-20 10:50 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -9026,7 +9336,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-04-19 09:49 UTC</t>
+          <t>2026-04-20 10:50 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -9051,7 +9361,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-04-19 09:49 UTC</t>
+          <t>2026-04-20 10:50 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -9076,7 +9386,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-19 09:49 UTC</t>
+          <t>2026-04-20 10:50 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -9101,7 +9411,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-04-19 09:49 UTC</t>
+          <t>2026-04-20 10:50 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -9126,7 +9436,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-04-19 09:49 UTC</t>
+          <t>2026-04-20 10:50 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -9151,7 +9461,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-04-19 09:49 UTC</t>
+          <t>2026-04-20 10:50 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -9176,7 +9486,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-04-19 09:49 UTC</t>
+          <t>2026-04-20 10:50 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -9201,7 +9511,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-19 09:49 UTC</t>
+          <t>2026-04-20 10:50 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -9226,7 +9536,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-19 09:49 UTC</t>
+          <t>2026-04-20 10:50 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -9235,6 +9545,76 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.276ff2ba54c8e48abf3a.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.eeea495b597ca09b845b.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.f3bd1b5b095bb64711ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.a198328c15c6d468eaf3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3978fb6ce2deb4c39aa0.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-04-21
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H221"/>
+  <dimension ref="A1:H231"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -8937,6 +8937,386 @@
         </is>
       </c>
       <c r="H221" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="222" ht="15" customHeight="1">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>2026-04-21 10:19 UTC</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E222" t="n">
+        <v>0</v>
+      </c>
+      <c r="F222" t="n">
+        <v>0</v>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="223" ht="15" customHeight="1">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>2026-04-21 10:19 UTC</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E223" t="n">
+        <v>0</v>
+      </c>
+      <c r="F223" t="n">
+        <v>0</v>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="224" ht="15" customHeight="1">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>2026-04-21 10:19 UTC</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E224" t="n">
+        <v>0</v>
+      </c>
+      <c r="F224" t="n">
+        <v>0</v>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="225" ht="15" customHeight="1">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>2026-04-21 10:19 UTC</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E225" t="n">
+        <v>0</v>
+      </c>
+      <c r="F225" t="n">
+        <v>0</v>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="226" ht="15" customHeight="1">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>2026-04-21 10:19 UTC</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E226" t="n">
+        <v>0</v>
+      </c>
+      <c r="F226" t="n">
+        <v>0</v>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="227" ht="15" customHeight="1">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>2026-04-21 10:19 UTC</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E227" t="n">
+        <v>0</v>
+      </c>
+      <c r="F227" t="n">
+        <v>0</v>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="228" ht="15" customHeight="1">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>2026-04-21 10:19 UTC</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E228" t="n">
+        <v>0</v>
+      </c>
+      <c r="F228" t="n">
+        <v>0</v>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="229" ht="15" customHeight="1">
+      <c r="A229" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-21 10:19 UTC</t>
+        </is>
+      </c>
+      <c r="B229" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C229" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D229" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E229" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F229" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G229" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.832252dc3bb9e4adb6d6.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8ccc1f017d7b94cfd357.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H229" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.276ff2ba54c8e48abf3a.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.eeea495b597ca09b845b.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="230" ht="15" customHeight="1">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>2026-04-21 10:19 UTC</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E230" t="n">
+        <v>0</v>
+      </c>
+      <c r="F230" t="n">
+        <v>0</v>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="231" ht="15" customHeight="1">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>2026-04-21 10:19 UTC</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E231" t="n">
+        <v>0</v>
+      </c>
+      <c r="F231" t="n">
+        <v>0</v>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -9311,7 +9691,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-20 10:50 UTC</t>
+          <t>2026-04-21 10:19 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -9336,7 +9716,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-04-20 10:50 UTC</t>
+          <t>2026-04-21 10:19 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -9361,7 +9741,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-04-20 10:50 UTC</t>
+          <t>2026-04-21 10:19 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -9386,7 +9766,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-20 10:50 UTC</t>
+          <t>2026-04-21 10:19 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -9411,7 +9791,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-04-20 10:50 UTC</t>
+          <t>2026-04-21 10:19 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -9436,7 +9816,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-04-20 10:50 UTC</t>
+          <t>2026-04-21 10:19 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -9461,7 +9841,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-04-20 10:50 UTC</t>
+          <t>2026-04-21 10:19 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -9486,7 +9866,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-04-20 10:50 UTC</t>
+          <t>2026-04-21 10:19 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -9511,7 +9891,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-20 10:50 UTC</t>
+          <t>2026-04-21 10:19 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -9536,7 +9916,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-20 10:50 UTC</t>
+          <t>2026-04-21 10:19 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -9597,7 +9977,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.276ff2ba54c8e48abf3a.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.eeea495b597ca09b845b.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.832252dc3bb9e4adb6d6.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8ccc1f017d7b94cfd357.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -9614,7 +9994,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.f3bd1b5b095bb64711ca.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.a198328c15c6d468eaf3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.3978fb6ce2deb4c39aa0.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.276ff2ba54c8e48abf3a.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.eeea495b597ca09b845b.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-04-22
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H231"/>
+  <dimension ref="A1:H241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -9317,6 +9317,386 @@
         </is>
       </c>
       <c r="H231" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="232" ht="15" customHeight="1">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>2026-04-22 10:20 UTC</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E232" t="n">
+        <v>0</v>
+      </c>
+      <c r="F232" t="n">
+        <v>0</v>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="233" ht="15" customHeight="1">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>2026-04-22 10:20 UTC</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E233" t="n">
+        <v>0</v>
+      </c>
+      <c r="F233" t="n">
+        <v>0</v>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="234" ht="15" customHeight="1">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>2026-04-22 10:20 UTC</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E234" t="n">
+        <v>0</v>
+      </c>
+      <c r="F234" t="n">
+        <v>0</v>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="235" ht="15" customHeight="1">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>2026-04-22 10:20 UTC</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E235" t="n">
+        <v>0</v>
+      </c>
+      <c r="F235" t="n">
+        <v>0</v>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="236" ht="15" customHeight="1">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>2026-04-22 10:20 UTC</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E236" t="n">
+        <v>0</v>
+      </c>
+      <c r="F236" t="n">
+        <v>0</v>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="237" ht="15" customHeight="1">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>2026-04-22 10:20 UTC</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E237" t="n">
+        <v>0</v>
+      </c>
+      <c r="F237" t="n">
+        <v>0</v>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="238" ht="15" customHeight="1">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>2026-04-22 10:20 UTC</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E238" t="n">
+        <v>0</v>
+      </c>
+      <c r="F238" t="n">
+        <v>0</v>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="239" ht="15" customHeight="1">
+      <c r="A239" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-22 10:20 UTC</t>
+        </is>
+      </c>
+      <c r="B239" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C239" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D239" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E239" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F239" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G239" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.bdc09c5683feee7ef5cb.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8ccc1f017d7b94cfd357.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H239" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.832252dc3bb9e4adb6d6.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8ccc1f017d7b94cfd357.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="240" ht="15" customHeight="1">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>2026-04-22 10:20 UTC</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E240" t="n">
+        <v>0</v>
+      </c>
+      <c r="F240" t="n">
+        <v>0</v>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="241" ht="15" customHeight="1">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>2026-04-22 10:20 UTC</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E241" t="n">
+        <v>0</v>
+      </c>
+      <c r="F241" t="n">
+        <v>0</v>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -9691,7 +10071,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-21 10:19 UTC</t>
+          <t>2026-04-22 10:20 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -9716,7 +10096,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-04-21 10:19 UTC</t>
+          <t>2026-04-22 10:20 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -9741,7 +10121,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-04-21 10:19 UTC</t>
+          <t>2026-04-22 10:20 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -9766,7 +10146,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-21 10:19 UTC</t>
+          <t>2026-04-22 10:20 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -9791,7 +10171,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-04-21 10:19 UTC</t>
+          <t>2026-04-22 10:20 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -9816,7 +10196,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-04-21 10:19 UTC</t>
+          <t>2026-04-22 10:20 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -9841,7 +10221,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-04-21 10:19 UTC</t>
+          <t>2026-04-22 10:20 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -9866,7 +10246,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-04-21 10:19 UTC</t>
+          <t>2026-04-22 10:20 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -9891,7 +10271,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-21 10:19 UTC</t>
+          <t>2026-04-22 10:20 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -9916,7 +10296,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-21 10:19 UTC</t>
+          <t>2026-04-22 10:20 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -9977,7 +10357,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.832252dc3bb9e4adb6d6.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8ccc1f017d7b94cfd357.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.bdc09c5683feee7ef5cb.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8ccc1f017d7b94cfd357.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -9994,7 +10374,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.276ff2ba54c8e48abf3a.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.eeea495b597ca09b845b.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.832252dc3bb9e4adb6d6.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8ccc1f017d7b94cfd357.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-04-23
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H241"/>
+  <dimension ref="A1:H251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -9697,6 +9697,386 @@
         </is>
       </c>
       <c r="H241" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="242" ht="15" customHeight="1">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:22 UTC</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E242" t="n">
+        <v>0</v>
+      </c>
+      <c r="F242" t="n">
+        <v>0</v>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="243" ht="15" customHeight="1">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:22 UTC</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E243" t="n">
+        <v>0</v>
+      </c>
+      <c r="F243" t="n">
+        <v>0</v>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="244" ht="15" customHeight="1">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:22 UTC</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E244" t="n">
+        <v>0</v>
+      </c>
+      <c r="F244" t="n">
+        <v>0</v>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="245" ht="15" customHeight="1">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:22 UTC</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E245" t="n">
+        <v>0</v>
+      </c>
+      <c r="F245" t="n">
+        <v>0</v>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="246" ht="15" customHeight="1">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:22 UTC</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E246" t="n">
+        <v>0</v>
+      </c>
+      <c r="F246" t="n">
+        <v>0</v>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="247" ht="15" customHeight="1">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:22 UTC</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E247" t="n">
+        <v>0</v>
+      </c>
+      <c r="F247" t="n">
+        <v>0</v>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="248" ht="15" customHeight="1">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:22 UTC</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E248" t="n">
+        <v>0</v>
+      </c>
+      <c r="F248" t="n">
+        <v>0</v>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="249" ht="15" customHeight="1">
+      <c r="A249" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:22 UTC</t>
+        </is>
+      </c>
+      <c r="B249" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C249" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D249" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E249" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F249" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G249" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9c76d463468b2ab9e0fd.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.72a4cbf72571ebffd265.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H249" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.bdc09c5683feee7ef5cb.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8ccc1f017d7b94cfd357.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="250" ht="15" customHeight="1">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:22 UTC</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E250" t="n">
+        <v>0</v>
+      </c>
+      <c r="F250" t="n">
+        <v>0</v>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="251" ht="15" customHeight="1">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>2026-04-23 10:22 UTC</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E251" t="n">
+        <v>0</v>
+      </c>
+      <c r="F251" t="n">
+        <v>0</v>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -10071,7 +10451,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-22 10:20 UTC</t>
+          <t>2026-04-23 10:22 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -10096,7 +10476,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-04-22 10:20 UTC</t>
+          <t>2026-04-23 10:22 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -10121,7 +10501,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-04-22 10:20 UTC</t>
+          <t>2026-04-23 10:22 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -10146,7 +10526,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-22 10:20 UTC</t>
+          <t>2026-04-23 10:22 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -10171,7 +10551,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-04-22 10:20 UTC</t>
+          <t>2026-04-23 10:22 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -10196,7 +10576,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-04-22 10:20 UTC</t>
+          <t>2026-04-23 10:22 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -10221,7 +10601,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-04-22 10:20 UTC</t>
+          <t>2026-04-23 10:22 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -10246,7 +10626,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-04-22 10:20 UTC</t>
+          <t>2026-04-23 10:22 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -10271,7 +10651,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-22 10:20 UTC</t>
+          <t>2026-04-23 10:22 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -10296,7 +10676,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-22 10:20 UTC</t>
+          <t>2026-04-23 10:22 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -10357,7 +10737,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.bdc09c5683feee7ef5cb.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8ccc1f017d7b94cfd357.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9c76d463468b2ab9e0fd.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.72a4cbf72571ebffd265.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -10374,7 +10754,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.832252dc3bb9e4adb6d6.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8ccc1f017d7b94cfd357.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.bdc09c5683feee7ef5cb.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8ccc1f017d7b94cfd357.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-04-24
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -8,17 +8,17 @@
   </bookViews>
   <sheets>
     <sheet name="Change Log" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="amc_com_ads_txt" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="amc_com_app-ads_txt" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="bbca_com_ads_txt" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="bbca_com_app-ads_txt" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="ifc_com_ads_txt" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ifc_com_app-ads_txt" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Current Snapshot" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="amc_com_ads_txt" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="amc_com_app-ads_txt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="bbca_com_ads_txt" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="bbca_com_app-ads_txt" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="ifc_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="ifc_com_app-ads_txt" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="sundancetv_com_ads_txt" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="wetv_com_ads_txt" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="wetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H251"/>
+  <dimension ref="A1:H261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -10082,6 +10082,458 @@
         </is>
       </c>
     </row>
+    <row r="252" ht="15" customHeight="1">
+      <c r="A252" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-24 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B252" s="3" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C252" s="3" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D252" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E252" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F252" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G252" s="3" t="inlineStr">
+        <is>
+          <t>#Wurl: wurl.com, 55562, DIRECT
+#PrismRiot: freewheel.tv, 543709, RESELLER
+#PrismRiot: freewheel.tv, sg1303005, RESELLER
+#PrismRiot: freewheel.tv, 543709-r-523319, RESELLER
+#PrismRiot: freewheel.tv, 543709-r-524565, RESELLER
+#Olyzon: pubmatic.com, 167424, RESELLER, 5d62403b186f2ace
+#Olyzon: olyzon.tv, 76794, PUBLISHER
+#Nexxen: lkqd.net, 1100060088, RESELLER 59c49fa9598a0117
+#Infolinks: Infolinks.com, 3444795, DIRECT</t>
+        </is>
+      </c>
+      <c r="H252" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="253" ht="15" customHeight="1">
+      <c r="A253" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-24 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B253" s="3" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C253" s="3" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D253" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E253" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F253" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G253" s="3" t="inlineStr">
+        <is>
+          <t>#Wurl: wurl.com, 55562, DIRECT
+#PrismRiot: freewheel.tv, 543709, RESELLER
+#PrismRiot: freewheel.tv, sg1303005, RESELLER
+#PrismRiot: freewheel.tv, 543709-r-523319, RESELLER
+#PrismRiot: freewheel.tv, 543709-r-524565, RESELLER
+#Olyzon: pubmatic.com, 167424, RESELLER, 5d62403b186f2ace
+#Olyzon: olyzon.tv, 76794, PUBLISHER
+#Nexxen: lkqd.net, 1100060088, RESELLER 59c49fa9598a0117
+#Infolinks: Infolinks.com, 3444795, DIRECT</t>
+        </is>
+      </c>
+      <c r="H253" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="254" ht="15" customHeight="1">
+      <c r="A254" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-24 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B254" s="3" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C254" s="3" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D254" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E254" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F254" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G254" s="3" t="inlineStr">
+        <is>
+          <t>#Wurl: wurl.com, 55562, DIRECT
+#PrismRiot: freewheel.tv, 543709, RESELLER
+#PrismRiot: freewheel.tv, sg1303005, RESELLER
+#PrismRiot: freewheel.tv, 543709-r-523319, RESELLER
+#PrismRiot: freewheel.tv, 543709-r-524565, RESELLER
+#Olyzon: pubmatic.com, 167424, RESELLER, 5d62403b186f2ace
+#Olyzon: olyzon.tv, 76794, PUBLISHER
+#Nexxen: lkqd.net, 1100060088, RESELLER 59c49fa9598a0117
+#Infolinks: Infolinks.com, 3444795, DIRECT</t>
+        </is>
+      </c>
+      <c r="H254" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="255" ht="15" customHeight="1">
+      <c r="A255" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-24 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B255" s="3" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C255" s="3" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D255" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E255" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F255" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G255" s="3" t="inlineStr">
+        <is>
+          <t>#Wurl: wurl.com, 55562, DIRECT
+#PrismRiot: freewheel.tv, 543709, RESELLER
+#PrismRiot: freewheel.tv, sg1303005, RESELLER
+#PrismRiot: freewheel.tv, 543709-r-523319, RESELLER
+#PrismRiot: freewheel.tv, 543709-r-524565, RESELLER
+#Olyzon: pubmatic.com, 167424, RESELLER, 5d62403b186f2ace
+#Olyzon: olyzon.tv, 76794, PUBLISHER
+#Nexxen: lkqd.net, 1100060088, RESELLER 59c49fa9598a0117
+#Infolinks: Infolinks.com, 3444795, DIRECT</t>
+        </is>
+      </c>
+      <c r="H255" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="256" ht="15" customHeight="1">
+      <c r="A256" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-24 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B256" s="3" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C256" s="3" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D256" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E256" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F256" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G256" s="3" t="inlineStr">
+        <is>
+          <t>#Wurl: wurl.com, 55562, DIRECT
+#PrismRiot: freewheel.tv, 543709, RESELLER
+#PrismRiot: freewheel.tv, sg1303005, RESELLER
+#PrismRiot: freewheel.tv, 543709-r-523319, RESELLER
+#PrismRiot: freewheel.tv, 543709-r-524565, RESELLER
+#Olyzon: pubmatic.com, 167424, RESELLER, 5d62403b186f2ace
+#Olyzon: olyzon.tv, 76794, PUBLISHER
+#Nexxen: lkqd.net, 1100060088, RESELLER 59c49fa9598a0117
+#Infolinks: Infolinks.com, 3444795, DIRECT</t>
+        </is>
+      </c>
+      <c r="H256" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="257" ht="15" customHeight="1">
+      <c r="A257" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-24 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B257" s="3" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C257" s="3" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D257" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E257" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F257" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G257" s="3" t="inlineStr">
+        <is>
+          <t>#Wurl: wurl.com, 55562, DIRECT
+#PrismRiot: freewheel.tv, 543709, RESELLER
+#PrismRiot: freewheel.tv, sg1303005, RESELLER
+#PrismRiot: freewheel.tv, 543709-r-523319, RESELLER
+#PrismRiot: freewheel.tv, 543709-r-524565, RESELLER
+#Olyzon: pubmatic.com, 167424, RESELLER, 5d62403b186f2ace
+#Olyzon: olyzon.tv, 76794, PUBLISHER
+#Nexxen: lkqd.net, 1100060088, RESELLER 59c49fa9598a0117
+#Infolinks: Infolinks.com, 3444795, DIRECT</t>
+        </is>
+      </c>
+      <c r="H257" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="258" ht="15" customHeight="1">
+      <c r="A258" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-24 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B258" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C258" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D258" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E258" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F258" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G258" s="3" t="inlineStr">
+        <is>
+          <t>#Wurl: wurl.com, 55562, DIRECT
+#PrismRiot: freewheel.tv, 543709, RESELLER
+#PrismRiot: freewheel.tv, sg1303005, RESELLER
+#PrismRiot: freewheel.tv, 543709-r-523319, RESELLER
+#PrismRiot: freewheel.tv, 543709-r-524565, RESELLER
+#Olyzon: pubmatic.com, 167424, RESELLER, 5d62403b186f2ace
+#Olyzon: olyzon.tv, 76794, PUBLISHER
+#Nexxen: lkqd.net, 1100060088, RESELLER 59c49fa9598a0117
+#Infolinks: Infolinks.com, 3444795, DIRECT</t>
+        </is>
+      </c>
+      <c r="H258" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="259" ht="15" customHeight="1">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>2026-04-24 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E259" t="n">
+        <v>0</v>
+      </c>
+      <c r="F259" t="n">
+        <v>0</v>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="260" ht="15" customHeight="1">
+      <c r="A260" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-24 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B260" s="3" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C260" s="3" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D260" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E260" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F260" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G260" s="3" t="inlineStr">
+        <is>
+          <t>#Wurl: wurl.com, 55562, DIRECT
+#PrismRiot: freewheel.tv, 543709, RESELLER
+#PrismRiot: freewheel.tv, sg1303005, RESELLER
+#PrismRiot: freewheel.tv, 543709-r-523319, RESELLER
+#PrismRiot: freewheel.tv, 543709-r-524565, RESELLER
+#Olyzon: pubmatic.com, 167424, RESELLER, 5d62403b186f2ace
+#Olyzon: olyzon.tv, 76794, PUBLISHER
+#Nexxen: lkqd.net, 1100060088, RESELLER 59c49fa9598a0117
+#Infolinks: Infolinks.com, 3444795, DIRECT</t>
+        </is>
+      </c>
+      <c r="H260" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="261" ht="15" customHeight="1">
+      <c r="A261" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-24 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B261" s="3" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C261" s="3" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D261" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E261" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="F261" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G261" s="3" t="inlineStr">
+        <is>
+          <t>#Wurl: wurl.com, 55562, DIRECT
+#PrismRiot: freewheel.tv, 543709, RESELLER
+#PrismRiot: freewheel.tv, sg1303005, RESELLER
+#PrismRiot: freewheel.tv, 543709-r-523319, RESELLER
+#PrismRiot: freewheel.tv, 543709-r-524565, RESELLER
+#Olyzon: pubmatic.com, 167424, RESELLER, 5d62403b186f2ace
+#Olyzon: olyzon.tv, 76794, PUBLISHER
+#Nexxen: lkqd.net, 1100060088, RESELLER 59c49fa9598a0117
+#Infolinks: Infolinks.com, 3444795, DIRECT</t>
+        </is>
+      </c>
+      <c r="H261" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10093,7 +10545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10126,12 +10578,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Sonobi</t>
+          <t>#Wurl</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>oxiem.com, 7d3ac7564a, DIRECT, d1a215d9eb5aee9e</t>
+          <t>wurl.com, 55562, DIRECT</t>
         </is>
       </c>
     </row>
@@ -10143,12 +10595,12 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>#Sonobi</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>oxiem.com, 7d3ac7564a, DIRECT, b7aba0bfd04aa6b6</t>
+          <t>freewheel.tv, 543709, RESELLER</t>
         </is>
       </c>
     </row>
@@ -10160,12 +10612,12 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>connatix.com, 101557, DIRECT, 2af98acdee0e81ed</t>
+          <t>freewheel.tv, sg1303005, RESELLER</t>
         </is>
       </c>
     </row>
@@ -10177,12 +10629,12 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>pubmatic.com, 166226, RESELLER, 5d62403b186f2ace</t>
+          <t>freewheel.tv, 543709-r-523319, RESELLER</t>
         </is>
       </c>
     </row>
@@ -10194,12 +10646,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, 535072-r-524565, RESELLER</t>
+          <t>freewheel.tv, 543709-r-524565, RESELLER</t>
         </is>
       </c>
     </row>
@@ -10211,12 +10663,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#Olyzon</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>appnexus.com, 17444, RESELLER, f5ab79cb980f11d1</t>
+          <t>pubmatic.com, 167424, RESELLER, 5d62403b186f2ace</t>
         </is>
       </c>
     </row>
@@ -10228,12 +10680,12 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#Olyzon</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>themediagrid.com, PCE1BO, RESELLER, 35d5010d7789b49d</t>
+          <t>olyzon.tv, 76794, PUBLISHER</t>
         </is>
       </c>
     </row>
@@ -10245,12 +10697,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#Nexxen</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>loopme.com, 11186, RESELLER, 6c8d5f95897a5a3b</t>
+          <t>lkqd.net, 1100060088, RESELLER 59c49fa9598a0117</t>
         </is>
       </c>
     </row>
@@ -10262,131 +10714,12 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>#Xapads</t>
+          <t>#Infolinks</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>videoheroes.tv, 212796, DIRECT, 064bc410192443d8</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>video.unrulymedia.com, 170071695, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 534963-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>lkqd.net, 1100060074, RESELLER, 59c49fa9598a0117</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>conversantmedia.com, 100718, RESELLER, 03113cd04947736d</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>safex.tv, 5078, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>media.net, 8CU406385, RESELLER</t>
+          <t>Infolinks.com, 3444795, DIRECT</t>
         </is>
       </c>
     </row>
@@ -10396,6 +10729,454 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>#Wurl</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>wurl.com, 55562, DIRECT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>#PrismRiot</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 543709, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>#PrismRiot</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, sg1303005, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>#PrismRiot</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 543709-r-523319, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>#PrismRiot</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 543709-r-524565, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>#Olyzon</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>pubmatic.com, 167424, RESELLER, 5d62403b186f2ace</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>#Olyzon</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>olyzon.tv, 76794, PUBLISHER</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>#Nexxen</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>lkqd.net, 1100060088, RESELLER 59c49fa9598a0117</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>#Infolinks</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Infolinks.com, 3444795, DIRECT</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>#Wurl</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>wurl.com, 55562, DIRECT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>#PrismRiot</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 543709, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>#PrismRiot</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, sg1303005, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>#PrismRiot</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 543709-r-523319, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>#PrismRiot</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 543709-r-524565, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>#Olyzon</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>pubmatic.com, 167424, RESELLER, 5d62403b186f2ace</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>#Olyzon</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>olyzon.tv, 76794, PUBLISHER</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>#Nexxen</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>lkqd.net, 1100060088, RESELLER 59c49fa9598a0117</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>#Infolinks</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Infolinks.com, 3444795, DIRECT</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9c76d463468b2ab9e0fd.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.72a4cbf72571ebffd265.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.bdc09c5683feee7ef5cb.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8ccc1f017d7b94cfd357.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10451,11 +11232,11 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-23 10:22 UTC</t>
+          <t>2026-04-24 10:23 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1127</v>
+        <v>1140</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -10476,11 +11257,11 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-04-23 10:22 UTC</t>
+          <t>2026-04-24 10:23 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1040</v>
+        <v>1054</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -10501,11 +11282,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-04-23 10:22 UTC</t>
+          <t>2026-04-24 10:23 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1127</v>
+        <v>1140</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -10526,11 +11307,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-23 10:22 UTC</t>
+          <t>2026-04-24 10:23 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1040</v>
+        <v>1054</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -10551,11 +11332,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-04-23 10:22 UTC</t>
+          <t>2026-04-24 10:23 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1127</v>
+        <v>1140</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -10576,11 +11357,11 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-04-23 10:22 UTC</t>
+          <t>2026-04-24 10:23 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1040</v>
+        <v>1054</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -10601,11 +11382,11 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-04-23 10:22 UTC</t>
+          <t>2026-04-24 10:23 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1127</v>
+        <v>1140</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -10626,7 +11407,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-04-23 10:22 UTC</t>
+          <t>2026-04-24 10:23 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -10651,11 +11432,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-23 10:22 UTC</t>
+          <t>2026-04-24 10:23 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1127</v>
+        <v>1140</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -10676,701 +11457,15 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-23 10:22 UTC</t>
+          <t>2026-04-24 10:23 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1040</v>
+        <v>1054</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9c76d463468b2ab9e0fd.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.72a4cbf72571ebffd265.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.bdc09c5683feee7ef5cb.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8ccc1f017d7b94cfd357.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>#Sonobi</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>oxiem.com, 7d3ac7564a, DIRECT, d1a215d9eb5aee9e</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>#Sonobi</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>oxiem.com, 7d3ac7564a, DIRECT, b7aba0bfd04aa6b6</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>#MyCode</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>connatix.com, 101557, DIRECT, 2af98acdee0e81ed</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>#MyCode</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 166226, RESELLER, 5d62403b186f2ace</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>#MyCode</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 535072-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>#MyCode</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>appnexus.com, 17444, RESELLER, f5ab79cb980f11d1</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>#MyCode</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>themediagrid.com, PCE1BO, RESELLER, 35d5010d7789b49d</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>#MyCode</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>loopme.com, 11186, RESELLER, 6c8d5f95897a5a3b</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>videoheroes.tv, 212796, DIRECT, 064bc410192443d8</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>video.unrulymedia.com, 170071695, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 534963-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>lkqd.net, 1100060074, RESELLER, 59c49fa9598a0117</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>conversantmedia.com, 100718, RESELLER, 03113cd04947736d</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>safex.tv, 5078, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>media.net, 8CU406385, RESELLER</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>#Sonobi</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>oxiem.com, 7d3ac7564a, DIRECT, d1a215d9eb5aee9e</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>#Sonobi</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>oxiem.com, 7d3ac7564a, DIRECT, b7aba0bfd04aa6b6</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>#MyCode</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>connatix.com, 101557, DIRECT, 2af98acdee0e81ed</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>#MyCode</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 166226, RESELLER, 5d62403b186f2ace</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>#MyCode</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 535072-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>#MyCode</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>appnexus.com, 17444, RESELLER, f5ab79cb980f11d1</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>#MyCode</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>themediagrid.com, PCE1BO, RESELLER, 35d5010d7789b49d</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>#MyCode</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>loopme.com, 11186, RESELLER, 6c8d5f95897a5a3b</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>videoheroes.tv, 212796, DIRECT, 064bc410192443d8</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>video.unrulymedia.com, 170071695, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 534963-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>lkqd.net, 1100060074, RESELLER, 59c49fa9598a0117</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>conversantmedia.com, 100718, RESELLER, 03113cd04947736d</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>safex.tv, 5078, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>media.net, 8CU406385, RESELLER</t>
         </is>
       </c>
     </row>
@@ -11385,7 +11480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11418,12 +11513,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Sonobi</t>
+          <t>#Wurl</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>oxiem.com, 7d3ac7564a, DIRECT, d1a215d9eb5aee9e</t>
+          <t>wurl.com, 55562, DIRECT</t>
         </is>
       </c>
     </row>
@@ -11435,12 +11530,12 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>#Sonobi</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>oxiem.com, 7d3ac7564a, DIRECT, b7aba0bfd04aa6b6</t>
+          <t>freewheel.tv, 543709, RESELLER</t>
         </is>
       </c>
     </row>
@@ -11452,12 +11547,12 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>connatix.com, 101557, DIRECT, 2af98acdee0e81ed</t>
+          <t>freewheel.tv, sg1303005, RESELLER</t>
         </is>
       </c>
     </row>
@@ -11469,12 +11564,12 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>pubmatic.com, 166226, RESELLER, 5d62403b186f2ace</t>
+          <t>freewheel.tv, 543709-r-523319, RESELLER</t>
         </is>
       </c>
     </row>
@@ -11486,12 +11581,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, 535072-r-524565, RESELLER</t>
+          <t>freewheel.tv, 543709-r-524565, RESELLER</t>
         </is>
       </c>
     </row>
@@ -11503,12 +11598,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#Olyzon</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>appnexus.com, 17444, RESELLER, f5ab79cb980f11d1</t>
+          <t>pubmatic.com, 167424, RESELLER, 5d62403b186f2ace</t>
         </is>
       </c>
     </row>
@@ -11520,12 +11615,12 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#Olyzon</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>themediagrid.com, PCE1BO, RESELLER, 35d5010d7789b49d</t>
+          <t>olyzon.tv, 76794, PUBLISHER</t>
         </is>
       </c>
     </row>
@@ -11537,12 +11632,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#Nexxen</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>loopme.com, 11186, RESELLER, 6c8d5f95897a5a3b</t>
+          <t>lkqd.net, 1100060088, RESELLER 59c49fa9598a0117</t>
         </is>
       </c>
     </row>
@@ -11554,131 +11649,12 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>#Xapads</t>
+          <t>#Infolinks</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>videoheroes.tv, 212796, DIRECT, 064bc410192443d8</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>video.unrulymedia.com, 170071695, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 534963-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>lkqd.net, 1100060074, RESELLER, 59c49fa9598a0117</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>conversantmedia.com, 100718, RESELLER, 03113cd04947736d</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>safex.tv, 5078, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>media.net, 8CU406385, RESELLER</t>
+          <t>Infolinks.com, 3444795, DIRECT</t>
         </is>
       </c>
     </row>
@@ -11693,7 +11669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11726,12 +11702,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Sonobi</t>
+          <t>#Wurl</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>oxiem.com, 7d3ac7564a, DIRECT, d1a215d9eb5aee9e</t>
+          <t>wurl.com, 55562, DIRECT</t>
         </is>
       </c>
     </row>
@@ -11743,12 +11719,12 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>#Sonobi</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>oxiem.com, 7d3ac7564a, DIRECT, b7aba0bfd04aa6b6</t>
+          <t>freewheel.tv, 543709, RESELLER</t>
         </is>
       </c>
     </row>
@@ -11760,12 +11736,12 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>connatix.com, 101557, DIRECT, 2af98acdee0e81ed</t>
+          <t>freewheel.tv, sg1303005, RESELLER</t>
         </is>
       </c>
     </row>
@@ -11777,12 +11753,12 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>pubmatic.com, 166226, RESELLER, 5d62403b186f2ace</t>
+          <t>freewheel.tv, 543709-r-523319, RESELLER</t>
         </is>
       </c>
     </row>
@@ -11794,12 +11770,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, 535072-r-524565, RESELLER</t>
+          <t>freewheel.tv, 543709-r-524565, RESELLER</t>
         </is>
       </c>
     </row>
@@ -11811,12 +11787,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#Olyzon</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>appnexus.com, 17444, RESELLER, f5ab79cb980f11d1</t>
+          <t>pubmatic.com, 167424, RESELLER, 5d62403b186f2ace</t>
         </is>
       </c>
     </row>
@@ -11828,12 +11804,12 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#Olyzon</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>themediagrid.com, PCE1BO, RESELLER, 35d5010d7789b49d</t>
+          <t>olyzon.tv, 76794, PUBLISHER</t>
         </is>
       </c>
     </row>
@@ -11845,12 +11821,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#Nexxen</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>loopme.com, 11186, RESELLER, 6c8d5f95897a5a3b</t>
+          <t>lkqd.net, 1100060088, RESELLER 59c49fa9598a0117</t>
         </is>
       </c>
     </row>
@@ -11862,131 +11838,12 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>#Xapads</t>
+          <t>#Infolinks</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>videoheroes.tv, 212796, DIRECT, 064bc410192443d8</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>video.unrulymedia.com, 170071695, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 534963-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>lkqd.net, 1100060074, RESELLER, 59c49fa9598a0117</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>conversantmedia.com, 100718, RESELLER, 03113cd04947736d</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>safex.tv, 5078, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>media.net, 8CU406385, RESELLER</t>
+          <t>Infolinks.com, 3444795, DIRECT</t>
         </is>
       </c>
     </row>
@@ -12001,7 +11858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12034,12 +11891,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Sonobi</t>
+          <t>#Wurl</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>oxiem.com, 7d3ac7564a, DIRECT, d1a215d9eb5aee9e</t>
+          <t>wurl.com, 55562, DIRECT</t>
         </is>
       </c>
     </row>
@@ -12051,12 +11908,12 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>#Sonobi</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>oxiem.com, 7d3ac7564a, DIRECT, b7aba0bfd04aa6b6</t>
+          <t>freewheel.tv, 543709, RESELLER</t>
         </is>
       </c>
     </row>
@@ -12068,12 +11925,12 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>connatix.com, 101557, DIRECT, 2af98acdee0e81ed</t>
+          <t>freewheel.tv, sg1303005, RESELLER</t>
         </is>
       </c>
     </row>
@@ -12085,12 +11942,12 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>pubmatic.com, 166226, RESELLER, 5d62403b186f2ace</t>
+          <t>freewheel.tv, 543709-r-523319, RESELLER</t>
         </is>
       </c>
     </row>
@@ -12102,12 +11959,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, 535072-r-524565, RESELLER</t>
+          <t>freewheel.tv, 543709-r-524565, RESELLER</t>
         </is>
       </c>
     </row>
@@ -12119,12 +11976,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#Olyzon</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>appnexus.com, 17444, RESELLER, f5ab79cb980f11d1</t>
+          <t>pubmatic.com, 167424, RESELLER, 5d62403b186f2ace</t>
         </is>
       </c>
     </row>
@@ -12136,12 +11993,12 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#Olyzon</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>themediagrid.com, PCE1BO, RESELLER, 35d5010d7789b49d</t>
+          <t>olyzon.tv, 76794, PUBLISHER</t>
         </is>
       </c>
     </row>
@@ -12153,12 +12010,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#Nexxen</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>loopme.com, 11186, RESELLER, 6c8d5f95897a5a3b</t>
+          <t>lkqd.net, 1100060088, RESELLER 59c49fa9598a0117</t>
         </is>
       </c>
     </row>
@@ -12170,131 +12027,12 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>#Xapads</t>
+          <t>#Infolinks</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>videoheroes.tv, 212796, DIRECT, 064bc410192443d8</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>video.unrulymedia.com, 170071695, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 534963-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>lkqd.net, 1100060074, RESELLER, 59c49fa9598a0117</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>conversantmedia.com, 100718, RESELLER, 03113cd04947736d</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>safex.tv, 5078, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>media.net, 8CU406385, RESELLER</t>
+          <t>Infolinks.com, 3444795, DIRECT</t>
         </is>
       </c>
     </row>
@@ -12309,7 +12047,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12342,12 +12080,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Sonobi</t>
+          <t>#Wurl</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>oxiem.com, 7d3ac7564a, DIRECT, d1a215d9eb5aee9e</t>
+          <t>wurl.com, 55562, DIRECT</t>
         </is>
       </c>
     </row>
@@ -12359,12 +12097,12 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>#Sonobi</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>oxiem.com, 7d3ac7564a, DIRECT, b7aba0bfd04aa6b6</t>
+          <t>freewheel.tv, 543709, RESELLER</t>
         </is>
       </c>
     </row>
@@ -12376,12 +12114,12 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>connatix.com, 101557, DIRECT, 2af98acdee0e81ed</t>
+          <t>freewheel.tv, sg1303005, RESELLER</t>
         </is>
       </c>
     </row>
@@ -12393,12 +12131,12 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>pubmatic.com, 166226, RESELLER, 5d62403b186f2ace</t>
+          <t>freewheel.tv, 543709-r-523319, RESELLER</t>
         </is>
       </c>
     </row>
@@ -12410,12 +12148,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, 535072-r-524565, RESELLER</t>
+          <t>freewheel.tv, 543709-r-524565, RESELLER</t>
         </is>
       </c>
     </row>
@@ -12427,12 +12165,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#Olyzon</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>appnexus.com, 17444, RESELLER, f5ab79cb980f11d1</t>
+          <t>pubmatic.com, 167424, RESELLER, 5d62403b186f2ace</t>
         </is>
       </c>
     </row>
@@ -12444,12 +12182,12 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#Olyzon</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>themediagrid.com, PCE1BO, RESELLER, 35d5010d7789b49d</t>
+          <t>olyzon.tv, 76794, PUBLISHER</t>
         </is>
       </c>
     </row>
@@ -12461,12 +12199,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#Nexxen</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>loopme.com, 11186, RESELLER, 6c8d5f95897a5a3b</t>
+          <t>lkqd.net, 1100060088, RESELLER 59c49fa9598a0117</t>
         </is>
       </c>
     </row>
@@ -12478,131 +12216,12 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>#Xapads</t>
+          <t>#Infolinks</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>videoheroes.tv, 212796, DIRECT, 064bc410192443d8</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>video.unrulymedia.com, 170071695, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 534963-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>lkqd.net, 1100060074, RESELLER, 59c49fa9598a0117</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>conversantmedia.com, 100718, RESELLER, 03113cd04947736d</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>safex.tv, 5078, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>media.net, 8CU406385, RESELLER</t>
+          <t>Infolinks.com, 3444795, DIRECT</t>
         </is>
       </c>
     </row>
@@ -12617,7 +12236,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12650,12 +12269,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Sonobi</t>
+          <t>#Wurl</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>oxiem.com, 7d3ac7564a, DIRECT, d1a215d9eb5aee9e</t>
+          <t>wurl.com, 55562, DIRECT</t>
         </is>
       </c>
     </row>
@@ -12667,12 +12286,12 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>#Sonobi</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>oxiem.com, 7d3ac7564a, DIRECT, b7aba0bfd04aa6b6</t>
+          <t>freewheel.tv, 543709, RESELLER</t>
         </is>
       </c>
     </row>
@@ -12684,12 +12303,12 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>connatix.com, 101557, DIRECT, 2af98acdee0e81ed</t>
+          <t>freewheel.tv, sg1303005, RESELLER</t>
         </is>
       </c>
     </row>
@@ -12701,12 +12320,12 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>pubmatic.com, 166226, RESELLER, 5d62403b186f2ace</t>
+          <t>freewheel.tv, 543709-r-523319, RESELLER</t>
         </is>
       </c>
     </row>
@@ -12718,12 +12337,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, 535072-r-524565, RESELLER</t>
+          <t>freewheel.tv, 543709-r-524565, RESELLER</t>
         </is>
       </c>
     </row>
@@ -12735,12 +12354,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#Olyzon</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>appnexus.com, 17444, RESELLER, f5ab79cb980f11d1</t>
+          <t>pubmatic.com, 167424, RESELLER, 5d62403b186f2ace</t>
         </is>
       </c>
     </row>
@@ -12752,12 +12371,12 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#Olyzon</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>themediagrid.com, PCE1BO, RESELLER, 35d5010d7789b49d</t>
+          <t>olyzon.tv, 76794, PUBLISHER</t>
         </is>
       </c>
     </row>
@@ -12769,12 +12388,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#Nexxen</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>loopme.com, 11186, RESELLER, 6c8d5f95897a5a3b</t>
+          <t>lkqd.net, 1100060088, RESELLER 59c49fa9598a0117</t>
         </is>
       </c>
     </row>
@@ -12786,131 +12405,12 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>#Xapads</t>
+          <t>#Infolinks</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>videoheroes.tv, 212796, DIRECT, 064bc410192443d8</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>video.unrulymedia.com, 170071695, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 534963-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>lkqd.net, 1100060074, RESELLER, 59c49fa9598a0117</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>conversantmedia.com, 100718, RESELLER, 03113cd04947736d</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>safex.tv, 5078, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>media.net, 8CU406385, RESELLER</t>
+          <t>Infolinks.com, 3444795, DIRECT</t>
         </is>
       </c>
     </row>
@@ -12925,7 +12425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12958,12 +12458,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Sonobi</t>
+          <t>#Wurl</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>oxiem.com, 7d3ac7564a, DIRECT, d1a215d9eb5aee9e</t>
+          <t>wurl.com, 55562, DIRECT</t>
         </is>
       </c>
     </row>
@@ -12975,12 +12475,12 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>#Sonobi</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>oxiem.com, 7d3ac7564a, DIRECT, b7aba0bfd04aa6b6</t>
+          <t>freewheel.tv, 543709, RESELLER</t>
         </is>
       </c>
     </row>
@@ -12992,12 +12492,12 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>connatix.com, 101557, DIRECT, 2af98acdee0e81ed</t>
+          <t>freewheel.tv, sg1303005, RESELLER</t>
         </is>
       </c>
     </row>
@@ -13009,12 +12509,12 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>pubmatic.com, 166226, RESELLER, 5d62403b186f2ace</t>
+          <t>freewheel.tv, 543709-r-523319, RESELLER</t>
         </is>
       </c>
     </row>
@@ -13026,12 +12526,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#PrismRiot</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, 535072-r-524565, RESELLER</t>
+          <t>freewheel.tv, 543709-r-524565, RESELLER</t>
         </is>
       </c>
     </row>
@@ -13043,12 +12543,12 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#Olyzon</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>appnexus.com, 17444, RESELLER, f5ab79cb980f11d1</t>
+          <t>pubmatic.com, 167424, RESELLER, 5d62403b186f2ace</t>
         </is>
       </c>
     </row>
@@ -13060,12 +12560,12 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#Olyzon</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>themediagrid.com, PCE1BO, RESELLER, 35d5010d7789b49d</t>
+          <t>olyzon.tv, 76794, PUBLISHER</t>
         </is>
       </c>
     </row>
@@ -13077,12 +12577,12 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>#MyCode</t>
+          <t>#Nexxen</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>loopme.com, 11186, RESELLER, 6c8d5f95897a5a3b</t>
+          <t>lkqd.net, 1100060088, RESELLER 59c49fa9598a0117</t>
         </is>
       </c>
     </row>
@@ -13094,131 +12594,12 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>#Xapads</t>
+          <t>#Infolinks</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>videoheroes.tv, 212796, DIRECT, 064bc410192443d8</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>video.unrulymedia.com, 170071695, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 534963-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>lkqd.net, 1100060074, RESELLER, 59c49fa9598a0117</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>conversantmedia.com, 100718, RESELLER, 03113cd04947736d</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>safex.tv, 5078, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>media.net, 8CU406385, RESELLER</t>
+          <t>Infolinks.com, 3444795, DIRECT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-04-25
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -9,16 +9,16 @@
   <sheets>
     <sheet name="Change Log" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="sundancetv_com_app-ads_txt" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Current Snapshot" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="amc_com_ads_txt" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="amc_com_app-ads_txt" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="bbca_com_ads_txt" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="bbca_com_app-ads_txt" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="ifc_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ifc_com_app-ads_txt" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="sundancetv_com_ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="wetv_com_ads_txt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="wetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="amc_com_ads_txt" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="amc_com_app-ads_txt" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="bbca_com_ads_txt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="bbca_com_app-ads_txt" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ifc_com_ads_txt" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="ifc_com_app-ads_txt" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="sundancetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="wetv_com_ads_txt" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="wetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H261"/>
+  <dimension ref="A1:H271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -10529,6 +10529,374 @@
         </is>
       </c>
       <c r="H261" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="262" ht="15" customHeight="1">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>2026-04-25 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E262" t="n">
+        <v>0</v>
+      </c>
+      <c r="F262" t="n">
+        <v>0</v>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="263" ht="15" customHeight="1">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>2026-04-25 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E263" t="n">
+        <v>0</v>
+      </c>
+      <c r="F263" t="n">
+        <v>0</v>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="264" ht="15" customHeight="1">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>2026-04-25 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E264" t="n">
+        <v>0</v>
+      </c>
+      <c r="F264" t="n">
+        <v>0</v>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="265" ht="15" customHeight="1">
+      <c r="A265" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-25 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="B265" s="6" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C265" s="6" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D265" s="6" t="inlineStr">
+        <is>
+          <t>Error: HTTPSConnectionPool(host='www.bbcamerica.com', port=443): Read timed out. (read timeout=15)</t>
+        </is>
+      </c>
+      <c r="E265" s="6" t="inlineStr"/>
+      <c r="F265" s="6" t="inlineStr"/>
+      <c r="G265" s="6" t="inlineStr"/>
+      <c r="H265" s="6" t="inlineStr"/>
+    </row>
+    <row r="266" ht="15" customHeight="1">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>2026-04-25 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E266" t="n">
+        <v>0</v>
+      </c>
+      <c r="F266" t="n">
+        <v>0</v>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="267" ht="15" customHeight="1">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-04-25 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E267" t="n">
+        <v>0</v>
+      </c>
+      <c r="F267" t="n">
+        <v>0</v>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="268" ht="15" customHeight="1">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-04-25 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E268" t="n">
+        <v>0</v>
+      </c>
+      <c r="F268" t="n">
+        <v>0</v>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="269" ht="15" customHeight="1">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-04-25 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E269" t="n">
+        <v>0</v>
+      </c>
+      <c r="F269" t="n">
+        <v>0</v>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="270" ht="15" customHeight="1">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-04-25 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E270" t="n">
+        <v>0</v>
+      </c>
+      <c r="F270" t="n">
+        <v>0</v>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="271" ht="15" customHeight="1">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-04-25 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E271" t="n">
+        <v>0</v>
+      </c>
+      <c r="F271" t="n">
+        <v>0</v>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -10923,181 +11291,292 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Section</t>
+          <t>File</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Line Content</t>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Line Count</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>#Wurl</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>wurl.com, 55562, DIRECT</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-04-25 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1140</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709, RESELLER</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-04-25 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1054</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, sg1303005, RESELLER</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-04-25 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1140</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709-r-523319, RESELLER</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-04-25 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Error: HTTPSConnectionPool(host='www.bbcamerica.com', port=443): Read timed out. (read timeout=15)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709-r-524565, RESELLER</t>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-04-25 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1140</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>#Olyzon</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 167424, RESELLER, 5d62403b186f2ace</t>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-04-25 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1054</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>#Olyzon</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>olyzon.tv, 76794, PUBLISHER</t>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-04-25 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1140</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>#Nexxen</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>lkqd.net, 1100060088, RESELLER 59c49fa9598a0117</t>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-04-25 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>19</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>#Infolinks</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Infolinks.com, 3444795, DIRECT</t>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-04-25 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1140</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-04-25 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1054</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -11182,290 +11661,181 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Partner</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>File</t>
+          <t>Section</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Last Updated</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Line Count</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
+          <t>Line Content</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>AMC Networks</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>amc.com/ads.txt</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2026-04-24 10:23 UTC</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>1140</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>#Wurl</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>wurl.com, 55562, DIRECT</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>AMC Networks</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>amc.com/app-ads.txt</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2026-04-24 10:23 UTC</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>1054</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>#PrismRiot</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 543709, RESELLER</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>BBC America</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>bbca.com/ads.txt</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2026-04-24 10:23 UTC</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>1140</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>#PrismRiot</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, sg1303005, RESELLER</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>BBC America</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>bbca.com/app-ads.txt</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2026-04-24 10:23 UTC</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>1054</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>#PrismRiot</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 543709-r-523319, RESELLER</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>IFC</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>ifc.com/ads.txt</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>2026-04-24 10:23 UTC</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>1140</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>#PrismRiot</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 543709-r-524565, RESELLER</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>IFC</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>ifc.com/app-ads.txt</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>2026-04-24 10:23 UTC</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>1054</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>#Olyzon</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>pubmatic.com, 167424, RESELLER, 5d62403b186f2ace</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Sundance TV</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>sundancetv.com/ads.txt</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2026-04-24 10:23 UTC</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>1140</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>#Olyzon</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>olyzon.tv, 76794, PUBLISHER</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Sundance TV</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>sundancetv.com/app-ads.txt</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>2026-04-24 10:23 UTC</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>19</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>#Nexxen</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>lkqd.net, 1100060088, RESELLER 59c49fa9598a0117</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>WE tv</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>wetv.com/ads.txt</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>2026-04-24 10:23 UTC</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>1140</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>WE tv</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>wetv.com/app-ads.txt</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>2026-04-24 10:23 UTC</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>1054</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>#Infolinks</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Infolinks.com, 3444795, DIRECT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-04-26
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H271"/>
+  <dimension ref="A1:H281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -10897,6 +10897,374 @@
         </is>
       </c>
       <c r="H271" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="272" ht="15" customHeight="1">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-04-26 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E272" t="n">
+        <v>0</v>
+      </c>
+      <c r="F272" t="n">
+        <v>0</v>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="273" ht="15" customHeight="1">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-04-26 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E273" t="n">
+        <v>0</v>
+      </c>
+      <c r="F273" t="n">
+        <v>0</v>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="274" ht="15" customHeight="1">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-04-26 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E274" t="n">
+        <v>0</v>
+      </c>
+      <c r="F274" t="n">
+        <v>0</v>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="275" ht="15" customHeight="1">
+      <c r="A275" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-26 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="B275" s="6" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C275" s="6" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D275" s="6" t="inlineStr">
+        <is>
+          <t>Error: HTTPSConnectionPool(host='www.bbcamerica.com', port=443): Read timed out. (read timeout=15)</t>
+        </is>
+      </c>
+      <c r="E275" s="6" t="inlineStr"/>
+      <c r="F275" s="6" t="inlineStr"/>
+      <c r="G275" s="6" t="inlineStr"/>
+      <c r="H275" s="6" t="inlineStr"/>
+    </row>
+    <row r="276" ht="15" customHeight="1">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026-04-26 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E276" t="n">
+        <v>0</v>
+      </c>
+      <c r="F276" t="n">
+        <v>0</v>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="277" ht="15" customHeight="1">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026-04-26 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E277" t="n">
+        <v>0</v>
+      </c>
+      <c r="F277" t="n">
+        <v>0</v>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="278" ht="15" customHeight="1">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026-04-26 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E278" t="n">
+        <v>0</v>
+      </c>
+      <c r="F278" t="n">
+        <v>0</v>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="279" ht="15" customHeight="1">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-04-26 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E279" t="n">
+        <v>0</v>
+      </c>
+      <c r="F279" t="n">
+        <v>0</v>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="280" ht="15" customHeight="1">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026-04-26 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E280" t="n">
+        <v>0</v>
+      </c>
+      <c r="F280" t="n">
+        <v>0</v>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="281" ht="15" customHeight="1">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026-04-26 09:54 UTC</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E281" t="n">
+        <v>0</v>
+      </c>
+      <c r="F281" t="n">
+        <v>0</v>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -11341,7 +11709,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-25 09:54 UTC</t>
+          <t>2026-04-26 09:54 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -11366,7 +11734,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-04-25 09:54 UTC</t>
+          <t>2026-04-26 09:54 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -11391,7 +11759,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-04-25 09:54 UTC</t>
+          <t>2026-04-26 09:54 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -11416,7 +11784,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-25 09:54 UTC</t>
+          <t>2026-04-26 09:54 UTC</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -11443,7 +11811,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-04-25 09:54 UTC</t>
+          <t>2026-04-26 09:54 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -11468,7 +11836,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-04-25 09:54 UTC</t>
+          <t>2026-04-26 09:54 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -11493,7 +11861,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-04-25 09:54 UTC</t>
+          <t>2026-04-26 09:54 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -11518,7 +11886,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-04-25 09:54 UTC</t>
+          <t>2026-04-26 09:54 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -11543,7 +11911,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-25 09:54 UTC</t>
+          <t>2026-04-26 09:54 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -11568,7 +11936,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-25 09:54 UTC</t>
+          <t>2026-04-26 09:54 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">

</xml_diff>

<commit_message>
chore: update snapshots 2026-04-27
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H281"/>
+  <dimension ref="A1:H291"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -11265,6 +11265,386 @@
         </is>
       </c>
       <c r="H281" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="282" ht="15" customHeight="1">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026-04-27 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E282" t="n">
+        <v>0</v>
+      </c>
+      <c r="F282" t="n">
+        <v>0</v>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="283" ht="15" customHeight="1">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026-04-27 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E283" t="n">
+        <v>0</v>
+      </c>
+      <c r="F283" t="n">
+        <v>0</v>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="284" ht="15" customHeight="1">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-04-27 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E284" t="n">
+        <v>0</v>
+      </c>
+      <c r="F284" t="n">
+        <v>0</v>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="285" ht="15" customHeight="1">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-04-27 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E285" t="n">
+        <v>0</v>
+      </c>
+      <c r="F285" t="n">
+        <v>0</v>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="286" ht="15" customHeight="1">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026-04-27 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E286" t="n">
+        <v>0</v>
+      </c>
+      <c r="F286" t="n">
+        <v>0</v>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="287" ht="15" customHeight="1">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026-04-27 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E287" t="n">
+        <v>0</v>
+      </c>
+      <c r="F287" t="n">
+        <v>0</v>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="288" ht="15" customHeight="1">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026-04-27 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E288" t="n">
+        <v>0</v>
+      </c>
+      <c r="F288" t="n">
+        <v>0</v>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="289" ht="15" customHeight="1">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026-04-27 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E289" t="n">
+        <v>0</v>
+      </c>
+      <c r="F289" t="n">
+        <v>0</v>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="290" ht="15" customHeight="1">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-04-27 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E290" t="n">
+        <v>0</v>
+      </c>
+      <c r="F290" t="n">
+        <v>0</v>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="291" ht="15" customHeight="1">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026-04-27 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E291" t="n">
+        <v>0</v>
+      </c>
+      <c r="F291" t="n">
+        <v>0</v>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -11666,7 +12046,7 @@
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11709,7 +12089,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-26 09:54 UTC</t>
+          <t>2026-04-27 11:06 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -11734,7 +12114,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-04-26 09:54 UTC</t>
+          <t>2026-04-27 11:06 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -11759,7 +12139,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-04-26 09:54 UTC</t>
+          <t>2026-04-27 11:06 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -11784,17 +12164,15 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-26 09:54 UTC</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>Error: HTTPSConnectionPool(host='www.bbcamerica.com', port=443): Read timed out. (read timeout=15)</t>
+          <t>2026-04-27 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1054</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -11811,7 +12189,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-04-26 09:54 UTC</t>
+          <t>2026-04-27 11:06 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -11836,7 +12214,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-04-26 09:54 UTC</t>
+          <t>2026-04-27 11:06 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -11861,7 +12239,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-04-26 09:54 UTC</t>
+          <t>2026-04-27 11:06 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -11886,7 +12264,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-04-26 09:54 UTC</t>
+          <t>2026-04-27 11:06 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -11911,7 +12289,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-26 09:54 UTC</t>
+          <t>2026-04-27 11:06 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -11936,7 +12314,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-26 09:54 UTC</t>
+          <t>2026-04-27 11:06 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">

</xml_diff>

<commit_message>
chore: update snapshots 2026-04-28
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -8,17 +8,17 @@
   </bookViews>
   <sheets>
     <sheet name="Change Log" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="amc_com_ads_txt" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="amc_com_app-ads_txt" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="bbca_com_ads_txt" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="bbca_com_app-ads_txt" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ifc_com_ads_txt" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="ifc_com_app-ads_txt" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="sundancetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="wetv_com_ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="wetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="amc_com_ads_txt" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="amc_com_app-ads_txt" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="bbca_com_ads_txt" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="bbca_com_app-ads_txt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ifc_com_ads_txt" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ifc_com_app-ads_txt" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H291"/>
+  <dimension ref="A1:H301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -11645,6 +11645,362 @@
         </is>
       </c>
       <c r="H291" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="292" ht="15" customHeight="1">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-04-28 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E292" t="n">
+        <v>0</v>
+      </c>
+      <c r="F292" t="n">
+        <v>0</v>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="293" ht="15" customHeight="1">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-04-28 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E293" t="n">
+        <v>0</v>
+      </c>
+      <c r="F293" t="n">
+        <v>0</v>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="294" ht="15" customHeight="1">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-04-28 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E294" t="n">
+        <v>0</v>
+      </c>
+      <c r="F294" t="n">
+        <v>0</v>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="295" ht="15" customHeight="1">
+      <c r="A295" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-28 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B295" s="6" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C295" s="6" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D295" s="6" t="inlineStr">
+        <is>
+          <t>Error: HTTPSConnectionPool(host='www.bbcamerica.com', port=443): Read timed out. (read timeout=15)</t>
+        </is>
+      </c>
+      <c r="E295" s="6" t="inlineStr"/>
+      <c r="F295" s="6" t="inlineStr"/>
+      <c r="G295" s="6" t="inlineStr"/>
+      <c r="H295" s="6" t="inlineStr"/>
+    </row>
+    <row r="296" ht="15" customHeight="1">
+      <c r="A296" s="6" t="inlineStr">
+        <is>
+          <t>2026-04-28 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B296" s="6" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C296" s="6" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D296" s="6" t="inlineStr">
+        <is>
+          <t>Error: HTTPSConnectionPool(host='www.ifc.com', port=443): Read timed out. (read timeout=15)</t>
+        </is>
+      </c>
+      <c r="E296" s="6" t="inlineStr"/>
+      <c r="F296" s="6" t="inlineStr"/>
+      <c r="G296" s="6" t="inlineStr"/>
+      <c r="H296" s="6" t="inlineStr"/>
+    </row>
+    <row r="297" ht="15" customHeight="1">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026-04-28 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E297" t="n">
+        <v>0</v>
+      </c>
+      <c r="F297" t="n">
+        <v>0</v>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="298" ht="15" customHeight="1">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026-04-28 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E298" t="n">
+        <v>0</v>
+      </c>
+      <c r="F298" t="n">
+        <v>0</v>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="299" ht="15" customHeight="1">
+      <c r="A299" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-28 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B299" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C299" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D299" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E299" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F299" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G299" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.efd59aa2891eed23b550.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f8a313db7b6c5381dc3b.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H299" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9c76d463468b2ab9e0fd.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.72a4cbf72571ebffd265.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="300" ht="15" customHeight="1">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2026-04-28 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E300" t="n">
+        <v>0</v>
+      </c>
+      <c r="F300" t="n">
+        <v>0</v>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="301" ht="15" customHeight="1">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2026-04-28 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E301" t="n">
+        <v>0</v>
+      </c>
+      <c r="F301" t="n">
+        <v>0</v>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -11850,195 +12206,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>#Wurl</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>wurl.com, 55562, DIRECT</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, sg1303005, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709-r-523319, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>#Olyzon</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 167424, RESELLER, 5d62403b186f2ace</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>#Olyzon</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>olyzon.tv, 76794, PUBLISHER</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>#Nexxen</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>lkqd.net, 1100060088, RESELLER 59c49fa9598a0117</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>#Infolinks</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Infolinks.com, 3444795, DIRECT</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -12046,7 +12213,7 @@
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12089,7 +12256,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-27 11:06 UTC</t>
+          <t>2026-04-28 11:06 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -12114,7 +12281,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-04-27 11:06 UTC</t>
+          <t>2026-04-28 11:06 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -12139,7 +12306,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-04-27 11:06 UTC</t>
+          <t>2026-04-28 11:06 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -12164,15 +12331,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-27 11:06 UTC</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>1054</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>OK</t>
+          <t>2026-04-28 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Error: HTTPSConnectionPool(host='www.bbcamerica.com', port=443): Read timed out. (read timeout=15)</t>
         </is>
       </c>
     </row>
@@ -12189,15 +12358,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-04-27 11:06 UTC</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>1140</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>OK</t>
+          <t>2026-04-28 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Error: HTTPSConnectionPool(host='www.ifc.com', port=443): Read timed out. (read timeout=15)</t>
         </is>
       </c>
     </row>
@@ -12214,7 +12385,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-04-27 11:06 UTC</t>
+          <t>2026-04-28 11:06 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -12239,7 +12410,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-04-27 11:06 UTC</t>
+          <t>2026-04-28 11:06 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -12264,7 +12435,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-04-27 11:06 UTC</t>
+          <t>2026-04-28 11:06 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -12289,7 +12460,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-27 11:06 UTC</t>
+          <t>2026-04-28 11:06 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -12314,7 +12485,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-27 11:06 UTC</t>
+          <t>2026-04-28 11:06 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -12331,7 +12502,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12375,7 +12546,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9c76d463468b2ab9e0fd.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.72a4cbf72571ebffd265.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.efd59aa2891eed23b550.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f8a313db7b6c5381dc3b.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -12392,7 +12563,196 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.3aa44342103b9d642241.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.bdc09c5683feee7ef5cb.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.8ccc1f017d7b94cfd357.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9c76d463468b2ab9e0fd.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.72a4cbf72571ebffd265.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>#Wurl</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>wurl.com, 55562, DIRECT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>#PrismRiot</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 543709, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>#PrismRiot</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, sg1303005, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>#PrismRiot</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 543709-r-523319, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>#PrismRiot</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 543709-r-524565, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>#Olyzon</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>pubmatic.com, 167424, RESELLER, 5d62403b186f2ace</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>#Olyzon</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>olyzon.tv, 76794, PUBLISHER</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>#Nexxen</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>lkqd.net, 1100060088, RESELLER 59c49fa9598a0117</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>#Infolinks</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Infolinks.com, 3444795, DIRECT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-04-29
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H301"/>
+  <dimension ref="A1:H311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -12001,6 +12001,386 @@
         </is>
       </c>
       <c r="H301" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="302" ht="15" customHeight="1">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:58 UTC</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E302" t="n">
+        <v>0</v>
+      </c>
+      <c r="F302" t="n">
+        <v>0</v>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="303" ht="15" customHeight="1">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:58 UTC</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E303" t="n">
+        <v>0</v>
+      </c>
+      <c r="F303" t="n">
+        <v>0</v>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="304" ht="15" customHeight="1">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:58 UTC</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E304" t="n">
+        <v>0</v>
+      </c>
+      <c r="F304" t="n">
+        <v>0</v>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="305" ht="15" customHeight="1">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:58 UTC</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E305" t="n">
+        <v>0</v>
+      </c>
+      <c r="F305" t="n">
+        <v>0</v>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="306" ht="15" customHeight="1">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:58 UTC</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E306" t="n">
+        <v>0</v>
+      </c>
+      <c r="F306" t="n">
+        <v>0</v>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="307" ht="15" customHeight="1">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:58 UTC</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E307" t="n">
+        <v>0</v>
+      </c>
+      <c r="F307" t="n">
+        <v>0</v>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="308" ht="15" customHeight="1">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:58 UTC</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E308" t="n">
+        <v>0</v>
+      </c>
+      <c r="F308" t="n">
+        <v>0</v>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="309" ht="15" customHeight="1">
+      <c r="A309" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:58 UTC</t>
+        </is>
+      </c>
+      <c r="B309" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C309" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D309" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E309" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F309" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G309" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8b7a782ded1310fc1510.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H309" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.efd59aa2891eed23b550.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f8a313db7b6c5381dc3b.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="310" ht="15" customHeight="1">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:58 UTC</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E310" t="n">
+        <v>0</v>
+      </c>
+      <c r="F310" t="n">
+        <v>0</v>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="311" ht="15" customHeight="1">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2026-04-29 10:58 UTC</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E311" t="n">
+        <v>0</v>
+      </c>
+      <c r="F311" t="n">
+        <v>0</v>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -12213,7 +12593,7 @@
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12256,7 +12636,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-28 11:06 UTC</t>
+          <t>2026-04-29 10:58 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -12281,7 +12661,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-04-28 11:06 UTC</t>
+          <t>2026-04-29 10:58 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -12306,7 +12686,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-04-28 11:06 UTC</t>
+          <t>2026-04-29 10:58 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -12331,17 +12711,15 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-28 11:06 UTC</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>Error: HTTPSConnectionPool(host='www.bbcamerica.com', port=443): Read timed out. (read timeout=15)</t>
+          <t>2026-04-29 10:58 UTC</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1054</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -12358,17 +12736,15 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-04-28 11:06 UTC</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>Error: HTTPSConnectionPool(host='www.ifc.com', port=443): Read timed out. (read timeout=15)</t>
+          <t>2026-04-29 10:58 UTC</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1140</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -12385,7 +12761,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-04-28 11:06 UTC</t>
+          <t>2026-04-29 10:58 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -12410,7 +12786,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-04-28 11:06 UTC</t>
+          <t>2026-04-29 10:58 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -12435,7 +12811,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-04-28 11:06 UTC</t>
+          <t>2026-04-29 10:58 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -12460,7 +12836,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-28 11:06 UTC</t>
+          <t>2026-04-29 10:58 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -12485,7 +12861,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-28 11:06 UTC</t>
+          <t>2026-04-29 10:58 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -12546,7 +12922,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.efd59aa2891eed23b550.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f8a313db7b6c5381dc3b.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8b7a782ded1310fc1510.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -12563,7 +12939,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.2bad9518e36a64fbd660.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.1aa8db3a9f0ea808a97d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/5790.7dd733e2fbc9888192e3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9c76d463468b2ab9e0fd.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/5790.27446ca8abbfc55c5698.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.72a4cbf72571ebffd265.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.efd59aa2891eed23b550.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f8a313db7b6c5381dc3b.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-04-30
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H311"/>
+  <dimension ref="A1:H321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -12381,6 +12381,386 @@
         </is>
       </c>
       <c r="H311" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="312" ht="15" customHeight="1">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:56 UTC</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E312" t="n">
+        <v>0</v>
+      </c>
+      <c r="F312" t="n">
+        <v>0</v>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="313" ht="15" customHeight="1">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:56 UTC</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E313" t="n">
+        <v>0</v>
+      </c>
+      <c r="F313" t="n">
+        <v>0</v>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="314" ht="15" customHeight="1">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:56 UTC</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E314" t="n">
+        <v>0</v>
+      </c>
+      <c r="F314" t="n">
+        <v>0</v>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="315" ht="15" customHeight="1">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:56 UTC</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E315" t="n">
+        <v>0</v>
+      </c>
+      <c r="F315" t="n">
+        <v>0</v>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="316" ht="15" customHeight="1">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:56 UTC</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E316" t="n">
+        <v>0</v>
+      </c>
+      <c r="F316" t="n">
+        <v>0</v>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="317" ht="15" customHeight="1">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:56 UTC</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E317" t="n">
+        <v>0</v>
+      </c>
+      <c r="F317" t="n">
+        <v>0</v>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="318" ht="15" customHeight="1">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:56 UTC</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E318" t="n">
+        <v>0</v>
+      </c>
+      <c r="F318" t="n">
+        <v>0</v>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="319" ht="15" customHeight="1">
+      <c r="A319" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:56 UTC</t>
+        </is>
+      </c>
+      <c r="B319" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C319" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D319" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E319" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F319" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G319" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9ce82bb4d750a524c082.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H319" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8b7a782ded1310fc1510.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="320" ht="15" customHeight="1">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:56 UTC</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E320" t="n">
+        <v>0</v>
+      </c>
+      <c r="F320" t="n">
+        <v>0</v>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="321" ht="15" customHeight="1">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2026-04-30 10:56 UTC</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E321" t="n">
+        <v>0</v>
+      </c>
+      <c r="F321" t="n">
+        <v>0</v>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -12636,7 +13016,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-29 10:58 UTC</t>
+          <t>2026-04-30 10:56 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -12661,7 +13041,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-04-29 10:58 UTC</t>
+          <t>2026-04-30 10:56 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -12686,7 +13066,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-04-29 10:58 UTC</t>
+          <t>2026-04-30 10:56 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -12711,7 +13091,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-29 10:58 UTC</t>
+          <t>2026-04-30 10:56 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -12736,7 +13116,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-04-29 10:58 UTC</t>
+          <t>2026-04-30 10:56 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -12761,7 +13141,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-04-29 10:58 UTC</t>
+          <t>2026-04-30 10:56 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -12786,7 +13166,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-04-29 10:58 UTC</t>
+          <t>2026-04-30 10:56 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -12811,7 +13191,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-04-29 10:58 UTC</t>
+          <t>2026-04-30 10:56 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -12836,7 +13216,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-29 10:58 UTC</t>
+          <t>2026-04-30 10:56 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -12861,7 +13241,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-29 10:58 UTC</t>
+          <t>2026-04-30 10:56 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -12922,7 +13302,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8b7a782ded1310fc1510.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9ce82bb4d750a524c082.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -12939,7 +13319,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.efd59aa2891eed23b550.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f8a313db7b6c5381dc3b.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8b7a782ded1310fc1510.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-01
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H321"/>
+  <dimension ref="A1:H331"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -12761,6 +12761,386 @@
         </is>
       </c>
       <c r="H321" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="322" ht="15" customHeight="1">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026-05-01 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E322" t="n">
+        <v>0</v>
+      </c>
+      <c r="F322" t="n">
+        <v>0</v>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="323" ht="15" customHeight="1">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2026-05-01 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E323" t="n">
+        <v>0</v>
+      </c>
+      <c r="F323" t="n">
+        <v>0</v>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="324" ht="15" customHeight="1">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2026-05-01 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E324" t="n">
+        <v>0</v>
+      </c>
+      <c r="F324" t="n">
+        <v>0</v>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="325" ht="15" customHeight="1">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2026-05-01 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E325" t="n">
+        <v>0</v>
+      </c>
+      <c r="F325" t="n">
+        <v>0</v>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="326" ht="15" customHeight="1">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2026-05-01 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E326" t="n">
+        <v>0</v>
+      </c>
+      <c r="F326" t="n">
+        <v>0</v>
+      </c>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="327" ht="15" customHeight="1">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>2026-05-01 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E327" t="n">
+        <v>0</v>
+      </c>
+      <c r="F327" t="n">
+        <v>0</v>
+      </c>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="328" ht="15" customHeight="1">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>2026-05-01 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E328" t="n">
+        <v>0</v>
+      </c>
+      <c r="F328" t="n">
+        <v>0</v>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="329" ht="15" customHeight="1">
+      <c r="A329" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-01 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B329" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C329" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D329" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E329" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F329" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G329" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d162a07c451f872b6951.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H329" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9ce82bb4d750a524c082.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="330" ht="15" customHeight="1">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2026-05-01 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E330" t="n">
+        <v>0</v>
+      </c>
+      <c r="F330" t="n">
+        <v>0</v>
+      </c>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="331" ht="15" customHeight="1">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>2026-05-01 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E331" t="n">
+        <v>0</v>
+      </c>
+      <c r="F331" t="n">
+        <v>0</v>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H331" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -13016,7 +13396,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-04-30 10:56 UTC</t>
+          <t>2026-05-01 10:23 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -13041,7 +13421,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-04-30 10:56 UTC</t>
+          <t>2026-05-01 10:23 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -13066,7 +13446,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-04-30 10:56 UTC</t>
+          <t>2026-05-01 10:23 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -13091,7 +13471,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-30 10:56 UTC</t>
+          <t>2026-05-01 10:23 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -13116,7 +13496,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-04-30 10:56 UTC</t>
+          <t>2026-05-01 10:23 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -13141,7 +13521,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-04-30 10:56 UTC</t>
+          <t>2026-05-01 10:23 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -13166,7 +13546,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-04-30 10:56 UTC</t>
+          <t>2026-05-01 10:23 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -13191,7 +13571,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-04-30 10:56 UTC</t>
+          <t>2026-05-01 10:23 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -13216,7 +13596,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-04-30 10:56 UTC</t>
+          <t>2026-05-01 10:23 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -13241,7 +13621,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-04-30 10:56 UTC</t>
+          <t>2026-05-01 10:23 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -13302,7 +13682,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9ce82bb4d750a524c082.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d162a07c451f872b6951.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -13319,7 +13699,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8b7a782ded1310fc1510.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9ce82bb4d750a524c082.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-02
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H331"/>
+  <dimension ref="A1:H341"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -13141,6 +13141,386 @@
         </is>
       </c>
       <c r="H331" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="332" ht="15" customHeight="1">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>2026-05-02 09:59 UTC</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E332" t="n">
+        <v>0</v>
+      </c>
+      <c r="F332" t="n">
+        <v>0</v>
+      </c>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="333" ht="15" customHeight="1">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>2026-05-02 09:59 UTC</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E333" t="n">
+        <v>0</v>
+      </c>
+      <c r="F333" t="n">
+        <v>0</v>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="334" ht="15" customHeight="1">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>2026-05-02 09:59 UTC</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E334" t="n">
+        <v>0</v>
+      </c>
+      <c r="F334" t="n">
+        <v>0</v>
+      </c>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="335" ht="15" customHeight="1">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>2026-05-02 09:59 UTC</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E335" t="n">
+        <v>0</v>
+      </c>
+      <c r="F335" t="n">
+        <v>0</v>
+      </c>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="336" ht="15" customHeight="1">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>2026-05-02 09:59 UTC</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E336" t="n">
+        <v>0</v>
+      </c>
+      <c r="F336" t="n">
+        <v>0</v>
+      </c>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="337" ht="15" customHeight="1">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>2026-05-02 09:59 UTC</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E337" t="n">
+        <v>0</v>
+      </c>
+      <c r="F337" t="n">
+        <v>0</v>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="338" ht="15" customHeight="1">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>2026-05-02 09:59 UTC</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E338" t="n">
+        <v>0</v>
+      </c>
+      <c r="F338" t="n">
+        <v>0</v>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="339" ht="15" customHeight="1">
+      <c r="A339" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-02 09:59 UTC</t>
+        </is>
+      </c>
+      <c r="B339" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C339" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D339" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E339" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F339" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G339" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.6f77781eb84d891a42f0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H339" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d162a07c451f872b6951.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="340" ht="15" customHeight="1">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>2026-05-02 09:59 UTC</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E340" t="n">
+        <v>0</v>
+      </c>
+      <c r="F340" t="n">
+        <v>0</v>
+      </c>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="341" ht="15" customHeight="1">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>2026-05-02 09:59 UTC</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E341" t="n">
+        <v>0</v>
+      </c>
+      <c r="F341" t="n">
+        <v>0</v>
+      </c>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H341" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -13396,7 +13776,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-01 10:23 UTC</t>
+          <t>2026-05-02 09:59 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -13421,7 +13801,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-01 10:23 UTC</t>
+          <t>2026-05-02 09:59 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -13446,7 +13826,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-01 10:23 UTC</t>
+          <t>2026-05-02 09:59 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -13471,7 +13851,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-01 10:23 UTC</t>
+          <t>2026-05-02 09:59 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -13496,7 +13876,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-01 10:23 UTC</t>
+          <t>2026-05-02 09:59 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -13521,7 +13901,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-01 10:23 UTC</t>
+          <t>2026-05-02 09:59 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -13546,7 +13926,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-01 10:23 UTC</t>
+          <t>2026-05-02 09:59 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -13571,7 +13951,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-01 10:23 UTC</t>
+          <t>2026-05-02 09:59 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -13596,7 +13976,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-01 10:23 UTC</t>
+          <t>2026-05-02 09:59 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -13621,7 +14001,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-01 10:23 UTC</t>
+          <t>2026-05-02 09:59 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -13682,7 +14062,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d162a07c451f872b6951.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.6f77781eb84d891a42f0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -13699,7 +14079,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9ce82bb4d750a524c082.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d162a07c451f872b6951.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-03
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H341"/>
+  <dimension ref="A1:H351"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -13521,6 +13521,386 @@
         </is>
       </c>
       <c r="H341" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="342" ht="15" customHeight="1">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>2026-05-03 10:06 UTC</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E342" t="n">
+        <v>0</v>
+      </c>
+      <c r="F342" t="n">
+        <v>0</v>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="343" ht="15" customHeight="1">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>2026-05-03 10:06 UTC</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E343" t="n">
+        <v>0</v>
+      </c>
+      <c r="F343" t="n">
+        <v>0</v>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="344" ht="15" customHeight="1">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>2026-05-03 10:06 UTC</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E344" t="n">
+        <v>0</v>
+      </c>
+      <c r="F344" t="n">
+        <v>0</v>
+      </c>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="345" ht="15" customHeight="1">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>2026-05-03 10:06 UTC</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E345" t="n">
+        <v>0</v>
+      </c>
+      <c r="F345" t="n">
+        <v>0</v>
+      </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="346" ht="15" customHeight="1">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>2026-05-03 10:06 UTC</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E346" t="n">
+        <v>0</v>
+      </c>
+      <c r="F346" t="n">
+        <v>0</v>
+      </c>
+      <c r="G346" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="347" ht="15" customHeight="1">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>2026-05-03 10:06 UTC</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E347" t="n">
+        <v>0</v>
+      </c>
+      <c r="F347" t="n">
+        <v>0</v>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="348" ht="15" customHeight="1">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>2026-05-03 10:06 UTC</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E348" t="n">
+        <v>0</v>
+      </c>
+      <c r="F348" t="n">
+        <v>0</v>
+      </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="349" ht="15" customHeight="1">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>2026-05-03 10:06 UTC</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E349" t="n">
+        <v>0</v>
+      </c>
+      <c r="F349" t="n">
+        <v>0</v>
+      </c>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="350" ht="15" customHeight="1">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>2026-05-03 10:06 UTC</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E350" t="n">
+        <v>0</v>
+      </c>
+      <c r="F350" t="n">
+        <v>0</v>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="351" ht="15" customHeight="1">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2026-05-03 10:06 UTC</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E351" t="n">
+        <v>0</v>
+      </c>
+      <c r="F351" t="n">
+        <v>0</v>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -13726,6 +14106,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.6f77781eb84d891a42f0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d162a07c451f872b6951.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -13776,7 +14226,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-02 09:59 UTC</t>
+          <t>2026-05-03 10:06 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -13801,7 +14251,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-02 09:59 UTC</t>
+          <t>2026-05-03 10:06 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -13826,7 +14276,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-02 09:59 UTC</t>
+          <t>2026-05-03 10:06 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -13851,7 +14301,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-02 09:59 UTC</t>
+          <t>2026-05-03 10:06 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -13876,7 +14326,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-02 09:59 UTC</t>
+          <t>2026-05-03 10:06 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -13901,7 +14351,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-02 09:59 UTC</t>
+          <t>2026-05-03 10:06 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -13926,7 +14376,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-02 09:59 UTC</t>
+          <t>2026-05-03 10:06 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -13951,7 +14401,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-02 09:59 UTC</t>
+          <t>2026-05-03 10:06 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -13976,7 +14426,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-02 09:59 UTC</t>
+          <t>2026-05-03 10:06 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -14001,7 +14451,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-02 09:59 UTC</t>
+          <t>2026-05-03 10:06 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -14010,76 +14460,6 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.6f77781eb84d891a42f0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d162a07c451f872b6951.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-04
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H351"/>
+  <dimension ref="A1:H361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -13901,6 +13901,386 @@
         </is>
       </c>
       <c r="H351" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="352" ht="15" customHeight="1">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2026-05-04 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E352" t="n">
+        <v>0</v>
+      </c>
+      <c r="F352" t="n">
+        <v>0</v>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="353" ht="15" customHeight="1">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2026-05-04 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E353" t="n">
+        <v>0</v>
+      </c>
+      <c r="F353" t="n">
+        <v>0</v>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="354" ht="15" customHeight="1">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>2026-05-04 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E354" t="n">
+        <v>0</v>
+      </c>
+      <c r="F354" t="n">
+        <v>0</v>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="355" ht="15" customHeight="1">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2026-05-04 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E355" t="n">
+        <v>0</v>
+      </c>
+      <c r="F355" t="n">
+        <v>0</v>
+      </c>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="356" ht="15" customHeight="1">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>2026-05-04 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E356" t="n">
+        <v>0</v>
+      </c>
+      <c r="F356" t="n">
+        <v>0</v>
+      </c>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H356" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="357" ht="15" customHeight="1">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>2026-05-04 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E357" t="n">
+        <v>0</v>
+      </c>
+      <c r="F357" t="n">
+        <v>0</v>
+      </c>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H357" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="358" ht="15" customHeight="1">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>2026-05-04 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E358" t="n">
+        <v>0</v>
+      </c>
+      <c r="F358" t="n">
+        <v>0</v>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="359" ht="15" customHeight="1">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>2026-05-04 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E359" t="n">
+        <v>0</v>
+      </c>
+      <c r="F359" t="n">
+        <v>0</v>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="360" ht="15" customHeight="1">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>2026-05-04 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E360" t="n">
+        <v>0</v>
+      </c>
+      <c r="F360" t="n">
+        <v>0</v>
+      </c>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="361" ht="15" customHeight="1">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>2026-05-04 11:06 UTC</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E361" t="n">
+        <v>0</v>
+      </c>
+      <c r="F361" t="n">
+        <v>0</v>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H361" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -14226,7 +14606,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-03 10:06 UTC</t>
+          <t>2026-05-04 11:06 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -14251,7 +14631,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-03 10:06 UTC</t>
+          <t>2026-05-04 11:06 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -14276,7 +14656,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-03 10:06 UTC</t>
+          <t>2026-05-04 11:06 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -14301,7 +14681,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-03 10:06 UTC</t>
+          <t>2026-05-04 11:06 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -14326,7 +14706,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-03 10:06 UTC</t>
+          <t>2026-05-04 11:06 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -14351,7 +14731,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-03 10:06 UTC</t>
+          <t>2026-05-04 11:06 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -14376,7 +14756,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-03 10:06 UTC</t>
+          <t>2026-05-04 11:06 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -14401,7 +14781,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-03 10:06 UTC</t>
+          <t>2026-05-04 11:06 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -14426,7 +14806,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-03 10:06 UTC</t>
+          <t>2026-05-04 11:06 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -14451,7 +14831,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-03 10:06 UTC</t>
+          <t>2026-05-04 11:06 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-05
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H361"/>
+  <dimension ref="A1:H371"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -14281,6 +14281,386 @@
         </is>
       </c>
       <c r="H361" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="362" ht="15" customHeight="1">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>2026-05-05 10:47 UTC</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E362" t="n">
+        <v>0</v>
+      </c>
+      <c r="F362" t="n">
+        <v>0</v>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="363" ht="15" customHeight="1">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>2026-05-05 10:47 UTC</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E363" t="n">
+        <v>0</v>
+      </c>
+      <c r="F363" t="n">
+        <v>0</v>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="364" ht="15" customHeight="1">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>2026-05-05 10:47 UTC</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E364" t="n">
+        <v>0</v>
+      </c>
+      <c r="F364" t="n">
+        <v>0</v>
+      </c>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="365" ht="15" customHeight="1">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2026-05-05 10:47 UTC</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E365" t="n">
+        <v>0</v>
+      </c>
+      <c r="F365" t="n">
+        <v>0</v>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="366" ht="15" customHeight="1">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2026-05-05 10:47 UTC</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E366" t="n">
+        <v>0</v>
+      </c>
+      <c r="F366" t="n">
+        <v>0</v>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="367" ht="15" customHeight="1">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2026-05-05 10:47 UTC</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E367" t="n">
+        <v>0</v>
+      </c>
+      <c r="F367" t="n">
+        <v>0</v>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H367" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="368" ht="15" customHeight="1">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2026-05-05 10:47 UTC</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E368" t="n">
+        <v>0</v>
+      </c>
+      <c r="F368" t="n">
+        <v>0</v>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="369" ht="15" customHeight="1">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2026-05-05 10:47 UTC</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E369" t="n">
+        <v>0</v>
+      </c>
+      <c r="F369" t="n">
+        <v>0</v>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="370" ht="15" customHeight="1">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2026-05-05 10:47 UTC</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E370" t="n">
+        <v>0</v>
+      </c>
+      <c r="F370" t="n">
+        <v>0</v>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="371" ht="15" customHeight="1">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026-05-05 10:47 UTC</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E371" t="n">
+        <v>0</v>
+      </c>
+      <c r="F371" t="n">
+        <v>0</v>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H371" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -14606,7 +14986,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-04 11:06 UTC</t>
+          <t>2026-05-05 10:47 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -14631,7 +15011,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-04 11:06 UTC</t>
+          <t>2026-05-05 10:47 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -14656,7 +15036,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-04 11:06 UTC</t>
+          <t>2026-05-05 10:47 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -14681,7 +15061,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-04 11:06 UTC</t>
+          <t>2026-05-05 10:47 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -14706,7 +15086,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-04 11:06 UTC</t>
+          <t>2026-05-05 10:47 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -14731,7 +15111,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-04 11:06 UTC</t>
+          <t>2026-05-05 10:47 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -14756,7 +15136,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-04 11:06 UTC</t>
+          <t>2026-05-05 10:47 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -14781,7 +15161,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-04 11:06 UTC</t>
+          <t>2026-05-05 10:47 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -14806,7 +15186,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-04 11:06 UTC</t>
+          <t>2026-05-05 10:47 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -14831,7 +15211,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-04 11:06 UTC</t>
+          <t>2026-05-05 10:47 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-06
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H371"/>
+  <dimension ref="A1:H381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -14661,6 +14661,386 @@
         </is>
       </c>
       <c r="H371" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="372" ht="15" customHeight="1">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026-05-06 11:08 UTC</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E372" t="n">
+        <v>0</v>
+      </c>
+      <c r="F372" t="n">
+        <v>0</v>
+      </c>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H372" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="373" ht="15" customHeight="1">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2026-05-06 11:08 UTC</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E373" t="n">
+        <v>0</v>
+      </c>
+      <c r="F373" t="n">
+        <v>0</v>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="374" ht="15" customHeight="1">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2026-05-06 11:08 UTC</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E374" t="n">
+        <v>0</v>
+      </c>
+      <c r="F374" t="n">
+        <v>0</v>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="375" ht="15" customHeight="1">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2026-05-06 11:08 UTC</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E375" t="n">
+        <v>0</v>
+      </c>
+      <c r="F375" t="n">
+        <v>0</v>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="376" ht="15" customHeight="1">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2026-05-06 11:08 UTC</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E376" t="n">
+        <v>0</v>
+      </c>
+      <c r="F376" t="n">
+        <v>0</v>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="377" ht="15" customHeight="1">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2026-05-06 11:08 UTC</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E377" t="n">
+        <v>0</v>
+      </c>
+      <c r="F377" t="n">
+        <v>0</v>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="378" ht="15" customHeight="1">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2026-05-06 11:08 UTC</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E378" t="n">
+        <v>0</v>
+      </c>
+      <c r="F378" t="n">
+        <v>0</v>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="379" ht="15" customHeight="1">
+      <c r="A379" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-06 11:08 UTC</t>
+        </is>
+      </c>
+      <c r="B379" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C379" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D379" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E379" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F379" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G379" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.3f52521020997bbfb2bb.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H379" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.6f77781eb84d891a42f0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="380" ht="15" customHeight="1">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-05-06 11:08 UTC</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E380" t="n">
+        <v>0</v>
+      </c>
+      <c r="F380" t="n">
+        <v>0</v>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="381" ht="15" customHeight="1">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-05-06 11:08 UTC</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E381" t="n">
+        <v>0</v>
+      </c>
+      <c r="F381" t="n">
+        <v>0</v>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -14866,76 +15246,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.6f77781eb84d891a42f0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d162a07c451f872b6951.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -14986,7 +15296,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-05 10:47 UTC</t>
+          <t>2026-05-06 11:08 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -15011,7 +15321,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-05 10:47 UTC</t>
+          <t>2026-05-06 11:08 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -15036,7 +15346,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-05 10:47 UTC</t>
+          <t>2026-05-06 11:08 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -15061,7 +15371,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-05 10:47 UTC</t>
+          <t>2026-05-06 11:08 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -15086,7 +15396,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-05 10:47 UTC</t>
+          <t>2026-05-06 11:08 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -15111,7 +15421,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-05 10:47 UTC</t>
+          <t>2026-05-06 11:08 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -15136,7 +15446,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-05 10:47 UTC</t>
+          <t>2026-05-06 11:08 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -15161,7 +15471,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-05 10:47 UTC</t>
+          <t>2026-05-06 11:08 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -15186,7 +15496,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-05 10:47 UTC</t>
+          <t>2026-05-06 11:08 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -15211,7 +15521,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-05 10:47 UTC</t>
+          <t>2026-05-06 11:08 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -15220,6 +15530,76 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.3f52521020997bbfb2bb.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.6f77781eb84d891a42f0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-07
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H381"/>
+  <dimension ref="A1:H391"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -15041,6 +15041,350 @@
         </is>
       </c>
       <c r="H381" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="382" ht="15" customHeight="1">
+      <c r="A382" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-07 11:09 UTC</t>
+        </is>
+      </c>
+      <c r="B382" s="6" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C382" s="6" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D382" s="6" t="inlineStr">
+        <is>
+          <t>Error: HTTPSConnectionPool(host='www.amc.com', port=443): Read timed out. (read timeout=15)</t>
+        </is>
+      </c>
+      <c r="E382" s="6" t="inlineStr"/>
+      <c r="F382" s="6" t="inlineStr"/>
+      <c r="G382" s="6" t="inlineStr"/>
+      <c r="H382" s="6" t="inlineStr"/>
+    </row>
+    <row r="383" ht="15" customHeight="1">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2026-05-07 11:09 UTC</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E383" t="n">
+        <v>0</v>
+      </c>
+      <c r="F383" t="n">
+        <v>0</v>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="384" ht="15" customHeight="1">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2026-05-07 11:09 UTC</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E384" t="n">
+        <v>0</v>
+      </c>
+      <c r="F384" t="n">
+        <v>0</v>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="385" ht="15" customHeight="1">
+      <c r="A385" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-07 11:09 UTC</t>
+        </is>
+      </c>
+      <c r="B385" s="6" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C385" s="6" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D385" s="6" t="inlineStr">
+        <is>
+          <t>Error: HTTPSConnectionPool(host='www.bbcamerica.com', port=443): Read timed out. (read timeout=15)</t>
+        </is>
+      </c>
+      <c r="E385" s="6" t="inlineStr"/>
+      <c r="F385" s="6" t="inlineStr"/>
+      <c r="G385" s="6" t="inlineStr"/>
+      <c r="H385" s="6" t="inlineStr"/>
+    </row>
+    <row r="386" ht="15" customHeight="1">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2026-05-07 11:09 UTC</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E386" t="n">
+        <v>0</v>
+      </c>
+      <c r="F386" t="n">
+        <v>0</v>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="387" ht="15" customHeight="1">
+      <c r="A387" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-07 11:09 UTC</t>
+        </is>
+      </c>
+      <c r="B387" s="6" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C387" s="6" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D387" s="6" t="inlineStr">
+        <is>
+          <t>Error: HTTPSConnectionPool(host='www.ifc.com', port=443): Read timed out. (read timeout=15)</t>
+        </is>
+      </c>
+      <c r="E387" s="6" t="inlineStr"/>
+      <c r="F387" s="6" t="inlineStr"/>
+      <c r="G387" s="6" t="inlineStr"/>
+      <c r="H387" s="6" t="inlineStr"/>
+    </row>
+    <row r="388" ht="15" customHeight="1">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>2026-05-07 11:09 UTC</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E388" t="n">
+        <v>0</v>
+      </c>
+      <c r="F388" t="n">
+        <v>0</v>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="389" ht="15" customHeight="1">
+      <c r="A389" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07 11:09 UTC</t>
+        </is>
+      </c>
+      <c r="B389" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C389" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D389" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E389" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F389" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G389" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.ee80b25e8811396367cc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.69f230c0871da659cfdc.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H389" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.3f52521020997bbfb2bb.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="390" ht="15" customHeight="1">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>2026-05-07 11:09 UTC</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E390" t="n">
+        <v>0</v>
+      </c>
+      <c r="F390" t="n">
+        <v>0</v>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="391" ht="15" customHeight="1">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2026-05-07 11:09 UTC</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E391" t="n">
+        <v>0</v>
+      </c>
+      <c r="F391" t="n">
+        <v>0</v>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -15253,7 +15597,7 @@
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -15296,15 +15640,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-06 11:08 UTC</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>1140</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>OK</t>
+          <t>2026-05-07 11:09 UTC</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Error: HTTPSConnectionPool(host='www.amc.com', port=443): Read timed out. (read timeout=15)</t>
         </is>
       </c>
     </row>
@@ -15321,7 +15667,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-06 11:08 UTC</t>
+          <t>2026-05-07 11:09 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -15346,7 +15692,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-06 11:08 UTC</t>
+          <t>2026-05-07 11:09 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -15371,15 +15717,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-06 11:08 UTC</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>1054</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>OK</t>
+          <t>2026-05-07 11:09 UTC</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Error: HTTPSConnectionPool(host='www.bbcamerica.com', port=443): Read timed out. (read timeout=15)</t>
         </is>
       </c>
     </row>
@@ -15396,7 +15744,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-06 11:08 UTC</t>
+          <t>2026-05-07 11:09 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -15421,15 +15769,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-06 11:08 UTC</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>1054</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>OK</t>
+          <t>2026-05-07 11:09 UTC</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Error: HTTPSConnectionPool(host='www.ifc.com', port=443): Read timed out. (read timeout=15)</t>
         </is>
       </c>
     </row>
@@ -15446,7 +15796,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-06 11:08 UTC</t>
+          <t>2026-05-07 11:09 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -15471,7 +15821,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-06 11:08 UTC</t>
+          <t>2026-05-07 11:09 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -15496,7 +15846,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-06 11:08 UTC</t>
+          <t>2026-05-07 11:09 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -15521,7 +15871,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-06 11:08 UTC</t>
+          <t>2026-05-07 11:09 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -15582,7 +15932,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.3f52521020997bbfb2bb.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.ee80b25e8811396367cc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.69f230c0871da659cfdc.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -15599,7 +15949,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.6f77781eb84d891a42f0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.edc423e48fbc8ecb5630.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.3f52521020997bbfb2bb.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-08
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H391"/>
+  <dimension ref="A1:H401"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -15385,6 +15385,374 @@
         </is>
       </c>
       <c r="H391" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="392" ht="15" customHeight="1">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2026-05-08 10:25 UTC</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E392" t="n">
+        <v>0</v>
+      </c>
+      <c r="F392" t="n">
+        <v>0</v>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="393" ht="15" customHeight="1">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2026-05-08 10:25 UTC</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E393" t="n">
+        <v>0</v>
+      </c>
+      <c r="F393" t="n">
+        <v>0</v>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="394" ht="15" customHeight="1">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2026-05-08 10:25 UTC</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E394" t="n">
+        <v>0</v>
+      </c>
+      <c r="F394" t="n">
+        <v>0</v>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="395" ht="15" customHeight="1">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2026-05-08 10:25 UTC</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E395" t="n">
+        <v>0</v>
+      </c>
+      <c r="F395" t="n">
+        <v>0</v>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="396" ht="15" customHeight="1">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2026-05-08 10:25 UTC</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E396" t="n">
+        <v>0</v>
+      </c>
+      <c r="F396" t="n">
+        <v>0</v>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="397" ht="15" customHeight="1">
+      <c r="A397" s="6" t="inlineStr">
+        <is>
+          <t>2026-05-08 10:25 UTC</t>
+        </is>
+      </c>
+      <c r="B397" s="6" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C397" s="6" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D397" s="6" t="inlineStr">
+        <is>
+          <t>Error: HTTPSConnectionPool(host='www.ifc.com', port=443): Read timed out. (read timeout=15)</t>
+        </is>
+      </c>
+      <c r="E397" s="6" t="inlineStr"/>
+      <c r="F397" s="6" t="inlineStr"/>
+      <c r="G397" s="6" t="inlineStr"/>
+      <c r="H397" s="6" t="inlineStr"/>
+    </row>
+    <row r="398" ht="15" customHeight="1">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2026-05-08 10:25 UTC</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E398" t="n">
+        <v>0</v>
+      </c>
+      <c r="F398" t="n">
+        <v>0</v>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="399" ht="15" customHeight="1">
+      <c r="A399" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08 10:25 UTC</t>
+        </is>
+      </c>
+      <c r="B399" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C399" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D399" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E399" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F399" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G399" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.9c60c3f74bed29def584.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.28aaf9b56ef3a26a0244.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.79a8e48c33483561ca78.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.5d5537fe4edcab9b99d4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9ef1f8b90a816086ee2e.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H399" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.ee80b25e8811396367cc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.69f230c0871da659cfdc.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="400" ht="15" customHeight="1">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2026-05-08 10:25 UTC</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E400" t="n">
+        <v>0</v>
+      </c>
+      <c r="F400" t="n">
+        <v>0</v>
+      </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="401" ht="15" customHeight="1">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2026-05-08 10:25 UTC</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E401" t="n">
+        <v>0</v>
+      </c>
+      <c r="F401" t="n">
+        <v>0</v>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H401" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -15640,17 +16008,15 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-07 11:09 UTC</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>Error: HTTPSConnectionPool(host='www.amc.com', port=443): Read timed out. (read timeout=15)</t>
+          <t>2026-05-08 10:25 UTC</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1140</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -15667,7 +16033,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-07 11:09 UTC</t>
+          <t>2026-05-08 10:25 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -15692,7 +16058,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-07 11:09 UTC</t>
+          <t>2026-05-08 10:25 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -15717,17 +16083,15 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-07 11:09 UTC</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>Error: HTTPSConnectionPool(host='www.bbcamerica.com', port=443): Read timed out. (read timeout=15)</t>
+          <t>2026-05-08 10:25 UTC</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1054</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -15744,7 +16108,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-07 11:09 UTC</t>
+          <t>2026-05-08 10:25 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -15769,7 +16133,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-07 11:09 UTC</t>
+          <t>2026-05-08 10:25 UTC</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -15796,7 +16160,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-07 11:09 UTC</t>
+          <t>2026-05-08 10:25 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -15821,7 +16185,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-07 11:09 UTC</t>
+          <t>2026-05-08 10:25 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -15846,7 +16210,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-07 11:09 UTC</t>
+          <t>2026-05-08 10:25 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -15871,7 +16235,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-07 11:09 UTC</t>
+          <t>2026-05-08 10:25 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -15932,7 +16296,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.ee80b25e8811396367cc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.69f230c0871da659cfdc.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.9c60c3f74bed29def584.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.28aaf9b56ef3a26a0244.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.79a8e48c33483561ca78.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.5d5537fe4edcab9b99d4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9ef1f8b90a816086ee2e.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -15949,7 +16313,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.3f5acfa81699b3763eb3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.3f52521020997bbfb2bb.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.ee80b25e8811396367cc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.69f230c0871da659cfdc.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-09
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H401"/>
+  <dimension ref="A1:H411"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -15753,6 +15753,386 @@
         </is>
       </c>
       <c r="H401" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="402" ht="15" customHeight="1">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>2026-05-09 10:06 UTC</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E402" t="n">
+        <v>0</v>
+      </c>
+      <c r="F402" t="n">
+        <v>0</v>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="403" ht="15" customHeight="1">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>2026-05-09 10:06 UTC</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E403" t="n">
+        <v>0</v>
+      </c>
+      <c r="F403" t="n">
+        <v>0</v>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="404" ht="15" customHeight="1">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>2026-05-09 10:06 UTC</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E404" t="n">
+        <v>0</v>
+      </c>
+      <c r="F404" t="n">
+        <v>0</v>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="405" ht="15" customHeight="1">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>2026-05-09 10:06 UTC</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E405" t="n">
+        <v>0</v>
+      </c>
+      <c r="F405" t="n">
+        <v>0</v>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="406" ht="15" customHeight="1">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>2026-05-09 10:06 UTC</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E406" t="n">
+        <v>0</v>
+      </c>
+      <c r="F406" t="n">
+        <v>0</v>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="407" ht="15" customHeight="1">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>2026-05-09 10:06 UTC</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E407" t="n">
+        <v>0</v>
+      </c>
+      <c r="F407" t="n">
+        <v>0</v>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="408" ht="15" customHeight="1">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>2026-05-09 10:06 UTC</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E408" t="n">
+        <v>0</v>
+      </c>
+      <c r="F408" t="n">
+        <v>0</v>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="409" ht="15" customHeight="1">
+      <c r="A409" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-09 10:06 UTC</t>
+        </is>
+      </c>
+      <c r="B409" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C409" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D409" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E409" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F409" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G409" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.9c60c3f74bed29def584.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.28aaf9b56ef3a26a0244.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.79a8e48c33483561ca78.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.5d5537fe4edcab9b99d4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.1b21394316b5407803d3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H409" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.9c60c3f74bed29def584.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.28aaf9b56ef3a26a0244.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.79a8e48c33483561ca78.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.5d5537fe4edcab9b99d4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9ef1f8b90a816086ee2e.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="410" ht="15" customHeight="1">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>2026-05-09 10:06 UTC</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E410" t="n">
+        <v>0</v>
+      </c>
+      <c r="F410" t="n">
+        <v>0</v>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="411" ht="15" customHeight="1">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>2026-05-09 10:06 UTC</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E411" t="n">
+        <v>0</v>
+      </c>
+      <c r="F411" t="n">
+        <v>0</v>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H411" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -15965,7 +16345,7 @@
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -16008,7 +16388,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-08 10:25 UTC</t>
+          <t>2026-05-09 10:06 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -16033,7 +16413,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-08 10:25 UTC</t>
+          <t>2026-05-09 10:06 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -16058,7 +16438,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-08 10:25 UTC</t>
+          <t>2026-05-09 10:06 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -16083,7 +16463,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-08 10:25 UTC</t>
+          <t>2026-05-09 10:06 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -16108,7 +16488,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-08 10:25 UTC</t>
+          <t>2026-05-09 10:06 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -16133,17 +16513,15 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-08 10:25 UTC</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>Error: HTTPSConnectionPool(host='www.ifc.com', port=443): Read timed out. (read timeout=15)</t>
+          <t>2026-05-09 10:06 UTC</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1054</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -16160,7 +16538,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-08 10:25 UTC</t>
+          <t>2026-05-09 10:06 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -16185,7 +16563,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-08 10:25 UTC</t>
+          <t>2026-05-09 10:06 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -16210,7 +16588,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-08 10:25 UTC</t>
+          <t>2026-05-09 10:06 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -16235,7 +16613,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-08 10:25 UTC</t>
+          <t>2026-05-09 10:06 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -16296,7 +16674,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.9c60c3f74bed29def584.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.28aaf9b56ef3a26a0244.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.79a8e48c33483561ca78.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.5d5537fe4edcab9b99d4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9ef1f8b90a816086ee2e.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.9c60c3f74bed29def584.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.28aaf9b56ef3a26a0244.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.79a8e48c33483561ca78.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.5d5537fe4edcab9b99d4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.1b21394316b5407803d3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -16313,7 +16691,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.6c39467d21e115bf8f28.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.cc32d2dbdf574d730c04.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.ee80b25e8811396367cc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.dc3b5d0af4e08fd8866f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.69f230c0871da659cfdc.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.9c60c3f74bed29def584.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.28aaf9b56ef3a26a0244.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.79a8e48c33483561ca78.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.5d5537fe4edcab9b99d4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9ef1f8b90a816086ee2e.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-10
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H411"/>
+  <dimension ref="A1:H421"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -16133,6 +16133,386 @@
         </is>
       </c>
       <c r="H411" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="412" ht="15" customHeight="1">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>2026-05-10 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E412" t="n">
+        <v>0</v>
+      </c>
+      <c r="F412" t="n">
+        <v>0</v>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="413" ht="15" customHeight="1">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>2026-05-10 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E413" t="n">
+        <v>0</v>
+      </c>
+      <c r="F413" t="n">
+        <v>0</v>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="414" ht="15" customHeight="1">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>2026-05-10 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E414" t="n">
+        <v>0</v>
+      </c>
+      <c r="F414" t="n">
+        <v>0</v>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H414" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="415" ht="15" customHeight="1">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>2026-05-10 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E415" t="n">
+        <v>0</v>
+      </c>
+      <c r="F415" t="n">
+        <v>0</v>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="416" ht="15" customHeight="1">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>2026-05-10 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E416" t="n">
+        <v>0</v>
+      </c>
+      <c r="F416" t="n">
+        <v>0</v>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H416" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="417" ht="15" customHeight="1">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>2026-05-10 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E417" t="n">
+        <v>0</v>
+      </c>
+      <c r="F417" t="n">
+        <v>0</v>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H417" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="418" ht="15" customHeight="1">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>2026-05-10 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E418" t="n">
+        <v>0</v>
+      </c>
+      <c r="F418" t="n">
+        <v>0</v>
+      </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H418" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="419" ht="15" customHeight="1">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>2026-05-10 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E419" t="n">
+        <v>0</v>
+      </c>
+      <c r="F419" t="n">
+        <v>0</v>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="420" ht="15" customHeight="1">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>2026-05-10 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E420" t="n">
+        <v>0</v>
+      </c>
+      <c r="F420" t="n">
+        <v>0</v>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="421" ht="15" customHeight="1">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>2026-05-10 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E421" t="n">
+        <v>0</v>
+      </c>
+      <c r="F421" t="n">
+        <v>0</v>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H421" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -16338,6 +16718,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.9c60c3f74bed29def584.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.28aaf9b56ef3a26a0244.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.79a8e48c33483561ca78.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.5d5537fe4edcab9b99d4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.1b21394316b5407803d3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.9c60c3f74bed29def584.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.28aaf9b56ef3a26a0244.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.79a8e48c33483561ca78.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.5d5537fe4edcab9b99d4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9ef1f8b90a816086ee2e.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -16388,7 +16838,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-09 10:06 UTC</t>
+          <t>2026-05-10 10:17 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -16413,7 +16863,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-09 10:06 UTC</t>
+          <t>2026-05-10 10:17 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -16438,7 +16888,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-09 10:06 UTC</t>
+          <t>2026-05-10 10:17 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -16463,7 +16913,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-09 10:06 UTC</t>
+          <t>2026-05-10 10:17 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -16488,7 +16938,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-09 10:06 UTC</t>
+          <t>2026-05-10 10:17 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -16513,7 +16963,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-09 10:06 UTC</t>
+          <t>2026-05-10 10:17 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -16538,7 +16988,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-09 10:06 UTC</t>
+          <t>2026-05-10 10:17 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -16563,7 +17013,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-09 10:06 UTC</t>
+          <t>2026-05-10 10:17 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -16588,7 +17038,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-09 10:06 UTC</t>
+          <t>2026-05-10 10:17 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -16613,7 +17063,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-09 10:06 UTC</t>
+          <t>2026-05-10 10:17 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -16622,76 +17072,6 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.9c60c3f74bed29def584.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.28aaf9b56ef3a26a0244.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.79a8e48c33483561ca78.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.5d5537fe4edcab9b99d4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.1b21394316b5407803d3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.9c60c3f74bed29def584.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.28aaf9b56ef3a26a0244.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.79a8e48c33483561ca78.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.5d5537fe4edcab9b99d4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9ef1f8b90a816086ee2e.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-11
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H421"/>
+  <dimension ref="A1:H431"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -16513,6 +16513,386 @@
         </is>
       </c>
       <c r="H421" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="422" ht="15" customHeight="1">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>2026-05-11 12:11 UTC</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E422" t="n">
+        <v>0</v>
+      </c>
+      <c r="F422" t="n">
+        <v>0</v>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="423" ht="15" customHeight="1">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>2026-05-11 12:11 UTC</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E423" t="n">
+        <v>0</v>
+      </c>
+      <c r="F423" t="n">
+        <v>0</v>
+      </c>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="424" ht="15" customHeight="1">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>2026-05-11 12:11 UTC</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E424" t="n">
+        <v>0</v>
+      </c>
+      <c r="F424" t="n">
+        <v>0</v>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="425" ht="15" customHeight="1">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>2026-05-11 12:11 UTC</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E425" t="n">
+        <v>0</v>
+      </c>
+      <c r="F425" t="n">
+        <v>0</v>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H425" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="426" ht="15" customHeight="1">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>2026-05-11 12:11 UTC</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E426" t="n">
+        <v>0</v>
+      </c>
+      <c r="F426" t="n">
+        <v>0</v>
+      </c>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="427" ht="15" customHeight="1">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>2026-05-11 12:11 UTC</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E427" t="n">
+        <v>0</v>
+      </c>
+      <c r="F427" t="n">
+        <v>0</v>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="428" ht="15" customHeight="1">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>2026-05-11 12:11 UTC</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E428" t="n">
+        <v>0</v>
+      </c>
+      <c r="F428" t="n">
+        <v>0</v>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="429" ht="15" customHeight="1">
+      <c r="A429" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-11 12:11 UTC</t>
+        </is>
+      </c>
+      <c r="B429" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C429" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D429" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E429" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F429" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G429" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/401.ae93f895fdce492bb088.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.1d34910ba24e0ea7d73c.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.ffb72f8469a804455906.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.e0f65152fcb26a44d42f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.fef10f550a2ce9c29973.js"&gt;&lt;/script&gt;&lt;link href="/style/css/401.41aca791586de4cad0c1.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H429" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.9c60c3f74bed29def584.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.28aaf9b56ef3a26a0244.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.79a8e48c33483561ca78.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.5d5537fe4edcab9b99d4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.1b21394316b5407803d3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="430" ht="15" customHeight="1">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>2026-05-11 12:11 UTC</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E430" t="n">
+        <v>0</v>
+      </c>
+      <c r="F430" t="n">
+        <v>0</v>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="431" ht="15" customHeight="1">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>2026-05-11 12:11 UTC</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E431" t="n">
+        <v>0</v>
+      </c>
+      <c r="F431" t="n">
+        <v>0</v>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -16718,76 +17098,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.9c60c3f74bed29def584.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.28aaf9b56ef3a26a0244.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.79a8e48c33483561ca78.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.5d5537fe4edcab9b99d4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.1b21394316b5407803d3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.9c60c3f74bed29def584.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.28aaf9b56ef3a26a0244.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.79a8e48c33483561ca78.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.5d5537fe4edcab9b99d4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9ef1f8b90a816086ee2e.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -16838,7 +17148,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-10 10:17 UTC</t>
+          <t>2026-05-11 12:11 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -16863,7 +17173,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-10 10:17 UTC</t>
+          <t>2026-05-11 12:11 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -16888,7 +17198,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-10 10:17 UTC</t>
+          <t>2026-05-11 12:11 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -16913,7 +17223,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-10 10:17 UTC</t>
+          <t>2026-05-11 12:11 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -16938,7 +17248,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-10 10:17 UTC</t>
+          <t>2026-05-11 12:11 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -16963,7 +17273,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-10 10:17 UTC</t>
+          <t>2026-05-11 12:11 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -16988,7 +17298,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-10 10:17 UTC</t>
+          <t>2026-05-11 12:11 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -17013,7 +17323,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-10 10:17 UTC</t>
+          <t>2026-05-11 12:11 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -17038,7 +17348,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-10 10:17 UTC</t>
+          <t>2026-05-11 12:11 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -17063,7 +17373,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-10 10:17 UTC</t>
+          <t>2026-05-11 12:11 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -17072,6 +17382,76 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/401.ae93f895fdce492bb088.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.1d34910ba24e0ea7d73c.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.ffb72f8469a804455906.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.e0f65152fcb26a44d42f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.fef10f550a2ce9c29973.js"&gt;&lt;/script&gt;&lt;link href="/style/css/401.41aca791586de4cad0c1.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.9c60c3f74bed29def584.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.28aaf9b56ef3a26a0244.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.79a8e48c33483561ca78.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.5d5537fe4edcab9b99d4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.1b21394316b5407803d3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-12
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H431"/>
+  <dimension ref="A1:H441"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -16893,6 +16893,386 @@
         </is>
       </c>
       <c r="H431" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="432" ht="15" customHeight="1">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>2026-05-12 11:22 UTC</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E432" t="n">
+        <v>0</v>
+      </c>
+      <c r="F432" t="n">
+        <v>0</v>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="433" ht="15" customHeight="1">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>2026-05-12 11:22 UTC</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E433" t="n">
+        <v>0</v>
+      </c>
+      <c r="F433" t="n">
+        <v>0</v>
+      </c>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H433" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="434" ht="15" customHeight="1">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>2026-05-12 11:22 UTC</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E434" t="n">
+        <v>0</v>
+      </c>
+      <c r="F434" t="n">
+        <v>0</v>
+      </c>
+      <c r="G434" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H434" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="435" ht="15" customHeight="1">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>2026-05-12 11:22 UTC</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E435" t="n">
+        <v>0</v>
+      </c>
+      <c r="F435" t="n">
+        <v>0</v>
+      </c>
+      <c r="G435" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H435" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="436" ht="15" customHeight="1">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>2026-05-12 11:22 UTC</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E436" t="n">
+        <v>0</v>
+      </c>
+      <c r="F436" t="n">
+        <v>0</v>
+      </c>
+      <c r="G436" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H436" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="437" ht="15" customHeight="1">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>2026-05-12 11:22 UTC</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E437" t="n">
+        <v>0</v>
+      </c>
+      <c r="F437" t="n">
+        <v>0</v>
+      </c>
+      <c r="G437" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="438" ht="15" customHeight="1">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>2026-05-12 11:22 UTC</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E438" t="n">
+        <v>0</v>
+      </c>
+      <c r="F438" t="n">
+        <v>0</v>
+      </c>
+      <c r="G438" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H438" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="439" ht="15" customHeight="1">
+      <c r="A439" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-12 11:22 UTC</t>
+        </is>
+      </c>
+      <c r="B439" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C439" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D439" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E439" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F439" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G439" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/401.48b446e8305bfb561abd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.03447827fd317a0d372f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.94a1b6580ae294a277a9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.59808510eb5014c1e193.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.68ef677a9c50fab15f42.js"&gt;&lt;/script&gt;&lt;link href="/style/css/401.41aca791586de4cad0c1.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H439" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/401.ae93f895fdce492bb088.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.1d34910ba24e0ea7d73c.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.ffb72f8469a804455906.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.e0f65152fcb26a44d42f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.fef10f550a2ce9c29973.js"&gt;&lt;/script&gt;&lt;link href="/style/css/401.41aca791586de4cad0c1.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="440" ht="15" customHeight="1">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>2026-05-12 11:22 UTC</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E440" t="n">
+        <v>0</v>
+      </c>
+      <c r="F440" t="n">
+        <v>0</v>
+      </c>
+      <c r="G440" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H440" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="441" ht="15" customHeight="1">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>2026-05-12 11:22 UTC</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E441" t="n">
+        <v>0</v>
+      </c>
+      <c r="F441" t="n">
+        <v>0</v>
+      </c>
+      <c r="G441" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H441" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -17148,7 +17528,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-11 12:11 UTC</t>
+          <t>2026-05-12 11:22 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -17173,7 +17553,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-11 12:11 UTC</t>
+          <t>2026-05-12 11:22 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -17198,7 +17578,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-11 12:11 UTC</t>
+          <t>2026-05-12 11:22 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -17223,7 +17603,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-11 12:11 UTC</t>
+          <t>2026-05-12 11:22 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -17248,7 +17628,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-11 12:11 UTC</t>
+          <t>2026-05-12 11:22 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -17273,7 +17653,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-11 12:11 UTC</t>
+          <t>2026-05-12 11:22 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -17298,7 +17678,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-11 12:11 UTC</t>
+          <t>2026-05-12 11:22 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -17323,7 +17703,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-11 12:11 UTC</t>
+          <t>2026-05-12 11:22 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -17348,7 +17728,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-11 12:11 UTC</t>
+          <t>2026-05-12 11:22 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -17373,7 +17753,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-11 12:11 UTC</t>
+          <t>2026-05-12 11:22 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -17434,7 +17814,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/401.ae93f895fdce492bb088.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.1d34910ba24e0ea7d73c.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.ffb72f8469a804455906.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.e0f65152fcb26a44d42f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.fef10f550a2ce9c29973.js"&gt;&lt;/script&gt;&lt;link href="/style/css/401.41aca791586de4cad0c1.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/401.48b446e8305bfb561abd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.03447827fd317a0d372f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.94a1b6580ae294a277a9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.59808510eb5014c1e193.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.68ef677a9c50fab15f42.js"&gt;&lt;/script&gt;&lt;link href="/style/css/401.41aca791586de4cad0c1.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -17451,7 +17831,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1137.25e6159b20eb00a2d2c4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6901.9c60c3f74bed29def584.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.28aaf9b56ef3a26a0244.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.79a8e48c33483561ca78.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2018.5d5537fe4edcab9b99d4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.1b21394316b5407803d3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/6901.911f535d0d79976b7f73.css" rel="stylesheet"&gt;&lt;link href="/style/css/2018.eb0277fa41bd0ebb6625.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/401.ae93f895fdce492bb088.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.1d34910ba24e0ea7d73c.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.ffb72f8469a804455906.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.e0f65152fcb26a44d42f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.fef10f550a2ce9c29973.js"&gt;&lt;/script&gt;&lt;link href="/style/css/401.41aca791586de4cad0c1.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-13
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -8,17 +8,17 @@
   </bookViews>
   <sheets>
     <sheet name="Change Log" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="amc_com_ads_txt" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="amc_com_app-ads_txt" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="bbca_com_ads_txt" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="bbca_com_app-ads_txt" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="ifc_com_ads_txt" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ifc_com_app-ads_txt" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Current Snapshot" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="amc_com_ads_txt" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="amc_com_app-ads_txt" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="bbca_com_ads_txt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="bbca_com_app-ads_txt" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ifc_com_ads_txt" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="ifc_com_app-ads_txt" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="sundancetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="wetv_com_ads_txt" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="wetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H441"/>
+  <dimension ref="A1:H451"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -17278,6 +17278,395 @@
         </is>
       </c>
     </row>
+    <row r="442" ht="15" customHeight="1">
+      <c r="A442" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-13 11:30 UTC</t>
+        </is>
+      </c>
+      <c r="B442" s="3" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C442" s="3" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D442" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E442" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F442" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G442" s="3" t="inlineStr">
+        <is>
+          <t>#Oxiem: freewheel.tv, sg1306174, RESELLER
+#Oxiem: freewheel.tv, 545336-r-523319, RESELLER</t>
+        </is>
+      </c>
+      <c r="H442" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="443" ht="15" customHeight="1">
+      <c r="A443" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-13 11:30 UTC</t>
+        </is>
+      </c>
+      <c r="B443" s="3" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C443" s="3" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D443" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E443" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F443" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G443" s="3" t="inlineStr">
+        <is>
+          <t>#Oxiem: freewheel.tv, sg1306174, RESELLER
+#Oxiem: freewheel.tv, 545336-r-523319, RESELLER</t>
+        </is>
+      </c>
+      <c r="H443" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="444" ht="15" customHeight="1">
+      <c r="A444" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-13 11:30 UTC</t>
+        </is>
+      </c>
+      <c r="B444" s="3" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C444" s="3" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D444" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E444" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F444" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G444" s="3" t="inlineStr">
+        <is>
+          <t>#Oxiem: freewheel.tv, sg1306174, RESELLER
+#Oxiem: freewheel.tv, 545336-r-523319, RESELLER</t>
+        </is>
+      </c>
+      <c r="H444" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="445" ht="15" customHeight="1">
+      <c r="A445" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-13 11:30 UTC</t>
+        </is>
+      </c>
+      <c r="B445" s="3" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C445" s="3" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D445" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E445" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F445" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G445" s="3" t="inlineStr">
+        <is>
+          <t>#Oxiem: freewheel.tv, sg1306174, RESELLER
+#Oxiem: freewheel.tv, 545336-r-523319, RESELLER</t>
+        </is>
+      </c>
+      <c r="H445" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="446" ht="15" customHeight="1">
+      <c r="A446" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-13 11:30 UTC</t>
+        </is>
+      </c>
+      <c r="B446" s="3" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C446" s="3" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D446" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E446" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F446" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G446" s="3" t="inlineStr">
+        <is>
+          <t>#Oxiem: freewheel.tv, sg1306174, RESELLER
+#Oxiem: freewheel.tv, 545336-r-523319, RESELLER</t>
+        </is>
+      </c>
+      <c r="H446" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="447" ht="15" customHeight="1">
+      <c r="A447" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-13 11:30 UTC</t>
+        </is>
+      </c>
+      <c r="B447" s="3" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C447" s="3" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D447" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E447" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F447" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G447" s="3" t="inlineStr">
+        <is>
+          <t>#Oxiem: freewheel.tv, sg1306174, RESELLER
+#Oxiem: freewheel.tv, 545336-r-523319, RESELLER</t>
+        </is>
+      </c>
+      <c r="H447" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="448" ht="15" customHeight="1">
+      <c r="A448" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-13 11:30 UTC</t>
+        </is>
+      </c>
+      <c r="B448" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C448" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D448" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E448" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F448" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G448" s="3" t="inlineStr">
+        <is>
+          <t>#Oxiem: freewheel.tv, sg1306174, RESELLER
+#Oxiem: freewheel.tv, 545336-r-523319, RESELLER</t>
+        </is>
+      </c>
+      <c r="H448" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="449" ht="15" customHeight="1">
+      <c r="A449" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-13 11:30 UTC</t>
+        </is>
+      </c>
+      <c r="B449" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C449" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D449" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E449" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F449" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G449" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/401.48b446e8305bfb561abd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.03447827fd317a0d372f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.94a1b6580ae294a277a9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.59808510eb5014c1e193.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.58c156d942d0183bed7e.js"&gt;&lt;/script&gt;&lt;link href="/style/css/401.41aca791586de4cad0c1.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H449" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/401.48b446e8305bfb561abd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.03447827fd317a0d372f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.94a1b6580ae294a277a9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.59808510eb5014c1e193.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.68ef677a9c50fab15f42.js"&gt;&lt;/script&gt;&lt;link href="/style/css/401.41aca791586de4cad0c1.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="450" ht="15" customHeight="1">
+      <c r="A450" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-13 11:30 UTC</t>
+        </is>
+      </c>
+      <c r="B450" s="3" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C450" s="3" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D450" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E450" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F450" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G450" s="3" t="inlineStr">
+        <is>
+          <t>#Oxiem: freewheel.tv, sg1306174, RESELLER
+#Oxiem: freewheel.tv, 545336-r-523319, RESELLER</t>
+        </is>
+      </c>
+      <c r="H450" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="451" ht="15" customHeight="1">
+      <c r="A451" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-13 11:30 UTC</t>
+        </is>
+      </c>
+      <c r="B451" s="3" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C451" s="3" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D451" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E451" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F451" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G451" s="3" t="inlineStr">
+        <is>
+          <t>#Oxiem: freewheel.tv, sg1306174, RESELLER
+#Oxiem: freewheel.tv, 545336-r-523319, RESELLER</t>
+        </is>
+      </c>
+      <c r="H451" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -17289,7 +17678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17322,148 +17711,29 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Wurl</t>
+          <t>(no section)</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>wurl.com, 55562, DIRECT</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/401.48b446e8305bfb561abd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.03447827fd317a0d372f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.94a1b6580ae294a277a9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.59808510eb5014c1e193.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.58c156d942d0183bed7e.js"&gt;&lt;/script&gt;&lt;link href="/style/css/401.41aca791586de4cad0c1.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, sg1303005, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709-r-523319, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>#Olyzon</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 167424, RESELLER, 5d62403b186f2ace</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>#Olyzon</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>olyzon.tv, 76794, PUBLISHER</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>#Nexxen</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>lkqd.net, 1100060088, RESELLER 59c49fa9598a0117</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>#Infolinks</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Infolinks.com, 3444795, DIRECT</t>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/401.48b446e8305bfb561abd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.03447827fd317a0d372f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.94a1b6580ae294a277a9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.59808510eb5014c1e193.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.68ef677a9c50fab15f42.js"&gt;&lt;/script&gt;&lt;link href="/style/css/401.41aca791586de4cad0c1.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -17478,290 +17748,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Partner</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>File</t>
+          <t>Section</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Last Updated</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Line Count</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
+          <t>Line Content</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>AMC Networks</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>amc.com/ads.txt</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2026-05-12 11:22 UTC</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>1140</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>#Oxiem</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, sg1306174, RESELLER</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>AMC Networks</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>amc.com/app-ads.txt</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2026-05-12 11:22 UTC</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>1054</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>BBC America</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>bbca.com/ads.txt</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2026-05-12 11:22 UTC</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>1140</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>BBC America</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>bbca.com/app-ads.txt</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2026-05-12 11:22 UTC</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>1054</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>IFC</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>ifc.com/ads.txt</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>2026-05-12 11:22 UTC</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>1140</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>IFC</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>ifc.com/app-ads.txt</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>2026-05-12 11:22 UTC</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>1054</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Sundance TV</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>sundancetv.com/ads.txt</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2026-05-12 11:22 UTC</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>1140</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Sundance TV</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>sundancetv.com/app-ads.txt</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>2026-05-12 11:22 UTC</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>19</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>WE tv</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>wetv.com/ads.txt</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>2026-05-12 11:22 UTC</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>1140</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>WE tv</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>wetv.com/app-ads.txt</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>2026-05-12 11:22 UTC</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>1054</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>#Oxiem</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 545336-r-523319, RESELLER</t>
         </is>
       </c>
     </row>
@@ -17809,29 +17851,29 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>(no section)</t>
+          <t>#Oxiem</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/401.48b446e8305bfb561abd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.03447827fd317a0d372f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.94a1b6580ae294a277a9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.59808510eb5014c1e193.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.68ef677a9c50fab15f42.js"&gt;&lt;/script&gt;&lt;link href="/style/css/401.41aca791586de4cad0c1.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>freewheel.tv, sg1306174, RESELLER</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/401.ae93f895fdce492bb088.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.1d34910ba24e0ea7d73c.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.ffb72f8469a804455906.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.e0f65152fcb26a44d42f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.fef10f550a2ce9c29973.js"&gt;&lt;/script&gt;&lt;link href="/style/css/401.41aca791586de4cad0c1.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>#Oxiem</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 545336-r-523319, RESELLER</t>
         </is>
       </c>
     </row>
@@ -17846,181 +17888,290 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Section</t>
+          <t>File</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Line Content</t>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Line Count</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>#Wurl</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>wurl.com, 55562, DIRECT</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-05-13 11:30 UTC</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1142</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709, RESELLER</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-05-13 11:30 UTC</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1056</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, sg1303005, RESELLER</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-05-13 11:30 UTC</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1142</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709-r-523319, RESELLER</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-05-13 11:30 UTC</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1056</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709-r-524565, RESELLER</t>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-05-13 11:30 UTC</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1142</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>#Olyzon</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 167424, RESELLER, 5d62403b186f2ace</t>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-05-13 11:30 UTC</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1056</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>#Olyzon</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>olyzon.tv, 76794, PUBLISHER</t>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-05-13 11:30 UTC</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1142</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>#Nexxen</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>lkqd.net, 1100060088, RESELLER 59c49fa9598a0117</t>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-05-13 11:30 UTC</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>19</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>#Infolinks</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Infolinks.com, 3444795, DIRECT</t>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-05-13 11:30 UTC</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1142</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-05-13 11:30 UTC</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1056</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -18035,7 +18186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18068,12 +18219,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Wurl</t>
+          <t>#Oxiem</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>wurl.com, 55562, DIRECT</t>
+          <t>freewheel.tv, sg1306174, RESELLER</t>
         </is>
       </c>
     </row>
@@ -18085,131 +18236,12 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>#PrismRiot</t>
+          <t>#Oxiem</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, 543709, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, sg1303005, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709-r-523319, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>#Olyzon</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 167424, RESELLER, 5d62403b186f2ace</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>#Olyzon</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>olyzon.tv, 76794, PUBLISHER</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>#Nexxen</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>lkqd.net, 1100060088, RESELLER 59c49fa9598a0117</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>#Infolinks</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Infolinks.com, 3444795, DIRECT</t>
+          <t>freewheel.tv, 545336-r-523319, RESELLER</t>
         </is>
       </c>
     </row>
@@ -18224,7 +18256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18257,12 +18289,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Wurl</t>
+          <t>#Oxiem</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>wurl.com, 55562, DIRECT</t>
+          <t>freewheel.tv, sg1306174, RESELLER</t>
         </is>
       </c>
     </row>
@@ -18274,131 +18306,12 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>#PrismRiot</t>
+          <t>#Oxiem</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, 543709, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, sg1303005, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709-r-523319, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>#Olyzon</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 167424, RESELLER, 5d62403b186f2ace</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>#Olyzon</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>olyzon.tv, 76794, PUBLISHER</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>#Nexxen</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>lkqd.net, 1100060088, RESELLER 59c49fa9598a0117</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>#Infolinks</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Infolinks.com, 3444795, DIRECT</t>
+          <t>freewheel.tv, 545336-r-523319, RESELLER</t>
         </is>
       </c>
     </row>
@@ -18413,7 +18326,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18446,12 +18359,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Wurl</t>
+          <t>#Oxiem</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>wurl.com, 55562, DIRECT</t>
+          <t>freewheel.tv, sg1306174, RESELLER</t>
         </is>
       </c>
     </row>
@@ -18463,131 +18376,12 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>#PrismRiot</t>
+          <t>#Oxiem</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, 543709, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, sg1303005, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709-r-523319, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>#Olyzon</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 167424, RESELLER, 5d62403b186f2ace</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>#Olyzon</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>olyzon.tv, 76794, PUBLISHER</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>#Nexxen</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>lkqd.net, 1100060088, RESELLER 59c49fa9598a0117</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>#Infolinks</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Infolinks.com, 3444795, DIRECT</t>
+          <t>freewheel.tv, 545336-r-523319, RESELLER</t>
         </is>
       </c>
     </row>
@@ -18602,7 +18396,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18635,12 +18429,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Wurl</t>
+          <t>#Oxiem</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>wurl.com, 55562, DIRECT</t>
+          <t>freewheel.tv, sg1306174, RESELLER</t>
         </is>
       </c>
     </row>
@@ -18652,131 +18446,12 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>#PrismRiot</t>
+          <t>#Oxiem</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, 543709, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, sg1303005, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709-r-523319, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>#Olyzon</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 167424, RESELLER, 5d62403b186f2ace</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>#Olyzon</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>olyzon.tv, 76794, PUBLISHER</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>#Nexxen</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>lkqd.net, 1100060088, RESELLER 59c49fa9598a0117</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>#Infolinks</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Infolinks.com, 3444795, DIRECT</t>
+          <t>freewheel.tv, 545336-r-523319, RESELLER</t>
         </is>
       </c>
     </row>
@@ -18791,7 +18466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -18824,12 +18499,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Wurl</t>
+          <t>#Oxiem</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>wurl.com, 55562, DIRECT</t>
+          <t>freewheel.tv, sg1306174, RESELLER</t>
         </is>
       </c>
     </row>
@@ -18841,131 +18516,12 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>#PrismRiot</t>
+          <t>#Oxiem</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, 543709, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, sg1303005, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709-r-523319, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>#Olyzon</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 167424, RESELLER, 5d62403b186f2ace</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>#Olyzon</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>olyzon.tv, 76794, PUBLISHER</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>#Nexxen</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>lkqd.net, 1100060088, RESELLER 59c49fa9598a0117</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>#Infolinks</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Infolinks.com, 3444795, DIRECT</t>
+          <t>freewheel.tv, 545336-r-523319, RESELLER</t>
         </is>
       </c>
     </row>
@@ -18980,7 +18536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19013,12 +18569,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Wurl</t>
+          <t>#Oxiem</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>wurl.com, 55562, DIRECT</t>
+          <t>freewheel.tv, sg1306174, RESELLER</t>
         </is>
       </c>
     </row>
@@ -19030,131 +18586,12 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>#PrismRiot</t>
+          <t>#Oxiem</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, 543709, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, sg1303005, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709-r-523319, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>#Olyzon</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 167424, RESELLER, 5d62403b186f2ace</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>#Olyzon</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>olyzon.tv, 76794, PUBLISHER</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>#Nexxen</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>lkqd.net, 1100060088, RESELLER 59c49fa9598a0117</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>#Infolinks</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Infolinks.com, 3444795, DIRECT</t>
+          <t>freewheel.tv, 545336-r-523319, RESELLER</t>
         </is>
       </c>
     </row>
@@ -19169,7 +18606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19202,12 +18639,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Wurl</t>
+          <t>#Oxiem</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>wurl.com, 55562, DIRECT</t>
+          <t>freewheel.tv, sg1306174, RESELLER</t>
         </is>
       </c>
     </row>
@@ -19219,131 +18656,12 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>#PrismRiot</t>
+          <t>#Oxiem</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, 543709, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, sg1303005, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709-r-523319, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>#PrismRiot</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 543709-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>#Olyzon</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 167424, RESELLER, 5d62403b186f2ace</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>#Olyzon</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>olyzon.tv, 76794, PUBLISHER</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>#Nexxen</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>lkqd.net, 1100060088, RESELLER 59c49fa9598a0117</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>#Infolinks</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Infolinks.com, 3444795, DIRECT</t>
+          <t>freewheel.tv, 545336-r-523319, RESELLER</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-14
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -8,17 +8,17 @@
   </bookViews>
   <sheets>
     <sheet name="Change Log" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Current Snapshot" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="amc_com_ads_txt" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="amc_com_app-ads_txt" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="bbca_com_ads_txt" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="bbca_com_app-ads_txt" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ifc_com_ads_txt" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="ifc_com_app-ads_txt" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="sundancetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="wetv_com_ads_txt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="wetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="amc_com_ads_txt" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="amc_com_app-ads_txt" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="bbca_com_ads_txt" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="bbca_com_app-ads_txt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ifc_com_ads_txt" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ifc_com_app-ads_txt" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H451"/>
+  <dimension ref="A1:H461"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -17662,6 +17662,386 @@
         </is>
       </c>
       <c r="H451" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="452" ht="15" customHeight="1">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>2026-05-14 11:13 UTC</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E452" t="n">
+        <v>0</v>
+      </c>
+      <c r="F452" t="n">
+        <v>0</v>
+      </c>
+      <c r="G452" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H452" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="453" ht="15" customHeight="1">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>2026-05-14 11:13 UTC</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E453" t="n">
+        <v>0</v>
+      </c>
+      <c r="F453" t="n">
+        <v>0</v>
+      </c>
+      <c r="G453" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H453" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="454" ht="15" customHeight="1">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>2026-05-14 11:13 UTC</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E454" t="n">
+        <v>0</v>
+      </c>
+      <c r="F454" t="n">
+        <v>0</v>
+      </c>
+      <c r="G454" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H454" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="455" ht="15" customHeight="1">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>2026-05-14 11:13 UTC</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E455" t="n">
+        <v>0</v>
+      </c>
+      <c r="F455" t="n">
+        <v>0</v>
+      </c>
+      <c r="G455" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H455" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="456" ht="15" customHeight="1">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>2026-05-14 11:13 UTC</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E456" t="n">
+        <v>0</v>
+      </c>
+      <c r="F456" t="n">
+        <v>0</v>
+      </c>
+      <c r="G456" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H456" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="457" ht="15" customHeight="1">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>2026-05-14 11:13 UTC</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E457" t="n">
+        <v>0</v>
+      </c>
+      <c r="F457" t="n">
+        <v>0</v>
+      </c>
+      <c r="G457" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H457" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="458" ht="15" customHeight="1">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>2026-05-14 11:13 UTC</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E458" t="n">
+        <v>0</v>
+      </c>
+      <c r="F458" t="n">
+        <v>0</v>
+      </c>
+      <c r="G458" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H458" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="459" ht="15" customHeight="1">
+      <c r="A459" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14 11:13 UTC</t>
+        </is>
+      </c>
+      <c r="B459" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C459" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D459" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E459" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F459" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G459" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/401.48b446e8305bfb561abd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.03447827fd317a0d372f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.94a1b6580ae294a277a9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.59808510eb5014c1e193.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9a5502c0a93c149f589f.js"&gt;&lt;/script&gt;&lt;link href="/style/css/401.41aca791586de4cad0c1.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H459" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/401.48b446e8305bfb561abd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.03447827fd317a0d372f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.94a1b6580ae294a277a9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.59808510eb5014c1e193.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.58c156d942d0183bed7e.js"&gt;&lt;/script&gt;&lt;link href="/style/css/401.41aca791586de4cad0c1.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="460" ht="15" customHeight="1">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>2026-05-14 11:13 UTC</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E460" t="n">
+        <v>0</v>
+      </c>
+      <c r="F460" t="n">
+        <v>0</v>
+      </c>
+      <c r="G460" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H460" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="461" ht="15" customHeight="1">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>2026-05-14 11:13 UTC</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E461" t="n">
+        <v>0</v>
+      </c>
+      <c r="F461" t="n">
+        <v>0</v>
+      </c>
+      <c r="G461" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H461" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -17711,29 +18091,29 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>(no section)</t>
+          <t>#Oxiem</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/401.48b446e8305bfb561abd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.03447827fd317a0d372f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.94a1b6580ae294a277a9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.59808510eb5014c1e193.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.58c156d942d0183bed7e.js"&gt;&lt;/script&gt;&lt;link href="/style/css/401.41aca791586de4cad0c1.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>freewheel.tv, sg1306174, RESELLER</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/401.48b446e8305bfb561abd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.03447827fd317a0d372f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.94a1b6580ae294a277a9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.59808510eb5014c1e193.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.68ef677a9c50fab15f42.js"&gt;&lt;/script&gt;&lt;link href="/style/css/401.41aca791586de4cad0c1.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>#Oxiem</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 545336-r-523319, RESELLER</t>
         </is>
       </c>
     </row>
@@ -17748,62 +18128,290 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Section</t>
+          <t>File</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Line Content</t>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Line Count</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>#Oxiem</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, sg1306174, RESELLER</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-05-14 11:13 UTC</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1142</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>#Oxiem</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 545336-r-523319, RESELLER</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-05-14 11:13 UTC</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1056</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-05-14 11:13 UTC</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1142</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-05-14 11:13 UTC</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1056</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-05-14 11:13 UTC</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1142</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-05-14 11:13 UTC</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1056</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-05-14 11:13 UTC</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1142</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-05-14 11:13 UTC</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>19</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-05-14 11:13 UTC</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1142</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-05-14 11:13 UTC</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1056</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -17851,29 +18459,29 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Oxiem</t>
+          <t>(no section)</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, sg1306174, RESELLER</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/401.48b446e8305bfb561abd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.03447827fd317a0d372f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.94a1b6580ae294a277a9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.59808510eb5014c1e193.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9a5502c0a93c149f589f.js"&gt;&lt;/script&gt;&lt;link href="/style/css/401.41aca791586de4cad0c1.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>#Oxiem</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 545336-r-523319, RESELLER</t>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/401.48b446e8305bfb561abd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.03447827fd317a0d372f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.94a1b6580ae294a277a9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.59808510eb5014c1e193.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.58c156d942d0183bed7e.js"&gt;&lt;/script&gt;&lt;link href="/style/css/401.41aca791586de4cad0c1.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -17888,290 +18496,62 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Partner</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>File</t>
+          <t>Section</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Last Updated</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Line Count</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
+          <t>Line Content</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>AMC Networks</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>amc.com/ads.txt</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2026-05-13 11:30 UTC</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>1142</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>#Oxiem</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, sg1306174, RESELLER</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>AMC Networks</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>amc.com/app-ads.txt</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2026-05-13 11:30 UTC</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>1056</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>BBC America</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>bbca.com/ads.txt</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2026-05-13 11:30 UTC</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>1142</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>BBC America</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>bbca.com/app-ads.txt</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2026-05-13 11:30 UTC</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>1056</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>IFC</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>ifc.com/ads.txt</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>2026-05-13 11:30 UTC</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>1142</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>IFC</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>ifc.com/app-ads.txt</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>2026-05-13 11:30 UTC</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>1056</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Sundance TV</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>sundancetv.com/ads.txt</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2026-05-13 11:30 UTC</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>1142</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Sundance TV</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>sundancetv.com/app-ads.txt</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>2026-05-13 11:30 UTC</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>19</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>WE tv</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>wetv.com/ads.txt</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>2026-05-13 11:30 UTC</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>1142</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>WE tv</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>wetv.com/app-ads.txt</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>2026-05-13 11:30 UTC</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>1056</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>#Oxiem</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 545336-r-523319, RESELLER</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-15
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H461"/>
+  <dimension ref="A1:H471"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -18042,6 +18042,386 @@
         </is>
       </c>
       <c r="H461" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="462" ht="15" customHeight="1">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>2026-05-15 11:22 UTC</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E462" t="n">
+        <v>0</v>
+      </c>
+      <c r="F462" t="n">
+        <v>0</v>
+      </c>
+      <c r="G462" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H462" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="463" ht="15" customHeight="1">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>2026-05-15 11:22 UTC</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E463" t="n">
+        <v>0</v>
+      </c>
+      <c r="F463" t="n">
+        <v>0</v>
+      </c>
+      <c r="G463" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H463" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="464" ht="15" customHeight="1">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>2026-05-15 11:22 UTC</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E464" t="n">
+        <v>0</v>
+      </c>
+      <c r="F464" t="n">
+        <v>0</v>
+      </c>
+      <c r="G464" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H464" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="465" ht="15" customHeight="1">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>2026-05-15 11:22 UTC</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E465" t="n">
+        <v>0</v>
+      </c>
+      <c r="F465" t="n">
+        <v>0</v>
+      </c>
+      <c r="G465" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H465" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="466" ht="15" customHeight="1">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>2026-05-15 11:22 UTC</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E466" t="n">
+        <v>0</v>
+      </c>
+      <c r="F466" t="n">
+        <v>0</v>
+      </c>
+      <c r="G466" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H466" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="467" ht="15" customHeight="1">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>2026-05-15 11:22 UTC</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E467" t="n">
+        <v>0</v>
+      </c>
+      <c r="F467" t="n">
+        <v>0</v>
+      </c>
+      <c r="G467" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H467" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="468" ht="15" customHeight="1">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>2026-05-15 11:22 UTC</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E468" t="n">
+        <v>0</v>
+      </c>
+      <c r="F468" t="n">
+        <v>0</v>
+      </c>
+      <c r="G468" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H468" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="469" ht="15" customHeight="1">
+      <c r="A469" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15 11:22 UTC</t>
+        </is>
+      </c>
+      <c r="B469" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C469" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D469" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E469" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F469" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G469" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.fae045a1158903fc8baa.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8d990b08b0b28aa5de58.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H469" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/401.48b446e8305bfb561abd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.03447827fd317a0d372f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.94a1b6580ae294a277a9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.59808510eb5014c1e193.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9a5502c0a93c149f589f.js"&gt;&lt;/script&gt;&lt;link href="/style/css/401.41aca791586de4cad0c1.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="470" ht="15" customHeight="1">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>2026-05-15 11:22 UTC</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E470" t="n">
+        <v>0</v>
+      </c>
+      <c r="F470" t="n">
+        <v>0</v>
+      </c>
+      <c r="G470" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H470" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="471" ht="15" customHeight="1">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>2026-05-15 11:22 UTC</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E471" t="n">
+        <v>0</v>
+      </c>
+      <c r="F471" t="n">
+        <v>0</v>
+      </c>
+      <c r="G471" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H471" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -18178,7 +18558,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-14 11:13 UTC</t>
+          <t>2026-05-15 11:22 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -18203,7 +18583,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-14 11:13 UTC</t>
+          <t>2026-05-15 11:22 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -18228,7 +18608,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-14 11:13 UTC</t>
+          <t>2026-05-15 11:22 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -18253,7 +18633,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-14 11:13 UTC</t>
+          <t>2026-05-15 11:22 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -18278,7 +18658,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-14 11:13 UTC</t>
+          <t>2026-05-15 11:22 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -18303,7 +18683,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-14 11:13 UTC</t>
+          <t>2026-05-15 11:22 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -18328,7 +18708,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-14 11:13 UTC</t>
+          <t>2026-05-15 11:22 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -18353,7 +18733,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-14 11:13 UTC</t>
+          <t>2026-05-15 11:22 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -18378,7 +18758,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-14 11:13 UTC</t>
+          <t>2026-05-15 11:22 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -18403,7 +18783,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-14 11:13 UTC</t>
+          <t>2026-05-15 11:22 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -18464,7 +18844,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/401.48b446e8305bfb561abd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.03447827fd317a0d372f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.94a1b6580ae294a277a9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.59808510eb5014c1e193.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9a5502c0a93c149f589f.js"&gt;&lt;/script&gt;&lt;link href="/style/css/401.41aca791586de4cad0c1.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.fae045a1158903fc8baa.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8d990b08b0b28aa5de58.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -18481,7 +18861,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/401.48b446e8305bfb561abd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.03447827fd317a0d372f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.94a1b6580ae294a277a9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.59808510eb5014c1e193.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.58c156d942d0183bed7e.js"&gt;&lt;/script&gt;&lt;link href="/style/css/401.41aca791586de4cad0c1.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/401.48b446e8305bfb561abd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.03447827fd317a0d372f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.94a1b6580ae294a277a9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.59808510eb5014c1e193.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9a5502c0a93c149f589f.js"&gt;&lt;/script&gt;&lt;link href="/style/css/401.41aca791586de4cad0c1.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-16
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H471"/>
+  <dimension ref="A1:H481"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -18422,6 +18422,386 @@
         </is>
       </c>
       <c r="H471" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="472" ht="15" customHeight="1">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>2026-05-16 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E472" t="n">
+        <v>0</v>
+      </c>
+      <c r="F472" t="n">
+        <v>0</v>
+      </c>
+      <c r="G472" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H472" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="473" ht="15" customHeight="1">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>2026-05-16 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E473" t="n">
+        <v>0</v>
+      </c>
+      <c r="F473" t="n">
+        <v>0</v>
+      </c>
+      <c r="G473" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H473" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="474" ht="15" customHeight="1">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>2026-05-16 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E474" t="n">
+        <v>0</v>
+      </c>
+      <c r="F474" t="n">
+        <v>0</v>
+      </c>
+      <c r="G474" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H474" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="475" ht="15" customHeight="1">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>2026-05-16 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E475" t="n">
+        <v>0</v>
+      </c>
+      <c r="F475" t="n">
+        <v>0</v>
+      </c>
+      <c r="G475" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H475" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="476" ht="15" customHeight="1">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>2026-05-16 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E476" t="n">
+        <v>0</v>
+      </c>
+      <c r="F476" t="n">
+        <v>0</v>
+      </c>
+      <c r="G476" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H476" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="477" ht="15" customHeight="1">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>2026-05-16 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E477" t="n">
+        <v>0</v>
+      </c>
+      <c r="F477" t="n">
+        <v>0</v>
+      </c>
+      <c r="G477" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H477" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="478" ht="15" customHeight="1">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>2026-05-16 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E478" t="n">
+        <v>0</v>
+      </c>
+      <c r="F478" t="n">
+        <v>0</v>
+      </c>
+      <c r="G478" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H478" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="479" ht="15" customHeight="1">
+      <c r="A479" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B479" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C479" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D479" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E479" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F479" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G479" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.fae045a1158903fc8baa.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.c31208edeb76d274f394.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H479" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.fae045a1158903fc8baa.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8d990b08b0b28aa5de58.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="480" ht="15" customHeight="1">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>2026-05-16 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E480" t="n">
+        <v>0</v>
+      </c>
+      <c r="F480" t="n">
+        <v>0</v>
+      </c>
+      <c r="G480" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H480" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="481" ht="15" customHeight="1">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>2026-05-16 10:17 UTC</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E481" t="n">
+        <v>0</v>
+      </c>
+      <c r="F481" t="n">
+        <v>0</v>
+      </c>
+      <c r="G481" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H481" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -18558,7 +18938,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-15 11:22 UTC</t>
+          <t>2026-05-16 10:17 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -18583,7 +18963,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-15 11:22 UTC</t>
+          <t>2026-05-16 10:17 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -18608,7 +18988,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-15 11:22 UTC</t>
+          <t>2026-05-16 10:17 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -18633,7 +19013,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-15 11:22 UTC</t>
+          <t>2026-05-16 10:17 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -18658,7 +19038,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-15 11:22 UTC</t>
+          <t>2026-05-16 10:17 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -18683,7 +19063,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-15 11:22 UTC</t>
+          <t>2026-05-16 10:17 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -18708,7 +19088,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-15 11:22 UTC</t>
+          <t>2026-05-16 10:17 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -18733,7 +19113,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-15 11:22 UTC</t>
+          <t>2026-05-16 10:17 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -18758,7 +19138,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-15 11:22 UTC</t>
+          <t>2026-05-16 10:17 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -18783,7 +19163,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-15 11:22 UTC</t>
+          <t>2026-05-16 10:17 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -18844,7 +19224,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.fae045a1158903fc8baa.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8d990b08b0b28aa5de58.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.fae045a1158903fc8baa.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.c31208edeb76d274f394.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -18861,7 +19241,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/401.48b446e8305bfb561abd.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.03447827fd317a0d372f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.615f2be175bb2fef89fe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.94a1b6580ae294a277a9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.59808510eb5014c1e193.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9a5502c0a93c149f589f.js"&gt;&lt;/script&gt;&lt;link href="/style/css/401.41aca791586de4cad0c1.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.fae045a1158903fc8baa.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8d990b08b0b28aa5de58.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-17
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H481"/>
+  <dimension ref="A1:H491"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -18802,6 +18802,386 @@
         </is>
       </c>
       <c r="H481" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="482" ht="15" customHeight="1">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>2026-05-17 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E482" t="n">
+        <v>0</v>
+      </c>
+      <c r="F482" t="n">
+        <v>0</v>
+      </c>
+      <c r="G482" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H482" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="483" ht="15" customHeight="1">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>2026-05-17 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E483" t="n">
+        <v>0</v>
+      </c>
+      <c r="F483" t="n">
+        <v>0</v>
+      </c>
+      <c r="G483" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H483" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="484" ht="15" customHeight="1">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>2026-05-17 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E484" t="n">
+        <v>0</v>
+      </c>
+      <c r="F484" t="n">
+        <v>0</v>
+      </c>
+      <c r="G484" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H484" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="485" ht="15" customHeight="1">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>2026-05-17 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E485" t="n">
+        <v>0</v>
+      </c>
+      <c r="F485" t="n">
+        <v>0</v>
+      </c>
+      <c r="G485" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H485" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="486" ht="15" customHeight="1">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>2026-05-17 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E486" t="n">
+        <v>0</v>
+      </c>
+      <c r="F486" t="n">
+        <v>0</v>
+      </c>
+      <c r="G486" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H486" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="487" ht="15" customHeight="1">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>2026-05-17 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E487" t="n">
+        <v>0</v>
+      </c>
+      <c r="F487" t="n">
+        <v>0</v>
+      </c>
+      <c r="G487" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H487" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="488" ht="15" customHeight="1">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>2026-05-17 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E488" t="n">
+        <v>0</v>
+      </c>
+      <c r="F488" t="n">
+        <v>0</v>
+      </c>
+      <c r="G488" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H488" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="489" ht="15" customHeight="1">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>2026-05-17 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E489" t="n">
+        <v>0</v>
+      </c>
+      <c r="F489" t="n">
+        <v>0</v>
+      </c>
+      <c r="G489" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H489" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="490" ht="15" customHeight="1">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>2026-05-17 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E490" t="n">
+        <v>0</v>
+      </c>
+      <c r="F490" t="n">
+        <v>0</v>
+      </c>
+      <c r="G490" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H490" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="491" ht="15" customHeight="1">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>2026-05-17 10:23 UTC</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E491" t="n">
+        <v>0</v>
+      </c>
+      <c r="F491" t="n">
+        <v>0</v>
+      </c>
+      <c r="G491" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H491" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -18888,6 +19268,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.fae045a1158903fc8baa.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.c31208edeb76d274f394.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.fae045a1158903fc8baa.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8d990b08b0b28aa5de58.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -18938,7 +19388,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-16 10:17 UTC</t>
+          <t>2026-05-17 10:23 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -18963,7 +19413,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-16 10:17 UTC</t>
+          <t>2026-05-17 10:23 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -18988,7 +19438,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-16 10:17 UTC</t>
+          <t>2026-05-17 10:23 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -19013,7 +19463,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-16 10:17 UTC</t>
+          <t>2026-05-17 10:23 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -19038,7 +19488,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-16 10:17 UTC</t>
+          <t>2026-05-17 10:23 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -19063,7 +19513,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-16 10:17 UTC</t>
+          <t>2026-05-17 10:23 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -19088,7 +19538,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-16 10:17 UTC</t>
+          <t>2026-05-17 10:23 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -19113,7 +19563,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-16 10:17 UTC</t>
+          <t>2026-05-17 10:23 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -19138,7 +19588,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-16 10:17 UTC</t>
+          <t>2026-05-17 10:23 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -19163,7 +19613,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-16 10:17 UTC</t>
+          <t>2026-05-17 10:23 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -19172,76 +19622,6 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.fae045a1158903fc8baa.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.c31208edeb76d274f394.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.fae045a1158903fc8baa.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8d990b08b0b28aa5de58.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-18
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H491"/>
+  <dimension ref="A1:H501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -19182,6 +19182,386 @@
         </is>
       </c>
       <c r="H491" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="492" ht="15" customHeight="1">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>2026-05-18 12:33 UTC</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E492" t="n">
+        <v>0</v>
+      </c>
+      <c r="F492" t="n">
+        <v>0</v>
+      </c>
+      <c r="G492" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H492" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="493" ht="15" customHeight="1">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>2026-05-18 12:33 UTC</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E493" t="n">
+        <v>0</v>
+      </c>
+      <c r="F493" t="n">
+        <v>0</v>
+      </c>
+      <c r="G493" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H493" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="494" ht="15" customHeight="1">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>2026-05-18 12:33 UTC</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E494" t="n">
+        <v>0</v>
+      </c>
+      <c r="F494" t="n">
+        <v>0</v>
+      </c>
+      <c r="G494" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H494" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="495" ht="15" customHeight="1">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>2026-05-18 12:33 UTC</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E495" t="n">
+        <v>0</v>
+      </c>
+      <c r="F495" t="n">
+        <v>0</v>
+      </c>
+      <c r="G495" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H495" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="496" ht="15" customHeight="1">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>2026-05-18 12:33 UTC</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E496" t="n">
+        <v>0</v>
+      </c>
+      <c r="F496" t="n">
+        <v>0</v>
+      </c>
+      <c r="G496" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H496" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="497" ht="15" customHeight="1">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>2026-05-18 12:33 UTC</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E497" t="n">
+        <v>0</v>
+      </c>
+      <c r="F497" t="n">
+        <v>0</v>
+      </c>
+      <c r="G497" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H497" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="498" ht="15" customHeight="1">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>2026-05-18 12:33 UTC</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E498" t="n">
+        <v>0</v>
+      </c>
+      <c r="F498" t="n">
+        <v>0</v>
+      </c>
+      <c r="G498" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H498" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="499" ht="15" customHeight="1">
+      <c r="A499" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18 12:33 UTC</t>
+        </is>
+      </c>
+      <c r="B499" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C499" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D499" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E499" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F499" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G499" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.fae045a1158903fc8baa.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d7dd78d37688f764db64.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H499" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.fae045a1158903fc8baa.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.c31208edeb76d274f394.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="500" ht="15" customHeight="1">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>2026-05-18 12:33 UTC</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E500" t="n">
+        <v>0</v>
+      </c>
+      <c r="F500" t="n">
+        <v>0</v>
+      </c>
+      <c r="G500" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H500" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="501" ht="15" customHeight="1">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>2026-05-18 12:33 UTC</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E501" t="n">
+        <v>0</v>
+      </c>
+      <c r="F501" t="n">
+        <v>0</v>
+      </c>
+      <c r="G501" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H501" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -19268,76 +19648,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.fae045a1158903fc8baa.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.c31208edeb76d274f394.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.fae045a1158903fc8baa.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8d990b08b0b28aa5de58.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -19388,7 +19698,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-17 10:23 UTC</t>
+          <t>2026-05-18 12:33 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -19413,7 +19723,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-17 10:23 UTC</t>
+          <t>2026-05-18 12:33 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -19438,7 +19748,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-17 10:23 UTC</t>
+          <t>2026-05-18 12:33 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -19463,7 +19773,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-17 10:23 UTC</t>
+          <t>2026-05-18 12:33 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -19488,7 +19798,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-17 10:23 UTC</t>
+          <t>2026-05-18 12:33 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -19513,7 +19823,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-17 10:23 UTC</t>
+          <t>2026-05-18 12:33 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -19538,7 +19848,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-17 10:23 UTC</t>
+          <t>2026-05-18 12:33 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -19563,7 +19873,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-17 10:23 UTC</t>
+          <t>2026-05-18 12:33 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -19588,7 +19898,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-17 10:23 UTC</t>
+          <t>2026-05-18 12:33 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -19613,7 +19923,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-17 10:23 UTC</t>
+          <t>2026-05-18 12:33 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -19622,6 +19932,76 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.fae045a1158903fc8baa.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d7dd78d37688f764db64.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.fae045a1158903fc8baa.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.c31208edeb76d274f394.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-19
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H501"/>
+  <dimension ref="A1:H511"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -19562,6 +19562,386 @@
         </is>
       </c>
       <c r="H501" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="502" ht="15" customHeight="1">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:12 UTC</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E502" t="n">
+        <v>0</v>
+      </c>
+      <c r="F502" t="n">
+        <v>0</v>
+      </c>
+      <c r="G502" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H502" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="503" ht="15" customHeight="1">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:12 UTC</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E503" t="n">
+        <v>0</v>
+      </c>
+      <c r="F503" t="n">
+        <v>0</v>
+      </c>
+      <c r="G503" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H503" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="504" ht="15" customHeight="1">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:12 UTC</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E504" t="n">
+        <v>0</v>
+      </c>
+      <c r="F504" t="n">
+        <v>0</v>
+      </c>
+      <c r="G504" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H504" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="505" ht="15" customHeight="1">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:12 UTC</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E505" t="n">
+        <v>0</v>
+      </c>
+      <c r="F505" t="n">
+        <v>0</v>
+      </c>
+      <c r="G505" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H505" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="506" ht="15" customHeight="1">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:12 UTC</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E506" t="n">
+        <v>0</v>
+      </c>
+      <c r="F506" t="n">
+        <v>0</v>
+      </c>
+      <c r="G506" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H506" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="507" ht="15" customHeight="1">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:12 UTC</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E507" t="n">
+        <v>0</v>
+      </c>
+      <c r="F507" t="n">
+        <v>0</v>
+      </c>
+      <c r="G507" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H507" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="508" ht="15" customHeight="1">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:12 UTC</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E508" t="n">
+        <v>0</v>
+      </c>
+      <c r="F508" t="n">
+        <v>0</v>
+      </c>
+      <c r="G508" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H508" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="509" ht="15" customHeight="1">
+      <c r="A509" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:12 UTC</t>
+        </is>
+      </c>
+      <c r="B509" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C509" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D509" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E509" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F509" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G509" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.711f019df493afab78f0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.184e39e78fa1a338db4d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H509" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.fae045a1158903fc8baa.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d7dd78d37688f764db64.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="510" ht="15" customHeight="1">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:12 UTC</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E510" t="n">
+        <v>0</v>
+      </c>
+      <c r="F510" t="n">
+        <v>0</v>
+      </c>
+      <c r="G510" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H510" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="511" ht="15" customHeight="1">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>2026-05-19 12:12 UTC</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E511" t="n">
+        <v>0</v>
+      </c>
+      <c r="F511" t="n">
+        <v>0</v>
+      </c>
+      <c r="G511" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H511" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -19698,7 +20078,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-18 12:33 UTC</t>
+          <t>2026-05-19 12:12 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -19723,7 +20103,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-18 12:33 UTC</t>
+          <t>2026-05-19 12:12 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -19748,7 +20128,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-18 12:33 UTC</t>
+          <t>2026-05-19 12:12 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -19773,7 +20153,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-18 12:33 UTC</t>
+          <t>2026-05-19 12:12 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -19798,7 +20178,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-18 12:33 UTC</t>
+          <t>2026-05-19 12:12 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -19823,7 +20203,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-18 12:33 UTC</t>
+          <t>2026-05-19 12:12 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -19848,7 +20228,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-18 12:33 UTC</t>
+          <t>2026-05-19 12:12 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -19873,7 +20253,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-18 12:33 UTC</t>
+          <t>2026-05-19 12:12 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -19898,7 +20278,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-18 12:33 UTC</t>
+          <t>2026-05-19 12:12 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -19923,7 +20303,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-18 12:33 UTC</t>
+          <t>2026-05-19 12:12 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -19984,7 +20364,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.fae045a1158903fc8baa.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d7dd78d37688f764db64.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.711f019df493afab78f0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.184e39e78fa1a338db4d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -20001,7 +20381,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.fae045a1158903fc8baa.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.c31208edeb76d274f394.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.fae045a1158903fc8baa.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d7dd78d37688f764db64.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-20
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H511"/>
+  <dimension ref="A1:H521"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -19942,6 +19942,386 @@
         </is>
       </c>
       <c r="H511" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="512" ht="15" customHeight="1">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>2026-05-20 11:49 UTC</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E512" t="n">
+        <v>0</v>
+      </c>
+      <c r="F512" t="n">
+        <v>0</v>
+      </c>
+      <c r="G512" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H512" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="513" ht="15" customHeight="1">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>2026-05-20 11:49 UTC</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E513" t="n">
+        <v>0</v>
+      </c>
+      <c r="F513" t="n">
+        <v>0</v>
+      </c>
+      <c r="G513" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H513" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="514" ht="15" customHeight="1">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>2026-05-20 11:49 UTC</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E514" t="n">
+        <v>0</v>
+      </c>
+      <c r="F514" t="n">
+        <v>0</v>
+      </c>
+      <c r="G514" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H514" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="515" ht="15" customHeight="1">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>2026-05-20 11:49 UTC</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E515" t="n">
+        <v>0</v>
+      </c>
+      <c r="F515" t="n">
+        <v>0</v>
+      </c>
+      <c r="G515" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H515" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="516" ht="15" customHeight="1">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>2026-05-20 11:49 UTC</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E516" t="n">
+        <v>0</v>
+      </c>
+      <c r="F516" t="n">
+        <v>0</v>
+      </c>
+      <c r="G516" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H516" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="517" ht="15" customHeight="1">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>2026-05-20 11:49 UTC</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E517" t="n">
+        <v>0</v>
+      </c>
+      <c r="F517" t="n">
+        <v>0</v>
+      </c>
+      <c r="G517" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H517" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="518" ht="15" customHeight="1">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>2026-05-20 11:49 UTC</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E518" t="n">
+        <v>0</v>
+      </c>
+      <c r="F518" t="n">
+        <v>0</v>
+      </c>
+      <c r="G518" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H518" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="519" ht="15" customHeight="1">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>2026-05-20 11:49 UTC</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E519" t="n">
+        <v>0</v>
+      </c>
+      <c r="F519" t="n">
+        <v>0</v>
+      </c>
+      <c r="G519" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H519" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="520" ht="15" customHeight="1">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>2026-05-20 11:49 UTC</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E520" t="n">
+        <v>0</v>
+      </c>
+      <c r="F520" t="n">
+        <v>0</v>
+      </c>
+      <c r="G520" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H520" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="521" ht="15" customHeight="1">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>2026-05-20 11:49 UTC</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E521" t="n">
+        <v>0</v>
+      </c>
+      <c r="F521" t="n">
+        <v>0</v>
+      </c>
+      <c r="G521" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H521" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -20028,6 +20408,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.711f019df493afab78f0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.184e39e78fa1a338db4d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.fae045a1158903fc8baa.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d7dd78d37688f764db64.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -20078,7 +20528,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-19 12:12 UTC</t>
+          <t>2026-05-20 11:49 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -20103,7 +20553,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-19 12:12 UTC</t>
+          <t>2026-05-20 11:49 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -20128,7 +20578,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-19 12:12 UTC</t>
+          <t>2026-05-20 11:49 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -20153,7 +20603,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-19 12:12 UTC</t>
+          <t>2026-05-20 11:49 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -20178,7 +20628,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-19 12:12 UTC</t>
+          <t>2026-05-20 11:49 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -20203,7 +20653,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-19 12:12 UTC</t>
+          <t>2026-05-20 11:49 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -20228,7 +20678,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-19 12:12 UTC</t>
+          <t>2026-05-20 11:49 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -20253,7 +20703,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-19 12:12 UTC</t>
+          <t>2026-05-20 11:49 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -20278,7 +20728,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-19 12:12 UTC</t>
+          <t>2026-05-20 11:49 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -20303,7 +20753,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-19 12:12 UTC</t>
+          <t>2026-05-20 11:49 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -20312,76 +20762,6 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.711f019df493afab78f0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.184e39e78fa1a338db4d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.fae045a1158903fc8baa.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d7dd78d37688f764db64.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-21
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -8,17 +8,17 @@
   </bookViews>
   <sheets>
     <sheet name="Change Log" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="amc_com_ads_txt" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="amc_com_app-ads_txt" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="bbca_com_ads_txt" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="bbca_com_app-ads_txt" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="ifc_com_ads_txt" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ifc_com_app-ads_txt" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Current Snapshot" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="amc_com_ads_txt" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="amc_com_app-ads_txt" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="bbca_com_ads_txt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="bbca_com_app-ads_txt" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ifc_com_ads_txt" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="ifc_com_app-ads_txt" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="sundancetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="wetv_com_ads_txt" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="wetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H521"/>
+  <dimension ref="A1:H531"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -20322,6 +20322,431 @@
         </is>
       </c>
       <c r="H521" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="522" ht="15" customHeight="1">
+      <c r="A522" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 12:15 UTC</t>
+        </is>
+      </c>
+      <c r="B522" s="3" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C522" s="3" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D522" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E522" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F522" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G522" s="3" t="inlineStr">
+        <is>
+          <t>#Adtelligent: triplelift.com, 13152, RESELLER, 6c33edb13117fd86
+#Adtelligent: triplelift.com, 13152-EB, RESELLER, 6c33edb13117fd86
+#Xapads: lemmatechnologies.com, 2421, DIRECT, 7829010c5bebd1fb
+#Xapads: boldcollective.co, 774398, RESELLER
+#Xapads: sharethrough.com, 5855, RESELLER, d53b998a7bd4ecd3
+#Xapads: triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
+        </is>
+      </c>
+      <c r="H522" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="523" ht="15" customHeight="1">
+      <c r="A523" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 12:15 UTC</t>
+        </is>
+      </c>
+      <c r="B523" s="3" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C523" s="3" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D523" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E523" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F523" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G523" s="3" t="inlineStr">
+        <is>
+          <t>#Adtelligent: triplelift.com, 13152, RESELLER, 6c33edb13117fd86
+#Adtelligent: triplelift.com, 13152-EB, RESELLER, 6c33edb13117fd86
+#Xapads: lemmatechnologies.com, 2421, DIRECT, 7829010c5bebd1fb
+#Xapads: boldcollective.co, 774398, RESELLER
+#Xapads: sharethrough.com, 5855, RESELLER, d53b998a7bd4ecd3
+#Xapads: triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
+        </is>
+      </c>
+      <c r="H523" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="524" ht="15" customHeight="1">
+      <c r="A524" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 12:15 UTC</t>
+        </is>
+      </c>
+      <c r="B524" s="3" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C524" s="3" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D524" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E524" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F524" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G524" s="3" t="inlineStr">
+        <is>
+          <t>#Adtelligent: triplelift.com, 13152, RESELLER, 6c33edb13117fd86
+#Adtelligent: triplelift.com, 13152-EB, RESELLER, 6c33edb13117fd86
+#Xapads: lemmatechnologies.com, 2421, DIRECT, 7829010c5bebd1fb
+#Xapads: boldcollective.co, 774398, RESELLER
+#Xapads: sharethrough.com, 5855, RESELLER, d53b998a7bd4ecd3
+#Xapads: triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
+        </is>
+      </c>
+      <c r="H524" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="525" ht="15" customHeight="1">
+      <c r="A525" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 12:15 UTC</t>
+        </is>
+      </c>
+      <c r="B525" s="3" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C525" s="3" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D525" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E525" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F525" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G525" s="3" t="inlineStr">
+        <is>
+          <t>#Adtelligent: triplelift.com, 13152, RESELLER, 6c33edb13117fd86
+#Adtelligent: triplelift.com, 13152-EB, RESELLER, 6c33edb13117fd86
+#Xapads: lemmatechnologies.com, 2421, DIRECT, 7829010c5bebd1fb
+#Xapads: boldcollective.co, 774398, RESELLER
+#Xapads: sharethrough.com, 5855, RESELLER, d53b998a7bd4ecd3
+#Xapads: triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
+        </is>
+      </c>
+      <c r="H525" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="526" ht="15" customHeight="1">
+      <c r="A526" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 12:15 UTC</t>
+        </is>
+      </c>
+      <c r="B526" s="3" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C526" s="3" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D526" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E526" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F526" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G526" s="3" t="inlineStr">
+        <is>
+          <t>#Adtelligent: triplelift.com, 13152, RESELLER, 6c33edb13117fd86
+#Adtelligent: triplelift.com, 13152-EB, RESELLER, 6c33edb13117fd86
+#Xapads: lemmatechnologies.com, 2421, DIRECT, 7829010c5bebd1fb
+#Xapads: boldcollective.co, 774398, RESELLER
+#Xapads: sharethrough.com, 5855, RESELLER, d53b998a7bd4ecd3
+#Xapads: triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
+        </is>
+      </c>
+      <c r="H526" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="527" ht="15" customHeight="1">
+      <c r="A527" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 12:15 UTC</t>
+        </is>
+      </c>
+      <c r="B527" s="3" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C527" s="3" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D527" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E527" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F527" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G527" s="3" t="inlineStr">
+        <is>
+          <t>#Adtelligent: triplelift.com, 13152, RESELLER, 6c33edb13117fd86
+#Adtelligent: triplelift.com, 13152-EB, RESELLER, 6c33edb13117fd86
+#Xapads: lemmatechnologies.com, 2421, DIRECT, 7829010c5bebd1fb
+#Xapads: boldcollective.co, 774398, RESELLER
+#Xapads: sharethrough.com, 5855, RESELLER, d53b998a7bd4ecd3
+#Xapads: triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
+        </is>
+      </c>
+      <c r="H527" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="528" ht="15" customHeight="1">
+      <c r="A528" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 12:15 UTC</t>
+        </is>
+      </c>
+      <c r="B528" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C528" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D528" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E528" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F528" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G528" s="3" t="inlineStr">
+        <is>
+          <t>#Adtelligent: triplelift.com, 13152, RESELLER, 6c33edb13117fd86
+#Adtelligent: triplelift.com, 13152-EB, RESELLER, 6c33edb13117fd86
+#Xapads: lemmatechnologies.com, 2421, DIRECT, 7829010c5bebd1fb
+#Xapads: boldcollective.co, 774398, RESELLER
+#Xapads: sharethrough.com, 5855, RESELLER, d53b998a7bd4ecd3
+#Xapads: triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
+        </is>
+      </c>
+      <c r="H528" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="529" ht="15" customHeight="1">
+      <c r="A529" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 12:15 UTC</t>
+        </is>
+      </c>
+      <c r="B529" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C529" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D529" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E529" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F529" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G529" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.050cb33f285398d0fb3e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.711f019df493afab78f0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.434aaba86b25a73d6a00.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H529" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.711f019df493afab78f0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.184e39e78fa1a338db4d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="530" ht="15" customHeight="1">
+      <c r="A530" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 12:15 UTC</t>
+        </is>
+      </c>
+      <c r="B530" s="3" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C530" s="3" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D530" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E530" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F530" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G530" s="3" t="inlineStr">
+        <is>
+          <t>#Adtelligent: triplelift.com, 13152, RESELLER, 6c33edb13117fd86
+#Adtelligent: triplelift.com, 13152-EB, RESELLER, 6c33edb13117fd86
+#Xapads: lemmatechnologies.com, 2421, DIRECT, 7829010c5bebd1fb
+#Xapads: boldcollective.co, 774398, RESELLER
+#Xapads: sharethrough.com, 5855, RESELLER, d53b998a7bd4ecd3
+#Xapads: triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
+        </is>
+      </c>
+      <c r="H530" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="531" ht="15" customHeight="1">
+      <c r="A531" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-21 12:15 UTC</t>
+        </is>
+      </c>
+      <c r="B531" s="3" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C531" s="3" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D531" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E531" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F531" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G531" s="3" t="inlineStr">
+        <is>
+          <t>#Adtelligent: triplelift.com, 13152, RESELLER, 6c33edb13117fd86
+#Adtelligent: triplelift.com, 13152-EB, RESELLER, 6c33edb13117fd86
+#Xapads: lemmatechnologies.com, 2421, DIRECT, 7829010c5bebd1fb
+#Xapads: boldcollective.co, 774398, RESELLER
+#Xapads: sharethrough.com, 5855, RESELLER, d53b998a7bd4ecd3
+#Xapads: triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
+        </is>
+      </c>
+      <c r="H531" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -20371,29 +20796,29 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Oxiem</t>
+          <t>(no section)</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, sg1306174, RESELLER</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.050cb33f285398d0fb3e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.711f019df493afab78f0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.434aaba86b25a73d6a00.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>#Oxiem</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 545336-r-523319, RESELLER</t>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.711f019df493afab78f0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.184e39e78fa1a338db4d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -20408,7 +20833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20441,29 +20866,97 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>(no section)</t>
+          <t>#Adtelligent</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.711f019df493afab78f0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.184e39e78fa1a338db4d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>triplelift.com, 13152, RESELLER, 6c33edb13117fd86</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.fae045a1158903fc8baa.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d7dd78d37688f764db64.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>#Adtelligent</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>triplelift.com, 13152-EB, RESELLER, 6c33edb13117fd86</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>lemmatechnologies.com, 2421, DIRECT, 7829010c5bebd1fb</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>boldcollective.co, 774398, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>sharethrough.com, 5855, RESELLER, d53b998a7bd4ecd3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
         </is>
       </c>
     </row>
@@ -20473,6 +20966,144 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>#Adtelligent</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>triplelift.com, 13152, RESELLER, 6c33edb13117fd86</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>#Adtelligent</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>triplelift.com, 13152-EB, RESELLER, 6c33edb13117fd86</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>lemmatechnologies.com, 2421, DIRECT, 7829010c5bebd1fb</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>boldcollective.co, 774398, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>sharethrough.com, 5855, RESELLER, d53b998a7bd4ecd3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20528,11 +21159,11 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-20 11:49 UTC</t>
+          <t>2026-05-21 12:15 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1142</v>
+        <v>1148</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -20553,11 +21184,11 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-20 11:49 UTC</t>
+          <t>2026-05-21 12:15 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1056</v>
+        <v>1062</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -20578,11 +21209,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-20 11:49 UTC</t>
+          <t>2026-05-21 12:15 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1142</v>
+        <v>1148</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -20603,11 +21234,11 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-20 11:49 UTC</t>
+          <t>2026-05-21 12:15 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1056</v>
+        <v>1062</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -20628,11 +21259,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-20 11:49 UTC</t>
+          <t>2026-05-21 12:15 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1142</v>
+        <v>1148</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -20653,11 +21284,11 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-20 11:49 UTC</t>
+          <t>2026-05-21 12:15 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1056</v>
+        <v>1062</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -20678,11 +21309,11 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-20 11:49 UTC</t>
+          <t>2026-05-21 12:15 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1142</v>
+        <v>1148</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -20703,7 +21334,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-20 11:49 UTC</t>
+          <t>2026-05-21 12:15 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -20728,11 +21359,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-20 11:49 UTC</t>
+          <t>2026-05-21 12:15 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1142</v>
+        <v>1148</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -20753,85 +21384,15 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-20 11:49 UTC</t>
+          <t>2026-05-21 12:15 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1056</v>
+        <v>1062</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>#Oxiem</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, sg1306174, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>#Oxiem</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 545336-r-523319, RESELLER</t>
         </is>
       </c>
     </row>
@@ -20846,7 +21407,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20879,12 +21440,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Oxiem</t>
+          <t>#Adtelligent</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, sg1306174, RESELLER</t>
+          <t>triplelift.com, 13152, RESELLER, 6c33edb13117fd86</t>
         </is>
       </c>
     </row>
@@ -20896,12 +21457,80 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>#Oxiem</t>
+          <t>#Adtelligent</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, 545336-r-523319, RESELLER</t>
+          <t>triplelift.com, 13152-EB, RESELLER, 6c33edb13117fd86</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>lemmatechnologies.com, 2421, DIRECT, 7829010c5bebd1fb</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>boldcollective.co, 774398, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>sharethrough.com, 5855, RESELLER, d53b998a7bd4ecd3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
         </is>
       </c>
     </row>
@@ -20916,7 +21545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20949,12 +21578,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Oxiem</t>
+          <t>#Adtelligent</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, sg1306174, RESELLER</t>
+          <t>triplelift.com, 13152, RESELLER, 6c33edb13117fd86</t>
         </is>
       </c>
     </row>
@@ -20966,12 +21595,80 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>#Oxiem</t>
+          <t>#Adtelligent</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, 545336-r-523319, RESELLER</t>
+          <t>triplelift.com, 13152-EB, RESELLER, 6c33edb13117fd86</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>lemmatechnologies.com, 2421, DIRECT, 7829010c5bebd1fb</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>boldcollective.co, 774398, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>sharethrough.com, 5855, RESELLER, d53b998a7bd4ecd3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
         </is>
       </c>
     </row>
@@ -20986,7 +21683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21019,12 +21716,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Oxiem</t>
+          <t>#Adtelligent</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, sg1306174, RESELLER</t>
+          <t>triplelift.com, 13152, RESELLER, 6c33edb13117fd86</t>
         </is>
       </c>
     </row>
@@ -21036,12 +21733,80 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>#Oxiem</t>
+          <t>#Adtelligent</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, 545336-r-523319, RESELLER</t>
+          <t>triplelift.com, 13152-EB, RESELLER, 6c33edb13117fd86</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>lemmatechnologies.com, 2421, DIRECT, 7829010c5bebd1fb</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>boldcollective.co, 774398, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>sharethrough.com, 5855, RESELLER, d53b998a7bd4ecd3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
         </is>
       </c>
     </row>
@@ -21056,7 +21821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21089,12 +21854,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Oxiem</t>
+          <t>#Adtelligent</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, sg1306174, RESELLER</t>
+          <t>triplelift.com, 13152, RESELLER, 6c33edb13117fd86</t>
         </is>
       </c>
     </row>
@@ -21106,12 +21871,80 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>#Oxiem</t>
+          <t>#Adtelligent</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, 545336-r-523319, RESELLER</t>
+          <t>triplelift.com, 13152-EB, RESELLER, 6c33edb13117fd86</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>lemmatechnologies.com, 2421, DIRECT, 7829010c5bebd1fb</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>boldcollective.co, 774398, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>sharethrough.com, 5855, RESELLER, d53b998a7bd4ecd3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
         </is>
       </c>
     </row>
@@ -21126,7 +21959,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21159,12 +21992,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Oxiem</t>
+          <t>#Adtelligent</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, sg1306174, RESELLER</t>
+          <t>triplelift.com, 13152, RESELLER, 6c33edb13117fd86</t>
         </is>
       </c>
     </row>
@@ -21176,12 +22009,80 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>#Oxiem</t>
+          <t>#Adtelligent</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, 545336-r-523319, RESELLER</t>
+          <t>triplelift.com, 13152-EB, RESELLER, 6c33edb13117fd86</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>lemmatechnologies.com, 2421, DIRECT, 7829010c5bebd1fb</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>boldcollective.co, 774398, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>sharethrough.com, 5855, RESELLER, d53b998a7bd4ecd3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
         </is>
       </c>
     </row>
@@ -21196,7 +22097,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21229,12 +22130,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Oxiem</t>
+          <t>#Adtelligent</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, sg1306174, RESELLER</t>
+          <t>triplelift.com, 13152, RESELLER, 6c33edb13117fd86</t>
         </is>
       </c>
     </row>
@@ -21246,12 +22147,80 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>#Oxiem</t>
+          <t>#Adtelligent</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, 545336-r-523319, RESELLER</t>
+          <t>triplelift.com, 13152-EB, RESELLER, 6c33edb13117fd86</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>lemmatechnologies.com, 2421, DIRECT, 7829010c5bebd1fb</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>boldcollective.co, 774398, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>sharethrough.com, 5855, RESELLER, d53b998a7bd4ecd3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
         </is>
       </c>
     </row>
@@ -21266,7 +22235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21299,12 +22268,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#Oxiem</t>
+          <t>#Adtelligent</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, sg1306174, RESELLER</t>
+          <t>triplelift.com, 13152, RESELLER, 6c33edb13117fd86</t>
         </is>
       </c>
     </row>
@@ -21316,12 +22285,80 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>#Oxiem</t>
+          <t>#Adtelligent</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>freewheel.tv, 545336-r-523319, RESELLER</t>
+          <t>triplelift.com, 13152-EB, RESELLER, 6c33edb13117fd86</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>lemmatechnologies.com, 2421, DIRECT, 7829010c5bebd1fb</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>boldcollective.co, 774398, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>sharethrough.com, 5855, RESELLER, d53b998a7bd4ecd3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-22
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -8,17 +8,17 @@
   </bookViews>
   <sheets>
     <sheet name="Change Log" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Current Snapshot" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="amc_com_ads_txt" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="amc_com_app-ads_txt" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="bbca_com_ads_txt" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="bbca_com_app-ads_txt" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ifc_com_ads_txt" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="ifc_com_app-ads_txt" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="sundancetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="wetv_com_ads_txt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="wetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="amc_com_ads_txt" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="amc_com_app-ads_txt" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="bbca_com_ads_txt" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="bbca_com_app-ads_txt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ifc_com_ads_txt" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ifc_com_app-ads_txt" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H531"/>
+  <dimension ref="A1:H541"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -20752,82 +20752,392 @@
         </is>
       </c>
     </row>
+    <row r="532" ht="15" customHeight="1">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>2026-05-22 11:46 UTC</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E532" t="n">
+        <v>0</v>
+      </c>
+      <c r="F532" t="n">
+        <v>0</v>
+      </c>
+      <c r="G532" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H532" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="533" ht="15" customHeight="1">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>2026-05-22 11:46 UTC</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E533" t="n">
+        <v>0</v>
+      </c>
+      <c r="F533" t="n">
+        <v>0</v>
+      </c>
+      <c r="G533" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H533" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="534" ht="15" customHeight="1">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>2026-05-22 11:46 UTC</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E534" t="n">
+        <v>0</v>
+      </c>
+      <c r="F534" t="n">
+        <v>0</v>
+      </c>
+      <c r="G534" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H534" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="535" ht="15" customHeight="1">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>2026-05-22 11:46 UTC</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E535" t="n">
+        <v>0</v>
+      </c>
+      <c r="F535" t="n">
+        <v>0</v>
+      </c>
+      <c r="G535" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H535" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="536" ht="15" customHeight="1">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>2026-05-22 11:46 UTC</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D536" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E536" t="n">
+        <v>0</v>
+      </c>
+      <c r="F536" t="n">
+        <v>0</v>
+      </c>
+      <c r="G536" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H536" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="537" ht="15" customHeight="1">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>2026-05-22 11:46 UTC</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D537" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E537" t="n">
+        <v>0</v>
+      </c>
+      <c r="F537" t="n">
+        <v>0</v>
+      </c>
+      <c r="G537" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H537" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="538" ht="15" customHeight="1">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>2026-05-22 11:46 UTC</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D538" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E538" t="n">
+        <v>0</v>
+      </c>
+      <c r="F538" t="n">
+        <v>0</v>
+      </c>
+      <c r="G538" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H538" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="539" ht="15" customHeight="1">
+      <c r="A539" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-22 11:46 UTC</t>
+        </is>
+      </c>
+      <c r="B539" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C539" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D539" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E539" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F539" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G539" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.050cb33f285398d0fb3e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.5cb52607615d3a459462.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8011.a103a7b41c1e8b8de75f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d4f5e9f0277f63619f95.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/8011.82613a08ccb02e6f6d26.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H539" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.050cb33f285398d0fb3e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.711f019df493afab78f0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.434aaba86b25a73d6a00.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="540" ht="15" customHeight="1">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>2026-05-22 11:46 UTC</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D540" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E540" t="n">
+        <v>0</v>
+      </c>
+      <c r="F540" t="n">
+        <v>0</v>
+      </c>
+      <c r="G540" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H540" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="541" ht="15" customHeight="1">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>2026-05-22 11:46 UTC</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D541" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E541" t="n">
+        <v>0</v>
+      </c>
+      <c r="F541" t="n">
+        <v>0</v>
+      </c>
+      <c r="G541" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H541" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.050cb33f285398d0fb3e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.711f019df493afab78f0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.434aaba86b25a73d6a00.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.aca7fbefb7eb135e1f3d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.711f019df493afab78f0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.184e39e78fa1a338db4d.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20965,145 +21275,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>#Adtelligent</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>triplelift.com, 13152, RESELLER, 6c33edb13117fd86</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>#Adtelligent</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>triplelift.com, 13152-EB, RESELLER, 6c33edb13117fd86</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>lemmatechnologies.com, 2421, DIRECT, 7829010c5bebd1fb</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>boldcollective.co, 774398, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>sharethrough.com, 5855, RESELLER, d53b998a7bd4ecd3</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>#Xapads</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21159,7 +21331,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-21 12:15 UTC</t>
+          <t>2026-05-22 11:46 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -21184,7 +21356,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-21 12:15 UTC</t>
+          <t>2026-05-22 11:46 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -21209,7 +21381,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-21 12:15 UTC</t>
+          <t>2026-05-22 11:46 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -21234,7 +21406,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-21 12:15 UTC</t>
+          <t>2026-05-22 11:46 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -21259,7 +21431,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-21 12:15 UTC</t>
+          <t>2026-05-22 11:46 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -21284,7 +21456,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-21 12:15 UTC</t>
+          <t>2026-05-22 11:46 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -21309,7 +21481,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-21 12:15 UTC</t>
+          <t>2026-05-22 11:46 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -21334,7 +21506,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-21 12:15 UTC</t>
+          <t>2026-05-22 11:46 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -21359,7 +21531,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-21 12:15 UTC</t>
+          <t>2026-05-22 11:46 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -21384,7 +21556,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-21 12:15 UTC</t>
+          <t>2026-05-22 11:46 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -21393,6 +21565,214 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.050cb33f285398d0fb3e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.5cb52607615d3a459462.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8011.a103a7b41c1e8b8de75f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d4f5e9f0277f63619f95.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/8011.82613a08ccb02e6f6d26.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.050cb33f285398d0fb3e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.711f019df493afab78f0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.434aaba86b25a73d6a00.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>#Adtelligent</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>triplelift.com, 13152, RESELLER, 6c33edb13117fd86</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>#Adtelligent</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>triplelift.com, 13152-EB, RESELLER, 6c33edb13117fd86</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>lemmatechnologies.com, 2421, DIRECT, 7829010c5bebd1fb</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>boldcollective.co, 774398, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>sharethrough.com, 5855, RESELLER, d53b998a7bd4ecd3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>#Xapads</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>triplelift.com, 14703, RESELLER, 6c33edb13117fd86</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-23
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H541"/>
+  <dimension ref="A1:H551"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -21127,6 +21127,386 @@
         </is>
       </c>
       <c r="H541" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="542" ht="15" customHeight="1">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>2026-05-23 10:26 UTC</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D542" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E542" t="n">
+        <v>0</v>
+      </c>
+      <c r="F542" t="n">
+        <v>0</v>
+      </c>
+      <c r="G542" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H542" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="543" ht="15" customHeight="1">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>2026-05-23 10:26 UTC</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D543" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E543" t="n">
+        <v>0</v>
+      </c>
+      <c r="F543" t="n">
+        <v>0</v>
+      </c>
+      <c r="G543" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H543" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="544" ht="15" customHeight="1">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>2026-05-23 10:26 UTC</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D544" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E544" t="n">
+        <v>0</v>
+      </c>
+      <c r="F544" t="n">
+        <v>0</v>
+      </c>
+      <c r="G544" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H544" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="545" ht="15" customHeight="1">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>2026-05-23 10:26 UTC</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D545" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E545" t="n">
+        <v>0</v>
+      </c>
+      <c r="F545" t="n">
+        <v>0</v>
+      </c>
+      <c r="G545" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H545" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="546" ht="15" customHeight="1">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>2026-05-23 10:26 UTC</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D546" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E546" t="n">
+        <v>0</v>
+      </c>
+      <c r="F546" t="n">
+        <v>0</v>
+      </c>
+      <c r="G546" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H546" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="547" ht="15" customHeight="1">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>2026-05-23 10:26 UTC</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D547" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E547" t="n">
+        <v>0</v>
+      </c>
+      <c r="F547" t="n">
+        <v>0</v>
+      </c>
+      <c r="G547" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H547" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="548" ht="15" customHeight="1">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>2026-05-23 10:26 UTC</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D548" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E548" t="n">
+        <v>0</v>
+      </c>
+      <c r="F548" t="n">
+        <v>0</v>
+      </c>
+      <c r="G548" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H548" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="549" ht="15" customHeight="1">
+      <c r="A549" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-23 10:26 UTC</t>
+        </is>
+      </c>
+      <c r="B549" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C549" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D549" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E549" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F549" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G549" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.f373aa0ed768a56d6f0e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8011.b6799ed0437c32506814.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.fba1426197a32f0e32aa.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8011.82613a08ccb02e6f6d26.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H549" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.050cb33f285398d0fb3e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.5cb52607615d3a459462.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8011.a103a7b41c1e8b8de75f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d4f5e9f0277f63619f95.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/8011.82613a08ccb02e6f6d26.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="550" ht="15" customHeight="1">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>2026-05-23 10:26 UTC</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D550" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E550" t="n">
+        <v>0</v>
+      </c>
+      <c r="F550" t="n">
+        <v>0</v>
+      </c>
+      <c r="G550" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H550" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="551" ht="15" customHeight="1">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>2026-05-23 10:26 UTC</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D551" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E551" t="n">
+        <v>0</v>
+      </c>
+      <c r="F551" t="n">
+        <v>0</v>
+      </c>
+      <c r="G551" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H551" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -21331,7 +21711,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-22 11:46 UTC</t>
+          <t>2026-05-23 10:26 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -21356,7 +21736,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-22 11:46 UTC</t>
+          <t>2026-05-23 10:26 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -21381,7 +21761,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-22 11:46 UTC</t>
+          <t>2026-05-23 10:26 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -21406,7 +21786,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-22 11:46 UTC</t>
+          <t>2026-05-23 10:26 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -21431,7 +21811,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-22 11:46 UTC</t>
+          <t>2026-05-23 10:26 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -21456,7 +21836,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-22 11:46 UTC</t>
+          <t>2026-05-23 10:26 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -21481,7 +21861,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-22 11:46 UTC</t>
+          <t>2026-05-23 10:26 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -21506,7 +21886,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-22 11:46 UTC</t>
+          <t>2026-05-23 10:26 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -21531,7 +21911,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-22 11:46 UTC</t>
+          <t>2026-05-23 10:26 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -21556,7 +21936,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-22 11:46 UTC</t>
+          <t>2026-05-23 10:26 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -21617,7 +21997,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.050cb33f285398d0fb3e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.5cb52607615d3a459462.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8011.a103a7b41c1e8b8de75f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d4f5e9f0277f63619f95.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/8011.82613a08ccb02e6f6d26.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.f373aa0ed768a56d6f0e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8011.b6799ed0437c32506814.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.fba1426197a32f0e32aa.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8011.82613a08ccb02e6f6d26.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -21634,7 +22014,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.050cb33f285398d0fb3e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.665a8dfa91838b83dbb0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/1694.711f019df493afab78f0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.434aaba86b25a73d6a00.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/1694.ccb7210da63f32716f75.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.050cb33f285398d0fb3e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.5cb52607615d3a459462.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8011.a103a7b41c1e8b8de75f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d4f5e9f0277f63619f95.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/8011.82613a08ccb02e6f6d26.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-24
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H551"/>
+  <dimension ref="A1:H561"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -21507,6 +21507,386 @@
         </is>
       </c>
       <c r="H551" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="552" ht="15" customHeight="1">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>2026-05-24 10:42 UTC</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E552" t="n">
+        <v>0</v>
+      </c>
+      <c r="F552" t="n">
+        <v>0</v>
+      </c>
+      <c r="G552" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H552" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="553" ht="15" customHeight="1">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>2026-05-24 10:42 UTC</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E553" t="n">
+        <v>0</v>
+      </c>
+      <c r="F553" t="n">
+        <v>0</v>
+      </c>
+      <c r="G553" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H553" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="554" ht="15" customHeight="1">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>2026-05-24 10:42 UTC</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E554" t="n">
+        <v>0</v>
+      </c>
+      <c r="F554" t="n">
+        <v>0</v>
+      </c>
+      <c r="G554" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H554" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="555" ht="15" customHeight="1">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>2026-05-24 10:42 UTC</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E555" t="n">
+        <v>0</v>
+      </c>
+      <c r="F555" t="n">
+        <v>0</v>
+      </c>
+      <c r="G555" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H555" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="556" ht="15" customHeight="1">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>2026-05-24 10:42 UTC</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E556" t="n">
+        <v>0</v>
+      </c>
+      <c r="F556" t="n">
+        <v>0</v>
+      </c>
+      <c r="G556" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H556" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="557" ht="15" customHeight="1">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>2026-05-24 10:42 UTC</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E557" t="n">
+        <v>0</v>
+      </c>
+      <c r="F557" t="n">
+        <v>0</v>
+      </c>
+      <c r="G557" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H557" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="558" ht="15" customHeight="1">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>2026-05-24 10:42 UTC</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E558" t="n">
+        <v>0</v>
+      </c>
+      <c r="F558" t="n">
+        <v>0</v>
+      </c>
+      <c r="G558" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H558" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="559" ht="15" customHeight="1">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>2026-05-24 10:42 UTC</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E559" t="n">
+        <v>0</v>
+      </c>
+      <c r="F559" t="n">
+        <v>0</v>
+      </c>
+      <c r="G559" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H559" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="560" ht="15" customHeight="1">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>2026-05-24 10:42 UTC</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E560" t="n">
+        <v>0</v>
+      </c>
+      <c r="F560" t="n">
+        <v>0</v>
+      </c>
+      <c r="G560" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H560" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="561" ht="15" customHeight="1">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>2026-05-24 10:42 UTC</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E561" t="n">
+        <v>0</v>
+      </c>
+      <c r="F561" t="n">
+        <v>0</v>
+      </c>
+      <c r="G561" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H561" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -21661,6 +22041,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.f373aa0ed768a56d6f0e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8011.b6799ed0437c32506814.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.fba1426197a32f0e32aa.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8011.82613a08ccb02e6f6d26.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.050cb33f285398d0fb3e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.5cb52607615d3a459462.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8011.a103a7b41c1e8b8de75f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d4f5e9f0277f63619f95.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/8011.82613a08ccb02e6f6d26.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -21711,7 +22161,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-23 10:26 UTC</t>
+          <t>2026-05-24 10:42 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -21736,7 +22186,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-23 10:26 UTC</t>
+          <t>2026-05-24 10:42 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -21761,7 +22211,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-23 10:26 UTC</t>
+          <t>2026-05-24 10:42 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -21786,7 +22236,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-23 10:26 UTC</t>
+          <t>2026-05-24 10:42 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -21811,7 +22261,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-23 10:26 UTC</t>
+          <t>2026-05-24 10:42 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -21836,7 +22286,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-23 10:26 UTC</t>
+          <t>2026-05-24 10:42 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -21861,7 +22311,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-23 10:26 UTC</t>
+          <t>2026-05-24 10:42 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -21886,7 +22336,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-23 10:26 UTC</t>
+          <t>2026-05-24 10:42 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -21911,7 +22361,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-23 10:26 UTC</t>
+          <t>2026-05-24 10:42 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -21936,7 +22386,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-23 10:26 UTC</t>
+          <t>2026-05-24 10:42 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -21945,76 +22395,6 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.f373aa0ed768a56d6f0e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8011.b6799ed0437c32506814.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.fba1426197a32f0e32aa.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8011.82613a08ccb02e6f6d26.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.050cb33f285398d0fb3e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.5cb52607615d3a459462.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8011.a103a7b41c1e8b8de75f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d4f5e9f0277f63619f95.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/8011.82613a08ccb02e6f6d26.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-25
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H561"/>
+  <dimension ref="A1:H571"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -21887,6 +21887,386 @@
         </is>
       </c>
       <c r="H561" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="562" ht="15" customHeight="1">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>2026-05-25 12:32 UTC</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E562" t="n">
+        <v>0</v>
+      </c>
+      <c r="F562" t="n">
+        <v>0</v>
+      </c>
+      <c r="G562" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H562" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="563" ht="15" customHeight="1">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>2026-05-25 12:32 UTC</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E563" t="n">
+        <v>0</v>
+      </c>
+      <c r="F563" t="n">
+        <v>0</v>
+      </c>
+      <c r="G563" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H563" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="564" ht="15" customHeight="1">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>2026-05-25 12:32 UTC</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E564" t="n">
+        <v>0</v>
+      </c>
+      <c r="F564" t="n">
+        <v>0</v>
+      </c>
+      <c r="G564" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H564" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="565" ht="15" customHeight="1">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>2026-05-25 12:32 UTC</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E565" t="n">
+        <v>0</v>
+      </c>
+      <c r="F565" t="n">
+        <v>0</v>
+      </c>
+      <c r="G565" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H565" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="566" ht="15" customHeight="1">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>2026-05-25 12:32 UTC</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E566" t="n">
+        <v>0</v>
+      </c>
+      <c r="F566" t="n">
+        <v>0</v>
+      </c>
+      <c r="G566" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H566" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="567" ht="15" customHeight="1">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>2026-05-25 12:32 UTC</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E567" t="n">
+        <v>0</v>
+      </c>
+      <c r="F567" t="n">
+        <v>0</v>
+      </c>
+      <c r="G567" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H567" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="568" ht="15" customHeight="1">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>2026-05-25 12:32 UTC</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E568" t="n">
+        <v>0</v>
+      </c>
+      <c r="F568" t="n">
+        <v>0</v>
+      </c>
+      <c r="G568" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H568" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="569" ht="15" customHeight="1">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>2026-05-25 12:32 UTC</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E569" t="n">
+        <v>0</v>
+      </c>
+      <c r="F569" t="n">
+        <v>0</v>
+      </c>
+      <c r="G569" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H569" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="570" ht="15" customHeight="1">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>2026-05-25 12:32 UTC</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E570" t="n">
+        <v>0</v>
+      </c>
+      <c r="F570" t="n">
+        <v>0</v>
+      </c>
+      <c r="G570" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H570" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="571" ht="15" customHeight="1">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>2026-05-25 12:32 UTC</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E571" t="n">
+        <v>0</v>
+      </c>
+      <c r="F571" t="n">
+        <v>0</v>
+      </c>
+      <c r="G571" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H571" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -22161,7 +22541,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-24 10:42 UTC</t>
+          <t>2026-05-25 12:32 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -22186,7 +22566,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-24 10:42 UTC</t>
+          <t>2026-05-25 12:32 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -22211,7 +22591,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-24 10:42 UTC</t>
+          <t>2026-05-25 12:32 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -22236,7 +22616,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-24 10:42 UTC</t>
+          <t>2026-05-25 12:32 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -22261,7 +22641,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-24 10:42 UTC</t>
+          <t>2026-05-25 12:32 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -22286,7 +22666,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-24 10:42 UTC</t>
+          <t>2026-05-25 12:32 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -22311,7 +22691,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-24 10:42 UTC</t>
+          <t>2026-05-25 12:32 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -22336,7 +22716,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-24 10:42 UTC</t>
+          <t>2026-05-25 12:32 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -22361,7 +22741,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-24 10:42 UTC</t>
+          <t>2026-05-25 12:32 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -22386,7 +22766,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-24 10:42 UTC</t>
+          <t>2026-05-25 12:32 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-27
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H571"/>
+  <dimension ref="A1:H581"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -22267,6 +22267,386 @@
         </is>
       </c>
       <c r="H571" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="572" ht="15" customHeight="1">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>2026-05-27 12:21 UTC</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E572" t="n">
+        <v>0</v>
+      </c>
+      <c r="F572" t="n">
+        <v>0</v>
+      </c>
+      <c r="G572" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H572" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="573" ht="15" customHeight="1">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>2026-05-27 12:21 UTC</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E573" t="n">
+        <v>0</v>
+      </c>
+      <c r="F573" t="n">
+        <v>0</v>
+      </c>
+      <c r="G573" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H573" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="574" ht="15" customHeight="1">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>2026-05-27 12:21 UTC</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E574" t="n">
+        <v>0</v>
+      </c>
+      <c r="F574" t="n">
+        <v>0</v>
+      </c>
+      <c r="G574" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H574" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="575" ht="15" customHeight="1">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>2026-05-27 12:21 UTC</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E575" t="n">
+        <v>0</v>
+      </c>
+      <c r="F575" t="n">
+        <v>0</v>
+      </c>
+      <c r="G575" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H575" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="576" ht="15" customHeight="1">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>2026-05-27 12:21 UTC</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E576" t="n">
+        <v>0</v>
+      </c>
+      <c r="F576" t="n">
+        <v>0</v>
+      </c>
+      <c r="G576" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H576" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="577" ht="15" customHeight="1">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>2026-05-27 12:21 UTC</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E577" t="n">
+        <v>0</v>
+      </c>
+      <c r="F577" t="n">
+        <v>0</v>
+      </c>
+      <c r="G577" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H577" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="578" ht="15" customHeight="1">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>2026-05-27 12:21 UTC</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E578" t="n">
+        <v>0</v>
+      </c>
+      <c r="F578" t="n">
+        <v>0</v>
+      </c>
+      <c r="G578" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H578" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="579" ht="15" customHeight="1">
+      <c r="A579" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-27 12:21 UTC</t>
+        </is>
+      </c>
+      <c r="B579" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C579" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D579" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E579" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F579" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G579" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8011.49bc5730da39751cebc3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.6c026d0f0a7324e83bfc.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8011.82613a08ccb02e6f6d26.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H579" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.f373aa0ed768a56d6f0e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8011.b6799ed0437c32506814.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.fba1426197a32f0e32aa.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8011.82613a08ccb02e6f6d26.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="580" ht="15" customHeight="1">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>2026-05-27 12:21 UTC</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E580" t="n">
+        <v>0</v>
+      </c>
+      <c r="F580" t="n">
+        <v>0</v>
+      </c>
+      <c r="G580" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H580" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="581" ht="15" customHeight="1">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>2026-05-27 12:21 UTC</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E581" t="n">
+        <v>0</v>
+      </c>
+      <c r="F581" t="n">
+        <v>0</v>
+      </c>
+      <c r="G581" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H581" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -22421,76 +22801,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.f373aa0ed768a56d6f0e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8011.b6799ed0437c32506814.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.fba1426197a32f0e32aa.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8011.82613a08ccb02e6f6d26.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/257.1fb5b028bc284f5b82cf.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.050cb33f285398d0fb3e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.5cb52607615d3a459462.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8011.a103a7b41c1e8b8de75f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d4f5e9f0277f63619f95.js"&gt;&lt;/script&gt;&lt;link href="/style/css/257.ca80321498efda8a07d3.css" rel="stylesheet"&gt;&lt;link href="/style/css/8011.82613a08ccb02e6f6d26.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -22541,7 +22851,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-25 12:32 UTC</t>
+          <t>2026-05-27 12:21 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -22566,7 +22876,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-25 12:32 UTC</t>
+          <t>2026-05-27 12:21 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -22591,7 +22901,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-25 12:32 UTC</t>
+          <t>2026-05-27 12:21 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -22616,7 +22926,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-25 12:32 UTC</t>
+          <t>2026-05-27 12:21 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -22641,7 +22951,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-25 12:32 UTC</t>
+          <t>2026-05-27 12:21 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -22666,7 +22976,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-25 12:32 UTC</t>
+          <t>2026-05-27 12:21 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -22691,7 +23001,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-25 12:32 UTC</t>
+          <t>2026-05-27 12:21 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -22716,7 +23026,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-25 12:32 UTC</t>
+          <t>2026-05-27 12:21 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -22741,7 +23051,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-25 12:32 UTC</t>
+          <t>2026-05-27 12:21 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -22766,7 +23076,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-25 12:32 UTC</t>
+          <t>2026-05-27 12:21 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -22775,6 +23085,76 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8011.49bc5730da39751cebc3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.6c026d0f0a7324e83bfc.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8011.82613a08ccb02e6f6d26.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.f373aa0ed768a56d6f0e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8011.b6799ed0437c32506814.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.fba1426197a32f0e32aa.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8011.82613a08ccb02e6f6d26.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-28
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H581"/>
+  <dimension ref="A1:H591"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -22647,6 +22647,386 @@
         </is>
       </c>
       <c r="H581" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="582" ht="15" customHeight="1">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>2026-05-28 12:28 UTC</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E582" t="n">
+        <v>0</v>
+      </c>
+      <c r="F582" t="n">
+        <v>0</v>
+      </c>
+      <c r="G582" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H582" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="583" ht="15" customHeight="1">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>2026-05-28 12:28 UTC</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E583" t="n">
+        <v>0</v>
+      </c>
+      <c r="F583" t="n">
+        <v>0</v>
+      </c>
+      <c r="G583" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H583" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="584" ht="15" customHeight="1">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>2026-05-28 12:28 UTC</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E584" t="n">
+        <v>0</v>
+      </c>
+      <c r="F584" t="n">
+        <v>0</v>
+      </c>
+      <c r="G584" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H584" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="585" ht="15" customHeight="1">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>2026-05-28 12:28 UTC</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E585" t="n">
+        <v>0</v>
+      </c>
+      <c r="F585" t="n">
+        <v>0</v>
+      </c>
+      <c r="G585" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H585" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="586" ht="15" customHeight="1">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>2026-05-28 12:28 UTC</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E586" t="n">
+        <v>0</v>
+      </c>
+      <c r="F586" t="n">
+        <v>0</v>
+      </c>
+      <c r="G586" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H586" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="587" ht="15" customHeight="1">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>2026-05-28 12:28 UTC</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E587" t="n">
+        <v>0</v>
+      </c>
+      <c r="F587" t="n">
+        <v>0</v>
+      </c>
+      <c r="G587" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H587" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="588" ht="15" customHeight="1">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>2026-05-28 12:28 UTC</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E588" t="n">
+        <v>0</v>
+      </c>
+      <c r="F588" t="n">
+        <v>0</v>
+      </c>
+      <c r="G588" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H588" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="589" ht="15" customHeight="1">
+      <c r="A589" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-28 12:28 UTC</t>
+        </is>
+      </c>
+      <c r="B589" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C589" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D589" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E589" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F589" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G589" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.6d2d8a5dcbf441ae99c9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.92dd16071b63ae3fa439.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H589" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8011.49bc5730da39751cebc3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.6c026d0f0a7324e83bfc.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8011.82613a08ccb02e6f6d26.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="590" ht="15" customHeight="1">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>2026-05-28 12:28 UTC</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E590" t="n">
+        <v>0</v>
+      </c>
+      <c r="F590" t="n">
+        <v>0</v>
+      </c>
+      <c r="G590" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H590" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="591" ht="15" customHeight="1">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>2026-05-28 12:28 UTC</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E591" t="n">
+        <v>0</v>
+      </c>
+      <c r="F591" t="n">
+        <v>0</v>
+      </c>
+      <c r="G591" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H591" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -22851,7 +23231,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-27 12:21 UTC</t>
+          <t>2026-05-28 12:28 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -22876,7 +23256,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-27 12:21 UTC</t>
+          <t>2026-05-28 12:28 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -22901,7 +23281,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-27 12:21 UTC</t>
+          <t>2026-05-28 12:28 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -22926,7 +23306,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-27 12:21 UTC</t>
+          <t>2026-05-28 12:28 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -22951,7 +23331,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-27 12:21 UTC</t>
+          <t>2026-05-28 12:28 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -22976,7 +23356,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-27 12:21 UTC</t>
+          <t>2026-05-28 12:28 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -23001,7 +23381,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-27 12:21 UTC</t>
+          <t>2026-05-28 12:28 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -23026,7 +23406,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-27 12:21 UTC</t>
+          <t>2026-05-28 12:28 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -23051,7 +23431,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-27 12:21 UTC</t>
+          <t>2026-05-28 12:28 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -23076,7 +23456,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-27 12:21 UTC</t>
+          <t>2026-05-28 12:28 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -23137,7 +23517,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8011.49bc5730da39751cebc3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.6c026d0f0a7324e83bfc.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8011.82613a08ccb02e6f6d26.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.6d2d8a5dcbf441ae99c9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.92dd16071b63ae3fa439.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -23154,7 +23534,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.f373aa0ed768a56d6f0e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8011.b6799ed0437c32506814.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.fba1426197a32f0e32aa.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8011.82613a08ccb02e6f6d26.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8011.49bc5730da39751cebc3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.6c026d0f0a7324e83bfc.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8011.82613a08ccb02e6f6d26.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-29
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H591"/>
+  <dimension ref="A1:H601"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -23027,6 +23027,386 @@
         </is>
       </c>
       <c r="H591" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="592" ht="15" customHeight="1">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:16 UTC</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E592" t="n">
+        <v>0</v>
+      </c>
+      <c r="F592" t="n">
+        <v>0</v>
+      </c>
+      <c r="G592" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H592" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="593" ht="15" customHeight="1">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:16 UTC</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E593" t="n">
+        <v>0</v>
+      </c>
+      <c r="F593" t="n">
+        <v>0</v>
+      </c>
+      <c r="G593" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H593" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="594" ht="15" customHeight="1">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:16 UTC</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E594" t="n">
+        <v>0</v>
+      </c>
+      <c r="F594" t="n">
+        <v>0</v>
+      </c>
+      <c r="G594" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H594" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="595" ht="15" customHeight="1">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:16 UTC</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E595" t="n">
+        <v>0</v>
+      </c>
+      <c r="F595" t="n">
+        <v>0</v>
+      </c>
+      <c r="G595" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H595" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="596" ht="15" customHeight="1">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:16 UTC</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E596" t="n">
+        <v>0</v>
+      </c>
+      <c r="F596" t="n">
+        <v>0</v>
+      </c>
+      <c r="G596" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H596" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="597" ht="15" customHeight="1">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:16 UTC</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E597" t="n">
+        <v>0</v>
+      </c>
+      <c r="F597" t="n">
+        <v>0</v>
+      </c>
+      <c r="G597" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H597" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="598" ht="15" customHeight="1">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:16 UTC</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E598" t="n">
+        <v>0</v>
+      </c>
+      <c r="F598" t="n">
+        <v>0</v>
+      </c>
+      <c r="G598" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H598" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="599" ht="15" customHeight="1">
+      <c r="A599" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:16 UTC</t>
+        </is>
+      </c>
+      <c r="B599" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C599" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D599" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E599" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F599" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G599" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.dab3471e8a96dc86b9f5.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H599" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.6d2d8a5dcbf441ae99c9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.92dd16071b63ae3fa439.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="600" ht="15" customHeight="1">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:16 UTC</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E600" t="n">
+        <v>0</v>
+      </c>
+      <c r="F600" t="n">
+        <v>0</v>
+      </c>
+      <c r="G600" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H600" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="601" ht="15" customHeight="1">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>2026-05-29 12:16 UTC</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E601" t="n">
+        <v>0</v>
+      </c>
+      <c r="F601" t="n">
+        <v>0</v>
+      </c>
+      <c r="G601" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H601" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -23231,7 +23611,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-28 12:28 UTC</t>
+          <t>2026-05-29 12:16 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -23256,7 +23636,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-28 12:28 UTC</t>
+          <t>2026-05-29 12:16 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -23281,7 +23661,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-28 12:28 UTC</t>
+          <t>2026-05-29 12:16 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -23306,7 +23686,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-28 12:28 UTC</t>
+          <t>2026-05-29 12:16 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -23331,7 +23711,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-28 12:28 UTC</t>
+          <t>2026-05-29 12:16 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -23356,7 +23736,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-28 12:28 UTC</t>
+          <t>2026-05-29 12:16 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -23381,7 +23761,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-28 12:28 UTC</t>
+          <t>2026-05-29 12:16 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -23406,7 +23786,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-28 12:28 UTC</t>
+          <t>2026-05-29 12:16 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -23431,7 +23811,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-28 12:28 UTC</t>
+          <t>2026-05-29 12:16 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -23456,7 +23836,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-28 12:28 UTC</t>
+          <t>2026-05-29 12:16 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -23517,7 +23897,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.6d2d8a5dcbf441ae99c9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.92dd16071b63ae3fa439.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.dab3471e8a96dc86b9f5.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -23534,7 +23914,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8011.49bc5730da39751cebc3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.6c026d0f0a7324e83bfc.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8011.82613a08ccb02e6f6d26.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.6d2d8a5dcbf441ae99c9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.92dd16071b63ae3fa439.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-05-31
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -8,17 +8,17 @@
   </bookViews>
   <sheets>
     <sheet name="Change Log" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Current Snapshot" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="amc_com_ads_txt" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="amc_com_app-ads_txt" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="bbca_com_ads_txt" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="bbca_com_app-ads_txt" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ifc_com_ads_txt" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="ifc_com_app-ads_txt" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="sundancetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="wetv_com_ads_txt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="wetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="amc_com_ads_txt" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="amc_com_app-ads_txt" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="bbca_com_ads_txt" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="bbca_com_app-ads_txt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ifc_com_ads_txt" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ifc_com_app-ads_txt" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="wetv_com_ads_txt" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="wetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H611"/>
+  <dimension ref="A1:H621"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -23963,6 +23963,386 @@
         </is>
       </c>
     </row>
+    <row r="612" ht="15" customHeight="1">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>2026-05-31 10:59 UTC</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E612" t="n">
+        <v>0</v>
+      </c>
+      <c r="F612" t="n">
+        <v>0</v>
+      </c>
+      <c r="G612" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H612" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="613" ht="15" customHeight="1">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>2026-05-31 10:59 UTC</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E613" t="n">
+        <v>0</v>
+      </c>
+      <c r="F613" t="n">
+        <v>0</v>
+      </c>
+      <c r="G613" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H613" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="614" ht="15" customHeight="1">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>2026-05-31 10:59 UTC</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E614" t="n">
+        <v>0</v>
+      </c>
+      <c r="F614" t="n">
+        <v>0</v>
+      </c>
+      <c r="G614" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H614" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="615" ht="15" customHeight="1">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>2026-05-31 10:59 UTC</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E615" t="n">
+        <v>0</v>
+      </c>
+      <c r="F615" t="n">
+        <v>0</v>
+      </c>
+      <c r="G615" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H615" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="616" ht="15" customHeight="1">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>2026-05-31 10:59 UTC</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E616" t="n">
+        <v>0</v>
+      </c>
+      <c r="F616" t="n">
+        <v>0</v>
+      </c>
+      <c r="G616" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H616" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="617" ht="15" customHeight="1">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>2026-05-31 10:59 UTC</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E617" t="n">
+        <v>0</v>
+      </c>
+      <c r="F617" t="n">
+        <v>0</v>
+      </c>
+      <c r="G617" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H617" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="618" ht="15" customHeight="1">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>2026-05-31 10:59 UTC</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E618" t="n">
+        <v>0</v>
+      </c>
+      <c r="F618" t="n">
+        <v>0</v>
+      </c>
+      <c r="G618" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H618" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="619" ht="15" customHeight="1">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>2026-05-31 10:59 UTC</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E619" t="n">
+        <v>0</v>
+      </c>
+      <c r="F619" t="n">
+        <v>0</v>
+      </c>
+      <c r="G619" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H619" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="620" ht="15" customHeight="1">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>2026-05-31 10:59 UTC</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E620" t="n">
+        <v>0</v>
+      </c>
+      <c r="F620" t="n">
+        <v>0</v>
+      </c>
+      <c r="G620" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H620" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="621" ht="15" customHeight="1">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>2026-05-31 10:59 UTC</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E621" t="n">
+        <v>0</v>
+      </c>
+      <c r="F621" t="n">
+        <v>0</v>
+      </c>
+      <c r="G621" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H621" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -23974,7 +24354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -24007,29 +24387,573 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>(no section)</t>
+          <t>#KrushMedia</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.3571122d0e628a0190e4.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>krushmedia.com, AJxF6R612a9M6CaTvK, DIRECT</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.dab3471e8a96dc86b9f5.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, sg1256491, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 534465-r-523319, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>conversantmedia.com, 41784, RESELLER, 03113cd04947736d</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>smartadserver.com, 4478, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>video.unrulymedia.com, 2736329702851206590, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>connatix.com, 655569151931372, DIRECT, 2af98acdee0e81ed</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>wavefront.tv, 54409, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>smartadserver.com, 4579, RESELLER, 060d053dcf45cbf3</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>inmobi.com,758e432765224cf2852ed7e0ff5b35e7,RESELLER,83e75a7ae333ca9d</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>zetaglobal.net, 903, DIRECT</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>lijit.com, 245697, RESELLER, fafdf38b16bf6b2b</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Media.net, 8CUT87EOU, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>zmaticoo.com, 5135803, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>video.unrulymedia.com, 9085206363819624071, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>lijit.com, 569110, RESELLER, fafdf38b16bf6b2b #SOVRN</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>supply.colossusssp.com, 610, RESELLER, 6c5b49d96ec1b458</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Added.tv, 9b602b2c, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>smartyads.com, 1156, RESELLER, fd2bde0ff2e62c5d</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>sharethrough.com, j0nru1gr, RESELLER, d53b998a7bd4ecd2</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>smoot.ai , 100260, DIRECT</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>smoot.ai , 100260, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>zmaticoo.com, 5135884, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>improvedigital.com, 2570, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>pubmatic.com, 163797, RESELLER, 5d62403b186f2ace</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>pubmatic.com, 163799, RESELLER, 5d62403b186f2ace</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>lijit.com, 497492, RESELLER, fafdf38b16bf6b2b #SOVRN</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>showheroes.com, 7405, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>x.adprime.com, AJxF6R92a9M6CaTvK, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>voisetech.com, 1315, RESELLER, 9009ef0379162448</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>metaxsoft.com, 70780506, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>#C360</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>C360.com, 4175, DIRECT</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>#VoiseTech</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>voisetech.com, 1341, DIRECT, 9009ef0379162448</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>#VoiseTech</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>google.com, pub-1682595508078257, RESELLER, f08c47fec0942fa0</t>
         </is>
       </c>
     </row>
@@ -24658,620 +25582,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>krushmedia.com, AJxF6R612a9M6CaTvK, DIRECT</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, sg1256491, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 534465-r-523319, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>conversantmedia.com, 41784, RESELLER, 03113cd04947736d</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>smartadserver.com, 4478, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>video.unrulymedia.com, 2736329702851206590, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>connatix.com, 655569151931372, DIRECT, 2af98acdee0e81ed</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>wavefront.tv, 54409, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>smartadserver.com, 4579, RESELLER, 060d053dcf45cbf3</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>inmobi.com,758e432765224cf2852ed7e0ff5b35e7,RESELLER,83e75a7ae333ca9d</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>zetaglobal.net, 903, DIRECT</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>lijit.com, 245697, RESELLER, fafdf38b16bf6b2b</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Media.net, 8CUT87EOU, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>zmaticoo.com, 5135803, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>video.unrulymedia.com, 9085206363819624071, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>lijit.com, 569110, RESELLER, fafdf38b16bf6b2b #SOVRN</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>supply.colossusssp.com, 610, RESELLER, 6c5b49d96ec1b458</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Added.tv, 9b602b2c, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>smartyads.com, 1156, RESELLER, fd2bde0ff2e62c5d</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>sharethrough.com, j0nru1gr, RESELLER, d53b998a7bd4ecd2</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>smoot.ai , 100260, DIRECT</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>smoot.ai , 100260, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>zmaticoo.com, 5135884, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>improvedigital.com, 2570, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 163797, RESELLER, 5d62403b186f2ace</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 163799, RESELLER, 5d62403b186f2ace</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>lijit.com, 497492, RESELLER, fafdf38b16bf6b2b #SOVRN</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>showheroes.com, 7405, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>x.adprime.com, AJxF6R92a9M6CaTvK, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>voisetech.com, 1315, RESELLER, 9009ef0379162448</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>metaxsoft.com, 70780506, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>#C360</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>C360.com, 4175, DIRECT</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>#VoiseTech</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>voisetech.com, 1341, DIRECT, 9009ef0379162448</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>#VoiseTech</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>google.com, pub-1682595508078257, RESELLER, f08c47fec0942fa0</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -25322,7 +25632,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-30 10:47 UTC</t>
+          <t>2026-05-31 10:59 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -25347,7 +25657,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-30 10:47 UTC</t>
+          <t>2026-05-31 10:59 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -25372,7 +25682,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-30 10:47 UTC</t>
+          <t>2026-05-31 10:59 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -25397,7 +25707,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-30 10:47 UTC</t>
+          <t>2026-05-31 10:59 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -25422,7 +25732,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-30 10:47 UTC</t>
+          <t>2026-05-31 10:59 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -25447,7 +25757,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-30 10:47 UTC</t>
+          <t>2026-05-31 10:59 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -25472,7 +25782,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-30 10:47 UTC</t>
+          <t>2026-05-31 10:59 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -25497,7 +25807,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-30 10:47 UTC</t>
+          <t>2026-05-31 10:59 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -25522,7 +25832,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-30 10:47 UTC</t>
+          <t>2026-05-31 10:59 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -25547,7 +25857,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-30 10:47 UTC</t>
+          <t>2026-05-31 10:59 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -25556,6 +25866,620 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>krushmedia.com, AJxF6R612a9M6CaTvK, DIRECT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, sg1256491, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 534465-r-523319, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>conversantmedia.com, 41784, RESELLER, 03113cd04947736d</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>smartadserver.com, 4478, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>video.unrulymedia.com, 2736329702851206590, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>connatix.com, 655569151931372, DIRECT, 2af98acdee0e81ed</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>wavefront.tv, 54409, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>smartadserver.com, 4579, RESELLER, 060d053dcf45cbf3</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>inmobi.com,758e432765224cf2852ed7e0ff5b35e7,RESELLER,83e75a7ae333ca9d</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>zetaglobal.net, 903, DIRECT</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>lijit.com, 245697, RESELLER, fafdf38b16bf6b2b</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Media.net, 8CUT87EOU, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>zmaticoo.com, 5135803, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>video.unrulymedia.com, 9085206363819624071, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>lijit.com, 569110, RESELLER, fafdf38b16bf6b2b #SOVRN</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>supply.colossusssp.com, 610, RESELLER, 6c5b49d96ec1b458</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Added.tv, 9b602b2c, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>smartyads.com, 1156, RESELLER, fd2bde0ff2e62c5d</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>sharethrough.com, j0nru1gr, RESELLER, d53b998a7bd4ecd2</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>smoot.ai , 100260, DIRECT</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>smoot.ai , 100260, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>zmaticoo.com, 5135884, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>improvedigital.com, 2570, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>pubmatic.com, 163797, RESELLER, 5d62403b186f2ace</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>pubmatic.com, 163799, RESELLER, 5d62403b186f2ace</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>lijit.com, 497492, RESELLER, fafdf38b16bf6b2b #SOVRN</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>showheroes.com, 7405, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>x.adprime.com, AJxF6R92a9M6CaTvK, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>voisetech.com, 1315, RESELLER, 9009ef0379162448</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>metaxsoft.com, 70780506, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>#C360</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>C360.com, 4175, DIRECT</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>#VoiseTech</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>voisetech.com, 1341, DIRECT, 9009ef0379162448</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>#VoiseTech</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>google.com, pub-1682595508078257, RESELLER, f08c47fec0942fa0</t>
         </is>
       </c>
     </row>
@@ -29254,7 +30178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29287,573 +30211,29 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>#KrushMedia</t>
+          <t>(no section)</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>krushmedia.com, AJxF6R612a9M6CaTvK, DIRECT</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.3571122d0e628a0190e4.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, sg1256491, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 534465-r-523319, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>conversantmedia.com, 41784, RESELLER, 03113cd04947736d</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>smartadserver.com, 4478, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>video.unrulymedia.com, 2736329702851206590, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>connatix.com, 655569151931372, DIRECT, 2af98acdee0e81ed</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>wavefront.tv, 54409, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>smartadserver.com, 4579, RESELLER, 060d053dcf45cbf3</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>inmobi.com,758e432765224cf2852ed7e0ff5b35e7,RESELLER,83e75a7ae333ca9d</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>zetaglobal.net, 903, DIRECT</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>lijit.com, 245697, RESELLER, fafdf38b16bf6b2b</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Media.net, 8CUT87EOU, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>zmaticoo.com, 5135803, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>video.unrulymedia.com, 9085206363819624071, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>lijit.com, 569110, RESELLER, fafdf38b16bf6b2b #SOVRN</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>supply.colossusssp.com, 610, RESELLER, 6c5b49d96ec1b458</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Added.tv, 9b602b2c, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>smartyads.com, 1156, RESELLER, fd2bde0ff2e62c5d</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>sharethrough.com, j0nru1gr, RESELLER, d53b998a7bd4ecd2</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>smoot.ai , 100260, DIRECT</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>smoot.ai , 100260, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>zmaticoo.com, 5135884, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>improvedigital.com, 2570, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 163797, RESELLER, 5d62403b186f2ace</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 163799, RESELLER, 5d62403b186f2ace</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>lijit.com, 497492, RESELLER, fafdf38b16bf6b2b #SOVRN</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>showheroes.com, 7405, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>x.adprime.com, AJxF6R92a9M6CaTvK, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>voisetech.com, 1315, RESELLER, 9009ef0379162448</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>metaxsoft.com, 70780506, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>#C360</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>C360.com, 4175, DIRECT</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>#VoiseTech</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>voisetech.com, 1341, DIRECT, 9009ef0379162448</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>#VoiseTech</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>google.com, pub-1682595508078257, RESELLER, f08c47fec0942fa0</t>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.dab3471e8a96dc86b9f5.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-01
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -15,10 +15,10 @@
     <sheet name="ifc_com_ads_txt" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="ifc_com_app-ads_txt" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="wetv_com_ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="wetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H621"/>
+  <dimension ref="A1:H631"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -24338,6 +24338,386 @@
         </is>
       </c>
       <c r="H621" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="622" ht="15" customHeight="1">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>2026-06-01 15:22 UTC</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E622" t="n">
+        <v>0</v>
+      </c>
+      <c r="F622" t="n">
+        <v>0</v>
+      </c>
+      <c r="G622" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H622" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="623" ht="15" customHeight="1">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>2026-06-01 15:22 UTC</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E623" t="n">
+        <v>0</v>
+      </c>
+      <c r="F623" t="n">
+        <v>0</v>
+      </c>
+      <c r="G623" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H623" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="624" ht="15" customHeight="1">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>2026-06-01 15:22 UTC</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E624" t="n">
+        <v>0</v>
+      </c>
+      <c r="F624" t="n">
+        <v>0</v>
+      </c>
+      <c r="G624" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H624" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="625" ht="15" customHeight="1">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>2026-06-01 15:22 UTC</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D625" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E625" t="n">
+        <v>0</v>
+      </c>
+      <c r="F625" t="n">
+        <v>0</v>
+      </c>
+      <c r="G625" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H625" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="626" ht="15" customHeight="1">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>2026-06-01 15:22 UTC</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D626" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E626" t="n">
+        <v>0</v>
+      </c>
+      <c r="F626" t="n">
+        <v>0</v>
+      </c>
+      <c r="G626" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H626" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="627" ht="15" customHeight="1">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>2026-06-01 15:22 UTC</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D627" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E627" t="n">
+        <v>0</v>
+      </c>
+      <c r="F627" t="n">
+        <v>0</v>
+      </c>
+      <c r="G627" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H627" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="628" ht="15" customHeight="1">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>2026-06-01 15:22 UTC</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D628" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E628" t="n">
+        <v>0</v>
+      </c>
+      <c r="F628" t="n">
+        <v>0</v>
+      </c>
+      <c r="G628" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H628" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="629" ht="15" customHeight="1">
+      <c r="A629" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-01 15:22 UTC</t>
+        </is>
+      </c>
+      <c r="B629" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C629" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D629" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E629" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F629" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G629" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.471b4a814761e3d979c0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H629" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.3571122d0e628a0190e4.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="630" ht="15" customHeight="1">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>2026-06-01 15:22 UTC</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D630" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E630" t="n">
+        <v>0</v>
+      </c>
+      <c r="F630" t="n">
+        <v>0</v>
+      </c>
+      <c r="G630" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H630" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="631" ht="15" customHeight="1">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>2026-06-01 15:22 UTC</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D631" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E631" t="n">
+        <v>0</v>
+      </c>
+      <c r="F631" t="n">
+        <v>0</v>
+      </c>
+      <c r="G631" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H631" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -24968,620 +25348,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>krushmedia.com, AJxF6R612a9M6CaTvK, DIRECT</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, sg1256491, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 534465-r-523319, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>conversantmedia.com, 41784, RESELLER, 03113cd04947736d</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>smartadserver.com, 4478, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>video.unrulymedia.com, 2736329702851206590, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>connatix.com, 655569151931372, DIRECT, 2af98acdee0e81ed</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>wavefront.tv, 54409, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>smartadserver.com, 4579, RESELLER, 060d053dcf45cbf3</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>inmobi.com,758e432765224cf2852ed7e0ff5b35e7,RESELLER,83e75a7ae333ca9d</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>zetaglobal.net, 903, DIRECT</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>lijit.com, 245697, RESELLER, fafdf38b16bf6b2b</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Media.net, 8CUT87EOU, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>zmaticoo.com, 5135803, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>video.unrulymedia.com, 9085206363819624071, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>lijit.com, 569110, RESELLER, fafdf38b16bf6b2b #SOVRN</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>supply.colossusssp.com, 610, RESELLER, 6c5b49d96ec1b458</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Added.tv, 9b602b2c, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>smartyads.com, 1156, RESELLER, fd2bde0ff2e62c5d</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>#KrushMedia</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>sharethrough.com, j0nru1gr, RESELLER, d53b998a7bd4ecd2</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>smoot.ai , 100260, DIRECT</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>smoot.ai , 100260, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>zmaticoo.com, 5135884, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>improvedigital.com, 2570, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 163797, RESELLER, 5d62403b186f2ace</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 163799, RESELLER, 5d62403b186f2ace</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>lijit.com, 497492, RESELLER, fafdf38b16bf6b2b #SOVRN</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>showheroes.com, 7405, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>x.adprime.com, AJxF6R92a9M6CaTvK, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>voisetech.com, 1315, RESELLER, 9009ef0379162448</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>#Smoot</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>metaxsoft.com, 70780506, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>#C360</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>C360.com, 4175, DIRECT</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>#VoiseTech</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>voisetech.com, 1341, DIRECT, 9009ef0379162448</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>#VoiseTech</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>google.com, pub-1682595508078257, RESELLER, f08c47fec0942fa0</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -25632,7 +25398,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-05-31 10:59 UTC</t>
+          <t>2026-06-01 15:22 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -25657,7 +25423,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-05-31 10:59 UTC</t>
+          <t>2026-06-01 15:22 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -25682,7 +25448,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-05-31 10:59 UTC</t>
+          <t>2026-06-01 15:22 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -25707,7 +25473,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-05-31 10:59 UTC</t>
+          <t>2026-06-01 15:22 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -25732,7 +25498,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-05-31 10:59 UTC</t>
+          <t>2026-06-01 15:22 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -25757,7 +25523,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-05-31 10:59 UTC</t>
+          <t>2026-06-01 15:22 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -25782,7 +25548,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-05-31 10:59 UTC</t>
+          <t>2026-06-01 15:22 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -25807,7 +25573,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-05-31 10:59 UTC</t>
+          <t>2026-06-01 15:22 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -25832,7 +25598,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-05-31 10:59 UTC</t>
+          <t>2026-06-01 15:22 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -25857,7 +25623,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-05-31 10:59 UTC</t>
+          <t>2026-06-01 15:22 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -25866,6 +25632,76 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.471b4a814761e3d979c0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.3571122d0e628a0190e4.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -30178,7 +30014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -30211,29 +30047,573 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>(no section)</t>
+          <t>#KrushMedia</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.3571122d0e628a0190e4.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>krushmedia.com, AJxF6R612a9M6CaTvK, DIRECT</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.dab3471e8a96dc86b9f5.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, sg1256491, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 534465-r-523319, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>conversantmedia.com, 41784, RESELLER, 03113cd04947736d</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>smartadserver.com, 4478, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>video.unrulymedia.com, 2736329702851206590, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>connatix.com, 655569151931372, DIRECT, 2af98acdee0e81ed</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>wavefront.tv, 54409, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>smartadserver.com, 4579, RESELLER, 060d053dcf45cbf3</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>inmobi.com,758e432765224cf2852ed7e0ff5b35e7,RESELLER,83e75a7ae333ca9d</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>zetaglobal.net, 903, DIRECT</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>lijit.com, 245697, RESELLER, fafdf38b16bf6b2b</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Media.net, 8CUT87EOU, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>zmaticoo.com, 5135803, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>video.unrulymedia.com, 9085206363819624071, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>lijit.com, 569110, RESELLER, fafdf38b16bf6b2b #SOVRN</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>supply.colossusssp.com, 610, RESELLER, 6c5b49d96ec1b458</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Added.tv, 9b602b2c, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>smartyads.com, 1156, RESELLER, fd2bde0ff2e62c5d</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>#KrushMedia</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>sharethrough.com, j0nru1gr, RESELLER, d53b998a7bd4ecd2</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>smoot.ai , 100260, DIRECT</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>smoot.ai , 100260, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>zmaticoo.com, 5135884, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>improvedigital.com, 2570, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>pubmatic.com, 163797, RESELLER, 5d62403b186f2ace</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>pubmatic.com, 163799, RESELLER, 5d62403b186f2ace</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>lijit.com, 497492, RESELLER, fafdf38b16bf6b2b #SOVRN</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>showheroes.com, 7405, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>x.adprime.com, AJxF6R92a9M6CaTvK, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>voisetech.com, 1315, RESELLER, 9009ef0379162448</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>#Smoot</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>metaxsoft.com, 70780506, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>#C360</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>C360.com, 4175, DIRECT</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>#VoiseTech</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>voisetech.com, 1341, DIRECT, 9009ef0379162448</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>#VoiseTech</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>google.com, pub-1682595508078257, RESELLER, f08c47fec0942fa0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-02
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H631"/>
+  <dimension ref="A1:H641"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -24718,6 +24718,386 @@
         </is>
       </c>
       <c r="H631" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="632" ht="15" customHeight="1">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>2026-06-02 12:43 UTC</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E632" t="n">
+        <v>0</v>
+      </c>
+      <c r="F632" t="n">
+        <v>0</v>
+      </c>
+      <c r="G632" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H632" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="633" ht="15" customHeight="1">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>2026-06-02 12:43 UTC</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D633" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E633" t="n">
+        <v>0</v>
+      </c>
+      <c r="F633" t="n">
+        <v>0</v>
+      </c>
+      <c r="G633" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H633" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="634" ht="15" customHeight="1">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>2026-06-02 12:43 UTC</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D634" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E634" t="n">
+        <v>0</v>
+      </c>
+      <c r="F634" t="n">
+        <v>0</v>
+      </c>
+      <c r="G634" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H634" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="635" ht="15" customHeight="1">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>2026-06-02 12:43 UTC</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D635" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E635" t="n">
+        <v>0</v>
+      </c>
+      <c r="F635" t="n">
+        <v>0</v>
+      </c>
+      <c r="G635" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H635" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="636" ht="15" customHeight="1">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>2026-06-02 12:43 UTC</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D636" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E636" t="n">
+        <v>0</v>
+      </c>
+      <c r="F636" t="n">
+        <v>0</v>
+      </c>
+      <c r="G636" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H636" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="637" ht="15" customHeight="1">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>2026-06-02 12:43 UTC</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D637" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E637" t="n">
+        <v>0</v>
+      </c>
+      <c r="F637" t="n">
+        <v>0</v>
+      </c>
+      <c r="G637" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H637" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="638" ht="15" customHeight="1">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>2026-06-02 12:43 UTC</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D638" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E638" t="n">
+        <v>0</v>
+      </c>
+      <c r="F638" t="n">
+        <v>0</v>
+      </c>
+      <c r="G638" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H638" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="639" ht="15" customHeight="1">
+      <c r="A639" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-02 12:43 UTC</t>
+        </is>
+      </c>
+      <c r="B639" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C639" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D639" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E639" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F639" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G639" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9e2a8b87782171391613.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.5d122c943b202eb5ade7.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H639" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.471b4a814761e3d979c0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="640" ht="15" customHeight="1">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>2026-06-02 12:43 UTC</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D640" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E640" t="n">
+        <v>0</v>
+      </c>
+      <c r="F640" t="n">
+        <v>0</v>
+      </c>
+      <c r="G640" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H640" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="641" ht="15" customHeight="1">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>2026-06-02 12:43 UTC</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D641" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E641" t="n">
+        <v>0</v>
+      </c>
+      <c r="F641" t="n">
+        <v>0</v>
+      </c>
+      <c r="G641" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H641" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -25398,7 +25778,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-01 15:22 UTC</t>
+          <t>2026-06-02 12:43 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -25423,7 +25803,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-01 15:22 UTC</t>
+          <t>2026-06-02 12:43 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -25448,7 +25828,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-01 15:22 UTC</t>
+          <t>2026-06-02 12:43 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -25473,7 +25853,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-01 15:22 UTC</t>
+          <t>2026-06-02 12:43 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -25498,7 +25878,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-01 15:22 UTC</t>
+          <t>2026-06-02 12:43 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -25523,7 +25903,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-01 15:22 UTC</t>
+          <t>2026-06-02 12:43 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -25548,7 +25928,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-01 15:22 UTC</t>
+          <t>2026-06-02 12:43 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -25573,7 +25953,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-01 15:22 UTC</t>
+          <t>2026-06-02 12:43 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -25598,7 +25978,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-01 15:22 UTC</t>
+          <t>2026-06-02 12:43 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -25623,7 +26003,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-01 15:22 UTC</t>
+          <t>2026-06-02 12:43 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -25684,7 +26064,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.471b4a814761e3d979c0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9e2a8b87782171391613.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.5d122c943b202eb5ade7.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -25701,7 +26081,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.3571122d0e628a0190e4.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.471b4a814761e3d979c0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-03
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H641"/>
+  <dimension ref="A1:H651"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -25098,6 +25098,386 @@
         </is>
       </c>
       <c r="H641" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="642" ht="15" customHeight="1">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>2026-06-03 13:18 UTC</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D642" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E642" t="n">
+        <v>0</v>
+      </c>
+      <c r="F642" t="n">
+        <v>0</v>
+      </c>
+      <c r="G642" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H642" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="643" ht="15" customHeight="1">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>2026-06-03 13:18 UTC</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D643" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E643" t="n">
+        <v>0</v>
+      </c>
+      <c r="F643" t="n">
+        <v>0</v>
+      </c>
+      <c r="G643" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H643" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="644" ht="15" customHeight="1">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>2026-06-03 13:18 UTC</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D644" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E644" t="n">
+        <v>0</v>
+      </c>
+      <c r="F644" t="n">
+        <v>0</v>
+      </c>
+      <c r="G644" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H644" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="645" ht="15" customHeight="1">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>2026-06-03 13:18 UTC</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D645" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E645" t="n">
+        <v>0</v>
+      </c>
+      <c r="F645" t="n">
+        <v>0</v>
+      </c>
+      <c r="G645" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H645" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="646" ht="15" customHeight="1">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>2026-06-03 13:18 UTC</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D646" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E646" t="n">
+        <v>0</v>
+      </c>
+      <c r="F646" t="n">
+        <v>0</v>
+      </c>
+      <c r="G646" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H646" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="647" ht="15" customHeight="1">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>2026-06-03 13:18 UTC</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D647" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E647" t="n">
+        <v>0</v>
+      </c>
+      <c r="F647" t="n">
+        <v>0</v>
+      </c>
+      <c r="G647" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H647" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="648" ht="15" customHeight="1">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>2026-06-03 13:18 UTC</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D648" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E648" t="n">
+        <v>0</v>
+      </c>
+      <c r="F648" t="n">
+        <v>0</v>
+      </c>
+      <c r="G648" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H648" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="649" ht="15" customHeight="1">
+      <c r="A649" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-03 13:18 UTC</t>
+        </is>
+      </c>
+      <c r="B649" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C649" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D649" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E649" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F649" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G649" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.3376fb0bac2083f934e4.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.5d122c943b202eb5ade7.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H649" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9e2a8b87782171391613.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.5d122c943b202eb5ade7.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="650" ht="15" customHeight="1">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>2026-06-03 13:18 UTC</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D650" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E650" t="n">
+        <v>0</v>
+      </c>
+      <c r="F650" t="n">
+        <v>0</v>
+      </c>
+      <c r="G650" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H650" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="651" ht="15" customHeight="1">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>2026-06-03 13:18 UTC</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D651" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E651" t="n">
+        <v>0</v>
+      </c>
+      <c r="F651" t="n">
+        <v>0</v>
+      </c>
+      <c r="G651" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H651" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -25778,7 +26158,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-02 12:43 UTC</t>
+          <t>2026-06-03 13:18 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -25803,7 +26183,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-02 12:43 UTC</t>
+          <t>2026-06-03 13:18 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -25828,7 +26208,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-02 12:43 UTC</t>
+          <t>2026-06-03 13:18 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -25853,7 +26233,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-02 12:43 UTC</t>
+          <t>2026-06-03 13:18 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -25878,7 +26258,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-02 12:43 UTC</t>
+          <t>2026-06-03 13:18 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -25903,7 +26283,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-02 12:43 UTC</t>
+          <t>2026-06-03 13:18 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -25928,7 +26308,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-02 12:43 UTC</t>
+          <t>2026-06-03 13:18 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -25953,7 +26333,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-02 12:43 UTC</t>
+          <t>2026-06-03 13:18 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -25978,7 +26358,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-02 12:43 UTC</t>
+          <t>2026-06-03 13:18 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -26003,7 +26383,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-02 12:43 UTC</t>
+          <t>2026-06-03 13:18 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -26064,7 +26444,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9e2a8b87782171391613.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.5d122c943b202eb5ade7.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.3376fb0bac2083f934e4.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.5d122c943b202eb5ade7.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -26081,7 +26461,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.2089381f4334adfb64dc.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.471b4a814761e3d979c0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.68569ed74203d54e3508.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9e2a8b87782171391613.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.5d122c943b202eb5ade7.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-04
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H651"/>
+  <dimension ref="A1:H661"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -25478,6 +25478,386 @@
         </is>
       </c>
       <c r="H651" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="652" ht="15" customHeight="1">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>2026-06-04 11:55 UTC</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D652" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E652" t="n">
+        <v>0</v>
+      </c>
+      <c r="F652" t="n">
+        <v>0</v>
+      </c>
+      <c r="G652" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H652" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="653" ht="15" customHeight="1">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>2026-06-04 11:55 UTC</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D653" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E653" t="n">
+        <v>0</v>
+      </c>
+      <c r="F653" t="n">
+        <v>0</v>
+      </c>
+      <c r="G653" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H653" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="654" ht="15" customHeight="1">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>2026-06-04 11:55 UTC</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D654" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E654" t="n">
+        <v>0</v>
+      </c>
+      <c r="F654" t="n">
+        <v>0</v>
+      </c>
+      <c r="G654" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H654" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="655" ht="15" customHeight="1">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>2026-06-04 11:55 UTC</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D655" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E655" t="n">
+        <v>0</v>
+      </c>
+      <c r="F655" t="n">
+        <v>0</v>
+      </c>
+      <c r="G655" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H655" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="656" ht="15" customHeight="1">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>2026-06-04 11:55 UTC</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D656" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E656" t="n">
+        <v>0</v>
+      </c>
+      <c r="F656" t="n">
+        <v>0</v>
+      </c>
+      <c r="G656" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H656" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="657" ht="15" customHeight="1">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>2026-06-04 11:55 UTC</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D657" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E657" t="n">
+        <v>0</v>
+      </c>
+      <c r="F657" t="n">
+        <v>0</v>
+      </c>
+      <c r="G657" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H657" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="658" ht="15" customHeight="1">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>2026-06-04 11:55 UTC</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D658" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E658" t="n">
+        <v>0</v>
+      </c>
+      <c r="F658" t="n">
+        <v>0</v>
+      </c>
+      <c r="G658" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H658" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="659" ht="15" customHeight="1">
+      <c r="A659" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-04 11:55 UTC</t>
+        </is>
+      </c>
+      <c r="B659" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C659" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D659" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E659" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F659" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G659" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.7a0f9905929399e89442.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H659" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.3376fb0bac2083f934e4.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.5d122c943b202eb5ade7.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="660" ht="15" customHeight="1">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>2026-06-04 11:55 UTC</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D660" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E660" t="n">
+        <v>0</v>
+      </c>
+      <c r="F660" t="n">
+        <v>0</v>
+      </c>
+      <c r="G660" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H660" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="661" ht="15" customHeight="1">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>2026-06-04 11:55 UTC</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D661" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E661" t="n">
+        <v>0</v>
+      </c>
+      <c r="F661" t="n">
+        <v>0</v>
+      </c>
+      <c r="G661" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H661" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -26158,7 +26538,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-03 13:18 UTC</t>
+          <t>2026-06-04 11:55 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -26183,7 +26563,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-03 13:18 UTC</t>
+          <t>2026-06-04 11:55 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -26208,7 +26588,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-03 13:18 UTC</t>
+          <t>2026-06-04 11:55 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -26233,7 +26613,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-03 13:18 UTC</t>
+          <t>2026-06-04 11:55 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -26258,7 +26638,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-03 13:18 UTC</t>
+          <t>2026-06-04 11:55 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -26283,7 +26663,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-03 13:18 UTC</t>
+          <t>2026-06-04 11:55 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -26308,7 +26688,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-03 13:18 UTC</t>
+          <t>2026-06-04 11:55 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -26333,7 +26713,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-03 13:18 UTC</t>
+          <t>2026-06-04 11:55 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -26358,7 +26738,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-03 13:18 UTC</t>
+          <t>2026-06-04 11:55 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -26383,7 +26763,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-03 13:18 UTC</t>
+          <t>2026-06-04 11:55 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -26444,7 +26824,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.3376fb0bac2083f934e4.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.5d122c943b202eb5ade7.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.7a0f9905929399e89442.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -26461,7 +26841,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9e2a8b87782171391613.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.5d122c943b202eb5ade7.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.3376fb0bac2083f934e4.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.5d122c943b202eb5ade7.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-05
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H661"/>
+  <dimension ref="A1:H671"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -25858,6 +25858,386 @@
         </is>
       </c>
       <c r="H661" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="662" ht="15" customHeight="1">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>2026-06-05 12:09 UTC</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D662" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E662" t="n">
+        <v>0</v>
+      </c>
+      <c r="F662" t="n">
+        <v>0</v>
+      </c>
+      <c r="G662" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H662" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="663" ht="15" customHeight="1">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>2026-06-05 12:09 UTC</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E663" t="n">
+        <v>0</v>
+      </c>
+      <c r="F663" t="n">
+        <v>0</v>
+      </c>
+      <c r="G663" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H663" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="664" ht="15" customHeight="1">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>2026-06-05 12:09 UTC</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E664" t="n">
+        <v>0</v>
+      </c>
+      <c r="F664" t="n">
+        <v>0</v>
+      </c>
+      <c r="G664" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H664" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="665" ht="15" customHeight="1">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>2026-06-05 12:09 UTC</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E665" t="n">
+        <v>0</v>
+      </c>
+      <c r="F665" t="n">
+        <v>0</v>
+      </c>
+      <c r="G665" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H665" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="666" ht="15" customHeight="1">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>2026-06-05 12:09 UTC</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E666" t="n">
+        <v>0</v>
+      </c>
+      <c r="F666" t="n">
+        <v>0</v>
+      </c>
+      <c r="G666" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H666" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="667" ht="15" customHeight="1">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>2026-06-05 12:09 UTC</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E667" t="n">
+        <v>0</v>
+      </c>
+      <c r="F667" t="n">
+        <v>0</v>
+      </c>
+      <c r="G667" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H667" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="668" ht="15" customHeight="1">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>2026-06-05 12:09 UTC</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E668" t="n">
+        <v>0</v>
+      </c>
+      <c r="F668" t="n">
+        <v>0</v>
+      </c>
+      <c r="G668" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H668" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="669" ht="15" customHeight="1">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>2026-06-05 12:09 UTC</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E669" t="n">
+        <v>0</v>
+      </c>
+      <c r="F669" t="n">
+        <v>0</v>
+      </c>
+      <c r="G669" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H669" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="670" ht="15" customHeight="1">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>2026-06-05 12:09 UTC</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E670" t="n">
+        <v>0</v>
+      </c>
+      <c r="F670" t="n">
+        <v>0</v>
+      </c>
+      <c r="G670" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H670" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="671" ht="15" customHeight="1">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>2026-06-05 12:09 UTC</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E671" t="n">
+        <v>0</v>
+      </c>
+      <c r="F671" t="n">
+        <v>0</v>
+      </c>
+      <c r="G671" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H671" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -26488,6 +26868,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.7a0f9905929399e89442.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.3376fb0bac2083f934e4.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.5d122c943b202eb5ade7.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -26538,7 +26988,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-04 11:55 UTC</t>
+          <t>2026-06-05 12:09 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -26563,7 +27013,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-04 11:55 UTC</t>
+          <t>2026-06-05 12:09 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -26588,7 +27038,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-04 11:55 UTC</t>
+          <t>2026-06-05 12:09 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -26613,7 +27063,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-04 11:55 UTC</t>
+          <t>2026-06-05 12:09 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -26638,7 +27088,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-04 11:55 UTC</t>
+          <t>2026-06-05 12:09 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -26663,7 +27113,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-04 11:55 UTC</t>
+          <t>2026-06-05 12:09 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -26688,7 +27138,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-04 11:55 UTC</t>
+          <t>2026-06-05 12:09 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -26713,7 +27163,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-04 11:55 UTC</t>
+          <t>2026-06-05 12:09 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -26738,7 +27188,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-04 11:55 UTC</t>
+          <t>2026-06-05 12:09 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -26763,7 +27213,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-04 11:55 UTC</t>
+          <t>2026-06-05 12:09 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -26772,76 +27222,6 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.7a0f9905929399e89442.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.3376fb0bac2083f934e4.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.5d122c943b202eb5ade7.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-06
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H671"/>
+  <dimension ref="A1:H681"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -26238,6 +26238,386 @@
         </is>
       </c>
       <c r="H671" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="672" ht="15" customHeight="1">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>2026-06-06 10:54 UTC</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E672" t="n">
+        <v>0</v>
+      </c>
+      <c r="F672" t="n">
+        <v>0</v>
+      </c>
+      <c r="G672" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H672" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="673" ht="15" customHeight="1">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>2026-06-06 10:54 UTC</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E673" t="n">
+        <v>0</v>
+      </c>
+      <c r="F673" t="n">
+        <v>0</v>
+      </c>
+      <c r="G673" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H673" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="674" ht="15" customHeight="1">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>2026-06-06 10:54 UTC</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E674" t="n">
+        <v>0</v>
+      </c>
+      <c r="F674" t="n">
+        <v>0</v>
+      </c>
+      <c r="G674" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H674" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="675" ht="15" customHeight="1">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>2026-06-06 10:54 UTC</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E675" t="n">
+        <v>0</v>
+      </c>
+      <c r="F675" t="n">
+        <v>0</v>
+      </c>
+      <c r="G675" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H675" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="676" ht="15" customHeight="1">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>2026-06-06 10:54 UTC</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E676" t="n">
+        <v>0</v>
+      </c>
+      <c r="F676" t="n">
+        <v>0</v>
+      </c>
+      <c r="G676" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H676" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="677" ht="15" customHeight="1">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>2026-06-06 10:54 UTC</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E677" t="n">
+        <v>0</v>
+      </c>
+      <c r="F677" t="n">
+        <v>0</v>
+      </c>
+      <c r="G677" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H677" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="678" ht="15" customHeight="1">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>2026-06-06 10:54 UTC</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E678" t="n">
+        <v>0</v>
+      </c>
+      <c r="F678" t="n">
+        <v>0</v>
+      </c>
+      <c r="G678" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H678" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="679" ht="15" customHeight="1">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>2026-06-06 10:54 UTC</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E679" t="n">
+        <v>0</v>
+      </c>
+      <c r="F679" t="n">
+        <v>0</v>
+      </c>
+      <c r="G679" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H679" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="680" ht="15" customHeight="1">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>2026-06-06 10:54 UTC</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E680" t="n">
+        <v>0</v>
+      </c>
+      <c r="F680" t="n">
+        <v>0</v>
+      </c>
+      <c r="G680" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H680" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="681" ht="15" customHeight="1">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>2026-06-06 10:54 UTC</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E681" t="n">
+        <v>0</v>
+      </c>
+      <c r="F681" t="n">
+        <v>0</v>
+      </c>
+      <c r="G681" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H681" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -26988,7 +27368,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-05 12:09 UTC</t>
+          <t>2026-06-06 10:54 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -27013,7 +27393,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-05 12:09 UTC</t>
+          <t>2026-06-06 10:54 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -27038,7 +27418,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-05 12:09 UTC</t>
+          <t>2026-06-06 10:54 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -27063,7 +27443,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-05 12:09 UTC</t>
+          <t>2026-06-06 10:54 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -27088,7 +27468,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-05 12:09 UTC</t>
+          <t>2026-06-06 10:54 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -27113,7 +27493,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-05 12:09 UTC</t>
+          <t>2026-06-06 10:54 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -27138,7 +27518,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-05 12:09 UTC</t>
+          <t>2026-06-06 10:54 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -27163,7 +27543,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-05 12:09 UTC</t>
+          <t>2026-06-06 10:54 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -27188,7 +27568,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-05 12:09 UTC</t>
+          <t>2026-06-06 10:54 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -27213,7 +27593,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-05 12:09 UTC</t>
+          <t>2026-06-06 10:54 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-07
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H681"/>
+  <dimension ref="A1:H691"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -26618,6 +26618,386 @@
         </is>
       </c>
       <c r="H681" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="682" ht="15" customHeight="1">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>2026-06-07 11:09 UTC</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E682" t="n">
+        <v>0</v>
+      </c>
+      <c r="F682" t="n">
+        <v>0</v>
+      </c>
+      <c r="G682" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H682" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="683" ht="15" customHeight="1">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>2026-06-07 11:09 UTC</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E683" t="n">
+        <v>0</v>
+      </c>
+      <c r="F683" t="n">
+        <v>0</v>
+      </c>
+      <c r="G683" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H683" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="684" ht="15" customHeight="1">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>2026-06-07 11:09 UTC</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E684" t="n">
+        <v>0</v>
+      </c>
+      <c r="F684" t="n">
+        <v>0</v>
+      </c>
+      <c r="G684" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H684" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="685" ht="15" customHeight="1">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>2026-06-07 11:09 UTC</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E685" t="n">
+        <v>0</v>
+      </c>
+      <c r="F685" t="n">
+        <v>0</v>
+      </c>
+      <c r="G685" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H685" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="686" ht="15" customHeight="1">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>2026-06-07 11:09 UTC</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E686" t="n">
+        <v>0</v>
+      </c>
+      <c r="F686" t="n">
+        <v>0</v>
+      </c>
+      <c r="G686" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H686" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="687" ht="15" customHeight="1">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>2026-06-07 11:09 UTC</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E687" t="n">
+        <v>0</v>
+      </c>
+      <c r="F687" t="n">
+        <v>0</v>
+      </c>
+      <c r="G687" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H687" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="688" ht="15" customHeight="1">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>2026-06-07 11:09 UTC</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E688" t="n">
+        <v>0</v>
+      </c>
+      <c r="F688" t="n">
+        <v>0</v>
+      </c>
+      <c r="G688" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H688" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="689" ht="15" customHeight="1">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>2026-06-07 11:09 UTC</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E689" t="n">
+        <v>0</v>
+      </c>
+      <c r="F689" t="n">
+        <v>0</v>
+      </c>
+      <c r="G689" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H689" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="690" ht="15" customHeight="1">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>2026-06-07 11:09 UTC</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E690" t="n">
+        <v>0</v>
+      </c>
+      <c r="F690" t="n">
+        <v>0</v>
+      </c>
+      <c r="G690" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H690" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="691" ht="15" customHeight="1">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>2026-06-07 11:09 UTC</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E691" t="n">
+        <v>0</v>
+      </c>
+      <c r="F691" t="n">
+        <v>0</v>
+      </c>
+      <c r="G691" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H691" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -27368,7 +27748,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-06 10:54 UTC</t>
+          <t>2026-06-07 11:09 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -27393,7 +27773,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-06 10:54 UTC</t>
+          <t>2026-06-07 11:09 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -27418,7 +27798,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-06 10:54 UTC</t>
+          <t>2026-06-07 11:09 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -27443,7 +27823,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-06 10:54 UTC</t>
+          <t>2026-06-07 11:09 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -27468,7 +27848,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-06 10:54 UTC</t>
+          <t>2026-06-07 11:09 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -27493,7 +27873,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-06 10:54 UTC</t>
+          <t>2026-06-07 11:09 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -27518,7 +27898,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-06 10:54 UTC</t>
+          <t>2026-06-07 11:09 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -27543,7 +27923,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-06 10:54 UTC</t>
+          <t>2026-06-07 11:09 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -27568,7 +27948,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-06 10:54 UTC</t>
+          <t>2026-06-07 11:09 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -27593,7 +27973,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-06 10:54 UTC</t>
+          <t>2026-06-07 11:09 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-08
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H691"/>
+  <dimension ref="A1:H701"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -26998,6 +26998,386 @@
         </is>
       </c>
       <c r="H691" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="692" ht="15" customHeight="1">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>2026-06-08 13:08 UTC</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E692" t="n">
+        <v>0</v>
+      </c>
+      <c r="F692" t="n">
+        <v>0</v>
+      </c>
+      <c r="G692" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H692" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="693" ht="15" customHeight="1">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>2026-06-08 13:08 UTC</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E693" t="n">
+        <v>0</v>
+      </c>
+      <c r="F693" t="n">
+        <v>0</v>
+      </c>
+      <c r="G693" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H693" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="694" ht="15" customHeight="1">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>2026-06-08 13:08 UTC</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E694" t="n">
+        <v>0</v>
+      </c>
+      <c r="F694" t="n">
+        <v>0</v>
+      </c>
+      <c r="G694" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H694" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="695" ht="15" customHeight="1">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>2026-06-08 13:08 UTC</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E695" t="n">
+        <v>0</v>
+      </c>
+      <c r="F695" t="n">
+        <v>0</v>
+      </c>
+      <c r="G695" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H695" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="696" ht="15" customHeight="1">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>2026-06-08 13:08 UTC</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E696" t="n">
+        <v>0</v>
+      </c>
+      <c r="F696" t="n">
+        <v>0</v>
+      </c>
+      <c r="G696" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H696" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="697" ht="15" customHeight="1">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>2026-06-08 13:08 UTC</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E697" t="n">
+        <v>0</v>
+      </c>
+      <c r="F697" t="n">
+        <v>0</v>
+      </c>
+      <c r="G697" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H697" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="698" ht="15" customHeight="1">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>2026-06-08 13:08 UTC</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E698" t="n">
+        <v>0</v>
+      </c>
+      <c r="F698" t="n">
+        <v>0</v>
+      </c>
+      <c r="G698" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H698" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="699" ht="15" customHeight="1">
+      <c r="A699" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-08 13:08 UTC</t>
+        </is>
+      </c>
+      <c r="B699" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C699" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D699" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E699" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F699" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G699" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8b9da178a57d2f5b2372.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H699" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.7a0f9905929399e89442.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="700" ht="15" customHeight="1">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>2026-06-08 13:08 UTC</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D700" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E700" t="n">
+        <v>0</v>
+      </c>
+      <c r="F700" t="n">
+        <v>0</v>
+      </c>
+      <c r="G700" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H700" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="701" ht="15" customHeight="1">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>2026-06-08 13:08 UTC</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D701" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E701" t="n">
+        <v>0</v>
+      </c>
+      <c r="F701" t="n">
+        <v>0</v>
+      </c>
+      <c r="G701" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H701" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -27628,76 +28008,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.7a0f9905929399e89442.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.3376fb0bac2083f934e4.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.5d122c943b202eb5ade7.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -27748,7 +28058,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-07 11:09 UTC</t>
+          <t>2026-06-08 13:08 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -27773,7 +28083,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-07 11:09 UTC</t>
+          <t>2026-06-08 13:08 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -27798,7 +28108,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-07 11:09 UTC</t>
+          <t>2026-06-08 13:08 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -27823,7 +28133,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-07 11:09 UTC</t>
+          <t>2026-06-08 13:08 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -27848,7 +28158,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-07 11:09 UTC</t>
+          <t>2026-06-08 13:08 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -27873,7 +28183,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-07 11:09 UTC</t>
+          <t>2026-06-08 13:08 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -27898,7 +28208,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-07 11:09 UTC</t>
+          <t>2026-06-08 13:08 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -27923,7 +28233,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-07 11:09 UTC</t>
+          <t>2026-06-08 13:08 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -27948,7 +28258,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-07 11:09 UTC</t>
+          <t>2026-06-08 13:08 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -27973,7 +28283,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-07 11:09 UTC</t>
+          <t>2026-06-08 13:08 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -27982,6 +28292,76 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8b9da178a57d2f5b2372.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.7a0f9905929399e89442.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-09
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H701"/>
+  <dimension ref="A1:H711"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -27378,6 +27378,386 @@
         </is>
       </c>
       <c r="H701" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="702" ht="15" customHeight="1">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>2026-06-09 12:05 UTC</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D702" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E702" t="n">
+        <v>0</v>
+      </c>
+      <c r="F702" t="n">
+        <v>0</v>
+      </c>
+      <c r="G702" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H702" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="703" ht="15" customHeight="1">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>2026-06-09 12:05 UTC</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D703" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E703" t="n">
+        <v>0</v>
+      </c>
+      <c r="F703" t="n">
+        <v>0</v>
+      </c>
+      <c r="G703" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H703" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="704" ht="15" customHeight="1">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>2026-06-09 12:05 UTC</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E704" t="n">
+        <v>0</v>
+      </c>
+      <c r="F704" t="n">
+        <v>0</v>
+      </c>
+      <c r="G704" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H704" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="705" ht="15" customHeight="1">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>2026-06-09 12:05 UTC</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D705" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E705" t="n">
+        <v>0</v>
+      </c>
+      <c r="F705" t="n">
+        <v>0</v>
+      </c>
+      <c r="G705" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H705" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="706" ht="15" customHeight="1">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>2026-06-09 12:05 UTC</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D706" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E706" t="n">
+        <v>0</v>
+      </c>
+      <c r="F706" t="n">
+        <v>0</v>
+      </c>
+      <c r="G706" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H706" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="707" ht="15" customHeight="1">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>2026-06-09 12:05 UTC</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E707" t="n">
+        <v>0</v>
+      </c>
+      <c r="F707" t="n">
+        <v>0</v>
+      </c>
+      <c r="G707" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H707" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="708" ht="15" customHeight="1">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>2026-06-09 12:05 UTC</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D708" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E708" t="n">
+        <v>0</v>
+      </c>
+      <c r="F708" t="n">
+        <v>0</v>
+      </c>
+      <c r="G708" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H708" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="709" ht="15" customHeight="1">
+      <c r="A709" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-09 12:05 UTC</t>
+        </is>
+      </c>
+      <c r="B709" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C709" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D709" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E709" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F709" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G709" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.bc8021352f52d7e3be39.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H709" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8b9da178a57d2f5b2372.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="710" ht="15" customHeight="1">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>2026-06-09 12:05 UTC</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D710" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E710" t="n">
+        <v>0</v>
+      </c>
+      <c r="F710" t="n">
+        <v>0</v>
+      </c>
+      <c r="G710" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H710" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="711" ht="15" customHeight="1">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>2026-06-09 12:05 UTC</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D711" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E711" t="n">
+        <v>0</v>
+      </c>
+      <c r="F711" t="n">
+        <v>0</v>
+      </c>
+      <c r="G711" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H711" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -28058,7 +28438,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-08 13:08 UTC</t>
+          <t>2026-06-09 12:05 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -28083,7 +28463,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-08 13:08 UTC</t>
+          <t>2026-06-09 12:05 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -28108,7 +28488,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-08 13:08 UTC</t>
+          <t>2026-06-09 12:05 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -28133,7 +28513,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-08 13:08 UTC</t>
+          <t>2026-06-09 12:05 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -28158,7 +28538,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-08 13:08 UTC</t>
+          <t>2026-06-09 12:05 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -28183,7 +28563,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-08 13:08 UTC</t>
+          <t>2026-06-09 12:05 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -28208,7 +28588,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-08 13:08 UTC</t>
+          <t>2026-06-09 12:05 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -28233,7 +28613,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-08 13:08 UTC</t>
+          <t>2026-06-09 12:05 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -28258,7 +28638,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-08 13:08 UTC</t>
+          <t>2026-06-09 12:05 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -28283,7 +28663,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-08 13:08 UTC</t>
+          <t>2026-06-09 12:05 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -28344,7 +28724,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8b9da178a57d2f5b2372.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.bc8021352f52d7e3be39.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -28361,7 +28741,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.7a0f9905929399e89442.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8b9da178a57d2f5b2372.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-10
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H711"/>
+  <dimension ref="A1:H721"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -27758,6 +27758,386 @@
         </is>
       </c>
       <c r="H711" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="712" ht="15" customHeight="1">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>2026-06-10 12:22 UTC</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D712" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E712" t="n">
+        <v>0</v>
+      </c>
+      <c r="F712" t="n">
+        <v>0</v>
+      </c>
+      <c r="G712" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H712" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="713" ht="15" customHeight="1">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>2026-06-10 12:22 UTC</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D713" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E713" t="n">
+        <v>0</v>
+      </c>
+      <c r="F713" t="n">
+        <v>0</v>
+      </c>
+      <c r="G713" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H713" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="714" ht="15" customHeight="1">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>2026-06-10 12:22 UTC</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D714" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E714" t="n">
+        <v>0</v>
+      </c>
+      <c r="F714" t="n">
+        <v>0</v>
+      </c>
+      <c r="G714" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H714" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="715" ht="15" customHeight="1">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>2026-06-10 12:22 UTC</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D715" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E715" t="n">
+        <v>0</v>
+      </c>
+      <c r="F715" t="n">
+        <v>0</v>
+      </c>
+      <c r="G715" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H715" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="716" ht="15" customHeight="1">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>2026-06-10 12:22 UTC</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D716" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E716" t="n">
+        <v>0</v>
+      </c>
+      <c r="F716" t="n">
+        <v>0</v>
+      </c>
+      <c r="G716" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H716" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="717" ht="15" customHeight="1">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>2026-06-10 12:22 UTC</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D717" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E717" t="n">
+        <v>0</v>
+      </c>
+      <c r="F717" t="n">
+        <v>0</v>
+      </c>
+      <c r="G717" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H717" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="718" ht="15" customHeight="1">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>2026-06-10 12:22 UTC</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D718" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E718" t="n">
+        <v>0</v>
+      </c>
+      <c r="F718" t="n">
+        <v>0</v>
+      </c>
+      <c r="G718" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H718" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="719" ht="15" customHeight="1">
+      <c r="A719" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-10 12:22 UTC</t>
+        </is>
+      </c>
+      <c r="B719" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C719" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D719" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E719" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F719" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G719" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.ff447c6742c49aa252b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.7fd7a0d56e603552915b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.49a759d4d3aa4f3d68df.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.7cca543e0b2db8c438b1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.a3640e30322f2ba9f6c2.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H719" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.bc8021352f52d7e3be39.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="720" ht="15" customHeight="1">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>2026-06-10 12:22 UTC</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D720" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E720" t="n">
+        <v>0</v>
+      </c>
+      <c r="F720" t="n">
+        <v>0</v>
+      </c>
+      <c r="G720" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H720" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="721" ht="15" customHeight="1">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>2026-06-10 12:22 UTC</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D721" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E721" t="n">
+        <v>0</v>
+      </c>
+      <c r="F721" t="n">
+        <v>0</v>
+      </c>
+      <c r="G721" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H721" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -28438,7 +28818,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-09 12:05 UTC</t>
+          <t>2026-06-10 12:22 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -28463,7 +28843,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-09 12:05 UTC</t>
+          <t>2026-06-10 12:22 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -28488,7 +28868,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-09 12:05 UTC</t>
+          <t>2026-06-10 12:22 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -28513,7 +28893,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-09 12:05 UTC</t>
+          <t>2026-06-10 12:22 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -28538,7 +28918,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-09 12:05 UTC</t>
+          <t>2026-06-10 12:22 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -28563,7 +28943,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-09 12:05 UTC</t>
+          <t>2026-06-10 12:22 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -28588,7 +28968,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-09 12:05 UTC</t>
+          <t>2026-06-10 12:22 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -28613,7 +28993,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-09 12:05 UTC</t>
+          <t>2026-06-10 12:22 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -28638,7 +29018,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-09 12:05 UTC</t>
+          <t>2026-06-10 12:22 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -28663,7 +29043,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-09 12:05 UTC</t>
+          <t>2026-06-10 12:22 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -28724,7 +29104,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.bc8021352f52d7e3be39.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.ff447c6742c49aa252b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.7fd7a0d56e603552915b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.49a759d4d3aa4f3d68df.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.7cca543e0b2db8c438b1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.a3640e30322f2ba9f6c2.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -28741,7 +29121,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.8b9da178a57d2f5b2372.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.bc8021352f52d7e3be39.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-11
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H721"/>
+  <dimension ref="A1:H731"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -28138,6 +28138,386 @@
         </is>
       </c>
       <c r="H721" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="722" ht="15" customHeight="1">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>2026-06-11 12:47 UTC</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D722" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E722" t="n">
+        <v>0</v>
+      </c>
+      <c r="F722" t="n">
+        <v>0</v>
+      </c>
+      <c r="G722" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H722" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="723" ht="15" customHeight="1">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>2026-06-11 12:47 UTC</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D723" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E723" t="n">
+        <v>0</v>
+      </c>
+      <c r="F723" t="n">
+        <v>0</v>
+      </c>
+      <c r="G723" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H723" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="724" ht="15" customHeight="1">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>2026-06-11 12:47 UTC</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D724" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E724" t="n">
+        <v>0</v>
+      </c>
+      <c r="F724" t="n">
+        <v>0</v>
+      </c>
+      <c r="G724" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H724" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="725" ht="15" customHeight="1">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>2026-06-11 12:47 UTC</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D725" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E725" t="n">
+        <v>0</v>
+      </c>
+      <c r="F725" t="n">
+        <v>0</v>
+      </c>
+      <c r="G725" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H725" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="726" ht="15" customHeight="1">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>2026-06-11 12:47 UTC</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D726" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E726" t="n">
+        <v>0</v>
+      </c>
+      <c r="F726" t="n">
+        <v>0</v>
+      </c>
+      <c r="G726" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H726" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="727" ht="15" customHeight="1">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>2026-06-11 12:47 UTC</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D727" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E727" t="n">
+        <v>0</v>
+      </c>
+      <c r="F727" t="n">
+        <v>0</v>
+      </c>
+      <c r="G727" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H727" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="728" ht="15" customHeight="1">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>2026-06-11 12:47 UTC</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D728" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E728" t="n">
+        <v>0</v>
+      </c>
+      <c r="F728" t="n">
+        <v>0</v>
+      </c>
+      <c r="G728" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H728" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="729" ht="15" customHeight="1">
+      <c r="A729" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-11 12:47 UTC</t>
+        </is>
+      </c>
+      <c r="B729" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C729" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D729" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E729" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F729" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G729" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.400eb53b9c8f4c64bcbb.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2190.c4fdb659b113a5ae5306.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.57e0e8b8b1eed654344d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.2752c7587d9ab4a73355.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.056d3370ac491910f5c8.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H729" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.ff447c6742c49aa252b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.7fd7a0d56e603552915b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.49a759d4d3aa4f3d68df.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.7cca543e0b2db8c438b1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.a3640e30322f2ba9f6c2.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="730" ht="15" customHeight="1">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>2026-06-11 12:47 UTC</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D730" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E730" t="n">
+        <v>0</v>
+      </c>
+      <c r="F730" t="n">
+        <v>0</v>
+      </c>
+      <c r="G730" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H730" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="731" ht="15" customHeight="1">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>2026-06-11 12:47 UTC</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D731" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E731" t="n">
+        <v>0</v>
+      </c>
+      <c r="F731" t="n">
+        <v>0</v>
+      </c>
+      <c r="G731" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H731" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -28818,7 +29198,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-10 12:22 UTC</t>
+          <t>2026-06-11 12:47 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -28843,7 +29223,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-10 12:22 UTC</t>
+          <t>2026-06-11 12:47 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -28868,7 +29248,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-10 12:22 UTC</t>
+          <t>2026-06-11 12:47 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -28893,7 +29273,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-10 12:22 UTC</t>
+          <t>2026-06-11 12:47 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -28918,7 +29298,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-10 12:22 UTC</t>
+          <t>2026-06-11 12:47 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -28943,7 +29323,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-10 12:22 UTC</t>
+          <t>2026-06-11 12:47 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -28968,7 +29348,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-10 12:22 UTC</t>
+          <t>2026-06-11 12:47 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -28993,7 +29373,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-10 12:22 UTC</t>
+          <t>2026-06-11 12:47 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -29018,7 +29398,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-10 12:22 UTC</t>
+          <t>2026-06-11 12:47 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -29043,7 +29423,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-10 12:22 UTC</t>
+          <t>2026-06-11 12:47 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -29104,7 +29484,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.ff447c6742c49aa252b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.7fd7a0d56e603552915b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.49a759d4d3aa4f3d68df.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.7cca543e0b2db8c438b1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.a3640e30322f2ba9f6c2.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.400eb53b9c8f4c64bcbb.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2190.c4fdb659b113a5ae5306.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.57e0e8b8b1eed654344d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.2752c7587d9ab4a73355.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.056d3370ac491910f5c8.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -29121,7 +29501,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.dbd8340586cc379f6170.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.fb6519e99f352c540ea9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.8f5d94f112cd8efdb6b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8830.8b96a341d1d227a39ef4.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.bc8021352f52d7e3be39.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/8830.4d40243063cd2b940dc2.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.ff447c6742c49aa252b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.7fd7a0d56e603552915b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.49a759d4d3aa4f3d68df.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.7cca543e0b2db8c438b1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.a3640e30322f2ba9f6c2.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-12
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H731"/>
+  <dimension ref="A1:H741"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -28518,6 +28518,386 @@
         </is>
       </c>
       <c r="H731" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="732" ht="15" customHeight="1">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>2026-06-12 12:20 UTC</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D732" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E732" t="n">
+        <v>0</v>
+      </c>
+      <c r="F732" t="n">
+        <v>0</v>
+      </c>
+      <c r="G732" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H732" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="733" ht="15" customHeight="1">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>2026-06-12 12:20 UTC</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D733" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E733" t="n">
+        <v>0</v>
+      </c>
+      <c r="F733" t="n">
+        <v>0</v>
+      </c>
+      <c r="G733" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H733" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="734" ht="15" customHeight="1">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>2026-06-12 12:20 UTC</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D734" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E734" t="n">
+        <v>0</v>
+      </c>
+      <c r="F734" t="n">
+        <v>0</v>
+      </c>
+      <c r="G734" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H734" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="735" ht="15" customHeight="1">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>2026-06-12 12:20 UTC</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D735" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E735" t="n">
+        <v>0</v>
+      </c>
+      <c r="F735" t="n">
+        <v>0</v>
+      </c>
+      <c r="G735" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H735" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="736" ht="15" customHeight="1">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>2026-06-12 12:20 UTC</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D736" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E736" t="n">
+        <v>0</v>
+      </c>
+      <c r="F736" t="n">
+        <v>0</v>
+      </c>
+      <c r="G736" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H736" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="737" ht="15" customHeight="1">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>2026-06-12 12:20 UTC</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D737" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E737" t="n">
+        <v>0</v>
+      </c>
+      <c r="F737" t="n">
+        <v>0</v>
+      </c>
+      <c r="G737" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H737" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="738" ht="15" customHeight="1">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>2026-06-12 12:20 UTC</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D738" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E738" t="n">
+        <v>0</v>
+      </c>
+      <c r="F738" t="n">
+        <v>0</v>
+      </c>
+      <c r="G738" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H738" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="739" ht="15" customHeight="1">
+      <c r="A739" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-12 12:20 UTC</t>
+        </is>
+      </c>
+      <c r="B739" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C739" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D739" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E739" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F739" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G739" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.400eb53b9c8f4c64bcbb.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2190.c4fdb659b113a5ae5306.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c7c425282a97b589d123.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.df878c2bb31cb0ccf844.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.84a40ffd89ed3d652a84.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.98ee4f61222728715dd2.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H739" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.400eb53b9c8f4c64bcbb.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2190.c4fdb659b113a5ae5306.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.57e0e8b8b1eed654344d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.2752c7587d9ab4a73355.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.056d3370ac491910f5c8.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="740" ht="15" customHeight="1">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>2026-06-12 12:20 UTC</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D740" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E740" t="n">
+        <v>0</v>
+      </c>
+      <c r="F740" t="n">
+        <v>0</v>
+      </c>
+      <c r="G740" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H740" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="741" ht="15" customHeight="1">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>2026-06-12 12:20 UTC</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D741" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E741" t="n">
+        <v>0</v>
+      </c>
+      <c r="F741" t="n">
+        <v>0</v>
+      </c>
+      <c r="G741" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H741" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -29198,7 +29578,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-11 12:47 UTC</t>
+          <t>2026-06-12 12:20 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -29223,7 +29603,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-11 12:47 UTC</t>
+          <t>2026-06-12 12:20 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -29248,7 +29628,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-11 12:47 UTC</t>
+          <t>2026-06-12 12:20 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -29273,7 +29653,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-11 12:47 UTC</t>
+          <t>2026-06-12 12:20 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -29298,7 +29678,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-11 12:47 UTC</t>
+          <t>2026-06-12 12:20 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -29323,7 +29703,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-11 12:47 UTC</t>
+          <t>2026-06-12 12:20 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -29348,7 +29728,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-11 12:47 UTC</t>
+          <t>2026-06-12 12:20 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -29373,7 +29753,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-11 12:47 UTC</t>
+          <t>2026-06-12 12:20 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -29398,7 +29778,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-11 12:47 UTC</t>
+          <t>2026-06-12 12:20 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -29423,7 +29803,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-11 12:47 UTC</t>
+          <t>2026-06-12 12:20 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -29484,7 +29864,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.400eb53b9c8f4c64bcbb.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2190.c4fdb659b113a5ae5306.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.57e0e8b8b1eed654344d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.2752c7587d9ab4a73355.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.056d3370ac491910f5c8.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.400eb53b9c8f4c64bcbb.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2190.c4fdb659b113a5ae5306.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c7c425282a97b589d123.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.df878c2bb31cb0ccf844.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.84a40ffd89ed3d652a84.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.98ee4f61222728715dd2.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -29501,7 +29881,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.ff447c6742c49aa252b9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7345.7fd7a0d56e603552915b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.49a759d4d3aa4f3d68df.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.7cca543e0b2db8c438b1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.a3640e30322f2ba9f6c2.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.400eb53b9c8f4c64bcbb.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2190.c4fdb659b113a5ae5306.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.57e0e8b8b1eed654344d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.2752c7587d9ab4a73355.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.056d3370ac491910f5c8.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-13
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H741"/>
+  <dimension ref="A1:H751"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -28898,6 +28898,386 @@
         </is>
       </c>
       <c r="H741" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="742" ht="15" customHeight="1">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>2026-06-13 11:14 UTC</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D742" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E742" t="n">
+        <v>0</v>
+      </c>
+      <c r="F742" t="n">
+        <v>0</v>
+      </c>
+      <c r="G742" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H742" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="743" ht="15" customHeight="1">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>2026-06-13 11:14 UTC</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D743" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E743" t="n">
+        <v>0</v>
+      </c>
+      <c r="F743" t="n">
+        <v>0</v>
+      </c>
+      <c r="G743" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H743" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="744" ht="15" customHeight="1">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>2026-06-13 11:14 UTC</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D744" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E744" t="n">
+        <v>0</v>
+      </c>
+      <c r="F744" t="n">
+        <v>0</v>
+      </c>
+      <c r="G744" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H744" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="745" ht="15" customHeight="1">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>2026-06-13 11:14 UTC</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D745" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E745" t="n">
+        <v>0</v>
+      </c>
+      <c r="F745" t="n">
+        <v>0</v>
+      </c>
+      <c r="G745" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H745" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="746" ht="15" customHeight="1">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>2026-06-13 11:14 UTC</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D746" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E746" t="n">
+        <v>0</v>
+      </c>
+      <c r="F746" t="n">
+        <v>0</v>
+      </c>
+      <c r="G746" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H746" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="747" ht="15" customHeight="1">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>2026-06-13 11:14 UTC</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D747" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E747" t="n">
+        <v>0</v>
+      </c>
+      <c r="F747" t="n">
+        <v>0</v>
+      </c>
+      <c r="G747" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H747" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="748" ht="15" customHeight="1">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>2026-06-13 11:14 UTC</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D748" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E748" t="n">
+        <v>0</v>
+      </c>
+      <c r="F748" t="n">
+        <v>0</v>
+      </c>
+      <c r="G748" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H748" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="749" ht="15" customHeight="1">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>2026-06-13 11:14 UTC</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D749" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E749" t="n">
+        <v>0</v>
+      </c>
+      <c r="F749" t="n">
+        <v>0</v>
+      </c>
+      <c r="G749" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H749" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="750" ht="15" customHeight="1">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>2026-06-13 11:14 UTC</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D750" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E750" t="n">
+        <v>0</v>
+      </c>
+      <c r="F750" t="n">
+        <v>0</v>
+      </c>
+      <c r="G750" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H750" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="751" ht="15" customHeight="1">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>2026-06-13 11:14 UTC</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D751" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E751" t="n">
+        <v>0</v>
+      </c>
+      <c r="F751" t="n">
+        <v>0</v>
+      </c>
+      <c r="G751" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H751" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -29528,6 +29908,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.400eb53b9c8f4c64bcbb.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2190.c4fdb659b113a5ae5306.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c7c425282a97b589d123.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.df878c2bb31cb0ccf844.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.84a40ffd89ed3d652a84.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.98ee4f61222728715dd2.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.400eb53b9c8f4c64bcbb.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2190.c4fdb659b113a5ae5306.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.57e0e8b8b1eed654344d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.2752c7587d9ab4a73355.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.056d3370ac491910f5c8.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -29578,7 +30028,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-12 12:20 UTC</t>
+          <t>2026-06-13 11:14 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -29603,7 +30053,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-12 12:20 UTC</t>
+          <t>2026-06-13 11:14 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -29628,7 +30078,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-12 12:20 UTC</t>
+          <t>2026-06-13 11:14 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -29653,7 +30103,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-12 12:20 UTC</t>
+          <t>2026-06-13 11:14 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -29678,7 +30128,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-12 12:20 UTC</t>
+          <t>2026-06-13 11:14 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -29703,7 +30153,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-12 12:20 UTC</t>
+          <t>2026-06-13 11:14 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -29728,7 +30178,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-12 12:20 UTC</t>
+          <t>2026-06-13 11:14 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -29753,7 +30203,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-12 12:20 UTC</t>
+          <t>2026-06-13 11:14 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -29778,7 +30228,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-12 12:20 UTC</t>
+          <t>2026-06-13 11:14 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -29803,7 +30253,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-12 12:20 UTC</t>
+          <t>2026-06-13 11:14 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -29812,76 +30262,6 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.400eb53b9c8f4c64bcbb.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2190.c4fdb659b113a5ae5306.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c7c425282a97b589d123.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.df878c2bb31cb0ccf844.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.84a40ffd89ed3d652a84.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.98ee4f61222728715dd2.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.400eb53b9c8f4c64bcbb.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2190.c4fdb659b113a5ae5306.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.57e0e8b8b1eed654344d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.2752c7587d9ab4a73355.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.056d3370ac491910f5c8.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-14
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H751"/>
+  <dimension ref="A1:H761"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -29278,6 +29278,386 @@
         </is>
       </c>
       <c r="H751" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="752" ht="15" customHeight="1">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:31 UTC</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D752" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E752" t="n">
+        <v>0</v>
+      </c>
+      <c r="F752" t="n">
+        <v>0</v>
+      </c>
+      <c r="G752" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H752" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="753" ht="15" customHeight="1">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:31 UTC</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D753" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E753" t="n">
+        <v>0</v>
+      </c>
+      <c r="F753" t="n">
+        <v>0</v>
+      </c>
+      <c r="G753" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H753" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="754" ht="15" customHeight="1">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:31 UTC</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D754" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E754" t="n">
+        <v>0</v>
+      </c>
+      <c r="F754" t="n">
+        <v>0</v>
+      </c>
+      <c r="G754" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H754" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="755" ht="15" customHeight="1">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:31 UTC</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E755" t="n">
+        <v>0</v>
+      </c>
+      <c r="F755" t="n">
+        <v>0</v>
+      </c>
+      <c r="G755" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H755" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="756" ht="15" customHeight="1">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:31 UTC</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D756" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E756" t="n">
+        <v>0</v>
+      </c>
+      <c r="F756" t="n">
+        <v>0</v>
+      </c>
+      <c r="G756" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H756" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="757" ht="15" customHeight="1">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:31 UTC</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D757" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E757" t="n">
+        <v>0</v>
+      </c>
+      <c r="F757" t="n">
+        <v>0</v>
+      </c>
+      <c r="G757" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H757" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="758" ht="15" customHeight="1">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:31 UTC</t>
+        </is>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D758" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E758" t="n">
+        <v>0</v>
+      </c>
+      <c r="F758" t="n">
+        <v>0</v>
+      </c>
+      <c r="G758" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H758" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="759" ht="15" customHeight="1">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:31 UTC</t>
+        </is>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D759" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E759" t="n">
+        <v>0</v>
+      </c>
+      <c r="F759" t="n">
+        <v>0</v>
+      </c>
+      <c r="G759" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H759" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="760" ht="15" customHeight="1">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:31 UTC</t>
+        </is>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D760" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E760" t="n">
+        <v>0</v>
+      </c>
+      <c r="F760" t="n">
+        <v>0</v>
+      </c>
+      <c r="G760" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H760" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="761" ht="15" customHeight="1">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>2026-06-14 11:31 UTC</t>
+        </is>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D761" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E761" t="n">
+        <v>0</v>
+      </c>
+      <c r="F761" t="n">
+        <v>0</v>
+      </c>
+      <c r="G761" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H761" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -30028,7 +30408,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-13 11:14 UTC</t>
+          <t>2026-06-14 11:31 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -30053,7 +30433,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-13 11:14 UTC</t>
+          <t>2026-06-14 11:31 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -30078,7 +30458,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-13 11:14 UTC</t>
+          <t>2026-06-14 11:31 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -30103,7 +30483,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-13 11:14 UTC</t>
+          <t>2026-06-14 11:31 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -30128,7 +30508,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-13 11:14 UTC</t>
+          <t>2026-06-14 11:31 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -30153,7 +30533,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-13 11:14 UTC</t>
+          <t>2026-06-14 11:31 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -30178,7 +30558,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-13 11:14 UTC</t>
+          <t>2026-06-14 11:31 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -30203,7 +30583,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-13 11:14 UTC</t>
+          <t>2026-06-14 11:31 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -30228,7 +30608,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-13 11:14 UTC</t>
+          <t>2026-06-14 11:31 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -30253,7 +30633,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-13 11:14 UTC</t>
+          <t>2026-06-14 11:31 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-15
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H761"/>
+  <dimension ref="A1:H771"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -29658,6 +29658,386 @@
         </is>
       </c>
       <c r="H761" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="762" ht="15" customHeight="1">
+      <c r="A762" t="inlineStr">
+        <is>
+          <t>2026-06-15 15:16 UTC</t>
+        </is>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D762" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E762" t="n">
+        <v>0</v>
+      </c>
+      <c r="F762" t="n">
+        <v>0</v>
+      </c>
+      <c r="G762" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H762" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="763" ht="15" customHeight="1">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>2026-06-15 15:16 UTC</t>
+        </is>
+      </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C763" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D763" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E763" t="n">
+        <v>0</v>
+      </c>
+      <c r="F763" t="n">
+        <v>0</v>
+      </c>
+      <c r="G763" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H763" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="764" ht="15" customHeight="1">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>2026-06-15 15:16 UTC</t>
+        </is>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C764" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D764" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E764" t="n">
+        <v>0</v>
+      </c>
+      <c r="F764" t="n">
+        <v>0</v>
+      </c>
+      <c r="G764" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H764" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="765" ht="15" customHeight="1">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>2026-06-15 15:16 UTC</t>
+        </is>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D765" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E765" t="n">
+        <v>0</v>
+      </c>
+      <c r="F765" t="n">
+        <v>0</v>
+      </c>
+      <c r="G765" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H765" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="766" ht="15" customHeight="1">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>2026-06-15 15:16 UTC</t>
+        </is>
+      </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D766" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E766" t="n">
+        <v>0</v>
+      </c>
+      <c r="F766" t="n">
+        <v>0</v>
+      </c>
+      <c r="G766" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H766" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="767" ht="15" customHeight="1">
+      <c r="A767" t="inlineStr">
+        <is>
+          <t>2026-06-15 15:16 UTC</t>
+        </is>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C767" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D767" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E767" t="n">
+        <v>0</v>
+      </c>
+      <c r="F767" t="n">
+        <v>0</v>
+      </c>
+      <c r="G767" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H767" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="768" ht="15" customHeight="1">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>2026-06-15 15:16 UTC</t>
+        </is>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D768" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E768" t="n">
+        <v>0</v>
+      </c>
+      <c r="F768" t="n">
+        <v>0</v>
+      </c>
+      <c r="G768" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H768" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="769" ht="15" customHeight="1">
+      <c r="A769" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-15 15:16 UTC</t>
+        </is>
+      </c>
+      <c r="B769" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C769" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D769" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E769" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F769" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G769" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9407.471d80aa2b4d8b01e945.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2190.c4fdb659b113a5ae5306.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.ee4c9bb27ad55eaa06b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.94958693313d73cd8835.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.dee845e9a4cbeb6663fd.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9407.eb7339b4eb4dca647de9.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.98ee4f61222728715dd2.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H769" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.400eb53b9c8f4c64bcbb.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2190.c4fdb659b113a5ae5306.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c7c425282a97b589d123.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.df878c2bb31cb0ccf844.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.84a40ffd89ed3d652a84.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.98ee4f61222728715dd2.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="770" ht="15" customHeight="1">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>2026-06-15 15:16 UTC</t>
+        </is>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D770" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E770" t="n">
+        <v>0</v>
+      </c>
+      <c r="F770" t="n">
+        <v>0</v>
+      </c>
+      <c r="G770" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H770" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="771" ht="15" customHeight="1">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>2026-06-15 15:16 UTC</t>
+        </is>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D771" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E771" t="n">
+        <v>0</v>
+      </c>
+      <c r="F771" t="n">
+        <v>0</v>
+      </c>
+      <c r="G771" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H771" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -30288,76 +30668,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.400eb53b9c8f4c64bcbb.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2190.c4fdb659b113a5ae5306.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c7c425282a97b589d123.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.df878c2bb31cb0ccf844.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.84a40ffd89ed3d652a84.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.98ee4f61222728715dd2.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.400eb53b9c8f4c64bcbb.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2190.c4fdb659b113a5ae5306.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.57e0e8b8b1eed654344d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.2752c7587d9ab4a73355.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.056d3370ac491910f5c8.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.1d4e1a5a170d91156ebd.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -30408,7 +30718,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-14 11:31 UTC</t>
+          <t>2026-06-15 15:16 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -30433,7 +30743,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-14 11:31 UTC</t>
+          <t>2026-06-15 15:16 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -30458,7 +30768,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-14 11:31 UTC</t>
+          <t>2026-06-15 15:16 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -30483,7 +30793,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-14 11:31 UTC</t>
+          <t>2026-06-15 15:16 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -30508,7 +30818,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-14 11:31 UTC</t>
+          <t>2026-06-15 15:16 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -30533,7 +30843,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-14 11:31 UTC</t>
+          <t>2026-06-15 15:16 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -30558,7 +30868,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-14 11:31 UTC</t>
+          <t>2026-06-15 15:16 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -30583,7 +30893,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-14 11:31 UTC</t>
+          <t>2026-06-15 15:16 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -30608,7 +30918,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-14 11:31 UTC</t>
+          <t>2026-06-15 15:16 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -30633,7 +30943,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-14 11:31 UTC</t>
+          <t>2026-06-15 15:16 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -30642,6 +30952,76 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9407.471d80aa2b4d8b01e945.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2190.c4fdb659b113a5ae5306.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.ee4c9bb27ad55eaa06b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.94958693313d73cd8835.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.dee845e9a4cbeb6663fd.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9407.eb7339b4eb4dca647de9.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.98ee4f61222728715dd2.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.400eb53b9c8f4c64bcbb.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2190.c4fdb659b113a5ae5306.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c7c425282a97b589d123.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.df878c2bb31cb0ccf844.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.84a40ffd89ed3d652a84.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.98ee4f61222728715dd2.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-16
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H771"/>
+  <dimension ref="A1:H781"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -30038,6 +30038,386 @@
         </is>
       </c>
       <c r="H771" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="772" ht="15" customHeight="1">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>2026-06-16 13:28 UTC</t>
+        </is>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D772" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E772" t="n">
+        <v>0</v>
+      </c>
+      <c r="F772" t="n">
+        <v>0</v>
+      </c>
+      <c r="G772" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H772" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="773" ht="15" customHeight="1">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>2026-06-16 13:28 UTC</t>
+        </is>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D773" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E773" t="n">
+        <v>0</v>
+      </c>
+      <c r="F773" t="n">
+        <v>0</v>
+      </c>
+      <c r="G773" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H773" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="774" ht="15" customHeight="1">
+      <c r="A774" t="inlineStr">
+        <is>
+          <t>2026-06-16 13:28 UTC</t>
+        </is>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D774" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E774" t="n">
+        <v>0</v>
+      </c>
+      <c r="F774" t="n">
+        <v>0</v>
+      </c>
+      <c r="G774" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H774" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="775" ht="15" customHeight="1">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>2026-06-16 13:28 UTC</t>
+        </is>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D775" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E775" t="n">
+        <v>0</v>
+      </c>
+      <c r="F775" t="n">
+        <v>0</v>
+      </c>
+      <c r="G775" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H775" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="776" ht="15" customHeight="1">
+      <c r="A776" t="inlineStr">
+        <is>
+          <t>2026-06-16 13:28 UTC</t>
+        </is>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D776" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E776" t="n">
+        <v>0</v>
+      </c>
+      <c r="F776" t="n">
+        <v>0</v>
+      </c>
+      <c r="G776" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H776" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="777" ht="15" customHeight="1">
+      <c r="A777" t="inlineStr">
+        <is>
+          <t>2026-06-16 13:28 UTC</t>
+        </is>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D777" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E777" t="n">
+        <v>0</v>
+      </c>
+      <c r="F777" t="n">
+        <v>0</v>
+      </c>
+      <c r="G777" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H777" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="778" ht="15" customHeight="1">
+      <c r="A778" t="inlineStr">
+        <is>
+          <t>2026-06-16 13:28 UTC</t>
+        </is>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D778" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E778" t="n">
+        <v>0</v>
+      </c>
+      <c r="F778" t="n">
+        <v>0</v>
+      </c>
+      <c r="G778" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H778" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="779" ht="15" customHeight="1">
+      <c r="A779" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-16 13:28 UTC</t>
+        </is>
+      </c>
+      <c r="B779" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C779" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D779" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E779" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F779" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G779" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59407.c03a2b27cbc32f68c08e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.3db9da783e2d3d839bd7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.547e0e079804993d5940.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f41fdcc02fda2d017edc.js"&gt;&lt;/script&gt;&lt;link href="/style/css/59407.3e77c98aa45f5cb88e2d.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.38828fbbf387038ed84a.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H779" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9407.471d80aa2b4d8b01e945.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2190.c4fdb659b113a5ae5306.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.ee4c9bb27ad55eaa06b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.94958693313d73cd8835.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.dee845e9a4cbeb6663fd.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9407.eb7339b4eb4dca647de9.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.98ee4f61222728715dd2.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="780" ht="15" customHeight="1">
+      <c r="A780" t="inlineStr">
+        <is>
+          <t>2026-06-16 13:28 UTC</t>
+        </is>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D780" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E780" t="n">
+        <v>0</v>
+      </c>
+      <c r="F780" t="n">
+        <v>0</v>
+      </c>
+      <c r="G780" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H780" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="781" ht="15" customHeight="1">
+      <c r="A781" t="inlineStr">
+        <is>
+          <t>2026-06-16 13:28 UTC</t>
+        </is>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D781" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E781" t="n">
+        <v>0</v>
+      </c>
+      <c r="F781" t="n">
+        <v>0</v>
+      </c>
+      <c r="G781" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H781" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -30718,7 +31098,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-15 15:16 UTC</t>
+          <t>2026-06-16 13:28 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -30743,7 +31123,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-15 15:16 UTC</t>
+          <t>2026-06-16 13:28 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -30768,7 +31148,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-15 15:16 UTC</t>
+          <t>2026-06-16 13:28 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -30793,7 +31173,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-15 15:16 UTC</t>
+          <t>2026-06-16 13:28 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -30818,7 +31198,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-15 15:16 UTC</t>
+          <t>2026-06-16 13:28 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -30843,7 +31223,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-15 15:16 UTC</t>
+          <t>2026-06-16 13:28 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -30868,7 +31248,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-15 15:16 UTC</t>
+          <t>2026-06-16 13:28 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -30893,7 +31273,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-15 15:16 UTC</t>
+          <t>2026-06-16 13:28 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -30918,7 +31298,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-15 15:16 UTC</t>
+          <t>2026-06-16 13:28 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -30943,7 +31323,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-15 15:16 UTC</t>
+          <t>2026-06-16 13:28 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -31004,7 +31384,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9407.471d80aa2b4d8b01e945.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2190.c4fdb659b113a5ae5306.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.ee4c9bb27ad55eaa06b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.94958693313d73cd8835.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.dee845e9a4cbeb6663fd.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9407.eb7339b4eb4dca647de9.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.98ee4f61222728715dd2.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59407.c03a2b27cbc32f68c08e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.3db9da783e2d3d839bd7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.547e0e079804993d5940.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f41fdcc02fda2d017edc.js"&gt;&lt;/script&gt;&lt;link href="/style/css/59407.3e77c98aa45f5cb88e2d.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.38828fbbf387038ed84a.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -31021,7 +31401,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2331.400eb53b9c8f4c64bcbb.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2190.c4fdb659b113a5ae5306.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.c7c425282a97b589d123.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.df878c2bb31cb0ccf844.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.84a40ffd89ed3d652a84.js"&gt;&lt;/script&gt;&lt;link href="/style/css/2331.9d4787090d72b70ad27f.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.98ee4f61222728715dd2.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9407.471d80aa2b4d8b01e945.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2190.c4fdb659b113a5ae5306.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.ee4c9bb27ad55eaa06b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.94958693313d73cd8835.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.dee845e9a4cbeb6663fd.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9407.eb7339b4eb4dca647de9.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.98ee4f61222728715dd2.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-17
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H781"/>
+  <dimension ref="A1:H791"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -30418,6 +30418,386 @@
         </is>
       </c>
       <c r="H781" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="782" ht="15" customHeight="1">
+      <c r="A782" t="inlineStr">
+        <is>
+          <t>2026-06-17 12:52 UTC</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D782" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E782" t="n">
+        <v>0</v>
+      </c>
+      <c r="F782" t="n">
+        <v>0</v>
+      </c>
+      <c r="G782" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H782" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="783" ht="15" customHeight="1">
+      <c r="A783" t="inlineStr">
+        <is>
+          <t>2026-06-17 12:52 UTC</t>
+        </is>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D783" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E783" t="n">
+        <v>0</v>
+      </c>
+      <c r="F783" t="n">
+        <v>0</v>
+      </c>
+      <c r="G783" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H783" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="784" ht="15" customHeight="1">
+      <c r="A784" t="inlineStr">
+        <is>
+          <t>2026-06-17 12:52 UTC</t>
+        </is>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D784" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E784" t="n">
+        <v>0</v>
+      </c>
+      <c r="F784" t="n">
+        <v>0</v>
+      </c>
+      <c r="G784" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H784" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="785" ht="15" customHeight="1">
+      <c r="A785" t="inlineStr">
+        <is>
+          <t>2026-06-17 12:52 UTC</t>
+        </is>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D785" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E785" t="n">
+        <v>0</v>
+      </c>
+      <c r="F785" t="n">
+        <v>0</v>
+      </c>
+      <c r="G785" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H785" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="786" ht="15" customHeight="1">
+      <c r="A786" t="inlineStr">
+        <is>
+          <t>2026-06-17 12:52 UTC</t>
+        </is>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D786" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E786" t="n">
+        <v>0</v>
+      </c>
+      <c r="F786" t="n">
+        <v>0</v>
+      </c>
+      <c r="G786" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H786" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="787" ht="15" customHeight="1">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>2026-06-17 12:52 UTC</t>
+        </is>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D787" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E787" t="n">
+        <v>0</v>
+      </c>
+      <c r="F787" t="n">
+        <v>0</v>
+      </c>
+      <c r="G787" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H787" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="788" ht="15" customHeight="1">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>2026-06-17 12:52 UTC</t>
+        </is>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D788" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E788" t="n">
+        <v>0</v>
+      </c>
+      <c r="F788" t="n">
+        <v>0</v>
+      </c>
+      <c r="G788" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H788" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="789" ht="15" customHeight="1">
+      <c r="A789" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-17 12:52 UTC</t>
+        </is>
+      </c>
+      <c r="B789" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C789" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D789" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E789" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F789" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G789" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59407.c03a2b27cbc32f68c08e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.3db9da783e2d3d839bd7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.547e0e079804993d5940.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.19603c9825c840003a6b.js"&gt;&lt;/script&gt;&lt;link href="/style/css/59407.3e77c98aa45f5cb88e2d.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.38828fbbf387038ed84a.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H789" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59407.c03a2b27cbc32f68c08e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.3db9da783e2d3d839bd7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.547e0e079804993d5940.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f41fdcc02fda2d017edc.js"&gt;&lt;/script&gt;&lt;link href="/style/css/59407.3e77c98aa45f5cb88e2d.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.38828fbbf387038ed84a.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="790" ht="15" customHeight="1">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>2026-06-17 12:52 UTC</t>
+        </is>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D790" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E790" t="n">
+        <v>0</v>
+      </c>
+      <c r="F790" t="n">
+        <v>0</v>
+      </c>
+      <c r="G790" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H790" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="791" ht="15" customHeight="1">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>2026-06-17 12:52 UTC</t>
+        </is>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D791" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E791" t="n">
+        <v>0</v>
+      </c>
+      <c r="F791" t="n">
+        <v>0</v>
+      </c>
+      <c r="G791" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H791" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -31098,7 +31478,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-16 13:28 UTC</t>
+          <t>2026-06-17 12:52 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -31123,7 +31503,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-16 13:28 UTC</t>
+          <t>2026-06-17 12:52 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -31148,7 +31528,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-16 13:28 UTC</t>
+          <t>2026-06-17 12:52 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -31173,7 +31553,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-16 13:28 UTC</t>
+          <t>2026-06-17 12:52 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -31198,7 +31578,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-16 13:28 UTC</t>
+          <t>2026-06-17 12:52 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -31223,7 +31603,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-16 13:28 UTC</t>
+          <t>2026-06-17 12:52 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -31248,7 +31628,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-16 13:28 UTC</t>
+          <t>2026-06-17 12:52 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -31273,7 +31653,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-16 13:28 UTC</t>
+          <t>2026-06-17 12:52 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -31298,7 +31678,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-16 13:28 UTC</t>
+          <t>2026-06-17 12:52 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -31323,7 +31703,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-16 13:28 UTC</t>
+          <t>2026-06-17 12:52 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -31384,7 +31764,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59407.c03a2b27cbc32f68c08e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.3db9da783e2d3d839bd7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.547e0e079804993d5940.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f41fdcc02fda2d017edc.js"&gt;&lt;/script&gt;&lt;link href="/style/css/59407.3e77c98aa45f5cb88e2d.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.38828fbbf387038ed84a.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59407.c03a2b27cbc32f68c08e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.3db9da783e2d3d839bd7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.547e0e079804993d5940.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.19603c9825c840003a6b.js"&gt;&lt;/script&gt;&lt;link href="/style/css/59407.3e77c98aa45f5cb88e2d.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.38828fbbf387038ed84a.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -31401,7 +31781,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.cf74f9511a2f14918305.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/7350.b3bc42f9782366b4a369.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8287.0ba943154ca536a45aba.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/8173.6f1ef8dd8d9235a278ad.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9407.471d80aa2b4d8b01e945.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/2190.c4fdb659b113a5ae5306.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/4366.4ef84af9236589d9b57f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/6406.ee4c9bb27ad55eaa06b3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/9657.94958693313d73cd8835.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.dee845e9a4cbeb6663fd.js"&gt;&lt;/script&gt;&lt;link href="/style/css/9407.eb7339b4eb4dca647de9.css" rel="stylesheet"&gt;&lt;link href="/style/css/9657.83127141e6ed0bd27245.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.98ee4f61222728715dd2.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59407.c03a2b27cbc32f68c08e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.3db9da783e2d3d839bd7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.547e0e079804993d5940.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f41fdcc02fda2d017edc.js"&gt;&lt;/script&gt;&lt;link href="/style/css/59407.3e77c98aa45f5cb88e2d.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.38828fbbf387038ed84a.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-18
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H791"/>
+  <dimension ref="A1:H801"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -30798,6 +30798,386 @@
         </is>
       </c>
       <c r="H791" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="792" ht="15" customHeight="1">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>2026-06-18 12:27 UTC</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D792" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E792" t="n">
+        <v>0</v>
+      </c>
+      <c r="F792" t="n">
+        <v>0</v>
+      </c>
+      <c r="G792" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H792" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="793" ht="15" customHeight="1">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>2026-06-18 12:27 UTC</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D793" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E793" t="n">
+        <v>0</v>
+      </c>
+      <c r="F793" t="n">
+        <v>0</v>
+      </c>
+      <c r="G793" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H793" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="794" ht="15" customHeight="1">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>2026-06-18 12:27 UTC</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D794" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E794" t="n">
+        <v>0</v>
+      </c>
+      <c r="F794" t="n">
+        <v>0</v>
+      </c>
+      <c r="G794" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H794" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="795" ht="15" customHeight="1">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>2026-06-18 12:27 UTC</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D795" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E795" t="n">
+        <v>0</v>
+      </c>
+      <c r="F795" t="n">
+        <v>0</v>
+      </c>
+      <c r="G795" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H795" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="796" ht="15" customHeight="1">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>2026-06-18 12:27 UTC</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D796" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E796" t="n">
+        <v>0</v>
+      </c>
+      <c r="F796" t="n">
+        <v>0</v>
+      </c>
+      <c r="G796" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H796" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="797" ht="15" customHeight="1">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>2026-06-18 12:27 UTC</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D797" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E797" t="n">
+        <v>0</v>
+      </c>
+      <c r="F797" t="n">
+        <v>0</v>
+      </c>
+      <c r="G797" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H797" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="798" ht="15" customHeight="1">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>2026-06-18 12:27 UTC</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D798" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E798" t="n">
+        <v>0</v>
+      </c>
+      <c r="F798" t="n">
+        <v>0</v>
+      </c>
+      <c r="G798" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H798" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="799" ht="15" customHeight="1">
+      <c r="A799" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-18 12:27 UTC</t>
+        </is>
+      </c>
+      <c r="B799" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C799" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D799" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E799" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F799" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G799" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59407.c03a2b27cbc32f68c08e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.3db9da783e2d3d839bd7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.547e0e079804993d5940.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.53f466e4f012652d8137.js"&gt;&lt;/script&gt;&lt;link href="/style/css/59407.3e77c98aa45f5cb88e2d.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.38828fbbf387038ed84a.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H799" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59407.c03a2b27cbc32f68c08e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.3db9da783e2d3d839bd7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.547e0e079804993d5940.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.19603c9825c840003a6b.js"&gt;&lt;/script&gt;&lt;link href="/style/css/59407.3e77c98aa45f5cb88e2d.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.38828fbbf387038ed84a.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="800" ht="15" customHeight="1">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>2026-06-18 12:27 UTC</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D800" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E800" t="n">
+        <v>0</v>
+      </c>
+      <c r="F800" t="n">
+        <v>0</v>
+      </c>
+      <c r="G800" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H800" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="801" ht="15" customHeight="1">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>2026-06-18 12:27 UTC</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D801" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E801" t="n">
+        <v>0</v>
+      </c>
+      <c r="F801" t="n">
+        <v>0</v>
+      </c>
+      <c r="G801" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H801" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -31478,7 +31858,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-17 12:52 UTC</t>
+          <t>2026-06-18 12:27 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -31503,7 +31883,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-17 12:52 UTC</t>
+          <t>2026-06-18 12:27 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -31528,7 +31908,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-17 12:52 UTC</t>
+          <t>2026-06-18 12:27 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -31553,7 +31933,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-17 12:52 UTC</t>
+          <t>2026-06-18 12:27 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -31578,7 +31958,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-17 12:52 UTC</t>
+          <t>2026-06-18 12:27 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -31603,7 +31983,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-17 12:52 UTC</t>
+          <t>2026-06-18 12:27 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -31628,7 +32008,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-17 12:52 UTC</t>
+          <t>2026-06-18 12:27 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -31653,7 +32033,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-17 12:52 UTC</t>
+          <t>2026-06-18 12:27 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -31678,7 +32058,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-17 12:52 UTC</t>
+          <t>2026-06-18 12:27 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -31703,7 +32083,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-17 12:52 UTC</t>
+          <t>2026-06-18 12:27 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -31764,7 +32144,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59407.c03a2b27cbc32f68c08e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.3db9da783e2d3d839bd7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.547e0e079804993d5940.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.19603c9825c840003a6b.js"&gt;&lt;/script&gt;&lt;link href="/style/css/59407.3e77c98aa45f5cb88e2d.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.38828fbbf387038ed84a.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59407.c03a2b27cbc32f68c08e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.3db9da783e2d3d839bd7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.547e0e079804993d5940.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.53f466e4f012652d8137.js"&gt;&lt;/script&gt;&lt;link href="/style/css/59407.3e77c98aa45f5cb88e2d.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.38828fbbf387038ed84a.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -31781,7 +32161,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59407.c03a2b27cbc32f68c08e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.3db9da783e2d3d839bd7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.547e0e079804993d5940.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f41fdcc02fda2d017edc.js"&gt;&lt;/script&gt;&lt;link href="/style/css/59407.3e77c98aa45f5cb88e2d.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.38828fbbf387038ed84a.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59407.c03a2b27cbc32f68c08e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.3db9da783e2d3d839bd7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.547e0e079804993d5940.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.19603c9825c840003a6b.js"&gt;&lt;/script&gt;&lt;link href="/style/css/59407.3e77c98aa45f5cb88e2d.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.38828fbbf387038ed84a.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-21
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H821"/>
+  <dimension ref="A1:H831"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -32109,6 +32109,386 @@
         </is>
       </c>
       <c r="H821" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="822" ht="15" customHeight="1">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>2026-06-21 11:46 UTC</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D822" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E822" t="n">
+        <v>0</v>
+      </c>
+      <c r="F822" t="n">
+        <v>0</v>
+      </c>
+      <c r="G822" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H822" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="823" ht="15" customHeight="1">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>2026-06-21 11:46 UTC</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D823" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E823" t="n">
+        <v>0</v>
+      </c>
+      <c r="F823" t="n">
+        <v>0</v>
+      </c>
+      <c r="G823" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H823" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="824" ht="15" customHeight="1">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>2026-06-21 11:46 UTC</t>
+        </is>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D824" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E824" t="n">
+        <v>0</v>
+      </c>
+      <c r="F824" t="n">
+        <v>0</v>
+      </c>
+      <c r="G824" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H824" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="825" ht="15" customHeight="1">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>2026-06-21 11:46 UTC</t>
+        </is>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D825" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E825" t="n">
+        <v>0</v>
+      </c>
+      <c r="F825" t="n">
+        <v>0</v>
+      </c>
+      <c r="G825" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H825" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="826" ht="15" customHeight="1">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>2026-06-21 11:46 UTC</t>
+        </is>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D826" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E826" t="n">
+        <v>0</v>
+      </c>
+      <c r="F826" t="n">
+        <v>0</v>
+      </c>
+      <c r="G826" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H826" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="827" ht="15" customHeight="1">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>2026-06-21 11:46 UTC</t>
+        </is>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D827" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E827" t="n">
+        <v>0</v>
+      </c>
+      <c r="F827" t="n">
+        <v>0</v>
+      </c>
+      <c r="G827" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H827" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="828" ht="15" customHeight="1">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>2026-06-21 11:46 UTC</t>
+        </is>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D828" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E828" t="n">
+        <v>0</v>
+      </c>
+      <c r="F828" t="n">
+        <v>0</v>
+      </c>
+      <c r="G828" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H828" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="829" ht="15" customHeight="1">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>2026-06-21 11:46 UTC</t>
+        </is>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D829" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E829" t="n">
+        <v>0</v>
+      </c>
+      <c r="F829" t="n">
+        <v>0</v>
+      </c>
+      <c r="G829" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H829" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="830" ht="15" customHeight="1">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>2026-06-21 11:46 UTC</t>
+        </is>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D830" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E830" t="n">
+        <v>0</v>
+      </c>
+      <c r="F830" t="n">
+        <v>0</v>
+      </c>
+      <c r="G830" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H830" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="831" ht="15" customHeight="1">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>2026-06-21 11:46 UTC</t>
+        </is>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D831" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E831" t="n">
+        <v>0</v>
+      </c>
+      <c r="F831" t="n">
+        <v>0</v>
+      </c>
+      <c r="G831" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H831" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -34933,7 +35313,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-20 11:20 UTC</t>
+          <t>2026-06-21 11:46 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -34958,7 +35338,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-20 11:20 UTC</t>
+          <t>2026-06-21 11:46 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -34983,7 +35363,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-20 11:20 UTC</t>
+          <t>2026-06-21 11:46 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -35008,7 +35388,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-20 11:20 UTC</t>
+          <t>2026-06-21 11:46 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -35033,7 +35413,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-20 11:20 UTC</t>
+          <t>2026-06-21 11:46 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -35058,7 +35438,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-20 11:20 UTC</t>
+          <t>2026-06-21 11:46 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -35083,7 +35463,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-20 11:20 UTC</t>
+          <t>2026-06-21 11:46 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -35108,7 +35488,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-20 11:20 UTC</t>
+          <t>2026-06-21 11:46 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -35133,7 +35513,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-20 11:20 UTC</t>
+          <t>2026-06-21 11:46 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -35158,7 +35538,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-20 11:20 UTC</t>
+          <t>2026-06-21 11:46 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-22
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -15,10 +15,10 @@
     <sheet name="ifc_com_ads_txt" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="ifc_com_app-ads_txt" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="wetv_com_ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="wetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H831"/>
+  <dimension ref="A1:H841"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -32489,6 +32489,386 @@
         </is>
       </c>
       <c r="H831" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="832" ht="15" customHeight="1">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>2026-06-22 14:42 UTC</t>
+        </is>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D832" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E832" t="n">
+        <v>0</v>
+      </c>
+      <c r="F832" t="n">
+        <v>0</v>
+      </c>
+      <c r="G832" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H832" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="833" ht="15" customHeight="1">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>2026-06-22 14:42 UTC</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D833" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E833" t="n">
+        <v>0</v>
+      </c>
+      <c r="F833" t="n">
+        <v>0</v>
+      </c>
+      <c r="G833" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H833" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="834" ht="15" customHeight="1">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>2026-06-22 14:42 UTC</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D834" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E834" t="n">
+        <v>0</v>
+      </c>
+      <c r="F834" t="n">
+        <v>0</v>
+      </c>
+      <c r="G834" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H834" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="835" ht="15" customHeight="1">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>2026-06-22 14:42 UTC</t>
+        </is>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D835" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E835" t="n">
+        <v>0</v>
+      </c>
+      <c r="F835" t="n">
+        <v>0</v>
+      </c>
+      <c r="G835" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H835" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="836" ht="15" customHeight="1">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>2026-06-22 14:42 UTC</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D836" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E836" t="n">
+        <v>0</v>
+      </c>
+      <c r="F836" t="n">
+        <v>0</v>
+      </c>
+      <c r="G836" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H836" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="837" ht="15" customHeight="1">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>2026-06-22 14:42 UTC</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D837" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E837" t="n">
+        <v>0</v>
+      </c>
+      <c r="F837" t="n">
+        <v>0</v>
+      </c>
+      <c r="G837" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H837" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="838" ht="15" customHeight="1">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>2026-06-22 14:42 UTC</t>
+        </is>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D838" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E838" t="n">
+        <v>0</v>
+      </c>
+      <c r="F838" t="n">
+        <v>0</v>
+      </c>
+      <c r="G838" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H838" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="839" ht="15" customHeight="1">
+      <c r="A839" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-22 14:42 UTC</t>
+        </is>
+      </c>
+      <c r="B839" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C839" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D839" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E839" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F839" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G839" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/22192.1b405875efa9f607de5b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a945bdfdb5cf49bf4266.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.9e173e0a67ac7ac4a279.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f98cff8f6cbd7006bc03.js"&gt;&lt;/script&gt;&lt;link href="/style/css/22192.3628d6adb3505d1a8000.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H839" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/22192.1b405875efa9f607de5b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a945bdfdb5cf49bf4266.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.9e173e0a67ac7ac4a279.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9803df3f645dd7eb7a3c.js"&gt;&lt;/script&gt;&lt;link href="/style/css/22192.3628d6adb3505d1a8000.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.38828fbbf387038ed84a.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="840" ht="15" customHeight="1">
+      <c r="A840" t="inlineStr">
+        <is>
+          <t>2026-06-22 14:42 UTC</t>
+        </is>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D840" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E840" t="n">
+        <v>0</v>
+      </c>
+      <c r="F840" t="n">
+        <v>0</v>
+      </c>
+      <c r="G840" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H840" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="841" ht="15" customHeight="1">
+      <c r="A841" t="inlineStr">
+        <is>
+          <t>2026-06-22 14:42 UTC</t>
+        </is>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D841" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E841" t="n">
+        <v>0</v>
+      </c>
+      <c r="F841" t="n">
+        <v>0</v>
+      </c>
+      <c r="G841" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H841" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -33884,1385 +34264,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C80"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>conversantmedia.com, 101216, RESELLER, 03113cd04947736d</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>inmobi.com, 55049d2e109d4ac1820ca1432dda4e13, RESELLER, 83e75a7ae333ca9d</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>intenze.co, 200202, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>onlinemediasolutions.com, 20480, RESELLER, b3868b187e4b6402</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>admixer.net, a4fc102e-449c-483d-bdf8-b2a476a3f3bd, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>blasto.ai, 101, RESELLER, 7e936b1feafdaa61</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>advangelists.com, 9766527f2b5d3e95d4a733fcfb77bd7e, RESELLER, 60d26397ec060f98</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>app-stock.com, 343264, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 161802, RESELLER, 5d62403b186f2ace</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 164126, RESELLER, 5d62403b186f2ace</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>risecodes.com, 688215d1f9acce0001954fb1, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>selectmedia.asia, 645b5a31e427dc0a87095fc5, RESELLER, e365c871a27c655d</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>bematterfull.com, 92134446122, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>smartyads.com, 300019, RESELLER, fd2bde0ff2e62c5d</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>tredio.io, 357a6fdf7642bf815a88822c447d9dc436970, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>conversantmedia.com, 100364, RESELLER, 03113cd04947736d</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>boldcollective.co, 778226, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>lijit.com, 509976, RESELLER, fafdf38b16bf6b2b</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>brightmountainmedia.com, 268679, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>bold-win.com, 1104, RESELLER, 71746737d0bab951</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>tviq.io, 2116, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>lunamedia.io, d5b7a3e0bf7575046765e5c639e98ab0, RESELLER, 524ecb396915caaf</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 534990-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 534990-r-523319, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>pgamssp.com, 690a2e9d27800cf3f809f319, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 166643, RESELLER, 5d62403b186f2ace</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, sg1256512, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 535662-r-523319, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>zmaticoo.com, 5135985, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>x.adprime.com, AJxF6R99a9M6CaTvK, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>zetaglobal.net, 748, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>telaria.com, wixu4-vssbd, RESELLER, 1a4e959a1b50034a</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>tremorhub.com, wixu4-vssbd, RESELLER, 1a4e959a1b50034a</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>adipolo.com, 102032, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>appnexus.com, 16912, RESELLER, f5ab79cb980f11d1</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>improvedigital.com, 2836, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>supply.colossusssp.com, 892, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>pgamssp.com, 69a5d5c4d1f5f685e7085234, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>videoheroes.tv, 212459, RESELLER, 064bc410192443d8</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>sharethrough.com, f0oQSO2J, RESELLER, d53b998a7bd4ecd2</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 534605-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>media.net, 8CU76542S, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>video.unrulymedia.com, 2099898025, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>zetaglobal.net, 642, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C46" s="4" t="inlineStr">
-        <is>
-          <t>improvedigital.com, 2853, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B47" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 162588, RESELLER, 5d62403b186f2ace</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B48" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 167844, RESELLER, 5d62403b186f2ace</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B49" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C49" s="4" t="inlineStr">
-        <is>
-          <t>rubiconproject.com, 27386, RESELLER, 0bfd66d529a55807</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t>lijit.com, 587508, RESELLER, fafdf38b16bf6b2b</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B51" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C51" s="4" t="inlineStr">
-        <is>
-          <t>bidmachine.io, 1490, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B52" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C52" s="4" t="inlineStr">
-        <is>
-          <t>x.adprime.com, AJxF6R109a9M6CaTvK, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B53" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C53" s="4" t="inlineStr">
-        <is>
-          <t>152media.info, 152M1197, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B54" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C54" s="4" t="inlineStr">
-        <is>
-          <t>sharethrough.com, vQMCuYXA, RESELLER, d53b998a7bd4ecd2</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B55" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C55" s="4" t="inlineStr">
-        <is>
-          <t>smartbid.ai, SMB60005, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B56" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C56" s="4" t="inlineStr">
-        <is>
-          <t>lijit.com, 512908, RESELLER, fafdf38b16bf6b2b</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B57" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C57" s="4" t="inlineStr">
-        <is>
-          <t>rubiconproject.com, 24448, RESELLER, 0bfd66d529a55807</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B58" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C58" s="4" t="inlineStr">
-        <is>
-          <t>video.unrulymedia.com, 2613193077, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B59" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C59" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, sg1256366, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B60" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C60" s="4" t="inlineStr">
-        <is>
-          <t>lijit.com, 383910, RESELLER, fafdf38b16bf6b2b #SOVRN</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B61" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C61" s="4" t="inlineStr">
-        <is>
-          <t>rhebus.works, 1500765024, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B62" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C62" s="4" t="inlineStr">
-        <is>
-          <t>pubmatic.com, 167263, RESELLER,</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B63" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C63" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 535659-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B64" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C64" s="4" t="inlineStr">
-        <is>
-          <t>smartadserver.com, 4210, RESELLER, 060d053dcf45cbf3</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B65" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C65" s="4" t="inlineStr">
-        <is>
-          <t>smartstream.tv, 679, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B66" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C66" s="4" t="inlineStr">
-        <is>
-          <t>smaato.com, 1100050739, RESELLER, 07bcf65f187117b4</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B67" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C67" s="4" t="inlineStr">
-        <is>
-          <t>appnexus.com, 13709, RESELLER, f5ab79cb980f11d1</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B68" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C68" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 534605-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B69" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C69" s="4" t="inlineStr">
-        <is>
-          <t>media.net, 8CU76542S, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B70" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C70" s="4" t="inlineStr">
-        <is>
-          <t>zetaglobal.net, 808, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B71" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C71" s="4" t="inlineStr">
-        <is>
-          <t>video.unrulymedia.com, 2099898025, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B72" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C72" s="4" t="inlineStr">
-        <is>
-          <t>sharethrough.com, 4880, RESELLER, d53b998a7bd4ecd2</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B73" s="4" t="inlineStr">
-        <is>
-          <t>#VGI CTV/Verve:</t>
-        </is>
-      </c>
-      <c r="C73" s="4" t="inlineStr">
-        <is>
-          <t>smartadserver.com, 4199, RESELLER, 060d053dcf45cbf3</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B74" s="4" t="inlineStr">
-        <is>
-          <t>#Gateway</t>
-        </is>
-      </c>
-      <c r="C74" s="4" t="inlineStr">
-        <is>
-          <t>dauup.com, 44344, DIRECT, 4daba13e2b0dfd92</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B75" s="4" t="inlineStr">
-        <is>
-          <t>#Gateway</t>
-        </is>
-      </c>
-      <c r="C75" s="4" t="inlineStr">
-        <is>
-          <t>smartadserver.com, 5924, RESELLER, 060d053dcf45cbf3</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B76" s="4" t="inlineStr">
-        <is>
-          <t>#Gateway</t>
-        </is>
-      </c>
-      <c r="C76" s="4" t="inlineStr">
-        <is>
-          <t>video.unrulymedia.com, 389912353, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B77" s="4" t="inlineStr">
-        <is>
-          <t>#Gateway</t>
-        </is>
-      </c>
-      <c r="C77" s="4" t="inlineStr">
-        <is>
-          <t>video.unrulymedia.com, 2979066401945419350, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B78" s="4" t="inlineStr">
-        <is>
-          <t>#Gateway</t>
-        </is>
-      </c>
-      <c r="C78" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 545588-r-524565, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B79" s="4" t="inlineStr">
-        <is>
-          <t>#Gateway</t>
-        </is>
-      </c>
-      <c r="C79" s="4" t="inlineStr">
-        <is>
-          <t>freewheel.tv, 545588-r-523319, RESELLER</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B80" s="4" t="inlineStr">
-        <is>
-          <t>#Gateway</t>
-        </is>
-      </c>
-      <c r="C80" s="4" t="inlineStr">
-        <is>
-          <t>consumable.com, 2001664, RESELLER, aefcd3d2f45b5070</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -35313,7 +34314,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-21 11:46 UTC</t>
+          <t>2026-06-22 14:42 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -35338,7 +34339,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-21 11:46 UTC</t>
+          <t>2026-06-22 14:42 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -35363,7 +34364,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-21 11:46 UTC</t>
+          <t>2026-06-22 14:42 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -35388,7 +34389,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-21 11:46 UTC</t>
+          <t>2026-06-22 14:42 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -35413,7 +34414,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-21 11:46 UTC</t>
+          <t>2026-06-22 14:42 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -35438,7 +34439,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-21 11:46 UTC</t>
+          <t>2026-06-22 14:42 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -35463,7 +34464,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-21 11:46 UTC</t>
+          <t>2026-06-22 14:42 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -35488,7 +34489,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-21 11:46 UTC</t>
+          <t>2026-06-22 14:42 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -35513,7 +34514,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-21 11:46 UTC</t>
+          <t>2026-06-22 14:42 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -35538,7 +34539,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-21 11:46 UTC</t>
+          <t>2026-06-22 14:42 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -35547,6 +34548,76 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/22192.1b405875efa9f607de5b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a945bdfdb5cf49bf4266.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.9e173e0a67ac7ac4a279.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f98cff8f6cbd7006bc03.js"&gt;&lt;/script&gt;&lt;link href="/style/css/22192.3628d6adb3505d1a8000.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/22192.1b405875efa9f607de5b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a945bdfdb5cf49bf4266.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.9e173e0a67ac7ac4a279.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9803df3f645dd7eb7a3c.js"&gt;&lt;/script&gt;&lt;link href="/style/css/22192.3628d6adb3505d1a8000.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.38828fbbf387038ed84a.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -45214,7 +44285,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -45247,29 +44318,1338 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>(no section)</t>
+          <t>#VGI CTV/Verve:</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/22192.1b405875efa9f607de5b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a945bdfdb5cf49bf4266.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.9e173e0a67ac7ac4a279.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9803df3f645dd7eb7a3c.js"&gt;&lt;/script&gt;&lt;link href="/style/css/22192.3628d6adb3505d1a8000.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.38828fbbf387038ed84a.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>conversantmedia.com, 101216, RESELLER, 03113cd04947736d</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59407.c03a2b27cbc32f68c08e.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.3db9da783e2d3d839bd7.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.547e0e079804993d5940.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.53f466e4f012652d8137.js"&gt;&lt;/script&gt;&lt;link href="/style/css/59407.3e77c98aa45f5cb88e2d.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.38828fbbf387038ed84a.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>inmobi.com, 55049d2e109d4ac1820ca1432dda4e13, RESELLER, 83e75a7ae333ca9d</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>intenze.co, 200202, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>onlinemediasolutions.com, 20480, RESELLER, b3868b187e4b6402</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>admixer.net, a4fc102e-449c-483d-bdf8-b2a476a3f3bd, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>blasto.ai, 101, RESELLER, 7e936b1feafdaa61</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>advangelists.com, 9766527f2b5d3e95d4a733fcfb77bd7e, RESELLER, 60d26397ec060f98</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>app-stock.com, 343264, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>pubmatic.com, 161802, RESELLER, 5d62403b186f2ace</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>pubmatic.com, 164126, RESELLER, 5d62403b186f2ace</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>risecodes.com, 688215d1f9acce0001954fb1, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>selectmedia.asia, 645b5a31e427dc0a87095fc5, RESELLER, e365c871a27c655d</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>bematterfull.com, 92134446122, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>smartyads.com, 300019, RESELLER, fd2bde0ff2e62c5d</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>tredio.io, 357a6fdf7642bf815a88822c447d9dc436970, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>conversantmedia.com, 100364, RESELLER, 03113cd04947736d</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>boldcollective.co, 778226, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>lijit.com, 509976, RESELLER, fafdf38b16bf6b2b</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>brightmountainmedia.com, 268679, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>bold-win.com, 1104, RESELLER, 71746737d0bab951</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>tviq.io, 2116, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>lunamedia.io, d5b7a3e0bf7575046765e5c639e98ab0, RESELLER, 524ecb396915caaf</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 534990-r-524565, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 534990-r-523319, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>pgamssp.com, 690a2e9d27800cf3f809f319, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>pubmatic.com, 166643, RESELLER, 5d62403b186f2ace</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, sg1256512, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 535662-r-523319, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>zmaticoo.com, 5135985, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>x.adprime.com, AJxF6R99a9M6CaTvK, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>zetaglobal.net, 748, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>telaria.com, wixu4-vssbd, RESELLER, 1a4e959a1b50034a</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>tremorhub.com, wixu4-vssbd, RESELLER, 1a4e959a1b50034a</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>adipolo.com, 102032, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>appnexus.com, 16912, RESELLER, f5ab79cb980f11d1</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>improvedigital.com, 2836, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>supply.colossusssp.com, 892, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>pgamssp.com, 69a5d5c4d1f5f685e7085234, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>videoheroes.tv, 212459, RESELLER, 064bc410192443d8</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>sharethrough.com, f0oQSO2J, RESELLER, d53b998a7bd4ecd2</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 534605-r-524565, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>media.net, 8CU76542S, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>video.unrulymedia.com, 2099898025, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>zetaglobal.net, 642, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>improvedigital.com, 2853, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>pubmatic.com, 162588, RESELLER, 5d62403b186f2ace</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>pubmatic.com, 167844, RESELLER, 5d62403b186f2ace</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>rubiconproject.com, 27386, RESELLER, 0bfd66d529a55807</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>lijit.com, 587508, RESELLER, fafdf38b16bf6b2b</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>bidmachine.io, 1490, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>x.adprime.com, AJxF6R109a9M6CaTvK, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>152media.info, 152M1197, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>sharethrough.com, vQMCuYXA, RESELLER, d53b998a7bd4ecd2</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>smartbid.ai, SMB60005, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>lijit.com, 512908, RESELLER, fafdf38b16bf6b2b</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>rubiconproject.com, 24448, RESELLER, 0bfd66d529a55807</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>video.unrulymedia.com, 2613193077, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, sg1256366, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>lijit.com, 383910, RESELLER, fafdf38b16bf6b2b #SOVRN</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>rhebus.works, 1500765024, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>pubmatic.com, 167263, RESELLER,</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 535659-r-524565, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>smartadserver.com, 4210, RESELLER, 060d053dcf45cbf3</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>smartstream.tv, 679, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>smaato.com, 1100050739, RESELLER, 07bcf65f187117b4</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>appnexus.com, 13709, RESELLER, f5ab79cb980f11d1</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 534605-r-524565, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>media.net, 8CU76542S, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>zetaglobal.net, 808, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>video.unrulymedia.com, 2099898025, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>sharethrough.com, 4880, RESELLER, d53b998a7bd4ecd2</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>#VGI CTV/Verve:</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>smartadserver.com, 4199, RESELLER, 060d053dcf45cbf3</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>#Gateway</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>dauup.com, 44344, DIRECT, 4daba13e2b0dfd92</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>#Gateway</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>smartadserver.com, 5924, RESELLER, 060d053dcf45cbf3</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>#Gateway</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>video.unrulymedia.com, 389912353, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>#Gateway</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>video.unrulymedia.com, 2979066401945419350, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>#Gateway</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 545588-r-524565, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>#Gateway</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>freewheel.tv, 545588-r-523319, RESELLER</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>#Gateway</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>consumable.com, 2001664, RESELLER, aefcd3d2f45b5070</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-23
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H841"/>
+  <dimension ref="A1:H851"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -32869,6 +32869,386 @@
         </is>
       </c>
       <c r="H841" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="842" ht="15" customHeight="1">
+      <c r="A842" t="inlineStr">
+        <is>
+          <t>2026-06-23 12:08 UTC</t>
+        </is>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D842" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E842" t="n">
+        <v>0</v>
+      </c>
+      <c r="F842" t="n">
+        <v>0</v>
+      </c>
+      <c r="G842" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H842" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="843" ht="15" customHeight="1">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>2026-06-23 12:08 UTC</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D843" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E843" t="n">
+        <v>0</v>
+      </c>
+      <c r="F843" t="n">
+        <v>0</v>
+      </c>
+      <c r="G843" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H843" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="844" ht="15" customHeight="1">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>2026-06-23 12:08 UTC</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D844" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E844" t="n">
+        <v>0</v>
+      </c>
+      <c r="F844" t="n">
+        <v>0</v>
+      </c>
+      <c r="G844" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H844" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="845" ht="15" customHeight="1">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>2026-06-23 12:08 UTC</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D845" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E845" t="n">
+        <v>0</v>
+      </c>
+      <c r="F845" t="n">
+        <v>0</v>
+      </c>
+      <c r="G845" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H845" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="846" ht="15" customHeight="1">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>2026-06-23 12:08 UTC</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D846" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E846" t="n">
+        <v>0</v>
+      </c>
+      <c r="F846" t="n">
+        <v>0</v>
+      </c>
+      <c r="G846" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H846" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="847" ht="15" customHeight="1">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>2026-06-23 12:08 UTC</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D847" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E847" t="n">
+        <v>0</v>
+      </c>
+      <c r="F847" t="n">
+        <v>0</v>
+      </c>
+      <c r="G847" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H847" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="848" ht="15" customHeight="1">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>2026-06-23 12:08 UTC</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D848" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E848" t="n">
+        <v>0</v>
+      </c>
+      <c r="F848" t="n">
+        <v>0</v>
+      </c>
+      <c r="G848" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H848" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="849" ht="15" customHeight="1">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>2026-06-23 12:08 UTC</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D849" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E849" t="n">
+        <v>0</v>
+      </c>
+      <c r="F849" t="n">
+        <v>0</v>
+      </c>
+      <c r="G849" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H849" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="850" ht="15" customHeight="1">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>2026-06-23 12:08 UTC</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D850" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E850" t="n">
+        <v>0</v>
+      </c>
+      <c r="F850" t="n">
+        <v>0</v>
+      </c>
+      <c r="G850" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H850" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="851" ht="15" customHeight="1">
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>2026-06-23 12:08 UTC</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D851" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E851" t="n">
+        <v>0</v>
+      </c>
+      <c r="F851" t="n">
+        <v>0</v>
+      </c>
+      <c r="G851" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H851" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -34264,6 +34644,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/22192.1b405875efa9f607de5b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a945bdfdb5cf49bf4266.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.9e173e0a67ac7ac4a279.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f98cff8f6cbd7006bc03.js"&gt;&lt;/script&gt;&lt;link href="/style/css/22192.3628d6adb3505d1a8000.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/22192.1b405875efa9f607de5b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a945bdfdb5cf49bf4266.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.9e173e0a67ac7ac4a279.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9803df3f645dd7eb7a3c.js"&gt;&lt;/script&gt;&lt;link href="/style/css/22192.3628d6adb3505d1a8000.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.38828fbbf387038ed84a.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -34314,7 +34764,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-22 14:42 UTC</t>
+          <t>2026-06-23 12:08 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -34339,7 +34789,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-22 14:42 UTC</t>
+          <t>2026-06-23 12:08 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -34364,7 +34814,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-22 14:42 UTC</t>
+          <t>2026-06-23 12:08 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -34389,7 +34839,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-22 14:42 UTC</t>
+          <t>2026-06-23 12:08 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -34414,7 +34864,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-22 14:42 UTC</t>
+          <t>2026-06-23 12:08 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -34439,7 +34889,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-22 14:42 UTC</t>
+          <t>2026-06-23 12:08 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -34464,7 +34914,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-22 14:42 UTC</t>
+          <t>2026-06-23 12:08 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -34489,7 +34939,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-22 14:42 UTC</t>
+          <t>2026-06-23 12:08 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -34514,7 +34964,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-22 14:42 UTC</t>
+          <t>2026-06-23 12:08 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -34539,7 +34989,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-22 14:42 UTC</t>
+          <t>2026-06-23 12:08 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -34548,76 +34998,6 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/22192.1b405875efa9f607de5b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a945bdfdb5cf49bf4266.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.9e173e0a67ac7ac4a279.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f98cff8f6cbd7006bc03.js"&gt;&lt;/script&gt;&lt;link href="/style/css/22192.3628d6adb3505d1a8000.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/22192.1b405875efa9f607de5b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a945bdfdb5cf49bf4266.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.9e173e0a67ac7ac4a279.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9803df3f645dd7eb7a3c.js"&gt;&lt;/script&gt;&lt;link href="/style/css/22192.3628d6adb3505d1a8000.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.38828fbbf387038ed84a.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-24
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H851"/>
+  <dimension ref="A1:H861"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -33249,6 +33249,386 @@
         </is>
       </c>
       <c r="H851" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="852" ht="15" customHeight="1">
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D852" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E852" t="n">
+        <v>0</v>
+      </c>
+      <c r="F852" t="n">
+        <v>0</v>
+      </c>
+      <c r="G852" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H852" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="853" ht="15" customHeight="1">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D853" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E853" t="n">
+        <v>0</v>
+      </c>
+      <c r="F853" t="n">
+        <v>0</v>
+      </c>
+      <c r="G853" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H853" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="854" ht="15" customHeight="1">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D854" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E854" t="n">
+        <v>0</v>
+      </c>
+      <c r="F854" t="n">
+        <v>0</v>
+      </c>
+      <c r="G854" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H854" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="855" ht="15" customHeight="1">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D855" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E855" t="n">
+        <v>0</v>
+      </c>
+      <c r="F855" t="n">
+        <v>0</v>
+      </c>
+      <c r="G855" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H855" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="856" ht="15" customHeight="1">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D856" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E856" t="n">
+        <v>0</v>
+      </c>
+      <c r="F856" t="n">
+        <v>0</v>
+      </c>
+      <c r="G856" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H856" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="857" ht="15" customHeight="1">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D857" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E857" t="n">
+        <v>0</v>
+      </c>
+      <c r="F857" t="n">
+        <v>0</v>
+      </c>
+      <c r="G857" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H857" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="858" ht="15" customHeight="1">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D858" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E858" t="n">
+        <v>0</v>
+      </c>
+      <c r="F858" t="n">
+        <v>0</v>
+      </c>
+      <c r="G858" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H858" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="859" ht="15" customHeight="1">
+      <c r="A859" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D859" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E859" t="n">
+        <v>0</v>
+      </c>
+      <c r="F859" t="n">
+        <v>0</v>
+      </c>
+      <c r="G859" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H859" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="860" ht="15" customHeight="1">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D860" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E860" t="n">
+        <v>0</v>
+      </c>
+      <c r="F860" t="n">
+        <v>0</v>
+      </c>
+      <c r="G860" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H860" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="861" ht="15" customHeight="1">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>2026-06-24 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D861" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E861" t="n">
+        <v>0</v>
+      </c>
+      <c r="F861" t="n">
+        <v>0</v>
+      </c>
+      <c r="G861" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H861" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -34764,7 +35144,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-23 12:08 UTC</t>
+          <t>2026-06-24 11:45 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -34789,7 +35169,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-23 12:08 UTC</t>
+          <t>2026-06-24 11:45 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -34814,7 +35194,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-23 12:08 UTC</t>
+          <t>2026-06-24 11:45 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -34839,7 +35219,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-23 12:08 UTC</t>
+          <t>2026-06-24 11:45 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -34864,7 +35244,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-23 12:08 UTC</t>
+          <t>2026-06-24 11:45 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -34889,7 +35269,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-23 12:08 UTC</t>
+          <t>2026-06-24 11:45 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -34914,7 +35294,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-23 12:08 UTC</t>
+          <t>2026-06-24 11:45 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -34939,7 +35319,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-23 12:08 UTC</t>
+          <t>2026-06-24 11:45 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -34964,7 +35344,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-23 12:08 UTC</t>
+          <t>2026-06-24 11:45 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -34989,7 +35369,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-23 12:08 UTC</t>
+          <t>2026-06-24 11:45 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-25
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H861"/>
+  <dimension ref="A1:H871"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -33629,6 +33629,386 @@
         </is>
       </c>
       <c r="H861" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="862" ht="15" customHeight="1">
+      <c r="A862" t="inlineStr">
+        <is>
+          <t>2026-06-25 11:40 UTC</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D862" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E862" t="n">
+        <v>0</v>
+      </c>
+      <c r="F862" t="n">
+        <v>0</v>
+      </c>
+      <c r="G862" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H862" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="863" ht="15" customHeight="1">
+      <c r="A863" t="inlineStr">
+        <is>
+          <t>2026-06-25 11:40 UTC</t>
+        </is>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D863" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E863" t="n">
+        <v>0</v>
+      </c>
+      <c r="F863" t="n">
+        <v>0</v>
+      </c>
+      <c r="G863" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H863" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="864" ht="15" customHeight="1">
+      <c r="A864" t="inlineStr">
+        <is>
+          <t>2026-06-25 11:40 UTC</t>
+        </is>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D864" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E864" t="n">
+        <v>0</v>
+      </c>
+      <c r="F864" t="n">
+        <v>0</v>
+      </c>
+      <c r="G864" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H864" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="865" ht="15" customHeight="1">
+      <c r="A865" t="inlineStr">
+        <is>
+          <t>2026-06-25 11:40 UTC</t>
+        </is>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D865" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E865" t="n">
+        <v>0</v>
+      </c>
+      <c r="F865" t="n">
+        <v>0</v>
+      </c>
+      <c r="G865" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H865" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="866" ht="15" customHeight="1">
+      <c r="A866" t="inlineStr">
+        <is>
+          <t>2026-06-25 11:40 UTC</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D866" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E866" t="n">
+        <v>0</v>
+      </c>
+      <c r="F866" t="n">
+        <v>0</v>
+      </c>
+      <c r="G866" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H866" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="867" ht="15" customHeight="1">
+      <c r="A867" t="inlineStr">
+        <is>
+          <t>2026-06-25 11:40 UTC</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D867" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E867" t="n">
+        <v>0</v>
+      </c>
+      <c r="F867" t="n">
+        <v>0</v>
+      </c>
+      <c r="G867" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H867" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="868" ht="15" customHeight="1">
+      <c r="A868" t="inlineStr">
+        <is>
+          <t>2026-06-25 11:40 UTC</t>
+        </is>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D868" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E868" t="n">
+        <v>0</v>
+      </c>
+      <c r="F868" t="n">
+        <v>0</v>
+      </c>
+      <c r="G868" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H868" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="869" ht="15" customHeight="1">
+      <c r="A869" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-25 11:40 UTC</t>
+        </is>
+      </c>
+      <c r="B869" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C869" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D869" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E869" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F869" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G869" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/22192.1b405875efa9f607de5b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a945bdfdb5cf49bf4266.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.9e173e0a67ac7ac4a279.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f824f7f28e7e5e9a22c0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/22192.3628d6adb3505d1a8000.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H869" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/22192.1b405875efa9f607de5b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a945bdfdb5cf49bf4266.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.9e173e0a67ac7ac4a279.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f98cff8f6cbd7006bc03.js"&gt;&lt;/script&gt;&lt;link href="/style/css/22192.3628d6adb3505d1a8000.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="870" ht="15" customHeight="1">
+      <c r="A870" t="inlineStr">
+        <is>
+          <t>2026-06-25 11:40 UTC</t>
+        </is>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D870" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E870" t="n">
+        <v>0</v>
+      </c>
+      <c r="F870" t="n">
+        <v>0</v>
+      </c>
+      <c r="G870" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H870" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="871" ht="15" customHeight="1">
+      <c r="A871" t="inlineStr">
+        <is>
+          <t>2026-06-25 11:40 UTC</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D871" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E871" t="n">
+        <v>0</v>
+      </c>
+      <c r="F871" t="n">
+        <v>0</v>
+      </c>
+      <c r="G871" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H871" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -35024,76 +35404,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/22192.1b405875efa9f607de5b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a945bdfdb5cf49bf4266.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.9e173e0a67ac7ac4a279.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f98cff8f6cbd7006bc03.js"&gt;&lt;/script&gt;&lt;link href="/style/css/22192.3628d6adb3505d1a8000.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/22192.1b405875efa9f607de5b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a945bdfdb5cf49bf4266.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.9e173e0a67ac7ac4a279.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.9803df3f645dd7eb7a3c.js"&gt;&lt;/script&gt;&lt;link href="/style/css/22192.3628d6adb3505d1a8000.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.38828fbbf387038ed84a.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -35144,7 +35454,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-24 11:45 UTC</t>
+          <t>2026-06-25 11:40 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -35169,7 +35479,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-24 11:45 UTC</t>
+          <t>2026-06-25 11:40 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -35194,7 +35504,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-24 11:45 UTC</t>
+          <t>2026-06-25 11:40 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -35219,7 +35529,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-24 11:45 UTC</t>
+          <t>2026-06-25 11:40 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -35244,7 +35554,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-24 11:45 UTC</t>
+          <t>2026-06-25 11:40 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -35269,7 +35579,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-24 11:45 UTC</t>
+          <t>2026-06-25 11:40 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -35294,7 +35604,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-24 11:45 UTC</t>
+          <t>2026-06-25 11:40 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -35319,7 +35629,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-24 11:45 UTC</t>
+          <t>2026-06-25 11:40 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -35344,7 +35654,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-24 11:45 UTC</t>
+          <t>2026-06-25 11:40 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -35369,7 +35679,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-24 11:45 UTC</t>
+          <t>2026-06-25 11:40 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -35378,6 +35688,76 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/22192.1b405875efa9f607de5b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a945bdfdb5cf49bf4266.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.9e173e0a67ac7ac4a279.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f824f7f28e7e5e9a22c0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/22192.3628d6adb3505d1a8000.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/22192.1b405875efa9f607de5b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a945bdfdb5cf49bf4266.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.9e173e0a67ac7ac4a279.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f98cff8f6cbd7006bc03.js"&gt;&lt;/script&gt;&lt;link href="/style/css/22192.3628d6adb3505d1a8000.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-26
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H871"/>
+  <dimension ref="A1:H881"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -34009,6 +34009,386 @@
         </is>
       </c>
       <c r="H871" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="872" ht="15" customHeight="1">
+      <c r="A872" t="inlineStr">
+        <is>
+          <t>2026-06-26 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D872" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E872" t="n">
+        <v>0</v>
+      </c>
+      <c r="F872" t="n">
+        <v>0</v>
+      </c>
+      <c r="G872" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H872" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="873" ht="15" customHeight="1">
+      <c r="A873" t="inlineStr">
+        <is>
+          <t>2026-06-26 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D873" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E873" t="n">
+        <v>0</v>
+      </c>
+      <c r="F873" t="n">
+        <v>0</v>
+      </c>
+      <c r="G873" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H873" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="874" ht="15" customHeight="1">
+      <c r="A874" t="inlineStr">
+        <is>
+          <t>2026-06-26 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D874" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E874" t="n">
+        <v>0</v>
+      </c>
+      <c r="F874" t="n">
+        <v>0</v>
+      </c>
+      <c r="G874" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H874" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="875" ht="15" customHeight="1">
+      <c r="A875" t="inlineStr">
+        <is>
+          <t>2026-06-26 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D875" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E875" t="n">
+        <v>0</v>
+      </c>
+      <c r="F875" t="n">
+        <v>0</v>
+      </c>
+      <c r="G875" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H875" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="876" ht="15" customHeight="1">
+      <c r="A876" t="inlineStr">
+        <is>
+          <t>2026-06-26 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D876" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E876" t="n">
+        <v>0</v>
+      </c>
+      <c r="F876" t="n">
+        <v>0</v>
+      </c>
+      <c r="G876" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H876" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="877" ht="15" customHeight="1">
+      <c r="A877" t="inlineStr">
+        <is>
+          <t>2026-06-26 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D877" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E877" t="n">
+        <v>0</v>
+      </c>
+      <c r="F877" t="n">
+        <v>0</v>
+      </c>
+      <c r="G877" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H877" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="878" ht="15" customHeight="1">
+      <c r="A878" t="inlineStr">
+        <is>
+          <t>2026-06-26 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D878" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E878" t="n">
+        <v>0</v>
+      </c>
+      <c r="F878" t="n">
+        <v>0</v>
+      </c>
+      <c r="G878" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H878" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="879" ht="15" customHeight="1">
+      <c r="A879" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-26 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B879" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C879" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D879" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E879" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F879" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G879" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.911467eae813e10303d8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.60434250cc98abda43a3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.534b6cd5ad061662bef3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.e30d343e9c23810e140a.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H879" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/22192.1b405875efa9f607de5b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a945bdfdb5cf49bf4266.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.9e173e0a67ac7ac4a279.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f824f7f28e7e5e9a22c0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/22192.3628d6adb3505d1a8000.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="880" ht="15" customHeight="1">
+      <c r="A880" t="inlineStr">
+        <is>
+          <t>2026-06-26 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D880" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E880" t="n">
+        <v>0</v>
+      </c>
+      <c r="F880" t="n">
+        <v>0</v>
+      </c>
+      <c r="G880" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H880" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="881" ht="15" customHeight="1">
+      <c r="A881" t="inlineStr">
+        <is>
+          <t>2026-06-26 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D881" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E881" t="n">
+        <v>0</v>
+      </c>
+      <c r="F881" t="n">
+        <v>0</v>
+      </c>
+      <c r="G881" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H881" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -35454,7 +35834,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-25 11:40 UTC</t>
+          <t>2026-06-26 11:45 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -35479,7 +35859,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-25 11:40 UTC</t>
+          <t>2026-06-26 11:45 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -35504,7 +35884,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-25 11:40 UTC</t>
+          <t>2026-06-26 11:45 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -35529,7 +35909,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-25 11:40 UTC</t>
+          <t>2026-06-26 11:45 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -35554,7 +35934,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-25 11:40 UTC</t>
+          <t>2026-06-26 11:45 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -35579,7 +35959,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-25 11:40 UTC</t>
+          <t>2026-06-26 11:45 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -35604,7 +35984,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-25 11:40 UTC</t>
+          <t>2026-06-26 11:45 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -35629,7 +36009,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-25 11:40 UTC</t>
+          <t>2026-06-26 11:45 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -35654,7 +36034,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-25 11:40 UTC</t>
+          <t>2026-06-26 11:45 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -35679,7 +36059,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-25 11:40 UTC</t>
+          <t>2026-06-26 11:45 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -35740,7 +36120,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/22192.1b405875efa9f607de5b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a945bdfdb5cf49bf4266.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.9e173e0a67ac7ac4a279.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f824f7f28e7e5e9a22c0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/22192.3628d6adb3505d1a8000.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.911467eae813e10303d8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.60434250cc98abda43a3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.534b6cd5ad061662bef3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.e30d343e9c23810e140a.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -35757,7 +36137,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/22192.1b405875efa9f607de5b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a945bdfdb5cf49bf4266.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.9e173e0a67ac7ac4a279.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f98cff8f6cbd7006bc03.js"&gt;&lt;/script&gt;&lt;link href="/style/css/22192.3628d6adb3505d1a8000.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/22192.1b405875efa9f607de5b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a945bdfdb5cf49bf4266.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.9e173e0a67ac7ac4a279.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f824f7f28e7e5e9a22c0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/22192.3628d6adb3505d1a8000.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-27
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H881"/>
+  <dimension ref="A1:H891"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -34389,6 +34389,386 @@
         </is>
       </c>
       <c r="H881" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="882" ht="15" customHeight="1">
+      <c r="A882" t="inlineStr">
+        <is>
+          <t>2026-06-27 10:58 UTC</t>
+        </is>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C882" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D882" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E882" t="n">
+        <v>0</v>
+      </c>
+      <c r="F882" t="n">
+        <v>0</v>
+      </c>
+      <c r="G882" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H882" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="883" ht="15" customHeight="1">
+      <c r="A883" t="inlineStr">
+        <is>
+          <t>2026-06-27 10:58 UTC</t>
+        </is>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C883" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D883" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E883" t="n">
+        <v>0</v>
+      </c>
+      <c r="F883" t="n">
+        <v>0</v>
+      </c>
+      <c r="G883" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H883" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="884" ht="15" customHeight="1">
+      <c r="A884" t="inlineStr">
+        <is>
+          <t>2026-06-27 10:58 UTC</t>
+        </is>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C884" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D884" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E884" t="n">
+        <v>0</v>
+      </c>
+      <c r="F884" t="n">
+        <v>0</v>
+      </c>
+      <c r="G884" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H884" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="885" ht="15" customHeight="1">
+      <c r="A885" t="inlineStr">
+        <is>
+          <t>2026-06-27 10:58 UTC</t>
+        </is>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C885" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D885" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E885" t="n">
+        <v>0</v>
+      </c>
+      <c r="F885" t="n">
+        <v>0</v>
+      </c>
+      <c r="G885" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H885" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="886" ht="15" customHeight="1">
+      <c r="A886" t="inlineStr">
+        <is>
+          <t>2026-06-27 10:58 UTC</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D886" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E886" t="n">
+        <v>0</v>
+      </c>
+      <c r="F886" t="n">
+        <v>0</v>
+      </c>
+      <c r="G886" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H886" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="887" ht="15" customHeight="1">
+      <c r="A887" t="inlineStr">
+        <is>
+          <t>2026-06-27 10:58 UTC</t>
+        </is>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C887" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D887" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E887" t="n">
+        <v>0</v>
+      </c>
+      <c r="F887" t="n">
+        <v>0</v>
+      </c>
+      <c r="G887" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H887" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="888" ht="15" customHeight="1">
+      <c r="A888" t="inlineStr">
+        <is>
+          <t>2026-06-27 10:58 UTC</t>
+        </is>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C888" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D888" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E888" t="n">
+        <v>0</v>
+      </c>
+      <c r="F888" t="n">
+        <v>0</v>
+      </c>
+      <c r="G888" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H888" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="889" ht="15" customHeight="1">
+      <c r="A889" t="inlineStr">
+        <is>
+          <t>2026-06-27 10:58 UTC</t>
+        </is>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C889" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D889" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E889" t="n">
+        <v>0</v>
+      </c>
+      <c r="F889" t="n">
+        <v>0</v>
+      </c>
+      <c r="G889" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H889" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="890" ht="15" customHeight="1">
+      <c r="A890" t="inlineStr">
+        <is>
+          <t>2026-06-27 10:58 UTC</t>
+        </is>
+      </c>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C890" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D890" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E890" t="n">
+        <v>0</v>
+      </c>
+      <c r="F890" t="n">
+        <v>0</v>
+      </c>
+      <c r="G890" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H890" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="891" ht="15" customHeight="1">
+      <c r="A891" t="inlineStr">
+        <is>
+          <t>2026-06-27 10:58 UTC</t>
+        </is>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C891" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D891" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E891" t="n">
+        <v>0</v>
+      </c>
+      <c r="F891" t="n">
+        <v>0</v>
+      </c>
+      <c r="G891" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H891" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -35784,6 +36164,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.911467eae813e10303d8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.60434250cc98abda43a3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.534b6cd5ad061662bef3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.e30d343e9c23810e140a.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/22192.1b405875efa9f607de5b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a945bdfdb5cf49bf4266.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.9e173e0a67ac7ac4a279.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f824f7f28e7e5e9a22c0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/22192.3628d6adb3505d1a8000.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -35834,7 +36284,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-26 11:45 UTC</t>
+          <t>2026-06-27 10:58 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -35859,7 +36309,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-26 11:45 UTC</t>
+          <t>2026-06-27 10:58 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -35884,7 +36334,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-26 11:45 UTC</t>
+          <t>2026-06-27 10:58 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -35909,7 +36359,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-26 11:45 UTC</t>
+          <t>2026-06-27 10:58 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -35934,7 +36384,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-26 11:45 UTC</t>
+          <t>2026-06-27 10:58 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -35959,7 +36409,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-26 11:45 UTC</t>
+          <t>2026-06-27 10:58 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -35984,7 +36434,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-26 11:45 UTC</t>
+          <t>2026-06-27 10:58 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -36009,7 +36459,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-26 11:45 UTC</t>
+          <t>2026-06-27 10:58 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -36034,7 +36484,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-26 11:45 UTC</t>
+          <t>2026-06-27 10:58 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -36059,7 +36509,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-26 11:45 UTC</t>
+          <t>2026-06-27 10:58 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -36068,76 +36518,6 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.911467eae813e10303d8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.60434250cc98abda43a3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.534b6cd5ad061662bef3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.e30d343e9c23810e140a.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/22192.1b405875efa9f607de5b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a945bdfdb5cf49bf4266.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.9e173e0a67ac7ac4a279.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f824f7f28e7e5e9a22c0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/22192.3628d6adb3505d1a8000.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-28
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H891"/>
+  <dimension ref="A1:H901"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -34769,6 +34769,386 @@
         </is>
       </c>
       <c r="H891" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="892" ht="15" customHeight="1">
+      <c r="A892" t="inlineStr">
+        <is>
+          <t>2026-06-28 11:08 UTC</t>
+        </is>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D892" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E892" t="n">
+        <v>0</v>
+      </c>
+      <c r="F892" t="n">
+        <v>0</v>
+      </c>
+      <c r="G892" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H892" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="893" ht="15" customHeight="1">
+      <c r="A893" t="inlineStr">
+        <is>
+          <t>2026-06-28 11:08 UTC</t>
+        </is>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D893" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E893" t="n">
+        <v>0</v>
+      </c>
+      <c r="F893" t="n">
+        <v>0</v>
+      </c>
+      <c r="G893" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H893" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="894" ht="15" customHeight="1">
+      <c r="A894" t="inlineStr">
+        <is>
+          <t>2026-06-28 11:08 UTC</t>
+        </is>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D894" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E894" t="n">
+        <v>0</v>
+      </c>
+      <c r="F894" t="n">
+        <v>0</v>
+      </c>
+      <c r="G894" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H894" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="895" ht="15" customHeight="1">
+      <c r="A895" t="inlineStr">
+        <is>
+          <t>2026-06-28 11:08 UTC</t>
+        </is>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D895" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E895" t="n">
+        <v>0</v>
+      </c>
+      <c r="F895" t="n">
+        <v>0</v>
+      </c>
+      <c r="G895" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H895" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="896" ht="15" customHeight="1">
+      <c r="A896" t="inlineStr">
+        <is>
+          <t>2026-06-28 11:08 UTC</t>
+        </is>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D896" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E896" t="n">
+        <v>0</v>
+      </c>
+      <c r="F896" t="n">
+        <v>0</v>
+      </c>
+      <c r="G896" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H896" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="897" ht="15" customHeight="1">
+      <c r="A897" t="inlineStr">
+        <is>
+          <t>2026-06-28 11:08 UTC</t>
+        </is>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D897" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E897" t="n">
+        <v>0</v>
+      </c>
+      <c r="F897" t="n">
+        <v>0</v>
+      </c>
+      <c r="G897" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H897" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="898" ht="15" customHeight="1">
+      <c r="A898" t="inlineStr">
+        <is>
+          <t>2026-06-28 11:08 UTC</t>
+        </is>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D898" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E898" t="n">
+        <v>0</v>
+      </c>
+      <c r="F898" t="n">
+        <v>0</v>
+      </c>
+      <c r="G898" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H898" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="899" ht="15" customHeight="1">
+      <c r="A899" t="inlineStr">
+        <is>
+          <t>2026-06-28 11:08 UTC</t>
+        </is>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D899" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E899" t="n">
+        <v>0</v>
+      </c>
+      <c r="F899" t="n">
+        <v>0</v>
+      </c>
+      <c r="G899" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H899" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="900" ht="15" customHeight="1">
+      <c r="A900" t="inlineStr">
+        <is>
+          <t>2026-06-28 11:08 UTC</t>
+        </is>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D900" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E900" t="n">
+        <v>0</v>
+      </c>
+      <c r="F900" t="n">
+        <v>0</v>
+      </c>
+      <c r="G900" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H900" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="901" ht="15" customHeight="1">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>2026-06-28 11:08 UTC</t>
+        </is>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D901" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E901" t="n">
+        <v>0</v>
+      </c>
+      <c r="F901" t="n">
+        <v>0</v>
+      </c>
+      <c r="G901" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H901" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -36284,7 +36664,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-27 10:58 UTC</t>
+          <t>2026-06-28 11:08 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -36309,7 +36689,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-27 10:58 UTC</t>
+          <t>2026-06-28 11:08 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -36334,7 +36714,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-27 10:58 UTC</t>
+          <t>2026-06-28 11:08 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -36359,7 +36739,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-27 10:58 UTC</t>
+          <t>2026-06-28 11:08 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -36384,7 +36764,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-27 10:58 UTC</t>
+          <t>2026-06-28 11:08 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -36409,7 +36789,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-27 10:58 UTC</t>
+          <t>2026-06-28 11:08 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -36434,7 +36814,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-27 10:58 UTC</t>
+          <t>2026-06-28 11:08 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -36459,7 +36839,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-27 10:58 UTC</t>
+          <t>2026-06-28 11:08 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -36484,7 +36864,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-27 10:58 UTC</t>
+          <t>2026-06-28 11:08 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -36509,7 +36889,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-27 10:58 UTC</t>
+          <t>2026-06-28 11:08 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-29
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H901"/>
+  <dimension ref="A1:H911"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -35149,6 +35149,386 @@
         </is>
       </c>
       <c r="H901" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="902" ht="15" customHeight="1">
+      <c r="A902" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:08 UTC</t>
+        </is>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D902" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E902" t="n">
+        <v>0</v>
+      </c>
+      <c r="F902" t="n">
+        <v>0</v>
+      </c>
+      <c r="G902" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H902" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="903" ht="15" customHeight="1">
+      <c r="A903" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:08 UTC</t>
+        </is>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C903" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D903" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E903" t="n">
+        <v>0</v>
+      </c>
+      <c r="F903" t="n">
+        <v>0</v>
+      </c>
+      <c r="G903" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H903" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="904" ht="15" customHeight="1">
+      <c r="A904" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:08 UTC</t>
+        </is>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D904" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E904" t="n">
+        <v>0</v>
+      </c>
+      <c r="F904" t="n">
+        <v>0</v>
+      </c>
+      <c r="G904" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H904" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="905" ht="15" customHeight="1">
+      <c r="A905" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:08 UTC</t>
+        </is>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D905" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E905" t="n">
+        <v>0</v>
+      </c>
+      <c r="F905" t="n">
+        <v>0</v>
+      </c>
+      <c r="G905" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H905" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="906" ht="15" customHeight="1">
+      <c r="A906" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:08 UTC</t>
+        </is>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D906" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E906" t="n">
+        <v>0</v>
+      </c>
+      <c r="F906" t="n">
+        <v>0</v>
+      </c>
+      <c r="G906" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H906" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="907" ht="15" customHeight="1">
+      <c r="A907" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:08 UTC</t>
+        </is>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D907" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E907" t="n">
+        <v>0</v>
+      </c>
+      <c r="F907" t="n">
+        <v>0</v>
+      </c>
+      <c r="G907" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H907" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="908" ht="15" customHeight="1">
+      <c r="A908" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:08 UTC</t>
+        </is>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D908" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E908" t="n">
+        <v>0</v>
+      </c>
+      <c r="F908" t="n">
+        <v>0</v>
+      </c>
+      <c r="G908" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H908" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="909" ht="15" customHeight="1">
+      <c r="A909" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:08 UTC</t>
+        </is>
+      </c>
+      <c r="B909" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C909" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D909" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E909" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F909" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G909" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.911467eae813e10303d8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.60434250cc98abda43a3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.534b6cd5ad061662bef3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.aaac70ed2c864a7913f3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H909" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.911467eae813e10303d8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.60434250cc98abda43a3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.534b6cd5ad061662bef3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.e30d343e9c23810e140a.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="910" ht="15" customHeight="1">
+      <c r="A910" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:08 UTC</t>
+        </is>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C910" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D910" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E910" t="n">
+        <v>0</v>
+      </c>
+      <c r="F910" t="n">
+        <v>0</v>
+      </c>
+      <c r="G910" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H910" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="911" ht="15" customHeight="1">
+      <c r="A911" t="inlineStr">
+        <is>
+          <t>2026-06-29 13:08 UTC</t>
+        </is>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D911" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E911" t="n">
+        <v>0</v>
+      </c>
+      <c r="F911" t="n">
+        <v>0</v>
+      </c>
+      <c r="G911" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H911" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -36544,76 +36924,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.911467eae813e10303d8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.60434250cc98abda43a3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.534b6cd5ad061662bef3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.e30d343e9c23810e140a.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/22192.1b405875efa9f607de5b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.6aed261317d2be1c4217.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.a945bdfdb5cf49bf4266.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.9e173e0a67ac7ac4a279.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.f824f7f28e7e5e9a22c0.js"&gt;&lt;/script&gt;&lt;link href="/style/css/22192.3628d6adb3505d1a8000.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -36664,7 +36974,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-28 11:08 UTC</t>
+          <t>2026-06-29 13:08 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -36689,7 +36999,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-28 11:08 UTC</t>
+          <t>2026-06-29 13:08 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -36714,7 +37024,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-28 11:08 UTC</t>
+          <t>2026-06-29 13:08 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -36739,7 +37049,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-28 11:08 UTC</t>
+          <t>2026-06-29 13:08 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -36764,7 +37074,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-28 11:08 UTC</t>
+          <t>2026-06-29 13:08 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -36789,7 +37099,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-28 11:08 UTC</t>
+          <t>2026-06-29 13:08 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -36814,7 +37124,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-28 11:08 UTC</t>
+          <t>2026-06-29 13:08 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -36839,7 +37149,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-28 11:08 UTC</t>
+          <t>2026-06-29 13:08 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -36864,7 +37174,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-28 11:08 UTC</t>
+          <t>2026-06-29 13:08 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -36889,7 +37199,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-28 11:08 UTC</t>
+          <t>2026-06-29 13:08 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -36898,6 +37208,76 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.911467eae813e10303d8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.60434250cc98abda43a3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.534b6cd5ad061662bef3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.aaac70ed2c864a7913f3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.911467eae813e10303d8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.60434250cc98abda43a3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.534b6cd5ad061662bef3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.e30d343e9c23810e140a.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-06-30
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H911"/>
+  <dimension ref="A1:H921"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -35529,6 +35529,386 @@
         </is>
       </c>
       <c r="H911" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="912" ht="15" customHeight="1">
+      <c r="A912" t="inlineStr">
+        <is>
+          <t>2026-06-30 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C912" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D912" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E912" t="n">
+        <v>0</v>
+      </c>
+      <c r="F912" t="n">
+        <v>0</v>
+      </c>
+      <c r="G912" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H912" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="913" ht="15" customHeight="1">
+      <c r="A913" t="inlineStr">
+        <is>
+          <t>2026-06-30 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C913" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D913" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E913" t="n">
+        <v>0</v>
+      </c>
+      <c r="F913" t="n">
+        <v>0</v>
+      </c>
+      <c r="G913" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H913" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="914" ht="15" customHeight="1">
+      <c r="A914" t="inlineStr">
+        <is>
+          <t>2026-06-30 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C914" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D914" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E914" t="n">
+        <v>0</v>
+      </c>
+      <c r="F914" t="n">
+        <v>0</v>
+      </c>
+      <c r="G914" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H914" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="915" ht="15" customHeight="1">
+      <c r="A915" t="inlineStr">
+        <is>
+          <t>2026-06-30 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C915" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D915" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E915" t="n">
+        <v>0</v>
+      </c>
+      <c r="F915" t="n">
+        <v>0</v>
+      </c>
+      <c r="G915" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H915" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="916" ht="15" customHeight="1">
+      <c r="A916" t="inlineStr">
+        <is>
+          <t>2026-06-30 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C916" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D916" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E916" t="n">
+        <v>0</v>
+      </c>
+      <c r="F916" t="n">
+        <v>0</v>
+      </c>
+      <c r="G916" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H916" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="917" ht="15" customHeight="1">
+      <c r="A917" t="inlineStr">
+        <is>
+          <t>2026-06-30 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C917" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D917" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E917" t="n">
+        <v>0</v>
+      </c>
+      <c r="F917" t="n">
+        <v>0</v>
+      </c>
+      <c r="G917" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H917" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="918" ht="15" customHeight="1">
+      <c r="A918" t="inlineStr">
+        <is>
+          <t>2026-06-30 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C918" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D918" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E918" t="n">
+        <v>0</v>
+      </c>
+      <c r="F918" t="n">
+        <v>0</v>
+      </c>
+      <c r="G918" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H918" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="919" ht="15" customHeight="1">
+      <c r="A919" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-30 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B919" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C919" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D919" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E919" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F919" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G919" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.4a9de14f82daebe19ae6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.60434250cc98abda43a3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/57207.a8e14565905c3fcc5021.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.7f8d7d452ea1a913637b.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/57207.61390cb7d67d935e7d20.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.67c16a0cc37f2e42c801.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H919" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.911467eae813e10303d8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.60434250cc98abda43a3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.534b6cd5ad061662bef3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.aaac70ed2c864a7913f3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="920" ht="15" customHeight="1">
+      <c r="A920" t="inlineStr">
+        <is>
+          <t>2026-06-30 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C920" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D920" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E920" t="n">
+        <v>0</v>
+      </c>
+      <c r="F920" t="n">
+        <v>0</v>
+      </c>
+      <c r="G920" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H920" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="921" ht="15" customHeight="1">
+      <c r="A921" t="inlineStr">
+        <is>
+          <t>2026-06-30 11:45 UTC</t>
+        </is>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C921" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D921" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E921" t="n">
+        <v>0</v>
+      </c>
+      <c r="F921" t="n">
+        <v>0</v>
+      </c>
+      <c r="G921" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H921" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -36974,7 +37354,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-29 13:08 UTC</t>
+          <t>2026-06-30 11:45 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -36999,7 +37379,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-29 13:08 UTC</t>
+          <t>2026-06-30 11:45 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -37024,7 +37404,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-29 13:08 UTC</t>
+          <t>2026-06-30 11:45 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -37049,7 +37429,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-29 13:08 UTC</t>
+          <t>2026-06-30 11:45 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -37074,7 +37454,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-29 13:08 UTC</t>
+          <t>2026-06-30 11:45 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -37099,7 +37479,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-29 13:08 UTC</t>
+          <t>2026-06-30 11:45 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -37124,7 +37504,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-29 13:08 UTC</t>
+          <t>2026-06-30 11:45 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -37149,7 +37529,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-29 13:08 UTC</t>
+          <t>2026-06-30 11:45 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -37174,7 +37554,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-29 13:08 UTC</t>
+          <t>2026-06-30 11:45 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -37199,7 +37579,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-29 13:08 UTC</t>
+          <t>2026-06-30 11:45 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -37260,7 +37640,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.911467eae813e10303d8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.60434250cc98abda43a3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.534b6cd5ad061662bef3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.aaac70ed2c864a7913f3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.4a9de14f82daebe19ae6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.60434250cc98abda43a3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/57207.a8e14565905c3fcc5021.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.7f8d7d452ea1a913637b.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/57207.61390cb7d67d935e7d20.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.67c16a0cc37f2e42c801.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -37277,7 +37657,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.911467eae813e10303d8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.60434250cc98abda43a3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.534b6cd5ad061662bef3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.e30d343e9c23810e140a.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.911467eae813e10303d8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.60434250cc98abda43a3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.534b6cd5ad061662bef3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.aaac70ed2c864a7913f3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-07-01
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H921"/>
+  <dimension ref="A1:H931"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -35909,6 +35909,386 @@
         </is>
       </c>
       <c r="H921" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="922" ht="15" customHeight="1">
+      <c r="A922" t="inlineStr">
+        <is>
+          <t>2026-07-01 12:09 UTC</t>
+        </is>
+      </c>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C922" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D922" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E922" t="n">
+        <v>0</v>
+      </c>
+      <c r="F922" t="n">
+        <v>0</v>
+      </c>
+      <c r="G922" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H922" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="923" ht="15" customHeight="1">
+      <c r="A923" t="inlineStr">
+        <is>
+          <t>2026-07-01 12:09 UTC</t>
+        </is>
+      </c>
+      <c r="B923" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C923" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D923" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E923" t="n">
+        <v>0</v>
+      </c>
+      <c r="F923" t="n">
+        <v>0</v>
+      </c>
+      <c r="G923" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H923" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="924" ht="15" customHeight="1">
+      <c r="A924" t="inlineStr">
+        <is>
+          <t>2026-07-01 12:09 UTC</t>
+        </is>
+      </c>
+      <c r="B924" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C924" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D924" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E924" t="n">
+        <v>0</v>
+      </c>
+      <c r="F924" t="n">
+        <v>0</v>
+      </c>
+      <c r="G924" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H924" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="925" ht="15" customHeight="1">
+      <c r="A925" t="inlineStr">
+        <is>
+          <t>2026-07-01 12:09 UTC</t>
+        </is>
+      </c>
+      <c r="B925" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C925" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D925" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E925" t="n">
+        <v>0</v>
+      </c>
+      <c r="F925" t="n">
+        <v>0</v>
+      </c>
+      <c r="G925" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H925" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="926" ht="15" customHeight="1">
+      <c r="A926" t="inlineStr">
+        <is>
+          <t>2026-07-01 12:09 UTC</t>
+        </is>
+      </c>
+      <c r="B926" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C926" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D926" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E926" t="n">
+        <v>0</v>
+      </c>
+      <c r="F926" t="n">
+        <v>0</v>
+      </c>
+      <c r="G926" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H926" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="927" ht="15" customHeight="1">
+      <c r="A927" t="inlineStr">
+        <is>
+          <t>2026-07-01 12:09 UTC</t>
+        </is>
+      </c>
+      <c r="B927" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C927" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D927" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E927" t="n">
+        <v>0</v>
+      </c>
+      <c r="F927" t="n">
+        <v>0</v>
+      </c>
+      <c r="G927" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H927" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="928" ht="15" customHeight="1">
+      <c r="A928" t="inlineStr">
+        <is>
+          <t>2026-07-01 12:09 UTC</t>
+        </is>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C928" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D928" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E928" t="n">
+        <v>0</v>
+      </c>
+      <c r="F928" t="n">
+        <v>0</v>
+      </c>
+      <c r="G928" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H928" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="929" ht="15" customHeight="1">
+      <c r="A929" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-01 12:09 UTC</t>
+        </is>
+      </c>
+      <c r="B929" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C929" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D929" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E929" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F929" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G929" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.94520e97b52408272a94.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.54b3b755601bffb8d823.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/57207.a570470b3d8f23de0626.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.fec4a7350f714d70d4f5.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/57207.61390cb7d67d935e7d20.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f70f4a8131c9282b753c.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H929" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.4a9de14f82daebe19ae6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.60434250cc98abda43a3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/57207.a8e14565905c3fcc5021.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.7f8d7d452ea1a913637b.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/57207.61390cb7d67d935e7d20.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.67c16a0cc37f2e42c801.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="930" ht="15" customHeight="1">
+      <c r="A930" t="inlineStr">
+        <is>
+          <t>2026-07-01 12:09 UTC</t>
+        </is>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C930" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D930" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E930" t="n">
+        <v>0</v>
+      </c>
+      <c r="F930" t="n">
+        <v>0</v>
+      </c>
+      <c r="G930" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H930" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="931" ht="15" customHeight="1">
+      <c r="A931" t="inlineStr">
+        <is>
+          <t>2026-07-01 12:09 UTC</t>
+        </is>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C931" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D931" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E931" t="n">
+        <v>0</v>
+      </c>
+      <c r="F931" t="n">
+        <v>0</v>
+      </c>
+      <c r="G931" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H931" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -37354,7 +37734,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-06-30 11:45 UTC</t>
+          <t>2026-07-01 12:09 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -37379,7 +37759,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-06-30 11:45 UTC</t>
+          <t>2026-07-01 12:09 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -37404,7 +37784,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-06-30 11:45 UTC</t>
+          <t>2026-07-01 12:09 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -37429,7 +37809,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-06-30 11:45 UTC</t>
+          <t>2026-07-01 12:09 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -37454,7 +37834,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-06-30 11:45 UTC</t>
+          <t>2026-07-01 12:09 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -37479,7 +37859,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-06-30 11:45 UTC</t>
+          <t>2026-07-01 12:09 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -37504,7 +37884,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-06-30 11:45 UTC</t>
+          <t>2026-07-01 12:09 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -37529,7 +37909,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-06-30 11:45 UTC</t>
+          <t>2026-07-01 12:09 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -37554,7 +37934,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-06-30 11:45 UTC</t>
+          <t>2026-07-01 12:09 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -37579,7 +37959,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-06-30 11:45 UTC</t>
+          <t>2026-07-01 12:09 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -37640,7 +38020,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.4a9de14f82daebe19ae6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.60434250cc98abda43a3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/57207.a8e14565905c3fcc5021.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.7f8d7d452ea1a913637b.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/57207.61390cb7d67d935e7d20.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.67c16a0cc37f2e42c801.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.94520e97b52408272a94.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.54b3b755601bffb8d823.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/57207.a570470b3d8f23de0626.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.fec4a7350f714d70d4f5.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/57207.61390cb7d67d935e7d20.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f70f4a8131c9282b753c.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -37657,7 +38037,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.911467eae813e10303d8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.60434250cc98abda43a3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/52293.534b6cd5ad061662bef3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.aaac70ed2c864a7913f3.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/52293.6e6b705f9bd11d2648b5.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.ec75406207693cc685e6.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.4a9de14f82daebe19ae6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.60434250cc98abda43a3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/57207.a8e14565905c3fcc5021.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.7f8d7d452ea1a913637b.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/57207.61390cb7d67d935e7d20.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.67c16a0cc37f2e42c801.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-07-02
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H931"/>
+  <dimension ref="A1:H941"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -36289,6 +36289,386 @@
         </is>
       </c>
       <c r="H931" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="932" ht="15" customHeight="1">
+      <c r="A932" t="inlineStr">
+        <is>
+          <t>2026-07-02 11:34 UTC</t>
+        </is>
+      </c>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C932" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D932" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E932" t="n">
+        <v>0</v>
+      </c>
+      <c r="F932" t="n">
+        <v>0</v>
+      </c>
+      <c r="G932" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H932" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="933" ht="15" customHeight="1">
+      <c r="A933" t="inlineStr">
+        <is>
+          <t>2026-07-02 11:34 UTC</t>
+        </is>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C933" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D933" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E933" t="n">
+        <v>0</v>
+      </c>
+      <c r="F933" t="n">
+        <v>0</v>
+      </c>
+      <c r="G933" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H933" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="934" ht="15" customHeight="1">
+      <c r="A934" t="inlineStr">
+        <is>
+          <t>2026-07-02 11:34 UTC</t>
+        </is>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C934" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D934" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E934" t="n">
+        <v>0</v>
+      </c>
+      <c r="F934" t="n">
+        <v>0</v>
+      </c>
+      <c r="G934" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H934" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="935" ht="15" customHeight="1">
+      <c r="A935" t="inlineStr">
+        <is>
+          <t>2026-07-02 11:34 UTC</t>
+        </is>
+      </c>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C935" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D935" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E935" t="n">
+        <v>0</v>
+      </c>
+      <c r="F935" t="n">
+        <v>0</v>
+      </c>
+      <c r="G935" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H935" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="936" ht="15" customHeight="1">
+      <c r="A936" t="inlineStr">
+        <is>
+          <t>2026-07-02 11:34 UTC</t>
+        </is>
+      </c>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C936" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D936" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E936" t="n">
+        <v>0</v>
+      </c>
+      <c r="F936" t="n">
+        <v>0</v>
+      </c>
+      <c r="G936" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H936" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="937" ht="15" customHeight="1">
+      <c r="A937" t="inlineStr">
+        <is>
+          <t>2026-07-02 11:34 UTC</t>
+        </is>
+      </c>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C937" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D937" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E937" t="n">
+        <v>0</v>
+      </c>
+      <c r="F937" t="n">
+        <v>0</v>
+      </c>
+      <c r="G937" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H937" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="938" ht="15" customHeight="1">
+      <c r="A938" t="inlineStr">
+        <is>
+          <t>2026-07-02 11:34 UTC</t>
+        </is>
+      </c>
+      <c r="B938" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C938" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D938" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E938" t="n">
+        <v>0</v>
+      </c>
+      <c r="F938" t="n">
+        <v>0</v>
+      </c>
+      <c r="G938" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H938" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="939" ht="15" customHeight="1">
+      <c r="A939" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02 11:34 UTC</t>
+        </is>
+      </c>
+      <c r="B939" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C939" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D939" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E939" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F939" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G939" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.94520e97b52408272a94.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.54b3b755601bffb8d823.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/57207.0b85d3b8da354f298333.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.db1b797cc6e6192822f2.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/57207.61390cb7d67d935e7d20.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.fabd73c4415a302aef05.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H939" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.94520e97b52408272a94.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.54b3b755601bffb8d823.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/57207.a570470b3d8f23de0626.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.fec4a7350f714d70d4f5.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/57207.61390cb7d67d935e7d20.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f70f4a8131c9282b753c.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="940" ht="15" customHeight="1">
+      <c r="A940" t="inlineStr">
+        <is>
+          <t>2026-07-02 11:34 UTC</t>
+        </is>
+      </c>
+      <c r="B940" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C940" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D940" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E940" t="n">
+        <v>0</v>
+      </c>
+      <c r="F940" t="n">
+        <v>0</v>
+      </c>
+      <c r="G940" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H940" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="941" ht="15" customHeight="1">
+      <c r="A941" t="inlineStr">
+        <is>
+          <t>2026-07-02 11:34 UTC</t>
+        </is>
+      </c>
+      <c r="B941" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C941" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D941" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E941" t="n">
+        <v>0</v>
+      </c>
+      <c r="F941" t="n">
+        <v>0</v>
+      </c>
+      <c r="G941" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H941" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -37734,7 +38114,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-07-01 12:09 UTC</t>
+          <t>2026-07-02 11:34 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -37759,7 +38139,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-07-01 12:09 UTC</t>
+          <t>2026-07-02 11:34 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -37784,7 +38164,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-07-01 12:09 UTC</t>
+          <t>2026-07-02 11:34 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -37809,7 +38189,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-07-01 12:09 UTC</t>
+          <t>2026-07-02 11:34 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -37834,7 +38214,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-07-01 12:09 UTC</t>
+          <t>2026-07-02 11:34 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -37859,7 +38239,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-07-01 12:09 UTC</t>
+          <t>2026-07-02 11:34 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -37884,7 +38264,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-01 12:09 UTC</t>
+          <t>2026-07-02 11:34 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -37909,7 +38289,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-07-01 12:09 UTC</t>
+          <t>2026-07-02 11:34 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -37934,7 +38314,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-07-01 12:09 UTC</t>
+          <t>2026-07-02 11:34 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -37959,7 +38339,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-07-01 12:09 UTC</t>
+          <t>2026-07-02 11:34 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -38020,7 +38400,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.94520e97b52408272a94.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.54b3b755601bffb8d823.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/57207.a570470b3d8f23de0626.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.fec4a7350f714d70d4f5.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/57207.61390cb7d67d935e7d20.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f70f4a8131c9282b753c.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.94520e97b52408272a94.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.54b3b755601bffb8d823.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/57207.0b85d3b8da354f298333.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.db1b797cc6e6192822f2.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/57207.61390cb7d67d935e7d20.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.fabd73c4415a302aef05.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -38037,7 +38417,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.4a9de14f82daebe19ae6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.60434250cc98abda43a3.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/57207.a8e14565905c3fcc5021.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.7f8d7d452ea1a913637b.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/57207.61390cb7d67d935e7d20.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.67c16a0cc37f2e42c801.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.94520e97b52408272a94.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.54b3b755601bffb8d823.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/57207.a570470b3d8f23de0626.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.fec4a7350f714d70d4f5.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/57207.61390cb7d67d935e7d20.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f70f4a8131c9282b753c.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-07-03
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H941"/>
+  <dimension ref="A1:H951"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -36669,6 +36669,386 @@
         </is>
       </c>
       <c r="H941" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="942" ht="15" customHeight="1">
+      <c r="A942" t="inlineStr">
+        <is>
+          <t>2026-07-03 11:33 UTC</t>
+        </is>
+      </c>
+      <c r="B942" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C942" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D942" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E942" t="n">
+        <v>0</v>
+      </c>
+      <c r="F942" t="n">
+        <v>0</v>
+      </c>
+      <c r="G942" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H942" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="943" ht="15" customHeight="1">
+      <c r="A943" t="inlineStr">
+        <is>
+          <t>2026-07-03 11:33 UTC</t>
+        </is>
+      </c>
+      <c r="B943" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C943" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D943" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E943" t="n">
+        <v>0</v>
+      </c>
+      <c r="F943" t="n">
+        <v>0</v>
+      </c>
+      <c r="G943" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H943" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="944" ht="15" customHeight="1">
+      <c r="A944" t="inlineStr">
+        <is>
+          <t>2026-07-03 11:33 UTC</t>
+        </is>
+      </c>
+      <c r="B944" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C944" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D944" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E944" t="n">
+        <v>0</v>
+      </c>
+      <c r="F944" t="n">
+        <v>0</v>
+      </c>
+      <c r="G944" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H944" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="945" ht="15" customHeight="1">
+      <c r="A945" t="inlineStr">
+        <is>
+          <t>2026-07-03 11:33 UTC</t>
+        </is>
+      </c>
+      <c r="B945" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C945" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D945" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E945" t="n">
+        <v>0</v>
+      </c>
+      <c r="F945" t="n">
+        <v>0</v>
+      </c>
+      <c r="G945" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H945" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="946" ht="15" customHeight="1">
+      <c r="A946" t="inlineStr">
+        <is>
+          <t>2026-07-03 11:33 UTC</t>
+        </is>
+      </c>
+      <c r="B946" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C946" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D946" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E946" t="n">
+        <v>0</v>
+      </c>
+      <c r="F946" t="n">
+        <v>0</v>
+      </c>
+      <c r="G946" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H946" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="947" ht="15" customHeight="1">
+      <c r="A947" t="inlineStr">
+        <is>
+          <t>2026-07-03 11:33 UTC</t>
+        </is>
+      </c>
+      <c r="B947" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C947" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D947" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E947" t="n">
+        <v>0</v>
+      </c>
+      <c r="F947" t="n">
+        <v>0</v>
+      </c>
+      <c r="G947" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H947" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="948" ht="15" customHeight="1">
+      <c r="A948" t="inlineStr">
+        <is>
+          <t>2026-07-03 11:33 UTC</t>
+        </is>
+      </c>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C948" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D948" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E948" t="n">
+        <v>0</v>
+      </c>
+      <c r="F948" t="n">
+        <v>0</v>
+      </c>
+      <c r="G948" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H948" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="949" ht="15" customHeight="1">
+      <c r="A949" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03 11:33 UTC</t>
+        </is>
+      </c>
+      <c r="B949" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C949" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D949" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E949" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F949" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G949" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/54404.31e08a854d0fd4374ce8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.12a01112c8c4cad48368.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.f2f80bd523e1af625c43.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.744fb21b30974ce01948.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.77904bdf86d88439d913.js"&gt;&lt;/script&gt;&lt;link href="/style/css/54404.84820f13883e452f12ae.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.fabd73c4415a302aef05.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H949" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.94520e97b52408272a94.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.54b3b755601bffb8d823.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/57207.0b85d3b8da354f298333.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.db1b797cc6e6192822f2.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/57207.61390cb7d67d935e7d20.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.fabd73c4415a302aef05.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="950" ht="15" customHeight="1">
+      <c r="A950" t="inlineStr">
+        <is>
+          <t>2026-07-03 11:33 UTC</t>
+        </is>
+      </c>
+      <c r="B950" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C950" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D950" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E950" t="n">
+        <v>0</v>
+      </c>
+      <c r="F950" t="n">
+        <v>0</v>
+      </c>
+      <c r="G950" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H950" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="951" ht="15" customHeight="1">
+      <c r="A951" t="inlineStr">
+        <is>
+          <t>2026-07-03 11:33 UTC</t>
+        </is>
+      </c>
+      <c r="B951" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C951" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D951" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E951" t="n">
+        <v>0</v>
+      </c>
+      <c r="F951" t="n">
+        <v>0</v>
+      </c>
+      <c r="G951" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H951" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -38114,7 +38494,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-07-02 11:34 UTC</t>
+          <t>2026-07-03 11:33 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -38139,7 +38519,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-07-02 11:34 UTC</t>
+          <t>2026-07-03 11:33 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -38164,7 +38544,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-07-02 11:34 UTC</t>
+          <t>2026-07-03 11:33 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -38189,7 +38569,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-07-02 11:34 UTC</t>
+          <t>2026-07-03 11:33 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -38214,7 +38594,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-07-02 11:34 UTC</t>
+          <t>2026-07-03 11:33 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -38239,7 +38619,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-07-02 11:34 UTC</t>
+          <t>2026-07-03 11:33 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -38264,7 +38644,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-02 11:34 UTC</t>
+          <t>2026-07-03 11:33 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -38289,7 +38669,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-07-02 11:34 UTC</t>
+          <t>2026-07-03 11:33 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -38314,7 +38694,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-07-02 11:34 UTC</t>
+          <t>2026-07-03 11:33 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -38339,7 +38719,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-07-02 11:34 UTC</t>
+          <t>2026-07-03 11:33 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -38400,7 +38780,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.94520e97b52408272a94.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.54b3b755601bffb8d823.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/57207.0b85d3b8da354f298333.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.db1b797cc6e6192822f2.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/57207.61390cb7d67d935e7d20.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.fabd73c4415a302aef05.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/54404.31e08a854d0fd4374ce8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.12a01112c8c4cad48368.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.f2f80bd523e1af625c43.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.744fb21b30974ce01948.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.77904bdf86d88439d913.js"&gt;&lt;/script&gt;&lt;link href="/style/css/54404.84820f13883e452f12ae.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.fabd73c4415a302aef05.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -38417,7 +38797,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.94520e97b52408272a94.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.54b3b755601bffb8d823.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/57207.a570470b3d8f23de0626.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.fec4a7350f714d70d4f5.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/57207.61390cb7d67d935e7d20.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.f70f4a8131c9282b753c.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.94520e97b52408272a94.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.54b3b755601bffb8d823.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/57207.0b85d3b8da354f298333.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.db1b797cc6e6192822f2.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/57207.61390cb7d67d935e7d20.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.fabd73c4415a302aef05.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-07-04
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H951"/>
+  <dimension ref="A1:H961"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -37049,6 +37049,386 @@
         </is>
       </c>
       <c r="H951" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="952" ht="15" customHeight="1">
+      <c r="A952" t="inlineStr">
+        <is>
+          <t>2026-07-04 10:54 UTC</t>
+        </is>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D952" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E952" t="n">
+        <v>0</v>
+      </c>
+      <c r="F952" t="n">
+        <v>0</v>
+      </c>
+      <c r="G952" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H952" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="953" ht="15" customHeight="1">
+      <c r="A953" t="inlineStr">
+        <is>
+          <t>2026-07-04 10:54 UTC</t>
+        </is>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D953" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E953" t="n">
+        <v>0</v>
+      </c>
+      <c r="F953" t="n">
+        <v>0</v>
+      </c>
+      <c r="G953" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H953" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="954" ht="15" customHeight="1">
+      <c r="A954" t="inlineStr">
+        <is>
+          <t>2026-07-04 10:54 UTC</t>
+        </is>
+      </c>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D954" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E954" t="n">
+        <v>0</v>
+      </c>
+      <c r="F954" t="n">
+        <v>0</v>
+      </c>
+      <c r="G954" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H954" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="955" ht="15" customHeight="1">
+      <c r="A955" t="inlineStr">
+        <is>
+          <t>2026-07-04 10:54 UTC</t>
+        </is>
+      </c>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D955" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E955" t="n">
+        <v>0</v>
+      </c>
+      <c r="F955" t="n">
+        <v>0</v>
+      </c>
+      <c r="G955" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H955" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="956" ht="15" customHeight="1">
+      <c r="A956" t="inlineStr">
+        <is>
+          <t>2026-07-04 10:54 UTC</t>
+        </is>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C956" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D956" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E956" t="n">
+        <v>0</v>
+      </c>
+      <c r="F956" t="n">
+        <v>0</v>
+      </c>
+      <c r="G956" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H956" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="957" ht="15" customHeight="1">
+      <c r="A957" t="inlineStr">
+        <is>
+          <t>2026-07-04 10:54 UTC</t>
+        </is>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C957" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D957" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E957" t="n">
+        <v>0</v>
+      </c>
+      <c r="F957" t="n">
+        <v>0</v>
+      </c>
+      <c r="G957" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H957" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="958" ht="15" customHeight="1">
+      <c r="A958" t="inlineStr">
+        <is>
+          <t>2026-07-04 10:54 UTC</t>
+        </is>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D958" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E958" t="n">
+        <v>0</v>
+      </c>
+      <c r="F958" t="n">
+        <v>0</v>
+      </c>
+      <c r="G958" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H958" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="959" ht="15" customHeight="1">
+      <c r="A959" t="inlineStr">
+        <is>
+          <t>2026-07-04 10:54 UTC</t>
+        </is>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D959" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E959" t="n">
+        <v>0</v>
+      </c>
+      <c r="F959" t="n">
+        <v>0</v>
+      </c>
+      <c r="G959" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H959" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="960" ht="15" customHeight="1">
+      <c r="A960" t="inlineStr">
+        <is>
+          <t>2026-07-04 10:54 UTC</t>
+        </is>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D960" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E960" t="n">
+        <v>0</v>
+      </c>
+      <c r="F960" t="n">
+        <v>0</v>
+      </c>
+      <c r="G960" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H960" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="961" ht="15" customHeight="1">
+      <c r="A961" t="inlineStr">
+        <is>
+          <t>2026-07-04 10:54 UTC</t>
+        </is>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D961" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E961" t="n">
+        <v>0</v>
+      </c>
+      <c r="F961" t="n">
+        <v>0</v>
+      </c>
+      <c r="G961" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H961" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -38444,6 +38824,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/54404.31e08a854d0fd4374ce8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.12a01112c8c4cad48368.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.f2f80bd523e1af625c43.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.744fb21b30974ce01948.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.77904bdf86d88439d913.js"&gt;&lt;/script&gt;&lt;link href="/style/css/54404.84820f13883e452f12ae.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.fabd73c4415a302aef05.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.94520e97b52408272a94.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.54b3b755601bffb8d823.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/57207.0b85d3b8da354f298333.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.db1b797cc6e6192822f2.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/57207.61390cb7d67d935e7d20.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.fabd73c4415a302aef05.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -38494,7 +38944,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-07-03 11:33 UTC</t>
+          <t>2026-07-04 10:54 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -38519,7 +38969,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-07-03 11:33 UTC</t>
+          <t>2026-07-04 10:54 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -38544,7 +38994,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-07-03 11:33 UTC</t>
+          <t>2026-07-04 10:54 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -38569,7 +39019,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-07-03 11:33 UTC</t>
+          <t>2026-07-04 10:54 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -38594,7 +39044,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-07-03 11:33 UTC</t>
+          <t>2026-07-04 10:54 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -38619,7 +39069,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-07-03 11:33 UTC</t>
+          <t>2026-07-04 10:54 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -38644,7 +39094,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-03 11:33 UTC</t>
+          <t>2026-07-04 10:54 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -38669,7 +39119,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-07-03 11:33 UTC</t>
+          <t>2026-07-04 10:54 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -38694,7 +39144,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-07-03 11:33 UTC</t>
+          <t>2026-07-04 10:54 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -38719,7 +39169,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-07-03 11:33 UTC</t>
+          <t>2026-07-04 10:54 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -38728,76 +39178,6 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/54404.31e08a854d0fd4374ce8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.12a01112c8c4cad48368.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.f2f80bd523e1af625c43.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.744fb21b30974ce01948.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.77904bdf86d88439d913.js"&gt;&lt;/script&gt;&lt;link href="/style/css/54404.84820f13883e452f12ae.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.fabd73c4415a302aef05.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.94520e97b52408272a94.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.54b3b755601bffb8d823.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/57207.0b85d3b8da354f298333.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.db1b797cc6e6192822f2.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/57207.61390cb7d67d935e7d20.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.fabd73c4415a302aef05.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-07-05
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H961"/>
+  <dimension ref="A1:H971"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -37429,6 +37429,386 @@
         </is>
       </c>
       <c r="H961" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="962" ht="15" customHeight="1">
+      <c r="A962" t="inlineStr">
+        <is>
+          <t>2026-07-05 11:04 UTC</t>
+        </is>
+      </c>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C962" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D962" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E962" t="n">
+        <v>0</v>
+      </c>
+      <c r="F962" t="n">
+        <v>0</v>
+      </c>
+      <c r="G962" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H962" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="963" ht="15" customHeight="1">
+      <c r="A963" t="inlineStr">
+        <is>
+          <t>2026-07-05 11:04 UTC</t>
+        </is>
+      </c>
+      <c r="B963" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C963" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D963" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E963" t="n">
+        <v>0</v>
+      </c>
+      <c r="F963" t="n">
+        <v>0</v>
+      </c>
+      <c r="G963" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H963" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="964" ht="15" customHeight="1">
+      <c r="A964" t="inlineStr">
+        <is>
+          <t>2026-07-05 11:04 UTC</t>
+        </is>
+      </c>
+      <c r="B964" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C964" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D964" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E964" t="n">
+        <v>0</v>
+      </c>
+      <c r="F964" t="n">
+        <v>0</v>
+      </c>
+      <c r="G964" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H964" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="965" ht="15" customHeight="1">
+      <c r="A965" t="inlineStr">
+        <is>
+          <t>2026-07-05 11:04 UTC</t>
+        </is>
+      </c>
+      <c r="B965" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C965" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D965" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E965" t="n">
+        <v>0</v>
+      </c>
+      <c r="F965" t="n">
+        <v>0</v>
+      </c>
+      <c r="G965" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H965" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="966" ht="15" customHeight="1">
+      <c r="A966" t="inlineStr">
+        <is>
+          <t>2026-07-05 11:04 UTC</t>
+        </is>
+      </c>
+      <c r="B966" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C966" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D966" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E966" t="n">
+        <v>0</v>
+      </c>
+      <c r="F966" t="n">
+        <v>0</v>
+      </c>
+      <c r="G966" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H966" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="967" ht="15" customHeight="1">
+      <c r="A967" t="inlineStr">
+        <is>
+          <t>2026-07-05 11:04 UTC</t>
+        </is>
+      </c>
+      <c r="B967" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C967" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D967" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E967" t="n">
+        <v>0</v>
+      </c>
+      <c r="F967" t="n">
+        <v>0</v>
+      </c>
+      <c r="G967" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H967" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="968" ht="15" customHeight="1">
+      <c r="A968" t="inlineStr">
+        <is>
+          <t>2026-07-05 11:04 UTC</t>
+        </is>
+      </c>
+      <c r="B968" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C968" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D968" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E968" t="n">
+        <v>0</v>
+      </c>
+      <c r="F968" t="n">
+        <v>0</v>
+      </c>
+      <c r="G968" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H968" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="969" ht="15" customHeight="1">
+      <c r="A969" t="inlineStr">
+        <is>
+          <t>2026-07-05 11:04 UTC</t>
+        </is>
+      </c>
+      <c r="B969" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C969" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D969" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E969" t="n">
+        <v>0</v>
+      </c>
+      <c r="F969" t="n">
+        <v>0</v>
+      </c>
+      <c r="G969" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H969" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="970" ht="15" customHeight="1">
+      <c r="A970" t="inlineStr">
+        <is>
+          <t>2026-07-05 11:04 UTC</t>
+        </is>
+      </c>
+      <c r="B970" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C970" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D970" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E970" t="n">
+        <v>0</v>
+      </c>
+      <c r="F970" t="n">
+        <v>0</v>
+      </c>
+      <c r="G970" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H970" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="971" ht="15" customHeight="1">
+      <c r="A971" t="inlineStr">
+        <is>
+          <t>2026-07-05 11:04 UTC</t>
+        </is>
+      </c>
+      <c r="B971" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C971" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D971" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E971" t="n">
+        <v>0</v>
+      </c>
+      <c r="F971" t="n">
+        <v>0</v>
+      </c>
+      <c r="G971" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H971" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -38944,7 +39324,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-07-04 10:54 UTC</t>
+          <t>2026-07-05 11:04 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -38969,7 +39349,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-07-04 10:54 UTC</t>
+          <t>2026-07-05 11:04 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -38994,7 +39374,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-07-04 10:54 UTC</t>
+          <t>2026-07-05 11:04 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -39019,7 +39399,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-07-04 10:54 UTC</t>
+          <t>2026-07-05 11:04 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -39044,7 +39424,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-07-04 10:54 UTC</t>
+          <t>2026-07-05 11:04 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -39069,7 +39449,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-07-04 10:54 UTC</t>
+          <t>2026-07-05 11:04 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -39094,7 +39474,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-04 10:54 UTC</t>
+          <t>2026-07-05 11:04 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -39119,7 +39499,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-07-04 10:54 UTC</t>
+          <t>2026-07-05 11:04 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -39144,7 +39524,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-07-04 10:54 UTC</t>
+          <t>2026-07-05 11:04 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -39169,7 +39549,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-07-04 10:54 UTC</t>
+          <t>2026-07-05 11:04 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">

</xml_diff>

<commit_message>
chore: update snapshots 2026-07-06
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -17,8 +17,8 @@
     <sheet name="sundancetv_com_ads_txt" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="wetv_com_ads_txt" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="wetv_com_app-ads_txt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="sundancetv_com_app-ads_txt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Current Snapshot" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Current Snapshot" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="sundancetv_com_app-ads_txt" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H971"/>
+  <dimension ref="A1:H981"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -37809,6 +37809,386 @@
         </is>
       </c>
       <c r="H971" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="972" ht="15" customHeight="1">
+      <c r="A972" t="inlineStr">
+        <is>
+          <t>2026-07-06 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="B972" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C972" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D972" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E972" t="n">
+        <v>0</v>
+      </c>
+      <c r="F972" t="n">
+        <v>0</v>
+      </c>
+      <c r="G972" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H972" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="973" ht="15" customHeight="1">
+      <c r="A973" t="inlineStr">
+        <is>
+          <t>2026-07-06 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="B973" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C973" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D973" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E973" t="n">
+        <v>0</v>
+      </c>
+      <c r="F973" t="n">
+        <v>0</v>
+      </c>
+      <c r="G973" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H973" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="974" ht="15" customHeight="1">
+      <c r="A974" t="inlineStr">
+        <is>
+          <t>2026-07-06 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="B974" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C974" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D974" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E974" t="n">
+        <v>0</v>
+      </c>
+      <c r="F974" t="n">
+        <v>0</v>
+      </c>
+      <c r="G974" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H974" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="975" ht="15" customHeight="1">
+      <c r="A975" t="inlineStr">
+        <is>
+          <t>2026-07-06 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="B975" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C975" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D975" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E975" t="n">
+        <v>0</v>
+      </c>
+      <c r="F975" t="n">
+        <v>0</v>
+      </c>
+      <c r="G975" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H975" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="976" ht="15" customHeight="1">
+      <c r="A976" t="inlineStr">
+        <is>
+          <t>2026-07-06 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="B976" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C976" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D976" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E976" t="n">
+        <v>0</v>
+      </c>
+      <c r="F976" t="n">
+        <v>0</v>
+      </c>
+      <c r="G976" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H976" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="977" ht="15" customHeight="1">
+      <c r="A977" t="inlineStr">
+        <is>
+          <t>2026-07-06 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="B977" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C977" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D977" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E977" t="n">
+        <v>0</v>
+      </c>
+      <c r="F977" t="n">
+        <v>0</v>
+      </c>
+      <c r="G977" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H977" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="978" ht="15" customHeight="1">
+      <c r="A978" t="inlineStr">
+        <is>
+          <t>2026-07-06 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="B978" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C978" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D978" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E978" t="n">
+        <v>0</v>
+      </c>
+      <c r="F978" t="n">
+        <v>0</v>
+      </c>
+      <c r="G978" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H978" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="979" ht="15" customHeight="1">
+      <c r="A979" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="B979" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C979" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D979" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E979" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F979" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G979" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/54404.31e08a854d0fd4374ce8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.12a01112c8c4cad48368.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.f2f80bd523e1af625c43.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.744fb21b30974ce01948.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.27b030127caafe68e26e.js"&gt;&lt;/script&gt;&lt;link href="/style/css/54404.84820f13883e452f12ae.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.fabd73c4415a302aef05.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H979" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/54404.31e08a854d0fd4374ce8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.12a01112c8c4cad48368.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.f2f80bd523e1af625c43.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.744fb21b30974ce01948.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.77904bdf86d88439d913.js"&gt;&lt;/script&gt;&lt;link href="/style/css/54404.84820f13883e452f12ae.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.fabd73c4415a302aef05.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="980" ht="15" customHeight="1">
+      <c r="A980" t="inlineStr">
+        <is>
+          <t>2026-07-06 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="B980" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C980" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D980" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E980" t="n">
+        <v>0</v>
+      </c>
+      <c r="F980" t="n">
+        <v>0</v>
+      </c>
+      <c r="G980" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H980" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="981" ht="15" customHeight="1">
+      <c r="A981" t="inlineStr">
+        <is>
+          <t>2026-07-06 12:48 UTC</t>
+        </is>
+      </c>
+      <c r="B981" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C981" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D981" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E981" t="n">
+        <v>0</v>
+      </c>
+      <c r="F981" t="n">
+        <v>0</v>
+      </c>
+      <c r="G981" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H981" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -39204,76 +39584,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="80" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Section</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Line Content</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>+ Added</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/54404.31e08a854d0fd4374ce8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.12a01112c8c4cad48368.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.f2f80bd523e1af625c43.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.744fb21b30974ce01948.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.77904bdf86d88439d913.js"&gt;&lt;/script&gt;&lt;link href="/style/css/54404.84820f13883e452f12ae.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.fabd73c4415a302aef05.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>- Removed</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>(no section)</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/21799.dbbd0158a95cfab6d144.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.94520e97b52408272a94.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.35943f481f84f787f1e1.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.54b3b755601bffb8d823.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/57207.0b85d3b8da354f298333.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.db1b797cc6e6192822f2.js"&gt;&lt;/script&gt;&lt;link href="/style/css/21799.c3cfa9a841b5a9a3f7ab.css" rel="stylesheet"&gt;&lt;link href="/style/css/57207.61390cb7d67d935e7d20.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.fabd73c4415a302aef05.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -39324,7 +39634,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-07-05 11:04 UTC</t>
+          <t>2026-07-06 12:48 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -39349,7 +39659,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-07-05 11:04 UTC</t>
+          <t>2026-07-06 12:48 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -39374,7 +39684,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-07-05 11:04 UTC</t>
+          <t>2026-07-06 12:48 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -39399,7 +39709,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-07-05 11:04 UTC</t>
+          <t>2026-07-06 12:48 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -39424,7 +39734,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-07-05 11:04 UTC</t>
+          <t>2026-07-06 12:48 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -39449,7 +39759,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-07-05 11:04 UTC</t>
+          <t>2026-07-06 12:48 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -39474,7 +39784,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-05 11:04 UTC</t>
+          <t>2026-07-06 12:48 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -39499,7 +39809,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-07-05 11:04 UTC</t>
+          <t>2026-07-06 12:48 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -39524,7 +39834,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-07-05 11:04 UTC</t>
+          <t>2026-07-06 12:48 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -39549,7 +39859,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-07-05 11:04 UTC</t>
+          <t>2026-07-06 12:48 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -39558,6 +39868,76 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>OK</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Line Content</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>+ Added</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/54404.31e08a854d0fd4374ce8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.12a01112c8c4cad48368.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.f2f80bd523e1af625c43.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.744fb21b30974ce01948.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.27b030127caafe68e26e.js"&gt;&lt;/script&gt;&lt;link href="/style/css/54404.84820f13883e452f12ae.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.fabd73c4415a302aef05.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>- Removed</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>(no section)</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/54404.31e08a854d0fd4374ce8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.12a01112c8c4cad48368.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.f2f80bd523e1af625c43.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.744fb21b30974ce01948.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.77904bdf86d88439d913.js"&gt;&lt;/script&gt;&lt;link href="/style/css/54404.84820f13883e452f12ae.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.fabd73c4415a302aef05.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-07-07
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H981"/>
+  <dimension ref="A1:H991"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -38189,6 +38189,386 @@
         </is>
       </c>
       <c r="H981" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="982" ht="15" customHeight="1">
+      <c r="A982" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:51 UTC</t>
+        </is>
+      </c>
+      <c r="B982" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C982" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D982" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E982" t="n">
+        <v>0</v>
+      </c>
+      <c r="F982" t="n">
+        <v>0</v>
+      </c>
+      <c r="G982" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H982" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="983" ht="15" customHeight="1">
+      <c r="A983" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:51 UTC</t>
+        </is>
+      </c>
+      <c r="B983" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C983" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D983" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E983" t="n">
+        <v>0</v>
+      </c>
+      <c r="F983" t="n">
+        <v>0</v>
+      </c>
+      <c r="G983" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H983" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="984" ht="15" customHeight="1">
+      <c r="A984" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:51 UTC</t>
+        </is>
+      </c>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C984" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D984" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E984" t="n">
+        <v>0</v>
+      </c>
+      <c r="F984" t="n">
+        <v>0</v>
+      </c>
+      <c r="G984" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H984" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="985" ht="15" customHeight="1">
+      <c r="A985" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:51 UTC</t>
+        </is>
+      </c>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C985" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D985" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E985" t="n">
+        <v>0</v>
+      </c>
+      <c r="F985" t="n">
+        <v>0</v>
+      </c>
+      <c r="G985" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H985" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="986" ht="15" customHeight="1">
+      <c r="A986" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:51 UTC</t>
+        </is>
+      </c>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C986" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D986" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E986" t="n">
+        <v>0</v>
+      </c>
+      <c r="F986" t="n">
+        <v>0</v>
+      </c>
+      <c r="G986" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H986" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="987" ht="15" customHeight="1">
+      <c r="A987" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:51 UTC</t>
+        </is>
+      </c>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C987" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D987" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E987" t="n">
+        <v>0</v>
+      </c>
+      <c r="F987" t="n">
+        <v>0</v>
+      </c>
+      <c r="G987" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H987" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="988" ht="15" customHeight="1">
+      <c r="A988" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:51 UTC</t>
+        </is>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D988" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E988" t="n">
+        <v>0</v>
+      </c>
+      <c r="F988" t="n">
+        <v>0</v>
+      </c>
+      <c r="G988" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H988" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="989" ht="15" customHeight="1">
+      <c r="A989" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:51 UTC</t>
+        </is>
+      </c>
+      <c r="B989" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C989" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D989" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E989" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F989" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G989" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.1bbd04b5ea4f62a1b99d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/13478.c46563973d037c413983.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.b7dc1428d87f14ef4c0a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.1781af8f883e4e880fe8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.195b800435d996383cbe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.6dd4217276b7c80eb4c4.js"&gt;&lt;/script&gt;&lt;link href="/style/css/13478.b6c6e17ee03ac36e3ac5.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.6757f72f185cd2fa2433.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H989" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/54404.31e08a854d0fd4374ce8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.12a01112c8c4cad48368.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.f2f80bd523e1af625c43.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.744fb21b30974ce01948.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.27b030127caafe68e26e.js"&gt;&lt;/script&gt;&lt;link href="/style/css/54404.84820f13883e452f12ae.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.fabd73c4415a302aef05.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="990" ht="15" customHeight="1">
+      <c r="A990" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:51 UTC</t>
+        </is>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C990" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D990" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E990" t="n">
+        <v>0</v>
+      </c>
+      <c r="F990" t="n">
+        <v>0</v>
+      </c>
+      <c r="G990" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H990" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="991" ht="15" customHeight="1">
+      <c r="A991" t="inlineStr">
+        <is>
+          <t>2026-07-07 11:51 UTC</t>
+        </is>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C991" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D991" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E991" t="n">
+        <v>0</v>
+      </c>
+      <c r="F991" t="n">
+        <v>0</v>
+      </c>
+      <c r="G991" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H991" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -39634,7 +40014,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-07-06 12:48 UTC</t>
+          <t>2026-07-07 11:51 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -39659,7 +40039,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-07-06 12:48 UTC</t>
+          <t>2026-07-07 11:51 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -39684,7 +40064,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-07-06 12:48 UTC</t>
+          <t>2026-07-07 11:51 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -39709,7 +40089,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-07-06 12:48 UTC</t>
+          <t>2026-07-07 11:51 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -39734,7 +40114,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-07-06 12:48 UTC</t>
+          <t>2026-07-07 11:51 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -39759,7 +40139,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-07-06 12:48 UTC</t>
+          <t>2026-07-07 11:51 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -39784,7 +40164,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-06 12:48 UTC</t>
+          <t>2026-07-07 11:51 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -39809,7 +40189,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-07-06 12:48 UTC</t>
+          <t>2026-07-07 11:51 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -39834,7 +40214,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-07-06 12:48 UTC</t>
+          <t>2026-07-07 11:51 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -39859,7 +40239,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-07-06 12:48 UTC</t>
+          <t>2026-07-07 11:51 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -39920,7 +40300,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/54404.31e08a854d0fd4374ce8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.12a01112c8c4cad48368.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.f2f80bd523e1af625c43.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.744fb21b30974ce01948.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.27b030127caafe68e26e.js"&gt;&lt;/script&gt;&lt;link href="/style/css/54404.84820f13883e452f12ae.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.fabd73c4415a302aef05.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.1bbd04b5ea4f62a1b99d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/13478.c46563973d037c413983.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.b7dc1428d87f14ef4c0a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.1781af8f883e4e880fe8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.195b800435d996383cbe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.6dd4217276b7c80eb4c4.js"&gt;&lt;/script&gt;&lt;link href="/style/css/13478.b6c6e17ee03ac36e3ac5.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.6757f72f185cd2fa2433.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -39937,7 +40317,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/54404.31e08a854d0fd4374ce8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.12a01112c8c4cad48368.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.f2f80bd523e1af625c43.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.744fb21b30974ce01948.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.77904bdf86d88439d913.js"&gt;&lt;/script&gt;&lt;link href="/style/css/54404.84820f13883e452f12ae.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.fabd73c4415a302aef05.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/54404.31e08a854d0fd4374ce8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.12a01112c8c4cad48368.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.f2f80bd523e1af625c43.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.744fb21b30974ce01948.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.27b030127caafe68e26e.js"&gt;&lt;/script&gt;&lt;link href="/style/css/54404.84820f13883e452f12ae.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.fabd73c4415a302aef05.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-07-08
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H991"/>
+  <dimension ref="A1:H1001"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -38569,6 +38569,386 @@
         </is>
       </c>
       <c r="H991" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="992" ht="15" customHeight="1">
+      <c r="A992" t="inlineStr">
+        <is>
+          <t>2026-07-08 11:05 UTC</t>
+        </is>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C992" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D992" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E992" t="n">
+        <v>0</v>
+      </c>
+      <c r="F992" t="n">
+        <v>0</v>
+      </c>
+      <c r="G992" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H992" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="993" ht="15" customHeight="1">
+      <c r="A993" t="inlineStr">
+        <is>
+          <t>2026-07-08 11:05 UTC</t>
+        </is>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D993" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E993" t="n">
+        <v>0</v>
+      </c>
+      <c r="F993" t="n">
+        <v>0</v>
+      </c>
+      <c r="G993" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H993" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="994" ht="15" customHeight="1">
+      <c r="A994" t="inlineStr">
+        <is>
+          <t>2026-07-08 11:05 UTC</t>
+        </is>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C994" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D994" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E994" t="n">
+        <v>0</v>
+      </c>
+      <c r="F994" t="n">
+        <v>0</v>
+      </c>
+      <c r="G994" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H994" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="995" ht="15" customHeight="1">
+      <c r="A995" t="inlineStr">
+        <is>
+          <t>2026-07-08 11:05 UTC</t>
+        </is>
+      </c>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C995" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D995" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E995" t="n">
+        <v>0</v>
+      </c>
+      <c r="F995" t="n">
+        <v>0</v>
+      </c>
+      <c r="G995" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H995" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="996" ht="15" customHeight="1">
+      <c r="A996" t="inlineStr">
+        <is>
+          <t>2026-07-08 11:05 UTC</t>
+        </is>
+      </c>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C996" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D996" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E996" t="n">
+        <v>0</v>
+      </c>
+      <c r="F996" t="n">
+        <v>0</v>
+      </c>
+      <c r="G996" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H996" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="997" ht="15" customHeight="1">
+      <c r="A997" t="inlineStr">
+        <is>
+          <t>2026-07-08 11:05 UTC</t>
+        </is>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D997" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E997" t="n">
+        <v>0</v>
+      </c>
+      <c r="F997" t="n">
+        <v>0</v>
+      </c>
+      <c r="G997" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H997" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="998" ht="15" customHeight="1">
+      <c r="A998" t="inlineStr">
+        <is>
+          <t>2026-07-08 11:05 UTC</t>
+        </is>
+      </c>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C998" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D998" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E998" t="n">
+        <v>0</v>
+      </c>
+      <c r="F998" t="n">
+        <v>0</v>
+      </c>
+      <c r="G998" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H998" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="999" ht="15" customHeight="1">
+      <c r="A999" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08 11:05 UTC</t>
+        </is>
+      </c>
+      <c r="B999" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C999" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D999" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E999" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F999" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G999" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.1bbd04b5ea4f62a1b99d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/13478.112588974a8433af0e8f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.b7dc1428d87f14ef4c0a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.85f74134e8460f2fe12a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.35e30a3bca70b8ad5ec9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d9b0d546ab6083bcecc9.js"&gt;&lt;/script&gt;&lt;link href="/style/css/13478.b6c6e17ee03ac36e3ac5.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.6757f72f185cd2fa2433.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H999" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.1bbd04b5ea4f62a1b99d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/13478.c46563973d037c413983.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.b7dc1428d87f14ef4c0a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.1781af8f883e4e880fe8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.195b800435d996383cbe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.6dd4217276b7c80eb4c4.js"&gt;&lt;/script&gt;&lt;link href="/style/css/13478.b6c6e17ee03ac36e3ac5.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.6757f72f185cd2fa2433.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000" ht="15" customHeight="1">
+      <c r="A1000" t="inlineStr">
+        <is>
+          <t>2026-07-08 11:05 UTC</t>
+        </is>
+      </c>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1000" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1000" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1000" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1000" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1000" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1000" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001" ht="15" customHeight="1">
+      <c r="A1001" t="inlineStr">
+        <is>
+          <t>2026-07-08 11:05 UTC</t>
+        </is>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1001" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1001" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1001" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1001" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1001" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1001" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -40014,7 +40394,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-07-07 11:51 UTC</t>
+          <t>2026-07-08 11:05 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -40039,7 +40419,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-07-07 11:51 UTC</t>
+          <t>2026-07-08 11:05 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -40064,7 +40444,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-07-07 11:51 UTC</t>
+          <t>2026-07-08 11:05 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -40089,7 +40469,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-07-07 11:51 UTC</t>
+          <t>2026-07-08 11:05 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -40114,7 +40494,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-07-07 11:51 UTC</t>
+          <t>2026-07-08 11:05 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -40139,7 +40519,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-07-07 11:51 UTC</t>
+          <t>2026-07-08 11:05 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -40164,7 +40544,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-07 11:51 UTC</t>
+          <t>2026-07-08 11:05 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -40189,7 +40569,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-07-07 11:51 UTC</t>
+          <t>2026-07-08 11:05 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -40214,7 +40594,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-07-07 11:51 UTC</t>
+          <t>2026-07-08 11:05 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -40239,7 +40619,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-07-07 11:51 UTC</t>
+          <t>2026-07-08 11:05 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -40300,7 +40680,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.1bbd04b5ea4f62a1b99d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/13478.c46563973d037c413983.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.b7dc1428d87f14ef4c0a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.1781af8f883e4e880fe8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.195b800435d996383cbe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.6dd4217276b7c80eb4c4.js"&gt;&lt;/script&gt;&lt;link href="/style/css/13478.b6c6e17ee03ac36e3ac5.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.6757f72f185cd2fa2433.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.1bbd04b5ea4f62a1b99d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/13478.112588974a8433af0e8f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.b7dc1428d87f14ef4c0a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.85f74134e8460f2fe12a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.35e30a3bca70b8ad5ec9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d9b0d546ab6083bcecc9.js"&gt;&lt;/script&gt;&lt;link href="/style/css/13478.b6c6e17ee03ac36e3ac5.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.6757f72f185cd2fa2433.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -40317,7 +40697,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.55fd796c6c730af82dc0.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.c1299cc7c25b845c595b.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/54404.31e08a854d0fd4374ce8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.12a01112c8c4cad48368.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.f2f80bd523e1af625c43.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.744fb21b30974ce01948.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.27b030127caafe68e26e.js"&gt;&lt;/script&gt;&lt;link href="/style/css/54404.84820f13883e452f12ae.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.fabd73c4415a302aef05.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.1bbd04b5ea4f62a1b99d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/13478.c46563973d037c413983.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.b7dc1428d87f14ef4c0a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.1781af8f883e4e880fe8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.195b800435d996383cbe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.6dd4217276b7c80eb4c4.js"&gt;&lt;/script&gt;&lt;link href="/style/css/13478.b6c6e17ee03ac36e3ac5.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.6757f72f185cd2fa2433.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-07-09
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1001"/>
+  <dimension ref="A1:H1011"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -38949,6 +38949,386 @@
         </is>
       </c>
       <c r="H1001" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002" ht="15" customHeight="1">
+      <c r="A1002" t="inlineStr">
+        <is>
+          <t>2026-07-09 12:01 UTC</t>
+        </is>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1002" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1002" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1002" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1002" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1002" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1002" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003" ht="15" customHeight="1">
+      <c r="A1003" t="inlineStr">
+        <is>
+          <t>2026-07-09 12:01 UTC</t>
+        </is>
+      </c>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1003" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1003" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1003" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1003" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1003" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1003" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004" ht="15" customHeight="1">
+      <c r="A1004" t="inlineStr">
+        <is>
+          <t>2026-07-09 12:01 UTC</t>
+        </is>
+      </c>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1004" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1004" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1004" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1004" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1004" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1004" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1005" ht="15" customHeight="1">
+      <c r="A1005" t="inlineStr">
+        <is>
+          <t>2026-07-09 12:01 UTC</t>
+        </is>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1005" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1005" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1005" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1005" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1005" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1005" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006" ht="15" customHeight="1">
+      <c r="A1006" t="inlineStr">
+        <is>
+          <t>2026-07-09 12:01 UTC</t>
+        </is>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1006" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1006" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1006" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1006" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1006" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1007" ht="15" customHeight="1">
+      <c r="A1007" t="inlineStr">
+        <is>
+          <t>2026-07-09 12:01 UTC</t>
+        </is>
+      </c>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1007" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1007" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1007" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1007" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1007" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1007" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1008" ht="15" customHeight="1">
+      <c r="A1008" t="inlineStr">
+        <is>
+          <t>2026-07-09 12:01 UTC</t>
+        </is>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1008" t="inlineStr">
+        <is>
+          <t>sundancetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1008" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1008" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1008" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1008" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1008" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009" ht="15" customHeight="1">
+      <c r="A1009" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09 12:01 UTC</t>
+        </is>
+      </c>
+      <c r="B1009" s="3" t="inlineStr">
+        <is>
+          <t>Sundance TV</t>
+        </is>
+      </c>
+      <c r="C1009" s="3" t="inlineStr">
+        <is>
+          <t>sundancetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1009" s="3" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="E1009" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1009" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1009" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.1bbd04b5ea4f62a1b99d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/13478.112588974a8433af0e8f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.b7dc1428d87f14ef4c0a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.eeda2b038ad004d40dc6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.35e30a3bca70b8ad5ec9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.42203ec020d4388e4c5f.js"&gt;&lt;/script&gt;&lt;link href="/style/css/13478.b6c6e17ee03ac36e3ac5.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.6757f72f185cd2fa2433.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+      <c r="H1009" s="3" t="inlineStr">
+        <is>
+          <t>(no section): document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.1bbd04b5ea4f62a1b99d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/13478.112588974a8433af0e8f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.b7dc1428d87f14ef4c0a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.85f74134e8460f2fe12a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.35e30a3bca70b8ad5ec9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d9b0d546ab6083bcecc9.js"&gt;&lt;/script&gt;&lt;link href="/style/css/13478.b6c6e17ee03ac36e3ac5.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.6757f72f185cd2fa2433.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010" ht="15" customHeight="1">
+      <c r="A1010" t="inlineStr">
+        <is>
+          <t>2026-07-09 12:01 UTC</t>
+        </is>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1010" t="inlineStr">
+        <is>
+          <t>wetv.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1010" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1010" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1010" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1010" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1010" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011" ht="15" customHeight="1">
+      <c r="A1011" t="inlineStr">
+        <is>
+          <t>2026-07-09 12:01 UTC</t>
+        </is>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>WE tv</t>
+        </is>
+      </c>
+      <c r="C1011" t="inlineStr">
+        <is>
+          <t>wetv.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1011" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1011" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1011" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1011" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1011" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -40394,7 +40774,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-07-08 11:05 UTC</t>
+          <t>2026-07-09 12:01 UTC</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -40419,7 +40799,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-07-08 11:05 UTC</t>
+          <t>2026-07-09 12:01 UTC</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -40444,7 +40824,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-07-08 11:05 UTC</t>
+          <t>2026-07-09 12:01 UTC</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -40469,7 +40849,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-07-08 11:05 UTC</t>
+          <t>2026-07-09 12:01 UTC</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -40494,7 +40874,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-07-08 11:05 UTC</t>
+          <t>2026-07-09 12:01 UTC</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -40519,7 +40899,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-07-08 11:05 UTC</t>
+          <t>2026-07-09 12:01 UTC</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -40544,7 +40924,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07-08 11:05 UTC</t>
+          <t>2026-07-09 12:01 UTC</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -40569,7 +40949,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-07-08 11:05 UTC</t>
+          <t>2026-07-09 12:01 UTC</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -40594,7 +40974,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-07-08 11:05 UTC</t>
+          <t>2026-07-09 12:01 UTC</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -40619,7 +40999,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-07-08 11:05 UTC</t>
+          <t>2026-07-09 12:01 UTC</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -40680,7 +41060,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.1bbd04b5ea4f62a1b99d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/13478.112588974a8433af0e8f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.b7dc1428d87f14ef4c0a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.85f74134e8460f2fe12a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.35e30a3bca70b8ad5ec9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d9b0d546ab6083bcecc9.js"&gt;&lt;/script&gt;&lt;link href="/style/css/13478.b6c6e17ee03ac36e3ac5.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.6757f72f185cd2fa2433.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.1bbd04b5ea4f62a1b99d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/13478.112588974a8433af0e8f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.b7dc1428d87f14ef4c0a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.eeda2b038ad004d40dc6.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.35e30a3bca70b8ad5ec9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.42203ec020d4388e4c5f.js"&gt;&lt;/script&gt;&lt;link href="/style/css/13478.b6c6e17ee03ac36e3ac5.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.6757f72f185cd2fa2433.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>
@@ -40697,7 +41077,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.1bbd04b5ea4f62a1b99d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/13478.c46563973d037c413983.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.b7dc1428d87f14ef4c0a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.1781af8f883e4e880fe8.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.195b800435d996383cbe.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.6dd4217276b7c80eb4c4.js"&gt;&lt;/script&gt;&lt;link href="/style/css/13478.b6c6e17ee03ac36e3ac5.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.6757f72f185cd2fa2433.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
+          <t>document.head.appendChild(s);&lt;/script&gt;&lt;script defer="defer" src="/code/js/moment.23140bed602335b1278f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/17350.0d34ab3d4bf3536e570f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/48287.2e53575ea85279b62f3a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/10074.1bbd04b5ea4f62a1b99d.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/13478.112588974a8433af0e8f.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/45423.b7dc1428d87f14ef4c0a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/14366.de88e91af1d0d435f65a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/96406.85f74134e8460f2fe12a.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/59402.35e30a3bca70b8ad5ec9.js"&gt;&lt;/script&gt;&lt;script defer="defer" src="/code/js/app.d9b0d546ab6083bcecc9.js"&gt;&lt;/script&gt;&lt;link href="/style/css/13478.b6c6e17ee03ac36e3ac5.css" rel="stylesheet"&gt;&lt;link href="/style/css/59402.e156d0e2f61cc6f3d393.css" rel="stylesheet"&gt;&lt;link href="/style/css/app.6757f72f185cd2fa2433.css" rel="stylesheet"&gt;&lt;/head&gt;&lt;body class="resident-background-color"&gt;&lt;!--[if lt IE 9]&gt;</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update snapshots 2026-07-10
</commit_message>
<xml_diff>
--- a/adstxt_changes.xlsx
+++ b/adstxt_changes.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1011"/>
+  <dimension ref="A1:H1021"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -39329,6 +39329,386 @@
         </is>
       </c>
       <c r="H1011" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012" ht="15" customHeight="1">
+      <c r="A1012" t="inlineStr">
+        <is>
+          <t>2026-07-10 11:52 UTC</t>
+        </is>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>amc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1012" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1012" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1012" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1012" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1012" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013" ht="15" customHeight="1">
+      <c r="A1013" t="inlineStr">
+        <is>
+          <t>2026-07-10 11:52 UTC</t>
+        </is>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>AMC Networks</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>amc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1013" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1013" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1013" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1013" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1013" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014" ht="15" customHeight="1">
+      <c r="A1014" t="inlineStr">
+        <is>
+          <t>2026-07-10 11:52 UTC</t>
+        </is>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1014" t="inlineStr">
+        <is>
+          <t>bbca.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1014" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1014" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1014" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1014" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1014" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015" ht="15" customHeight="1">
+      <c r="A1015" t="inlineStr">
+        <is>
+          <t>2026-07-10 11:52 UTC</t>
+        </is>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>BBC America</t>
+        </is>
+      </c>
+      <c r="C1015" t="inlineStr">
+        <is>
+          <t>bbca.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1015" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1015" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1015" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1015" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1015" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016" ht="15" customHeight="1">
+      <c r="A1016" t="inlineStr">
+        <is>
+          <t>2026-07-10 11:52 UTC</t>
+        </is>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1016" t="inlineStr">
+        <is>
+          <t>ifc.com/ads.txt</t>
+        </is>
+      </c>
+      <c r="D1016" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1016" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1016" t="n">
+        <v>0</v>
+      </c>
+      <c r="G1016" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H1016" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017" ht="15" customHeight="1">
+      <c r="A1017" t="inlineStr">
+        <is>
+          <t>2026-07-10 11:52 UTC</t>
+        </is>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>IFC</t>
+        </is>
+      </c>
+      <c r="C1017" t="inlineStr">
+        <is>
+          <t>ifc.com/app-ads.txt</t>
+        </is>
+      </c>
+      <c r="D1017" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+      <c r="E1017" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1017" t="n">
+        <v>0</v